<commit_message>
FBH-Auslegung v0.19 - max. Volumenstrom je Kreis, Anleitung als Schritt-fuer-Schritt, Deckblatt-Pfeile
Grundeinstellungen: neuer Grenzwert 'Maximaler Volumenstrom je Kreis' (V_max, Default 150 l/h); Abschnitt umbenannt zu 'Stroemungsgrenzwerte'.

Auslegung: Volumenstrom je Kreis (AD) wird gegen V_max geprueft und per Ampel eingefaerbt (gruen unter, rot ueber Grenze); zusaetzliche Warnung im Blatt Kontrolle.

Anleitung: durchgehende Schritt-fuer-Schritt-Anleitung mit integriertem Revit-Export (vorgefertigte Bauteilliste muss nicht angelegt werden); redundanter Abschnitt 'Raeume aus Revit' und Hinweis zum direkten Kopieren entfernt; bleibt im Querformat.

Deckblatt: Pfeil-Spalten D/H breiter (6) und Pfeilgroesse 20 - Pfeile nicht mehr zu lang fuer die Spalte.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FBH_Auslegung.xlsx
+++ b/FBH_Auslegung.xlsx
@@ -20,16 +20,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Deckblatt'!$A$1:$K$29</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Anleitung'!$A$1:$D$40</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Anleitung'!$A$1:$D$31</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Grundeinstellungen'!$A$1:$M$25</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Auslegung'!$1:$6</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'Auslegung'!$A$1:$AK$206</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="4">'Kontrolle'!$A$1:$D$24</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'Kontrolle'!$A$1:$D$25</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="5">'HKV'!$A$1:$G$56</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="6">'Verifikation'!$A$1:$Q$26</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">'Methodik'!$A$1:$F$26</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="8">'Konstanten'!$A$1:$I$26</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="9">'Changelog'!$A$1:$C$69</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="9">'Changelog'!$A$1:$C$73</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -37,33 +37,34 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="26">
+  <numFmts count="27">
     <numFmt numFmtId="164" formatCode="0.0&quot; °C&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0&quot; K&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; m&quot;"/>
     <numFmt numFmtId="167" formatCode="#,##0&quot; Pa&quot;"/>
     <numFmt numFmtId="168" formatCode="0.0"/>
     <numFmt numFmtId="169" formatCode="0.00&quot; m/s&quot;"/>
-    <numFmt numFmtId="170" formatCode="0.000"/>
-    <numFmt numFmtId="171" formatCode="0.0&quot; W/m²&quot;"/>
-    <numFmt numFmtId="172" formatCode="0.0&quot; mm&quot;"/>
-    <numFmt numFmtId="173" formatCode="0.000&quot; mm&quot;"/>
-    <numFmt numFmtId="174" formatCode="0.0000&quot; m&quot;"/>
-    <numFmt numFmtId="175" formatCode="0.000000&quot; m²&quot;"/>
-    <numFmt numFmtId="176" formatCode="0.0&quot; m²&quot;"/>
-    <numFmt numFmtId="177" formatCode="#,##0&quot; W&quot;"/>
-    <numFmt numFmtId="178" formatCode="0&quot; mm&quot;"/>
-    <numFmt numFmtId="179" formatCode="0.0&quot; m&quot;"/>
-    <numFmt numFmtId="180" formatCode="0.00&quot; K&quot;"/>
-    <numFmt numFmtId="181" formatCode="0.0%"/>
-    <numFmt numFmtId="182" formatCode="0.0&quot; kg/h&quot;"/>
-    <numFmt numFmtId="183" formatCode="0.0&quot; l/h&quot;"/>
-    <numFmt numFmtId="184" formatCode="0.000&quot; m/s&quot;"/>
-    <numFmt numFmtId="185" formatCode="0.0000"/>
-    <numFmt numFmtId="186" formatCode="#,##0&quot; Pa/m&quot;"/>
-    <numFmt numFmtId="187" formatCode="#,##0&quot; kg/h&quot;"/>
-    <numFmt numFmtId="188" formatCode="#,##0&quot; l/h&quot;"/>
-    <numFmt numFmtId="189" formatCode="0&quot; °C&quot;"/>
+    <numFmt numFmtId="170" formatCode="0&quot; l/h&quot;"/>
+    <numFmt numFmtId="171" formatCode="0.000"/>
+    <numFmt numFmtId="172" formatCode="0.0&quot; W/m²&quot;"/>
+    <numFmt numFmtId="173" formatCode="0.0&quot; mm&quot;"/>
+    <numFmt numFmtId="174" formatCode="0.000&quot; mm&quot;"/>
+    <numFmt numFmtId="175" formatCode="0.0000&quot; m&quot;"/>
+    <numFmt numFmtId="176" formatCode="0.000000&quot; m²&quot;"/>
+    <numFmt numFmtId="177" formatCode="0.0&quot; m²&quot;"/>
+    <numFmt numFmtId="178" formatCode="#,##0&quot; W&quot;"/>
+    <numFmt numFmtId="179" formatCode="0&quot; mm&quot;"/>
+    <numFmt numFmtId="180" formatCode="0.0&quot; m&quot;"/>
+    <numFmt numFmtId="181" formatCode="0.00&quot; K&quot;"/>
+    <numFmt numFmtId="182" formatCode="0.0%"/>
+    <numFmt numFmtId="183" formatCode="0.0&quot; kg/h&quot;"/>
+    <numFmt numFmtId="184" formatCode="0.0&quot; l/h&quot;"/>
+    <numFmt numFmtId="185" formatCode="0.000&quot; m/s&quot;"/>
+    <numFmt numFmtId="186" formatCode="0.0000"/>
+    <numFmt numFmtId="187" formatCode="#,##0&quot; Pa/m&quot;"/>
+    <numFmt numFmtId="188" formatCode="#,##0&quot; kg/h&quot;"/>
+    <numFmt numFmtId="189" formatCode="#,##0&quot; l/h&quot;"/>
+    <numFmt numFmtId="190" formatCode="0&quot; °C&quot;"/>
   </numFmts>
   <fonts count="23">
     <font>
@@ -173,7 +174,7 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00E2001A"/>
-      <sz val="26"/>
+      <sz val="20"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -382,9 +383,6 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
@@ -410,7 +408,7 @@
     <xf numFmtId="168" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="170" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -425,7 +423,7 @@
     <xf numFmtId="167" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="171" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="172" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -434,19 +432,22 @@
     <xf numFmtId="11" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="172" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="173" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="169" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="173" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="174" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="175" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -473,55 +474,52 @@
     <xf numFmtId="0" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="176" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="177" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="177" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="178" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="171" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="172" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="170" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="178" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="179" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="179" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="180" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="180" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="181" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="171" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="172" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="177" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="178" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="182" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="183" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -530,19 +528,22 @@
     <xf numFmtId="184" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="185" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="185" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="186" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="167" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="186" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="187" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -551,10 +552,10 @@
     <xf numFmtId="3" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="181" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="182" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="170" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -566,20 +567,20 @@
     <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="187" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="188" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="188" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="189" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="172" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -598,7 +599,7 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="189" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="190" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="168" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -619,8 +620,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1483,11 +1484,11 @@
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="4" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="4" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
@@ -1884,7 +1885,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C69"/>
+  <dimension ref="A1:C73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1900,9 +1901,9 @@
       </c>
     </row>
     <row r="3">
-      <c r="C3" s="25" t="inlineStr">
-        <is>
-          <t>Version 0.18 · dh</t>
+      <c r="C3" s="24" t="inlineStr">
+        <is>
+          <t>Version 0.19 · dh</t>
         </is>
       </c>
     </row>
@@ -1926,7 +1927,7 @@
     <row r="6">
       <c r="A6" s="102" t="inlineStr">
         <is>
-          <t>0.18</t>
+          <t>0.19</t>
         </is>
       </c>
       <c r="B6" s="103" t="inlineStr">
@@ -1936,7 +1937,7 @@
       </c>
       <c r="C6" s="104" t="inlineStr">
         <is>
-          <t>• Auslegung: Eingabespalten neu sortiert – zuerst die Revit-Spalten (A HKV, B Raum-Nr., C Bezeichnung, D Raumfläche, E Raumtemperatur, F Heizlast), dann G spez. Heizlast (berechnet), danach die manuellen Felder (H aktiv. Fläche, I R-Wert, J Verlegeabstand, K Anz. Kreise, L Zuleitung, M Zone).</t>
+          <t>• Grundeinstellungen: neuer Grenzwert 'Maximaler Volumenstrom je Kreis' (V̇_max, Default 150 l/h); Abschnitt 'Strömungsgeschwindigkeit' → 'Strömungsgrenzwerte'.</t>
         </is>
       </c>
     </row>
@@ -1945,50 +1946,42 @@
       <c r="B7" s="105" t="n"/>
       <c r="C7" s="104" t="inlineStr">
         <is>
-          <t>• Anleitung: Excel-Export aus Revit ist jetzt der Standard-Workflow (direktes Kopieren funktioniert nicht); Spaltenliste an neue Reihenfolge angepasst.</t>
+          <t>• Auslegung: Volumenstrom je Kreis wird gegen V̇_max geprüft und per Ampel eingefärbt (grün ≤ Grenze, rot darüber); zusätzliche Warnung im Blatt 'Kontrolle'.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="102" t="inlineStr">
-        <is>
-          <t>0.17</t>
-        </is>
-      </c>
-      <c r="B8" s="103" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
+      <c r="A8" s="105" t="n"/>
+      <c r="B8" s="105" t="n"/>
       <c r="C8" s="104" t="inlineStr">
         <is>
-          <t>• Neues Blatt 'Anleitung' (2. Blatt): Aufbau der Mappe, Schritt-für-Schritt, Farblegende.</t>
+          <t>• Anleitung: durchgehende Schritt-für-Schritt-Anleitung mit integriertem Revit-Export (vorgefertigte Bauteilliste muss nicht erst angelegt werden); redundanter Abschnitt 'Räume aus Revit' und der Hinweis zum direkten Kopieren entfernt.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="105" t="n"/>
-      <c r="B9" s="105" t="n"/>
+      <c r="A9" s="106" t="n"/>
+      <c r="B9" s="106" t="n"/>
       <c r="C9" s="104" t="inlineStr">
         <is>
-          <t>• Anleitung enthält den Workflow zum Übernehmen der Räume aus Revit (Copy &amp; Paste, Schedule, Dynamo/Power Query).</t>
+          <t>• Deckblatt: Pfeil-Spalten breiter und Pfeilgröße angepasst (optisch sauberer).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="102" t="inlineStr">
         <is>
-          <t>0.16</t>
+          <t>0.18</t>
         </is>
       </c>
       <c r="B10" s="103" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="C10" s="104" t="inlineStr">
         <is>
-          <t>• Alle Blätter im A4-Querformat (nur Auslegung A3 quer); einheitlichere Schriftgrößen/Skalierung.</t>
+          <t>• Auslegung: Eingabespalten neu sortiert – zuerst die Revit-Spalten (A HKV, B Raum-Nr., C Bezeichnung, D Raumfläche, E Raumtemperatur, F Heizlast), dann G spez. Heizlast (berechnet), danach die manuellen Felder (H aktiv. Fläche, I R-Wert, J Verlegeabstand, K Anz. Kreise, L Zuleitung, M Zone).</t>
         </is>
       </c>
     </row>
@@ -1997,16 +1990,24 @@
       <c r="B11" s="106" t="n"/>
       <c r="C11" s="104" t="inlineStr">
         <is>
-          <t>• Grundeinstellungen zweispaltig (Einstellwerte teilweise nebeneinander).</t>
+          <t>• Anleitung: Excel-Export aus Revit ist jetzt der Standard-Workflow (direktes Kopieren funktioniert nicht); Spaltenliste an neue Reihenfolge angepasst.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="106" t="n"/>
-      <c r="B12" s="106" t="n"/>
+      <c r="A12" s="102" t="inlineStr">
+        <is>
+          <t>0.17</t>
+        </is>
+      </c>
+      <c r="B12" s="103" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
       <c r="C12" s="104" t="inlineStr">
         <is>
-          <t>• Verifikation: Diagramm rechts neben den Tabellen.</t>
+          <t>• Neues Blatt 'Anleitung' (2. Blatt): Aufbau der Mappe, Schritt-für-Schritt, Farblegende.</t>
         </is>
       </c>
     </row>
@@ -2015,16 +2016,24 @@
       <c r="B13" s="106" t="n"/>
       <c r="C13" s="104" t="inlineStr">
         <is>
-          <t>• Methodik: Formelzeichen links, Berechnungsschritte in zwei Spalten rechts.</t>
+          <t>• Anleitung enthält den Workflow zum Übernehmen der Räume aus Revit (Copy &amp; Paste, Schedule, Dynamo/Power Query).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="106" t="n"/>
-      <c r="B14" s="106" t="n"/>
+      <c r="A14" s="102" t="inlineStr">
+        <is>
+          <t>0.16</t>
+        </is>
+      </c>
+      <c r="B14" s="103" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
       <c r="C14" s="104" t="inlineStr">
         <is>
-          <t>• Konstanten: Tabellen teilweise nebeneinander.</t>
+          <t>• Alle Blätter im A4-Querformat (nur Auslegung A3 quer); einheitlichere Schriftgrößen/Skalierung.</t>
         </is>
       </c>
     </row>
@@ -2033,33 +2042,25 @@
       <c r="B15" s="105" t="n"/>
       <c r="C15" s="104" t="inlineStr">
         <is>
-          <t>• Auslegung: Spalte Zone mittig/schmaler, Raum-Nr. breiter; Verifikation-Korrekturfaktor vertikal mittig.</t>
+          <t>• Grundeinstellungen zweispaltig (Einstellwerte teilweise nebeneinander).</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="102" t="inlineStr">
-        <is>
-          <t>0.15</t>
-        </is>
-      </c>
-      <c r="B16" s="103" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
+      <c r="A16" s="105" t="n"/>
+      <c r="B16" s="105" t="n"/>
       <c r="C16" s="104" t="inlineStr">
         <is>
-          <t>• Deckblatt-Diagramm aus Excel-Zellen statt Bild – direkt in Excel bearbeitbar.</t>
+          <t>• Verifikation: Diagramm rechts neben den Tabellen.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="106" t="n"/>
-      <c r="B17" s="106" t="n"/>
+      <c r="A17" s="105" t="n"/>
+      <c r="B17" s="105" t="n"/>
       <c r="C17" s="104" t="inlineStr">
         <is>
-          <t>• Auslegung: Beispielräume mit gemischter Heizlast (≤ 50 W/m²); Formelzeichen in Zeile 5 ergänzt (Flächen u. a.).</t>
+          <t>• Methodik: Formelzeichen links, Berechnungsschritte in zwei Spalten rechts.</t>
         </is>
       </c>
     </row>
@@ -2068,50 +2069,42 @@
       <c r="B18" s="105" t="n"/>
       <c r="C18" s="104" t="inlineStr">
         <is>
-          <t>• Heizkreisverteiler: zusätzliche Spalte Spreizung [K].</t>
+          <t>• Konstanten: Tabellen teilweise nebeneinander.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="102" t="inlineStr">
-        <is>
-          <t>0.14</t>
-        </is>
-      </c>
-      <c r="B19" s="103" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
+      <c r="A19" s="106" t="n"/>
+      <c r="B19" s="106" t="n"/>
       <c r="C19" s="104" t="inlineStr">
         <is>
-          <t>• Deckblatt als erstes Blatt: Übersichtsdiagramm Eingaben → Verarbeitung → Ergebnisse (inkl. Vereinfachungen).</t>
+          <t>• Auslegung: Spalte Zone mittig/schmaler, Raum-Nr. breiter; Verifikation-Korrekturfaktor vertikal mittig.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="102" t="inlineStr">
         <is>
-          <t>0.13</t>
+          <t>0.15</t>
         </is>
       </c>
       <c r="B20" s="103" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="C20" s="104" t="inlineStr">
         <is>
-          <t>• Strömungsbereich dreistufig: laminar (Re &lt; 2300), Übergangsbereich (2300–4000), turbulent (Re &gt; 4000).</t>
+          <t>• Deckblatt-Diagramm aus Excel-Zellen statt Bild – direkt in Excel bearbeitbar.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="106" t="n"/>
-      <c r="B21" s="106" t="n"/>
+      <c r="A21" s="105" t="n"/>
+      <c r="B21" s="105" t="n"/>
       <c r="C21" s="104" t="inlineStr">
         <is>
-          <t>• Spalte 'Strömungsbereich' ausgeblendet (für die Auslegung nicht relevant) und ohne Färbung.</t>
+          <t>• Auslegung: Beispielräume mit gemischter Heizlast (≤ 50 W/m²); Formelzeichen in Zeile 5 ergänzt (Flächen u. a.).</t>
         </is>
       </c>
     </row>
@@ -2120,60 +2113,68 @@
       <c r="B22" s="106" t="n"/>
       <c r="C22" s="104" t="inlineStr">
         <is>
+          <t>• Heizkreisverteiler: zusätzliche Spalte Spreizung [K].</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="102" t="inlineStr">
+        <is>
+          <t>0.14</t>
+        </is>
+      </c>
+      <c r="B23" s="103" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="C23" s="104" t="inlineStr">
+        <is>
+          <t>• Deckblatt als erstes Blatt: Übersichtsdiagramm Eingaben → Verarbeitung → Ergebnisse (inkl. Vereinfachungen).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="102" t="inlineStr">
+        <is>
+          <t>0.13</t>
+        </is>
+      </c>
+      <c r="B24" s="103" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C24" s="104" t="inlineStr">
+        <is>
+          <t>• Strömungsbereich dreistufig: laminar (Re &lt; 2300), Übergangsbereich (2300–4000), turbulent (Re &gt; 4000).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="105" t="n"/>
+      <c r="B25" s="105" t="n"/>
+      <c r="C25" s="104" t="inlineStr">
+        <is>
+          <t>• Spalte 'Strömungsbereich' ausgeblendet (für die Auslegung nicht relevant) und ohne Färbung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="105" t="n"/>
+      <c r="B26" s="105" t="n"/>
+      <c r="C26" s="104" t="inlineStr">
+        <is>
           <t>• Auslegung schlanker: weitere Zwischenspalten standardmäßig ausgeblendet (jederzeit einblendbar).</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="106" t="n"/>
-      <c r="B23" s="106" t="n"/>
-      <c r="C23" s="104" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="105" t="n"/>
+      <c r="B27" s="105" t="n"/>
+      <c r="C27" s="104" t="inlineStr">
         <is>
           <t>• Verifikation: Korrekturfaktor kleiner dargestellt (passt nun vollständig in die Zelle).</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="105" t="n"/>
-      <c r="B24" s="105" t="n"/>
-      <c r="C24" s="104" t="inlineStr">
-        <is>
-          <t>• Changelog wieder ausführlich.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="102" t="inlineStr">
-        <is>
-          <t>0.12</t>
-        </is>
-      </c>
-      <c r="B25" s="103" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="C25" s="104" t="inlineStr">
-        <is>
-          <t>• Grundeinstellungen: Bezeichnungen ausgeschrieben (keine Abkürzungen).</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="106" t="n"/>
-      <c r="B26" s="106" t="n"/>
-      <c r="C26" s="104" t="inlineStr">
-        <is>
-          <t>• Neue Spalte 'spez. Heizlast [W/m²]' (Heizlast bezogen auf die Raumfläche).</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="106" t="n"/>
-      <c r="B27" s="106" t="n"/>
-      <c r="C27" s="104" t="inlineStr">
-        <is>
-          <t>• Massenstrom/Geschwindigkeit/Druckverlust auf Basis min(Leistung; Heizlast) + Verlust nach unten (realer Betriebspunkt).</t>
         </is>
       </c>
     </row>
@@ -2182,67 +2183,67 @@
       <c r="B28" s="106" t="n"/>
       <c r="C28" s="104" t="inlineStr">
         <is>
+          <t>• Changelog wieder ausführlich.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="102" t="inlineStr">
+        <is>
+          <t>0.12</t>
+        </is>
+      </c>
+      <c r="B29" s="103" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C29" s="104" t="inlineStr">
+        <is>
+          <t>• Grundeinstellungen: Bezeichnungen ausgeschrieben (keine Abkürzungen).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="105" t="n"/>
+      <c r="B30" s="105" t="n"/>
+      <c r="C30" s="104" t="inlineStr">
+        <is>
+          <t>• Neue Spalte 'spez. Heizlast [W/m²]' (Heizlast bezogen auf die Raumfläche).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="105" t="n"/>
+      <c r="B31" s="105" t="n"/>
+      <c r="C31" s="104" t="inlineStr">
+        <is>
+          <t>• Massenstrom/Geschwindigkeit/Druckverlust auf Basis min(Leistung; Heizlast) + Verlust nach unten (realer Betriebspunkt).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="105" t="n"/>
+      <c r="B32" s="105" t="n"/>
+      <c r="C32" s="104" t="inlineStr">
+        <is>
           <t>• Heizkreisverteiler zusätzlich mit Massenstrom [kg/h]; Zonen-Kürzel (AZ/RZ/BAD).</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="105" t="n"/>
-      <c r="B29" s="105" t="n"/>
-      <c r="C29" s="104" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="106" t="n"/>
+      <c r="B33" s="106" t="n"/>
+      <c r="C33" s="104" t="inlineStr">
         <is>
           <t>• Kapazität 200 Räume / 50 Verteiler; Auslegung A3 quer, übrige Blätter A4 hoch.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="102" t="inlineStr">
-        <is>
-          <t>0.11</t>
-        </is>
-      </c>
-      <c r="B30" s="103" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="C30" s="104" t="inlineStr">
-        <is>
-          <t>• Bugfixes: Hinweistext wurde als Formel interpretiert (Fehler 501); MAXIFS ersetzt (#NAME? in LibreOffice).</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="106" t="n"/>
-      <c r="B31" s="106" t="n"/>
-      <c r="C31" s="104" t="inlineStr">
-        <is>
-          <t>• Verifikation: Korrekturfaktor prominent oben; Hersteller-q direkt neben q berechnet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="106" t="n"/>
-      <c r="B32" s="106" t="n"/>
-      <c r="C32" s="104" t="inlineStr">
-        <is>
-          <t>• Konstanten: alle Tabellen untereinander, mit Leerzeilen für weitere Einträge.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="105" t="n"/>
-      <c r="B33" s="105" t="n"/>
-      <c r="C33" s="104" t="inlineStr">
-        <is>
-          <t>• Methodik: Variablen zuerst, dann Formeln mit Erklärung je Schritt; weitere Musterräume (Verwaltungsbau).</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="102" t="inlineStr">
         <is>
-          <t>0.10</t>
+          <t>0.11</t>
         </is>
       </c>
       <c r="B34" s="103" t="inlineStr">
@@ -2252,16 +2253,16 @@
       </c>
       <c r="C34" s="104" t="inlineStr">
         <is>
-          <t>• Heizkreisverteiler-Liste und Verifikation ohne dynamische Array-Funktionen → läuft in Excel UND LibreOffice.</t>
+          <t>• Bugfixes: Hinweistext wurde als Formel interpretiert (Fehler 501); MAXIFS ersetzt (#NAME? in LibreOffice).</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="106" t="n"/>
-      <c r="B35" s="106" t="n"/>
+      <c r="A35" s="105" t="n"/>
+      <c r="B35" s="105" t="n"/>
       <c r="C35" s="104" t="inlineStr">
         <is>
-          <t>• Verifikation mit Liniendiagramm; Konstanten/Bibliotheken in eigenes Blatt ausgelagert.</t>
+          <t>• Verifikation: Korrekturfaktor prominent oben; Hersteller-q direkt neben q berechnet.</t>
         </is>
       </c>
     </row>
@@ -2270,58 +2271,58 @@
       <c r="B36" s="105" t="n"/>
       <c r="C36" s="104" t="inlineStr">
         <is>
+          <t>• Konstanten: alle Tabellen untereinander, mit Leerzeilen für weitere Einträge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="106" t="n"/>
+      <c r="B37" s="106" t="n"/>
+      <c r="C37" s="104" t="inlineStr">
+        <is>
+          <t>• Methodik: Variablen zuerst, dann Formeln mit Erklärung je Schritt; weitere Musterräume (Verwaltungsbau).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="102" t="inlineStr">
+        <is>
+          <t>0.10</t>
+        </is>
+      </c>
+      <c r="B38" s="103" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C38" s="104" t="inlineStr">
+        <is>
+          <t>• Heizkreisverteiler-Liste und Verifikation ohne dynamische Array-Funktionen → läuft in Excel UND LibreOffice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="105" t="n"/>
+      <c r="B39" s="105" t="n"/>
+      <c r="C39" s="104" t="inlineStr">
+        <is>
+          <t>• Verifikation mit Liniendiagramm; Konstanten/Bibliotheken in eigenes Blatt ausgelagert.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="106" t="n"/>
+      <c r="B40" s="106" t="n"/>
+      <c r="C40" s="104" t="inlineStr">
+        <is>
           <t>• Gewähltes Rohrsystem mit Außen-/Innendurchmesser, Wandstärke und Rauheit im Druckbereich.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="102" t="inlineStr">
-        <is>
-          <t>0.9</t>
-        </is>
-      </c>
-      <c r="B37" s="103" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C37" s="104" t="inlineStr">
-        <is>
-          <t>• Neues Blatt 'Heizkreisverteiler' (Leistung, max. Druckverlust, Volumenstrom je HKV).</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="106" t="n"/>
-      <c r="B38" s="106" t="n"/>
-      <c r="C38" s="104" t="inlineStr">
-        <is>
-          <t>• Spaltenüberschriften der Auslegung dreizeilig (Name / Formelzeichen / Einheit).</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="106" t="n"/>
-      <c r="B39" s="106" t="n"/>
-      <c r="C39" s="104" t="inlineStr">
-        <is>
-          <t>• Korrekturfaktor f wird auf 'Verifikation' eingegeben (mit Vergleichsdiagramm).</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="105" t="n"/>
-      <c r="B40" s="105" t="n"/>
-      <c r="C40" s="104" t="inlineStr">
-        <is>
-          <t>• Geschwindigkeits-Grenzwerte v_min/v_max als Grundeinstellung.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="102" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>0.9</t>
         </is>
       </c>
       <c r="B41" s="103" t="inlineStr">
@@ -2331,41 +2332,41 @@
       </c>
       <c r="C41" s="104" t="inlineStr">
         <is>
-          <t>• Grundeinstellungen für A3 quer optimiert (Einstellungen links, Tabellen rechts).</t>
+          <t>• Neues Blatt 'Heizkreisverteiler' (Leistung, max. Druckverlust, Volumenstrom je HKV).</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="106" t="n"/>
-      <c r="B42" s="106" t="n"/>
+      <c r="A42" s="105" t="n"/>
+      <c r="B42" s="105" t="n"/>
       <c r="C42" s="104" t="inlineStr">
         <is>
-          <t>• Auslegung passt auf eine Seite breit; Korrekturfaktor Heizleistung zur Kalibrierung ergänzt.</t>
+          <t>• Spaltenüberschriften der Auslegung dreizeilig (Name / Formelzeichen / Einheit).</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="106" t="n"/>
-      <c r="B43" s="106" t="n"/>
+      <c r="A43" s="105" t="n"/>
+      <c r="B43" s="105" t="n"/>
       <c r="C43" s="104" t="inlineStr">
         <is>
-          <t>• Wärmeabgabe nach unten berücksichtigt (Verlust + Gesamtleistung).</t>
+          <t>• Korrekturfaktor f wird auf 'Verifikation' eingegeben (mit Vergleichsdiagramm).</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="105" t="n"/>
-      <c r="B44" s="105" t="n"/>
+      <c r="A44" s="106" t="n"/>
+      <c r="B44" s="106" t="n"/>
       <c r="C44" s="104" t="inlineStr">
         <is>
-          <t>• Blätter umbenannt: Raumliste → Auslegung, Übersicht → Kontrolle; zusätzliche Kontrollen.</t>
+          <t>• Geschwindigkeits-Grenzwerte v_min/v_max als Grundeinstellung.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="102" t="inlineStr">
         <is>
-          <t>0.7</t>
+          <t>0.8</t>
         </is>
       </c>
       <c r="B45" s="103" t="inlineStr">
@@ -2375,16 +2376,16 @@
       </c>
       <c r="C45" s="104" t="inlineStr">
         <is>
-          <t>• Deckung-%-Spalte färbt nur noch gefüllte Zellen (leere bleiben farblos).</t>
+          <t>• Grundeinstellungen für A3 quer optimiert (Einstellungen links, Tabellen rechts).</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="106" t="n"/>
-      <c r="B46" s="106" t="n"/>
+      <c r="A46" s="105" t="n"/>
+      <c r="B46" s="105" t="n"/>
       <c r="C46" s="104" t="inlineStr">
         <is>
-          <t>• Neues Blatt 'Verifikation'; neue Spalte 'Strömungsbereich' (laminar/turbulent).</t>
+          <t>• Auslegung passt auf eine Seite breit; Korrekturfaktor Heizleistung zur Kalibrierung ergänzt.</t>
         </is>
       </c>
     </row>
@@ -2393,31 +2394,23 @@
       <c r="B47" s="105" t="n"/>
       <c r="C47" s="104" t="inlineStr">
         <is>
-          <t>• Alle Blätter im A3-Querformat; einheitlicher Kopf je Blatt.</t>
+          <t>• Wärmeabgabe nach unten berücksichtigt (Verlust + Gesamtleistung).</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="102" t="inlineStr">
-        <is>
-          <t>0.6</t>
-        </is>
-      </c>
-      <c r="B48" s="103" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
+      <c r="A48" s="106" t="n"/>
+      <c r="B48" s="106" t="n"/>
       <c r="C48" s="104" t="inlineStr">
         <is>
-          <t>• Bugfix: Zellfärbung (bedingte Formatierung) wird jetzt auch in Excel angezeigt – dxf-Füllfarbe mit voller Deckkraft.</t>
+          <t>• Blätter umbenannt: Raumliste → Auslegung, Übersicht → Kontrolle; zusätzliche Kontrollen.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="102" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>0.7</t>
         </is>
       </c>
       <c r="B49" s="103" t="inlineStr">
@@ -2427,7 +2420,7 @@
       </c>
       <c r="C49" s="104" t="inlineStr">
         <is>
-          <t>• Versionsnummer und Autor werden nur noch im Changelog angezeigt.</t>
+          <t>• Deckung-%-Spalte färbt nur noch gefüllte Zellen (leere bleiben farblos).</t>
         </is>
       </c>
     </row>
@@ -2436,58 +2429,66 @@
       <c r="B50" s="105" t="n"/>
       <c r="C50" s="104" t="inlineStr">
         <is>
+          <t>• Neues Blatt 'Verifikation'; neue Spalte 'Strömungsbereich' (laminar/turbulent).</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="106" t="n"/>
+      <c r="B51" s="106" t="n"/>
+      <c r="C51" s="104" t="inlineStr">
+        <is>
+          <t>• Alle Blätter im A3-Querformat; einheitlicher Kopf je Blatt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="102" t="inlineStr">
+        <is>
+          <t>0.6</t>
+        </is>
+      </c>
+      <c r="B52" s="103" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="C52" s="104" t="inlineStr">
+        <is>
+          <t>• Bugfix: Zellfärbung (bedingte Formatierung) wird jetzt auch in Excel angezeigt – dxf-Füllfarbe mit voller Deckkraft.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="102" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="B53" s="103" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="C53" s="104" t="inlineStr">
+        <is>
+          <t>• Versionsnummer und Autor werden nur noch im Changelog angezeigt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="106" t="n"/>
+      <c r="B54" s="106" t="n"/>
+      <c r="C54" s="104" t="inlineStr">
+        <is>
           <t>• Editierbares Bearbeiter-Kürzel rechts oben unter dem Logo (Grundeinstellungen, Auslegung, Kontrolle, HKV).</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="102" t="inlineStr">
-        <is>
-          <t>0.4</t>
-        </is>
-      </c>
-      <c r="B51" s="103" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C51" s="104" t="inlineStr">
-        <is>
-          <t>• Status-Spalten entfernt – Bewertung erfolgt jetzt direkt als Zellfärbung (grün/rot).</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="106" t="n"/>
-      <c r="B52" s="106" t="n"/>
-      <c r="C52" s="104" t="inlineStr">
-        <is>
-          <t>• Methodik um die Formelzeichen-Legende erweitert.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="106" t="n"/>
-      <c r="B53" s="106" t="n"/>
-      <c r="C53" s="104" t="inlineStr">
-        <is>
-          <t>• Heizkreisverteiler (HKV) als erste Spalte der Auslegung; Standardwert max. Druckverlust 15.000 Pa.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="105" t="n"/>
-      <c r="B54" s="105" t="n"/>
-      <c r="C54" s="104" t="inlineStr">
-        <is>
-          <t>• Versionsschema 0.x eingeführt (1.0 erst nach Test); interner Autor (dh).</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="102" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="B55" s="103" t="inlineStr">
@@ -2497,25 +2498,25 @@
       </c>
       <c r="C55" s="104" t="inlineStr">
         <is>
-          <t>• Zonentypen (Aufenthalt/Rand/Bad) mit eigener zulässiger Oberflächentemperatur.</t>
+          <t>• Status-Spalten entfernt – Bewertung erfolgt jetzt direkt als Zellfärbung (grün/rot).</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="106" t="n"/>
-      <c r="B56" s="106" t="n"/>
+      <c r="A56" s="105" t="n"/>
+      <c r="B56" s="105" t="n"/>
       <c r="C56" s="104" t="inlineStr">
         <is>
-          <t>• Einheitlicher Kopf: Titel oben links, agn-Logo oben rechts, Projektkopf darunter.</t>
+          <t>• Methodik um die Formelzeichen-Legende erweitert.</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="106" t="n"/>
-      <c r="B57" s="106" t="n"/>
+      <c r="A57" s="105" t="n"/>
+      <c r="B57" s="105" t="n"/>
       <c r="C57" s="104" t="inlineStr">
         <is>
-          <t>• Oberflächentemperatur θF und Volumenstrom eingeblendet.</t>
+          <t>• Heizkreisverteiler (HKV) als erste Spalte der Auslegung; Standardwert max. Druckverlust 15.000 Pa.</t>
         </is>
       </c>
     </row>
@@ -2524,51 +2525,51 @@
       <c r="B58" s="106" t="n"/>
       <c r="C58" s="104" t="inlineStr">
         <is>
+          <t>• Versionsschema 0.x eingeführt (1.0 erst nach Test); interner Autor (dh).</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="102" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="B59" s="103" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="C59" s="104" t="inlineStr">
+        <is>
+          <t>• Zonentypen (Aufenthalt/Rand/Bad) mit eigener zulässiger Oberflächentemperatur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="105" t="n"/>
+      <c r="B60" s="105" t="n"/>
+      <c r="C60" s="104" t="inlineStr">
+        <is>
+          <t>• Einheitlicher Kopf: Titel oben links, agn-Logo oben rechts, Projektkopf darunter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="105" t="n"/>
+      <c r="B61" s="105" t="n"/>
+      <c r="C61" s="104" t="inlineStr">
+        <is>
+          <t>• Oberflächentemperatur θF und Volumenstrom eingeblendet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="105" t="n"/>
+      <c r="B62" s="105" t="n"/>
+      <c r="C62" s="104" t="inlineStr">
+        <is>
           <t>• Neue Spalten 'spez. Druckverlust [Pa/m]' und Eingabespalte 'Verteiler (Anbindung)'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="105" t="n"/>
-      <c r="B59" s="105" t="n"/>
-      <c r="C59" s="104" t="inlineStr">
-        <is>
-          <t>• Warnung (rot), wenn die aktivierbare Fläche größer als die Raumfläche ist.</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="102" t="inlineStr">
-        <is>
-          <t>0.2</t>
-        </is>
-      </c>
-      <c r="B60" s="103" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C60" s="104" t="inlineStr">
-        <is>
-          <t>• agn-Logo eingebunden und eigenes Changelog-Blatt ergänzt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="106" t="n"/>
-      <c r="B61" s="106" t="n"/>
-      <c r="C61" s="104" t="inlineStr">
-        <is>
-          <t>• Zuschlag Einzelwiderstände (5 %) und fester Verteiler-Aufschlag (500 Pa je Kreis).</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="106" t="n"/>
-      <c r="B62" s="106" t="n"/>
-      <c r="C62" s="104" t="inlineStr">
-        <is>
-          <t>• Einheiten als Zellformat; Projektnummer/Projektname erscheinen im Ausdruck.</t>
         </is>
       </c>
     </row>
@@ -2577,51 +2578,51 @@
       <c r="B63" s="106" t="n"/>
       <c r="C63" s="104" t="inlineStr">
         <is>
+          <t>• Warnung (rot), wenn die aktivierbare Fläche größer als die Raumfläche ist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="102" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="B64" s="103" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="C64" s="104" t="inlineStr">
+        <is>
+          <t>• agn-Logo eingebunden und eigenes Changelog-Blatt ergänzt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="105" t="n"/>
+      <c r="B65" s="105" t="n"/>
+      <c r="C65" s="104" t="inlineStr">
+        <is>
+          <t>• Zuschlag Einzelwiderstände (5 %) und fester Verteiler-Aufschlag (500 Pa je Kreis).</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="105" t="n"/>
+      <c r="B66" s="105" t="n"/>
+      <c r="C66" s="104" t="inlineStr">
+        <is>
+          <t>• Einheiten als Zellformat; Projektnummer/Projektname erscheinen im Ausdruck.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="105" t="n"/>
+      <c r="B67" s="105" t="n"/>
+      <c r="C67" s="104" t="inlineStr">
+        <is>
           <t>• Richtwert-Tabellen für R-Werte und Verlegeabstand-Faktoren; weitere Musterräume.</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="105" t="n"/>
-      <c r="B64" s="105" t="n"/>
-      <c r="C64" s="104" t="inlineStr">
-        <is>
-          <t>• Druckaufbereitung für DIN A4.</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="102" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="B65" s="103" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C65" s="104" t="inlineStr">
-        <is>
-          <t>• Ersterstellung mit den Blättern Grundeinstellungen, Raumliste, Übersicht und Methodik.</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="106" t="n"/>
-      <c r="B66" s="106" t="n"/>
-      <c r="C66" s="104" t="inlineStr">
-        <is>
-          <t>• Heizleistung über die logarithmische Übertemperatur (q = η · K_H · ΔθH).</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="106" t="n"/>
-      <c r="B67" s="106" t="n"/>
-      <c r="C67" s="104" t="inlineStr">
-        <is>
-          <t>• Druckverlustberechnung nach Darcy-Weisbach.</t>
         </is>
       </c>
     </row>
@@ -2630,53 +2631,99 @@
       <c r="B68" s="106" t="n"/>
       <c r="C68" s="104" t="inlineStr">
         <is>
+          <t>• Druckaufbereitung für DIN A4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="102" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="B69" s="103" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="C69" s="104" t="inlineStr">
+        <is>
+          <t>• Ersterstellung mit den Blättern Grundeinstellungen, Raumliste, Übersicht und Methodik.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="105" t="n"/>
+      <c r="B70" s="105" t="n"/>
+      <c r="C70" s="104" t="inlineStr">
+        <is>
+          <t>• Heizleistung über die logarithmische Übertemperatur (q = η · K_H · ΔθH).</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="105" t="n"/>
+      <c r="B71" s="105" t="n"/>
+      <c r="C71" s="104" t="inlineStr">
+        <is>
+          <t>• Druckverlustberechnung nach Darcy-Weisbach.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="105" t="n"/>
+      <c r="B72" s="105" t="n"/>
+      <c r="C72" s="104" t="inlineStr">
+        <is>
           <t>• Editierbare Rohrbibliothek und Verlegeabstand-Faktoren.</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="105" t="n"/>
-      <c r="B69" s="105" t="n"/>
-      <c r="C69" s="104" t="inlineStr">
+    <row r="73">
+      <c r="A73" s="106" t="n"/>
+      <c r="B73" s="106" t="n"/>
+      <c r="C73" s="104" t="inlineStr">
         <is>
           <t>• Prüfungen: Oberflächentemperatur, Heizlastdeckung, Kreislänge, Druckverlust.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="32">
-    <mergeCell ref="B51:B54"/>
-    <mergeCell ref="B60:B64"/>
-    <mergeCell ref="B34:B36"/>
-    <mergeCell ref="B65:B69"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="A20:A24"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="B55:B59"/>
-    <mergeCell ref="B45:B47"/>
-    <mergeCell ref="A34:A36"/>
-    <mergeCell ref="B20:B24"/>
+  <mergeCells count="34">
+    <mergeCell ref="B49:B51"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="B29:B33"/>
+    <mergeCell ref="A20:A22"/>
+    <mergeCell ref="A38:A40"/>
+    <mergeCell ref="A45:A48"/>
+    <mergeCell ref="B64:B68"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="B20:B22"/>
+    <mergeCell ref="A29:A33"/>
+    <mergeCell ref="B24:B28"/>
+    <mergeCell ref="A6:A9"/>
     <mergeCell ref="A41:A44"/>
-    <mergeCell ref="A37:A40"/>
-    <mergeCell ref="B16:B18"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="A45:A47"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="B25:B29"/>
-    <mergeCell ref="B30:B33"/>
-    <mergeCell ref="B37:B40"/>
-    <mergeCell ref="B10:B15"/>
-    <mergeCell ref="A60:A64"/>
-    <mergeCell ref="A16:A18"/>
-    <mergeCell ref="A25:A29"/>
-    <mergeCell ref="A65:A69"/>
-    <mergeCell ref="A10:A15"/>
-    <mergeCell ref="A49:A50"/>
-    <mergeCell ref="A55:A59"/>
+    <mergeCell ref="A55:A58"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="B14:B19"/>
+    <mergeCell ref="A49:A51"/>
+    <mergeCell ref="A59:A63"/>
+    <mergeCell ref="B59:B63"/>
+    <mergeCell ref="A64:A68"/>
+    <mergeCell ref="B53:B54"/>
+    <mergeCell ref="A24:A28"/>
+    <mergeCell ref="B34:B37"/>
+    <mergeCell ref="B6:B9"/>
+    <mergeCell ref="A69:A73"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="A14:A19"/>
+    <mergeCell ref="A53:A54"/>
+    <mergeCell ref="B55:B58"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="B38:B40"/>
+    <mergeCell ref="B45:B48"/>
     <mergeCell ref="B41:B44"/>
-    <mergeCell ref="A51:A54"/>
+    <mergeCell ref="B69:B73"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -2698,7 +2745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -2722,7 +2769,7 @@
       </c>
       <c r="D3" s="18" t="inlineStr">
         <is>
-          <t>Räume aus Revit übernehmen</t>
+          <t>Schritt für Schritt</t>
         </is>
       </c>
     </row>
@@ -2734,7 +2781,7 @@
       </c>
       <c r="D4" s="19" t="inlineStr">
         <is>
-          <t>Spalten der Auslegung (links → rechts):</t>
+          <t>1. Grundeinstellungen ausfüllen: Projekt, Temperaturen,</t>
         </is>
       </c>
     </row>
@@ -2746,7 +2793,7 @@
       </c>
       <c r="D5" s="19" t="inlineStr">
         <is>
-          <t>A HKV · B Raum-Nr. · C Bezeichnung · D Raumfläche ·</t>
+          <t xml:space="preserve">    Rohrsystem, Stoffwerte und Grenzwerte (Kreislänge,</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2805,7 @@
       </c>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>E Raumtemperatur · F Heizlast</t>
+          <t xml:space="preserve">    Druckverlust, Geschwindigkeit, Volumenstrom je Kreis).</t>
         </is>
       </c>
     </row>
@@ -2768,9 +2815,9 @@
           <t>• Auslegung – Raumliste mit allen Berechnungen</t>
         </is>
       </c>
-      <c r="D7" s="20" t="inlineStr">
-        <is>
-          <t>G spez. Heizlast – berechnet, nicht überschreiben!</t>
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>2. Konstanten prüfen / erweitern (Rohre, R-Werte, Zonen).</t>
         </is>
       </c>
     </row>
@@ -2782,7 +2829,7 @@
       </c>
       <c r="D8" s="19" t="inlineStr">
         <is>
-          <t>H aktiv. Fläche · I R-Wert · J Verlegeabstand ·</t>
+          <t>3. In Revit die vorgefertigte Bauteilliste öffnen – sie ist</t>
         </is>
       </c>
     </row>
@@ -2794,7 +2841,7 @@
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>K Anz. Kreise · L Zuleitung · M Zone</t>
+          <t xml:space="preserve">    bereits passend angelegt und enthält die Spalten A–F</t>
         </is>
       </c>
     </row>
@@ -2804,7 +2851,11 @@
           <t>• Verifikation – Abgleich mit Herstellerdaten</t>
         </is>
       </c>
-      <c r="D10" s="19" t="inlineStr"/>
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    (HKV, Raum-Nr., Bezeichnung, Raumfläche,</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="B11" s="19" t="inlineStr">
@@ -2812,9 +2863,9 @@
           <t>• Methodik – Formeln &amp; Annahmen</t>
         </is>
       </c>
-      <c r="D11" s="21" t="inlineStr">
-        <is>
-          <t>Workflow: Excel-Export aus Revit</t>
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Raumtemperatur, Heizlast).</t>
         </is>
       </c>
     </row>
@@ -2826,7 +2877,7 @@
       </c>
       <c r="D12" s="19" t="inlineStr">
         <is>
-          <t>Das direkte Kopieren aus Revit in Excel funktioniert nicht –</t>
+          <t>4. Bauteilliste aus Revit nach Excel exportieren</t>
         </is>
       </c>
     </row>
@@ -2838,7 +2889,7 @@
       </c>
       <c r="D13" s="19" t="inlineStr">
         <is>
-          <t>es muss zuerst ein Excel-Export aus Revit erzeugt werden.</t>
+          <t xml:space="preserve">    ('Exportieren → Bericht/Schedule').</t>
         </is>
       </c>
     </row>
@@ -2846,119 +2897,123 @@
       <c r="B14" s="19" t="inlineStr"/>
       <c r="D14" s="19" t="inlineStr">
         <is>
-          <t>1. In Revit eine Raumliste (Schedule) mit den Spalten A–F</t>
+          <t>5. Werte aus dem Export in die Auslegung übernehmen</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>Schritt für Schritt</t>
+          <t>Spalten der Auslegung</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">   anlegen: HKV, Raum-Nr., Bezeichnung, Raumfläche,</t>
+          <t xml:space="preserve">    (Spalten A–F, ab der ersten Datenzeile).</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="19" t="inlineStr">
-        <is>
-          <t>1. Grundeinstellungen ausfüllen (Projekt, Temperaturen,</t>
+      <c r="B16" s="20" t="inlineStr">
+        <is>
+          <t>Aus Revit (A–F):</t>
         </is>
       </c>
       <c r="D16" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Raumtemperatur, Heizlast.</t>
+          <t>6. Spalte G (spez. Heizlast) frei lassen – wird berechnet.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Rohrsystem, Grenzwerte).</t>
+          <t>HKV, Raum-Nr., Bezeichnung, Raumfläche,</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>2. Schedule über 'Exportieren → Bericht/Schedule' als</t>
+          <t>7. Spalten H–M je Raum ergänzen: aktivierbare Fläche,</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="19" t="inlineStr">
         <is>
-          <t>2. Konstanten prüfen / erweitern (Rohre, R-Werte, Zonen).</t>
+          <t>Raumtemperatur, Heizlast.</t>
         </is>
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Excel-/CSV-Datei ausgeben.</t>
+          <t xml:space="preserve">    R-Wert Bodenbelag, Verlegeabstand, Anzahl Kreise,</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="19" t="inlineStr">
-        <is>
-          <t>3. Räume in 'Auslegung' eintragen (blaue Spalten) –</t>
+      <c r="B19" s="20" t="inlineStr">
+        <is>
+          <t>Berechnet (G):</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>3. Werte aus dem Export in die Auslegung übernehmen –</t>
+          <t xml:space="preserve">    Zuleitungslänge, Zone.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">    siehe rechts: aus Revit übernehmen.</t>
+          <t>spez. Heizlast – nicht überschreiben.</t>
         </is>
       </c>
       <c r="D20" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Spalten A–F, ab erster Datenzeile ('Werte einfügen').</t>
+          <t>8. Ergebnisse prüfen: Ampel in der Auslegung und im</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="19" t="inlineStr">
-        <is>
-          <t>4. Ergebnisse prüfen: Ampel in Auslegung + Blatt 'Kontrolle'.</t>
+      <c r="B21" s="20" t="inlineStr">
+        <is>
+          <t>Im Tool ergänzen (H–M):</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>4. Spalte G (spez. Heizlast) frei lassen – wird berechnet.</t>
+          <t xml:space="preserve">    Blatt 'Kontrolle' (Deckung, Kreislänge, Druckverlust,</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="19" t="inlineStr">
         <is>
-          <t>5. Verifikation: Korrekturfaktor f an Herstellerdaten</t>
+          <t>aktiv. Fläche, R-Wert, Verlegeabstand,</t>
         </is>
       </c>
       <c r="D22" s="19" t="inlineStr">
         <is>
-          <t>5. Spalten H–M im Tool ergänzen (siehe unten).</t>
+          <t xml:space="preserve">    Geschwindigkeit, Volumenstrom je Kreis).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">    kalibrieren.</t>
-        </is>
-      </c>
-      <c r="D23" s="19" t="inlineStr"/>
+          <t>Anz. Kreise, Zuleitung, Zone.</t>
+        </is>
+      </c>
+      <c r="D23" s="19" t="inlineStr">
+        <is>
+          <t>9. Verifikation: Korrekturfaktor f an Herstellerdaten</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="B24" s="19" t="inlineStr"/>
-      <c r="D24" s="21" t="inlineStr">
-        <is>
-          <t>Was kommt aus Revit (A–F)?</t>
+      <c r="D24" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    kalibrieren.</t>
         </is>
       </c>
     </row>
@@ -2968,11 +3023,7 @@
           <t>Farblegende</t>
         </is>
       </c>
-      <c r="D25" s="19" t="inlineStr">
-        <is>
-          <t>• HKV, Raum-Nr., Bezeichnung, Raumfläche, Raumtemperatur.</t>
-        </is>
-      </c>
+      <c r="D25" s="19" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="B26" s="19" t="inlineStr">
@@ -2980,9 +3031,9 @@
           <t>• Blau (gelb hinterlegt) = Eingabe</t>
         </is>
       </c>
-      <c r="D26" s="19" t="inlineStr">
-        <is>
-          <t>• Heizlast: aus Heizlastberechnung (DIN 12831) bzw.</t>
+      <c r="D26" s="20" t="inlineStr">
+        <is>
+          <t>Hinweis</t>
         </is>
       </c>
     </row>
@@ -2994,17 +3045,21 @@
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Revit-Systemanalyse – im Schedule mitführen.</t>
+          <t>Die Bauteilliste in Revit muss nicht erst angelegt werden –</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="19" t="inlineStr">
         <is>
-          <t>• Grün = OK,  Rot = Warnung</t>
-        </is>
-      </c>
-      <c r="D28" s="19" t="inlineStr"/>
+          <t>• Grün = OK,  Rot = Warnung / Grenzwert überschritten</t>
+        </is>
+      </c>
+      <c r="D28" s="19" t="inlineStr">
+        <is>
+          <t>sie ist passend zur Auslegung vorbereitet. Bei Bedarf lassen</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="B29" s="19" t="inlineStr">
@@ -3012,75 +3067,16 @@
           <t>• Nur die blauen Eingabezellen bearbeiten.</t>
         </is>
       </c>
-      <c r="D29" s="21" t="inlineStr">
-        <is>
-          <t>Im Tool ergänzen (H–M)</t>
+      <c r="D29" s="19" t="inlineStr">
+        <is>
+          <t>sich auch die Felder H–M (z. B. Zone, Verlegeabstand) als</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="D30" s="19" t="inlineStr">
         <is>
-          <t>• aktivierbare Fläche, R-Wert Bodenbelag, Verlegeabstand,</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="D31" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Anzahl Heizkreise, Zuleitungslänge, Zone.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="D32" s="19" t="inlineStr">
-        <is>
-          <t>• Planungsentscheidungen – kommen nicht aus Revit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="D33" s="19" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="D34" s="21" t="inlineStr">
-        <is>
-          <t>Tipp</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="D35" s="19" t="inlineStr">
-        <is>
-          <t>• Auch H–M (Zone, Verlegeabstand …) lassen sich als</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="D36" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   gemeinsame Parameter in Revit pflegen und mit</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="D37" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   exportieren.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="D38" s="19" t="inlineStr">
-        <is>
-          <t>• Dynamo / pyRevit oder Power Query halten den Export</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="D39" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   aktualisierbar.</t>
+          <t>gemeinsame Parameter in Revit pflegen und mit exportieren.</t>
         </is>
       </c>
     </row>
@@ -3131,534 +3127,552 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="22" t="inlineStr">
+      <c r="A2" s="21" t="inlineStr">
         <is>
           <t>Projekt-Nr.</t>
         </is>
       </c>
-      <c r="C2" s="23" t="inlineStr"/>
-      <c r="D2" s="24" t="n"/>
-      <c r="L2" s="25" t="inlineStr">
+      <c r="C2" s="22" t="inlineStr"/>
+      <c r="D2" s="23" t="n"/>
+      <c r="L2" s="24" t="inlineStr">
         <is>
           <t>Bearbeiter:</t>
         </is>
       </c>
-      <c r="M2" s="26" t="inlineStr"/>
+      <c r="M2" s="25" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="22" t="inlineStr">
+      <c r="A3" s="21" t="inlineStr">
         <is>
           <t>Projektname</t>
         </is>
       </c>
-      <c r="C3" s="23" t="inlineStr"/>
-      <c r="D3" s="24" t="n"/>
+      <c r="C3" s="22" t="inlineStr"/>
+      <c r="D3" s="23" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>Heizmedium / Temperaturen</t>
         </is>
       </c>
-      <c r="B5" s="28" t="n"/>
-      <c r="C5" s="28" t="n"/>
-      <c r="D5" s="28" t="n"/>
-      <c r="E5" s="28" t="n"/>
-      <c r="F5" s="28" t="n"/>
-      <c r="H5" s="27" t="inlineStr">
+      <c r="B5" s="27" t="n"/>
+      <c r="C5" s="27" t="n"/>
+      <c r="D5" s="27" t="n"/>
+      <c r="E5" s="27" t="n"/>
+      <c r="F5" s="27" t="n"/>
+      <c r="H5" s="26" t="inlineStr">
         <is>
           <t>Wärmeübergang / Fußbodenaufbau</t>
         </is>
       </c>
-      <c r="I5" s="28" t="n"/>
-      <c r="J5" s="28" t="n"/>
-      <c r="K5" s="28" t="n"/>
-      <c r="L5" s="28" t="n"/>
-      <c r="M5" s="28" t="n"/>
+      <c r="I5" s="27" t="n"/>
+      <c r="J5" s="27" t="n"/>
+      <c r="K5" s="27" t="n"/>
+      <c r="L5" s="27" t="n"/>
+      <c r="M5" s="27" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="29" t="inlineStr">
+      <c r="A6" s="28" t="inlineStr">
         <is>
           <t>Vorlauftemperatur  θV</t>
         </is>
       </c>
-      <c r="C6" s="30" t="n">
+      <c r="C6" s="29" t="n">
         <v>35</v>
       </c>
-      <c r="D6" s="31" t="inlineStr">
+      <c r="D6" s="30" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="E6" s="32" t="inlineStr">
+      <c r="E6" s="31" t="inlineStr">
         <is>
           <t>Auslegungs-Vorlauftemperatur</t>
         </is>
       </c>
-      <c r="H6" s="29" t="inlineStr">
+      <c r="H6" s="28" t="inlineStr">
         <is>
           <t>Wärmeübergangskoeffizient Oberfläche  α</t>
         </is>
       </c>
-      <c r="J6" s="33" t="n">
+      <c r="J6" s="32" t="n">
         <v>10.8</v>
       </c>
-      <c r="K6" s="31" t="inlineStr">
+      <c r="K6" s="30" t="inlineStr">
         <is>
           <t>W/m²K</t>
         </is>
       </c>
-      <c r="L6" s="32" t="inlineStr">
+      <c r="L6" s="31" t="inlineStr">
         <is>
           <t>Boden → Raum (EN 1264)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="29" t="inlineStr">
+      <c r="A7" s="28" t="inlineStr">
         <is>
           <t>Rücklauftemperatur  θR</t>
         </is>
       </c>
-      <c r="C7" s="30" t="n">
+      <c r="C7" s="29" t="n">
         <v>28</v>
       </c>
-      <c r="D7" s="31" t="inlineStr">
+      <c r="D7" s="30" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="E7" s="32" t="inlineStr">
+      <c r="E7" s="31" t="inlineStr">
         <is>
           <t>Auslegungs-Rücklauftemperatur</t>
         </is>
       </c>
-      <c r="H7" s="29" t="inlineStr">
+      <c r="H7" s="28" t="inlineStr">
         <is>
           <t>Estrichüberdeckung über Rohr  s_ü</t>
         </is>
       </c>
-      <c r="J7" s="34" t="n">
+      <c r="J7" s="33" t="n">
         <v>0.045</v>
       </c>
-      <c r="K7" s="31" t="inlineStr">
+      <c r="K7" s="30" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="L7" s="32" t="inlineStr">
+      <c r="L7" s="31" t="inlineStr">
         <is>
           <t>Estrich über den Rohren</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="29" t="inlineStr">
+      <c r="A8" s="28" t="inlineStr">
         <is>
           <t>Spreizung  θV − θR</t>
         </is>
       </c>
-      <c r="C8" s="35">
+      <c r="C8" s="34">
         <f>C6-C7</f>
         <v/>
       </c>
-      <c r="D8" s="31" t="inlineStr">
+      <c r="D8" s="30" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="E8" s="32" t="inlineStr">
+      <c r="E8" s="31" t="inlineStr">
         <is>
           <t>berechnet</t>
         </is>
       </c>
-      <c r="H8" s="29" t="inlineStr">
+      <c r="H8" s="28" t="inlineStr">
         <is>
           <t>Wärmeleitfähigkeit Estrich  λ_E</t>
         </is>
       </c>
-      <c r="J8" s="36" t="n">
+      <c r="J8" s="35" t="n">
         <v>1.2</v>
       </c>
-      <c r="K8" s="31" t="inlineStr">
+      <c r="K8" s="30" t="inlineStr">
         <is>
           <t>W/mK</t>
         </is>
       </c>
-      <c r="L8" s="32" t="inlineStr">
+      <c r="L8" s="31" t="inlineStr">
         <is>
           <t>Zementestrich typ. 1,2</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="27" t="inlineStr">
+      <c r="A10" s="26" t="inlineStr">
         <is>
           <t>Grenzwerte</t>
         </is>
       </c>
-      <c r="B10" s="28" t="n"/>
-      <c r="C10" s="28" t="n"/>
-      <c r="D10" s="28" t="n"/>
-      <c r="E10" s="28" t="n"/>
-      <c r="F10" s="28" t="n"/>
-      <c r="H10" s="27" t="inlineStr">
+      <c r="B10" s="27" t="n"/>
+      <c r="C10" s="27" t="n"/>
+      <c r="D10" s="27" t="n"/>
+      <c r="E10" s="27" t="n"/>
+      <c r="F10" s="27" t="n"/>
+      <c r="H10" s="26" t="inlineStr">
         <is>
           <t>Wärmeabgabe nach unten (Dämmung, global)</t>
         </is>
       </c>
-      <c r="I10" s="28" t="n"/>
-      <c r="J10" s="28" t="n"/>
-      <c r="K10" s="28" t="n"/>
-      <c r="L10" s="28" t="n"/>
-      <c r="M10" s="28" t="n"/>
+      <c r="I10" s="27" t="n"/>
+      <c r="J10" s="27" t="n"/>
+      <c r="K10" s="27" t="n"/>
+      <c r="L10" s="27" t="n"/>
+      <c r="M10" s="27" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="29" t="inlineStr">
+      <c r="A11" s="28" t="inlineStr">
         <is>
           <t>Maximale zulässige Kreislänge</t>
         </is>
       </c>
-      <c r="C11" s="37" t="n">
+      <c r="C11" s="36" t="n">
         <v>120</v>
       </c>
-      <c r="D11" s="31" t="inlineStr">
+      <c r="D11" s="30" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="E11" s="32" t="inlineStr">
+      <c r="E11" s="31" t="inlineStr">
         <is>
           <t>Obergrenze je Heizkreis</t>
         </is>
       </c>
-      <c r="H11" s="29" t="inlineStr">
+      <c r="H11" s="28" t="inlineStr">
         <is>
           <t>Wärmedurchlasswiderstand nach unten  R_u</t>
         </is>
       </c>
-      <c r="J11" s="36" t="n">
+      <c r="J11" s="35" t="n">
         <v>2</v>
       </c>
-      <c r="K11" s="31" t="inlineStr">
+      <c r="K11" s="30" t="inlineStr">
         <is>
           <t>m²K/W</t>
         </is>
       </c>
-      <c r="L11" s="32" t="inlineStr">
+      <c r="L11" s="31" t="inlineStr">
         <is>
           <t>Dämmung + Aufbau unter den Rohren</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="29" t="inlineStr">
+      <c r="A12" s="28" t="inlineStr">
         <is>
           <t>Maximaler Druckverlust je Kreis</t>
         </is>
       </c>
-      <c r="C12" s="38" t="n">
+      <c r="C12" s="37" t="n">
         <v>15000</v>
       </c>
-      <c r="D12" s="31" t="inlineStr">
+      <c r="D12" s="30" t="inlineStr">
         <is>
           <t>Pa</t>
         </is>
       </c>
-      <c r="E12" s="32" t="inlineStr">
+      <c r="E12" s="31" t="inlineStr">
         <is>
           <t>Warnschwelle bei Überschreitung</t>
         </is>
       </c>
-      <c r="H12" s="29" t="inlineStr">
+      <c r="H12" s="28" t="inlineStr">
         <is>
           <t>Temperatur unter der Decke  θ_u</t>
         </is>
       </c>
-      <c r="J12" s="30" t="n">
+      <c r="J12" s="29" t="n">
         <v>10</v>
       </c>
-      <c r="K12" s="31" t="inlineStr">
+      <c r="K12" s="30" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="L12" s="32" t="inlineStr">
+      <c r="L12" s="31" t="inlineStr">
         <is>
           <t>Raum / Erdreich unter der FBH</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="H13" s="29" t="inlineStr">
+      <c r="H13" s="28" t="inlineStr">
         <is>
           <t>Wärmestrom nach unten  q_u</t>
         </is>
       </c>
-      <c r="J13" s="39">
+      <c r="J13" s="38">
         <f>((C6+C7)/2-J12)/J11</f>
         <v/>
       </c>
-      <c r="K13" s="31" t="inlineStr">
+      <c r="K13" s="30" t="inlineStr">
         <is>
           <t>W/m²</t>
         </is>
       </c>
-      <c r="L13" s="32" t="inlineStr">
+      <c r="L13" s="31" t="inlineStr">
         <is>
           <t>Mittel θm = (θV+θR)/2</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="27" t="inlineStr">
+      <c r="A14" s="26" t="inlineStr">
         <is>
           <t>Stoffwerte Heizmedium (Wasser ~30 °C)</t>
         </is>
       </c>
-      <c r="B14" s="28" t="n"/>
-      <c r="C14" s="28" t="n"/>
-      <c r="D14" s="28" t="n"/>
-      <c r="E14" s="28" t="n"/>
-      <c r="F14" s="28" t="n"/>
+      <c r="B14" s="27" t="n"/>
+      <c r="C14" s="27" t="n"/>
+      <c r="D14" s="27" t="n"/>
+      <c r="E14" s="27" t="n"/>
+      <c r="F14" s="27" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="29" t="inlineStr">
+      <c r="A15" s="28" t="inlineStr">
         <is>
           <t>Dichte  ρ</t>
         </is>
       </c>
-      <c r="C15" s="33" t="n">
+      <c r="C15" s="32" t="n">
         <v>995.7</v>
       </c>
-      <c r="D15" s="31" t="inlineStr">
+      <c r="D15" s="30" t="inlineStr">
         <is>
           <t>kg/m³</t>
         </is>
       </c>
-      <c r="E15" s="32" t="inlineStr">
+      <c r="E15" s="31" t="inlineStr">
         <is>
           <t>Dichte des Mediums</t>
         </is>
       </c>
-      <c r="H15" s="27" t="inlineStr">
+      <c r="H15" s="26" t="inlineStr">
         <is>
           <t>Rohrsystem-Auswahl (Werte aus Konstanten)</t>
         </is>
       </c>
-      <c r="I15" s="28" t="n"/>
-      <c r="J15" s="28" t="n"/>
-      <c r="K15" s="28" t="n"/>
-      <c r="L15" s="28" t="n"/>
-      <c r="M15" s="28" t="n"/>
+      <c r="I15" s="27" t="n"/>
+      <c r="J15" s="27" t="n"/>
+      <c r="K15" s="27" t="n"/>
+      <c r="L15" s="27" t="n"/>
+      <c r="M15" s="27" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="29" t="inlineStr">
+      <c r="A16" s="28" t="inlineStr">
         <is>
           <t>spezifische Wärmekapazität  c_p</t>
         </is>
       </c>
-      <c r="C16" s="40" t="n">
+      <c r="C16" s="39" t="n">
         <v>4180</v>
       </c>
-      <c r="D16" s="31" t="inlineStr">
+      <c r="D16" s="30" t="inlineStr">
         <is>
           <t>J/(kg·K)</t>
         </is>
       </c>
-      <c r="E16" s="32" t="inlineStr">
+      <c r="E16" s="31" t="inlineStr">
         <is>
           <t>spez. Wärmekapazität</t>
         </is>
       </c>
-      <c r="H16" s="29" t="inlineStr">
+      <c r="H16" s="28" t="inlineStr">
         <is>
           <t>Gewähltes Rohrsystem</t>
         </is>
       </c>
-      <c r="J16" s="26" t="inlineStr">
+      <c r="J16" s="25" t="inlineStr">
         <is>
           <t>PE-Xa 17x2</t>
         </is>
       </c>
-      <c r="K16" s="24" t="n"/>
-      <c r="L16" s="32" t="inlineStr">
+      <c r="K16" s="23" t="n"/>
+      <c r="L16" s="31" t="inlineStr">
         <is>
           <t>Dropdown</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="29" t="inlineStr">
+      <c r="A17" s="28" t="inlineStr">
         <is>
           <t>kinematische Viskosität  ν</t>
         </is>
       </c>
-      <c r="C17" s="41" t="n">
+      <c r="C17" s="40" t="n">
         <v>8.01e-07</v>
       </c>
-      <c r="D17" s="31" t="inlineStr">
+      <c r="D17" s="30" t="inlineStr">
         <is>
           <t>m²/s</t>
         </is>
       </c>
-      <c r="E17" s="32" t="inlineStr">
+      <c r="E17" s="31" t="inlineStr">
         <is>
           <t>für die Reynolds-Zahl</t>
         </is>
       </c>
-      <c r="H17" s="29" t="inlineStr">
+      <c r="H17" s="28" t="inlineStr">
         <is>
           <t>→ Außendurchmesser  da</t>
         </is>
       </c>
-      <c r="J17" s="42">
+      <c r="J17" s="41">
         <f>VLOOKUP($J$16,'Konstanten'!$A$18:$E$25,2,FALSE)</f>
         <v/>
       </c>
-      <c r="K17" s="31" t="inlineStr">
+      <c r="K17" s="30" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="L17" s="32" t="inlineStr">
+      <c r="L17" s="31" t="inlineStr">
         <is>
           <t>aus Rohrbibliothek</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="H18" s="29" t="inlineStr">
+      <c r="H18" s="28" t="inlineStr">
         <is>
           <t>→ Wandstärke  s</t>
         </is>
       </c>
-      <c r="J18" s="42">
+      <c r="J18" s="41">
         <f>VLOOKUP($J$16,'Konstanten'!$A$18:$E$25,3,FALSE)</f>
         <v/>
       </c>
-      <c r="K18" s="31" t="inlineStr">
+      <c r="K18" s="30" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="L18" s="32" t="inlineStr">
+      <c r="L18" s="31" t="inlineStr">
         <is>
           <t>aus Rohrbibliothek</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="27" t="inlineStr">
-        <is>
-          <t>Strömungsgeschwindigkeit (Empfehlung)</t>
-        </is>
-      </c>
-      <c r="B19" s="28" t="n"/>
-      <c r="C19" s="28" t="n"/>
-      <c r="D19" s="28" t="n"/>
-      <c r="E19" s="28" t="n"/>
-      <c r="F19" s="28" t="n"/>
-      <c r="H19" s="29" t="inlineStr">
+      <c r="A19" s="26" t="inlineStr">
+        <is>
+          <t>Strömungsgrenzwerte</t>
+        </is>
+      </c>
+      <c r="B19" s="27" t="n"/>
+      <c r="C19" s="27" t="n"/>
+      <c r="D19" s="27" t="n"/>
+      <c r="E19" s="27" t="n"/>
+      <c r="F19" s="27" t="n"/>
+      <c r="H19" s="28" t="inlineStr">
         <is>
           <t>→ Innendurchmesser  di</t>
         </is>
       </c>
-      <c r="J19" s="42">
+      <c r="J19" s="41">
         <f>VLOOKUP($J$16,'Konstanten'!$A$18:$E$25,4,FALSE)</f>
         <v/>
       </c>
-      <c r="K19" s="31" t="inlineStr">
+      <c r="K19" s="30" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="L19" s="32" t="inlineStr">
+      <c r="L19" s="31" t="inlineStr">
         <is>
           <t>di = da − 2·s</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="29" t="inlineStr">
+      <c r="A20" s="28" t="inlineStr">
         <is>
           <t>Minimale Strömungsgeschwindigkeit  v_min</t>
         </is>
       </c>
-      <c r="C20" s="43" t="n">
+      <c r="C20" s="42" t="n">
         <v>0.1</v>
       </c>
-      <c r="D20" s="31" t="inlineStr">
+      <c r="D20" s="30" t="inlineStr">
         <is>
           <t>m/s</t>
         </is>
       </c>
-      <c r="E20" s="32" t="inlineStr">
+      <c r="E20" s="31" t="inlineStr">
         <is>
           <t>untere empfohlene Grenze</t>
         </is>
       </c>
-      <c r="H20" s="29" t="inlineStr">
+      <c r="H20" s="28" t="inlineStr">
         <is>
           <t>→ Rauheit  k</t>
         </is>
       </c>
-      <c r="J20" s="44">
+      <c r="J20" s="43">
         <f>VLOOKUP($J$16,'Konstanten'!$A$18:$E$25,5,FALSE)</f>
         <v/>
       </c>
-      <c r="K20" s="31" t="inlineStr">
+      <c r="K20" s="30" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="L20" s="32" t="inlineStr">
+      <c r="L20" s="31" t="inlineStr">
         <is>
           <t>aus Rohrbibliothek</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="29" t="inlineStr">
+      <c r="A21" s="28" t="inlineStr">
         <is>
           <t>Maximale Strömungsgeschwindigkeit  v_max</t>
         </is>
       </c>
-      <c r="C21" s="43" t="n">
+      <c r="C21" s="42" t="n">
         <v>0.5</v>
       </c>
-      <c r="D21" s="31" t="inlineStr">
+      <c r="D21" s="30" t="inlineStr">
         <is>
           <t>m/s</t>
         </is>
       </c>
-      <c r="E21" s="32" t="inlineStr">
+      <c r="E21" s="31" t="inlineStr">
         <is>
           <t>obere empfohlene Grenze</t>
         </is>
       </c>
-      <c r="H21" s="29" t="inlineStr">
+      <c r="H21" s="28" t="inlineStr">
         <is>
           <t>→ Innendurchmesser  di</t>
         </is>
       </c>
-      <c r="J21" s="45">
+      <c r="J21" s="44">
         <f>J19/1000</f>
         <v/>
       </c>
-      <c r="K21" s="31" t="inlineStr">
+      <c r="K21" s="30" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="L21" s="32" t="inlineStr">
+      <c r="L21" s="31" t="inlineStr">
         <is>
           <t>für die Berechnung</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="H22" s="29" t="inlineStr">
+      <c r="A22" s="28" t="inlineStr">
+        <is>
+          <t>Maximaler Volumenstrom je Kreis  V̇_max</t>
+        </is>
+      </c>
+      <c r="C22" s="45" t="n">
+        <v>150</v>
+      </c>
+      <c r="D22" s="30" t="inlineStr">
+        <is>
+          <t>l/h</t>
+        </is>
+      </c>
+      <c r="E22" s="31" t="inlineStr">
+        <is>
+          <t>Warnschwelle je Heizkreis</t>
+        </is>
+      </c>
+      <c r="H22" s="28" t="inlineStr">
         <is>
           <t>→ Innenquerschnitt  A_i</t>
         </is>
@@ -3667,31 +3681,31 @@
         <f>PI()/4*J21^2</f>
         <v/>
       </c>
-      <c r="K22" s="31" t="inlineStr">
+      <c r="K22" s="30" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="L22" s="32" t="inlineStr">
+      <c r="L22" s="31" t="inlineStr">
         <is>
           <t>für die Berechnung</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="27" t="inlineStr">
+      <c r="A23" s="26" t="inlineStr">
         <is>
           <t>Druckverlust-Zuschläge</t>
         </is>
       </c>
-      <c r="B23" s="28" t="n"/>
-      <c r="C23" s="28" t="n"/>
-      <c r="D23" s="28" t="n"/>
-      <c r="E23" s="28" t="n"/>
-      <c r="F23" s="28" t="n"/>
+      <c r="B23" s="27" t="n"/>
+      <c r="C23" s="27" t="n"/>
+      <c r="D23" s="27" t="n"/>
+      <c r="E23" s="27" t="n"/>
+      <c r="F23" s="27" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="29" t="inlineStr">
+      <c r="A24" s="28" t="inlineStr">
         <is>
           <t>Zuschlag Einzelwiderstände</t>
         </is>
@@ -3699,39 +3713,39 @@
       <c r="C24" s="47" t="n">
         <v>0.05</v>
       </c>
-      <c r="D24" s="31" t="inlineStr">
+      <c r="D24" s="30" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E24" s="32" t="inlineStr">
+      <c r="E24" s="31" t="inlineStr">
         <is>
           <t>Rohr-Formstücke (0,05 = 5 %)</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="29" t="inlineStr">
+      <c r="A25" s="28" t="inlineStr">
         <is>
           <t>Aufschlag Verteiler je Kreis</t>
         </is>
       </c>
-      <c r="C25" s="38" t="n">
+      <c r="C25" s="37" t="n">
         <v>500</v>
       </c>
-      <c r="D25" s="31" t="inlineStr">
+      <c r="D25" s="30" t="inlineStr">
         <is>
           <t>Pa</t>
         </is>
       </c>
-      <c r="E25" s="32" t="inlineStr">
+      <c r="E25" s="31" t="inlineStr">
         <is>
           <t>fester Wert je Verteiler</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="55">
+  <mergeCells count="57">
     <mergeCell ref="E12:F12"/>
     <mergeCell ref="L17:M17"/>
     <mergeCell ref="A24:B24"/>
@@ -3775,6 +3789,7 @@
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="H13:I13"/>
     <mergeCell ref="L22:M22"/>
+    <mergeCell ref="A22:B22"/>
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="H12:I12"/>
     <mergeCell ref="E16:F16"/>
@@ -3784,6 +3799,7 @@
     <mergeCell ref="E25:F25"/>
     <mergeCell ref="H18:I18"/>
     <mergeCell ref="L11:M11"/>
+    <mergeCell ref="E22:F22"/>
     <mergeCell ref="H8:I8"/>
     <mergeCell ref="C3:D3"/>
     <mergeCell ref="E21:F21"/>
@@ -27520,24 +27536,32 @@
       <formula>AND($AB7&lt;&gt;"",$AB7&lt;='Grundeinstellungen'!$C$11)</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="AD7:AD206">
+    <cfRule type="expression" priority="7" dxfId="0">
+      <formula>AND($AD7&lt;&gt;"",$AD7&gt;'Grundeinstellungen'!$C$22)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="1">
+      <formula>AND($AD7&lt;&gt;"",$AD7&lt;='Grundeinstellungen'!$C$22)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="AK7:AK206">
-    <cfRule type="expression" priority="7" dxfId="0">
+    <cfRule type="expression" priority="9" dxfId="0">
       <formula>AND($AK7&lt;&gt;"",$AK7&gt;'Grundeinstellungen'!$C$12)</formula>
     </cfRule>
-    <cfRule type="expression" priority="8" dxfId="1">
+    <cfRule type="expression" priority="10" dxfId="1">
       <formula>AND($AK7&lt;&gt;"",$AK7&lt;='Grundeinstellungen'!$C$12)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AE7:AE206">
-    <cfRule type="expression" priority="9" dxfId="0">
+    <cfRule type="expression" priority="11" dxfId="0">
       <formula>AND($AE7&lt;&gt;"",OR($AE7&lt;'Grundeinstellungen'!$C$20,$AE7&gt;'Grundeinstellungen'!$C$21))</formula>
     </cfRule>
-    <cfRule type="expression" priority="10" dxfId="1">
+    <cfRule type="expression" priority="12" dxfId="1">
       <formula>AND($AE7&lt;&gt;"",$AE7&gt;='Grundeinstellungen'!$C$20,$AE7&lt;='Grundeinstellungen'!$C$21)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H7:H206">
-    <cfRule type="expression" priority="11" dxfId="0">
+    <cfRule type="expression" priority="13" dxfId="0">
       <formula>AND($H7&lt;&gt;"",$D7&lt;&gt;"",$H7&gt;$D7)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -27569,7 +27593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -27602,17 +27626,17 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>Summen / Kennzahlen</t>
         </is>
       </c>
-      <c r="B5" s="28" t="n"/>
-      <c r="C5" s="28" t="n"/>
-      <c r="D5" s="28" t="n"/>
+      <c r="B5" s="27" t="n"/>
+      <c r="C5" s="27" t="n"/>
+      <c r="D5" s="27" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="29" t="inlineStr">
+      <c r="A6" s="28" t="inlineStr">
         <is>
           <t>Anzahl Räume</t>
         </is>
@@ -27621,14 +27645,14 @@
         <f>COUNTA('Auslegung'!B7:B206)</f>
         <v/>
       </c>
-      <c r="C6" s="31" t="inlineStr">
+      <c r="C6" s="30" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="29" t="inlineStr">
+      <c r="A7" s="28" t="inlineStr">
         <is>
           <t>Gesamte Heizlast</t>
         </is>
@@ -27637,14 +27661,14 @@
         <f>SUM('Auslegung'!F7:F206)</f>
         <v/>
       </c>
-      <c r="C7" s="31" t="inlineStr">
+      <c r="C7" s="30" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="29" t="inlineStr">
+      <c r="A8" s="28" t="inlineStr">
         <is>
           <t>Gesamte FBH-Leistung (nach oben)</t>
         </is>
@@ -27653,14 +27677,14 @@
         <f>SUM('Auslegung'!T7:T206)</f>
         <v/>
       </c>
-      <c r="C8" s="31" t="inlineStr">
+      <c r="C8" s="30" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="29" t="inlineStr">
+      <c r="A9" s="28" t="inlineStr">
         <is>
           <t>Verlustleistung nach unten</t>
         </is>
@@ -27669,14 +27693,14 @@
         <f>SUM('Auslegung'!W7:W206)</f>
         <v/>
       </c>
-      <c r="C9" s="31" t="inlineStr">
+      <c r="C9" s="30" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="29" t="inlineStr">
+      <c r="A10" s="28" t="inlineStr">
         <is>
           <t>Maßgebliche Gesamtleistung (Hydraulik)</t>
         </is>
@@ -27685,14 +27709,14 @@
         <f>SUM('Auslegung'!X7:X206)</f>
         <v/>
       </c>
-      <c r="C10" s="31" t="inlineStr">
+      <c r="C10" s="30" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="29" t="inlineStr">
+      <c r="A11" s="28" t="inlineStr">
         <is>
           <t>Deckungsgrad gesamt</t>
         </is>
@@ -27701,14 +27725,14 @@
         <f>IFERROR(B8/B7,0)</f>
         <v/>
       </c>
-      <c r="C11" s="31" t="inlineStr">
+      <c r="C11" s="30" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="29" t="inlineStr">
+      <c r="A12" s="28" t="inlineStr">
         <is>
           <t>Gesamte Rohrlänge</t>
         </is>
@@ -27717,14 +27741,14 @@
         <f>SUM('Auslegung'!AA7:AA206)</f>
         <v/>
       </c>
-      <c r="C12" s="31" t="inlineStr">
+      <c r="C12" s="30" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="29" t="inlineStr">
+      <c r="A13" s="28" t="inlineStr">
         <is>
           <t>Anzahl Heizkreise gesamt</t>
         </is>
@@ -27733,14 +27757,14 @@
         <f>SUM('Auslegung'!K7:K206)</f>
         <v/>
       </c>
-      <c r="C13" s="31" t="inlineStr">
+      <c r="C13" s="30" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="29" t="inlineStr">
+      <c r="A14" s="28" t="inlineStr">
         <is>
           <t>Gesamtmassenstrom (Pumpe)</t>
         </is>
@@ -27749,14 +27773,14 @@
         <f>SUM('Auslegung'!AC7:AC206)</f>
         <v/>
       </c>
-      <c r="C14" s="31" t="inlineStr">
+      <c r="C14" s="30" t="inlineStr">
         <is>
           <t>kg/h</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="29" t="inlineStr">
+      <c r="A15" s="28" t="inlineStr">
         <is>
           <t>Gesamtvolumenstrom (Pumpe)</t>
         </is>
@@ -27765,14 +27789,14 @@
         <f>SUM('Auslegung'!AD7:AD206)</f>
         <v/>
       </c>
-      <c r="C15" s="31" t="inlineStr">
+      <c r="C15" s="30" t="inlineStr">
         <is>
           <t>l/h</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="29" t="inlineStr">
+      <c r="A16" s="28" t="inlineStr">
         <is>
           <t>Max. Druckverlust eines Kreises</t>
         </is>
@@ -27781,14 +27805,14 @@
         <f>IFERROR(MAX('Auslegung'!AK7:AK206),0)</f>
         <v/>
       </c>
-      <c r="C16" s="31" t="inlineStr">
+      <c r="C16" s="30" t="inlineStr">
         <is>
           <t>Pa</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="29" t="inlineStr">
+      <c r="A17" s="28" t="inlineStr">
         <is>
           <t>Max. Strömungsgeschwindigkeit</t>
         </is>
@@ -27797,24 +27821,24 @@
         <f>IFERROR(MAX('Auslegung'!AE7:AE206),0)</f>
         <v/>
       </c>
-      <c r="C17" s="31" t="inlineStr">
+      <c r="C17" s="30" t="inlineStr">
         <is>
           <t>m/s</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="27" t="inlineStr">
+      <c r="A19" s="26" t="inlineStr">
         <is>
           <t>Warnungen</t>
         </is>
       </c>
-      <c r="B19" s="28" t="n"/>
-      <c r="C19" s="28" t="n"/>
-      <c r="D19" s="28" t="n"/>
+      <c r="B19" s="27" t="n"/>
+      <c r="C19" s="27" t="n"/>
+      <c r="D19" s="27" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="29" t="inlineStr">
+      <c r="A20" s="28" t="inlineStr">
         <is>
           <t>Räume unterdeckt</t>
         </is>
@@ -27823,19 +27847,19 @@
         <f>COUNTIF('Auslegung'!V7:V206,"&lt;1")</f>
         <v/>
       </c>
-      <c r="C20" s="31" t="inlineStr">
+      <c r="C20" s="30" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D20" s="32" t="inlineStr">
+      <c r="D20" s="31" t="inlineStr">
         <is>
           <t>Heizlast nicht gedeckt</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="29" t="inlineStr">
+      <c r="A21" s="28" t="inlineStr">
         <is>
           <t>Kreise zu lang</t>
         </is>
@@ -27844,19 +27868,19 @@
         <f>COUNTIF('Auslegung'!AB7:AB206,"&gt;"&amp;'Grundeinstellungen'!$C$11)</f>
         <v/>
       </c>
-      <c r="C21" s="31" t="inlineStr">
+      <c r="C21" s="30" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D21" s="32" t="inlineStr">
+      <c r="D21" s="31" t="inlineStr">
         <is>
           <t>&gt; max. Kreislänge</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="29" t="inlineStr">
+      <c r="A22" s="28" t="inlineStr">
         <is>
           <t>Druckverlust über Warnschwelle</t>
         </is>
@@ -27865,14 +27889,14 @@
         <f>COUNTIF('Auslegung'!AK7:AK206,"&gt;"&amp;'Grundeinstellungen'!$C$12)</f>
         <v/>
       </c>
-      <c r="C22" s="31" t="inlineStr">
+      <c r="C22" s="30" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="29" t="inlineStr">
+      <c r="A23" s="28" t="inlineStr">
         <is>
           <t>Oberflächentemperatur zu hoch</t>
         </is>
@@ -27881,14 +27905,14 @@
         <f>SUMPRODUCT(('Auslegung'!R7:R206&lt;&gt;"")*('Auslegung'!R7:R206&gt;'Auslegung'!S7:S206))</f>
         <v/>
       </c>
-      <c r="C23" s="31" t="inlineStr">
+      <c r="C23" s="30" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="29" t="inlineStr">
+      <c r="A24" s="28" t="inlineStr">
         <is>
           <t>Geschwindigkeit außerhalb v_min–v_max</t>
         </is>
@@ -27897,14 +27921,35 @@
         <f>SUMPRODUCT(('Auslegung'!AE7:AE206&lt;&gt;"")*(('Auslegung'!AE7:AE206&lt;'Grundeinstellungen'!$C$20)+('Auslegung'!AE7:AE206&gt;'Grundeinstellungen'!$C$21)))</f>
         <v/>
       </c>
-      <c r="C24" s="31" t="inlineStr">
+      <c r="C24" s="30" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D24" s="32" t="inlineStr">
+      <c r="D24" s="31" t="inlineStr">
         <is>
           <t>Kreise</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="28" t="inlineStr">
+        <is>
+          <t>Volumenstrom je Kreis zu hoch</t>
+        </is>
+      </c>
+      <c r="B25" s="79">
+        <f>COUNTIF('Auslegung'!AD7:AD206,"&gt;"&amp;'Grundeinstellungen'!$C$22)</f>
+        <v/>
+      </c>
+      <c r="C25" s="30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D25" s="31" t="inlineStr">
+        <is>
+          <t>&gt; max. Volumenstrom</t>
         </is>
       </c>
     </row>
@@ -27949,6 +27994,14 @@
       <formula>$B$24=0</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B25">
+    <cfRule type="expression" priority="11" dxfId="0">
+      <formula>$B$25&gt;0</formula>
+    </cfRule>
+    <cfRule type="expression" priority="12" dxfId="1">
+      <formula>$B$25=0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
@@ -29542,7 +29595,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="32" t="inlineStr">
+      <c r="A56" s="31" t="inlineStr">
         <is>
           <t>Baut sich automatisch aus der Auslegung auf (Array-Formeln, Excel &amp; LibreOffice).</t>
         </is>
@@ -29622,83 +29675,83 @@
       <c r="C5" s="90" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="32" t="inlineStr">
+      <c r="D5" s="31" t="inlineStr">
         <is>
           <t>← an Herstellerdaten anpassen</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="27" t="inlineStr">
+      <c r="A7" s="26" t="inlineStr">
         <is>
           <t>Vergleichsbedingungen (fix)</t>
         </is>
       </c>
-      <c r="B7" s="28" t="n"/>
-      <c r="C7" s="28" t="n"/>
+      <c r="B7" s="27" t="n"/>
+      <c r="C7" s="27" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="29" t="inlineStr">
+      <c r="A8" s="28" t="inlineStr">
         <is>
           <t>Vorlauftemperatur  θV</t>
         </is>
       </c>
-      <c r="B8" s="30" t="n">
+      <c r="B8" s="29" t="n">
         <v>35</v>
       </c>
-      <c r="C8" s="31" t="inlineStr">
+      <c r="C8" s="30" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="29" t="inlineStr">
+      <c r="A9" s="28" t="inlineStr">
         <is>
           <t>Rücklauftemperatur  θR</t>
         </is>
       </c>
-      <c r="B9" s="30" t="n">
+      <c r="B9" s="29" t="n">
         <v>28</v>
       </c>
-      <c r="C9" s="31" t="inlineStr">
+      <c r="C9" s="30" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="29" t="inlineStr">
+      <c r="A10" s="28" t="inlineStr">
         <is>
           <t>Raumtemperatur  θi</t>
         </is>
       </c>
-      <c r="B10" s="30" t="n">
+      <c r="B10" s="29" t="n">
         <v>20</v>
       </c>
-      <c r="C10" s="31" t="inlineStr">
+      <c r="C10" s="30" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="29" t="inlineStr">
+      <c r="A11" s="28" t="inlineStr">
         <is>
           <t>R-Wert Bodenbelag</t>
         </is>
       </c>
-      <c r="B11" s="34" t="n">
+      <c r="B11" s="33" t="n">
         <v>0.1</v>
       </c>
-      <c r="C11" s="31" t="inlineStr">
+      <c r="C11" s="30" t="inlineStr">
         <is>
           <t>m²K/W</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="32" t="inlineStr">
+      <c r="A12" s="31" t="inlineStr">
         <is>
           <t>q berechnet = f · η(VA) · K_H · ΔθH</t>
         </is>
@@ -30010,21 +30063,21 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="29" t="inlineStr">
+      <c r="A25" s="28" t="inlineStr">
         <is>
           <t>• Vergleich EINES Berechnungsmodells mit EINEM Herstellermodell über den Verlegeabstand.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="29" t="inlineStr">
+      <c r="A26" s="28" t="inlineStr">
         <is>
           <t>• Hersteller-q je Verlegeabstand aus dem Datenblatt in Spalte C eintragen.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="32" t="inlineStr">
+      <c r="A27" s="31" t="inlineStr">
         <is>
           <t>• Korrekturfaktor f oben so einstellen, dass die Linien übereinanderliegen (Abweichung grün).</t>
         </is>
@@ -30410,7 +30463,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="32" t="inlineStr">
+      <c r="A3" s="31" t="inlineStr">
         <is>
           <t>Nachschlage-Tabellen (editierbar). Leerzeilen = Platz für weitere Einträge.</t>
         </is>

</xml_diff>

<commit_message>
FBH-Auslegung v0.23 - groessere Formelzeichen, saubere Kopfzeilen-Umbrueche, Druck-Hinweis entfernt
Auslegung: Formelzeichen-Zeile groesser (Schriftgrad 13, Zeilenhoehe 20) - Tiefstellungen jetzt gut lesbar.

Auslegung: Kopfzeilen mit manuellen Umbruechen an Silben-/Wortgrenzen (Heizkreis-/verteiler, Raum-/bezeichnung, aktivier-/bare Flaeche, R-Wert/Bodenbelag, Zuleitungs-/laenge, spez. Heiz-/leistung, Ober-/flaechen-/temperatur, Druck-/verlust); Spalten E/I/L/Q/R leicht breiter, damit kein Umbruch mitten im Wort.

Deckblatt: Druck-Hinweis-Box wieder entfernt (print_area zurueck auf A1:K29).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FBH_Auslegung.xlsx
+++ b/FBH_Auslegung.xlsx
@@ -19,7 +19,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changelog" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Deckblatt'!$A$1:$K$33</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Deckblatt'!$A$1:$K$29</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Grundeinstellungen'!$A$1:$M$25</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Auslegung'!$1:$6</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Auslegung'!$A$1:$AK$206</definedName>
@@ -29,7 +29,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="6">'Anleitung'!$A$1:$D$32</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">'Methodik'!$A$1:$F$26</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="8">'Konstanten'!$A$1:$I$26</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="9">'Changelog'!$A$1:$C$82</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="9">'Changelog'!$A$1:$C$84</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -66,7 +66,7 @@
     <numFmt numFmtId="189" formatCode="#,##0&quot; l/h&quot;"/>
     <numFmt numFmtId="190" formatCode="0&quot; °C&quot;"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="24">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -124,7 +124,19 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="001F4E78"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -185,12 +197,6 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00B88600"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
@@ -342,44 +348,38 @@
   </cellStyleXfs>
   <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -450,7 +450,7 @@
     <xf numFmtId="9" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -465,37 +465,43 @@
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="177" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="177" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="178" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="178" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="172" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="171" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="179" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="179" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="180" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="180" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="181" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -570,26 +576,26 @@
     <xf numFmtId="189" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="171" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="15" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="172" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -598,17 +604,17 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="190" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="190" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="168" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -626,8 +632,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1484,7 +1490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1863,55 +1869,8 @@
       <c r="J29" s="16" t="n"/>
       <c r="K29" s="16" t="n"/>
     </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="17" t="inlineStr">
-        <is>
-          <t>Drucken – Auslegungsunterlagen</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="n"/>
-      <c r="C31" s="5" t="n"/>
-      <c r="D31" s="5" t="n"/>
-      <c r="E31" s="5" t="n"/>
-      <c r="F31" s="5" t="n"/>
-      <c r="G31" s="5" t="n"/>
-      <c r="H31" s="5" t="n"/>
-      <c r="I31" s="5" t="n"/>
-      <c r="J31" s="5" t="n"/>
-      <c r="K31" s="5" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="18" t="inlineStr">
-        <is>
-          <t>Für die Ausgabe der Auslegung die Blätter  Deckblatt · Grundeinstellungen · Auslegung · Kontrolle · HKV · Anleitung  mit Strg gemeinsam markieren und  Datei &gt; Drucken &gt; 'Aktive Blätter drucken'  wählen.   (Verifikation, Methodik, Konstanten und Changelog sind Referenz und werden dabei nicht mitgedruckt.)</t>
-        </is>
-      </c>
-      <c r="B32" s="11" t="n"/>
-      <c r="C32" s="11" t="n"/>
-      <c r="D32" s="11" t="n"/>
-      <c r="E32" s="11" t="n"/>
-      <c r="F32" s="11" t="n"/>
-      <c r="G32" s="11" t="n"/>
-      <c r="H32" s="11" t="n"/>
-      <c r="I32" s="11" t="n"/>
-      <c r="J32" s="11" t="n"/>
-      <c r="K32" s="11" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="11" t="n"/>
-      <c r="B33" s="11" t="n"/>
-      <c r="C33" s="11" t="n"/>
-      <c r="D33" s="11" t="n"/>
-      <c r="E33" s="11" t="n"/>
-      <c r="F33" s="11" t="n"/>
-      <c r="G33" s="11" t="n"/>
-      <c r="H33" s="11" t="n"/>
-      <c r="I33" s="11" t="n"/>
-      <c r="J33" s="11" t="n"/>
-      <c r="K33" s="11" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="13">
     <mergeCell ref="E6:G24"/>
     <mergeCell ref="A6:C24"/>
     <mergeCell ref="A3:K3"/>
@@ -1923,10 +1882,8 @@
     <mergeCell ref="H6:H24"/>
     <mergeCell ref="A27:K29"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A32:K33"/>
     <mergeCell ref="D6:D24"/>
     <mergeCell ref="I6:K24"/>
-    <mergeCell ref="A31:K31"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.3" top="0.3" bottom="0.3" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
@@ -1940,7 +1897,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C82"/>
+  <dimension ref="A1:C84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1949,16 +1906,16 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>Changelog – FBH-Auslegung</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="C3" s="23" t="inlineStr">
-        <is>
-          <t>Version 0.22 · dh</t>
+      <c r="C3" s="21" t="inlineStr">
+        <is>
+          <t>Version 0.23 · dh</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1939,7 @@
     <row r="6">
       <c r="A6" s="104" t="inlineStr">
         <is>
-          <t>0.22</t>
+          <t>0.23</t>
         </is>
       </c>
       <c r="B6" s="105" t="inlineStr">
@@ -1992,7 +1949,7 @@
       </c>
       <c r="C6" s="106" t="inlineStr">
         <is>
-          <t>• Anleitung: neue Ampel-Legende (warum ist eine Zelle rot?) und Hinweis zur Auslegung mehrerer Verteiler/Geschosse; Blatt nach hinten verschoben (jetzt vor der Methodik).</t>
+          <t>• Auslegung: Formelzeichen größer (besser lesbare Tiefstellungen); Kopfzeilen-Umbrüche optimiert – keine Trennung mehr mitten im Wort.</t>
         </is>
       </c>
     </row>
@@ -2001,33 +1958,33 @@
       <c r="B7" s="107" t="n"/>
       <c r="C7" s="106" t="inlineStr">
         <is>
+          <t>• Deckblatt: Druck-Hinweis wieder entfernt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="104" t="inlineStr">
+        <is>
+          <t>0.22</t>
+        </is>
+      </c>
+      <c r="B8" s="105" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="C8" s="106" t="inlineStr">
+        <is>
+          <t>• Anleitung: neue Ampel-Legende (warum ist eine Zelle rot?) und Hinweis zur Auslegung mehrerer Verteiler/Geschosse; Blatt nach hinten verschoben (jetzt vor der Methodik).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="108" t="n"/>
+      <c r="B9" s="108" t="n"/>
+      <c r="C9" s="106" t="inlineStr">
+        <is>
           <t>• Deckblatt: Druck-Hinweis ergänzt – nur die relevanten Blätter (Deckblatt, Grundeinstellungen, Auslegung, Kontrolle, HKV, Anleitung) gemeinsam als 'Aktive Blätter' drucken.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="108" t="n"/>
-      <c r="B8" s="108" t="n"/>
-      <c r="C8" s="106" t="inlineStr">
-        <is>
-          <t>• Formelzeichen mit echten Tiefstellungen dargestellt (z. B. q_HL, R_λ,B, V̇_max) – kein Unterstrich mehr in den Kopfzeilen, Grundeinstellungen und der Methodik-Variablenliste.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="104" t="inlineStr">
-        <is>
-          <t>0.21</t>
-        </is>
-      </c>
-      <c r="B9" s="105" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="C9" s="106" t="inlineStr">
-        <is>
-          <t>• Auslegung jetzt auf A4-Querformat (vorher A3); sichtbare Spalten schmaler, damit das Blatt auf A4 passt.</t>
         </is>
       </c>
     </row>
@@ -2036,33 +1993,33 @@
       <c r="B10" s="107" t="n"/>
       <c r="C10" s="106" t="inlineStr">
         <is>
+          <t>• Formelzeichen mit echten Tiefstellungen dargestellt (z. B. q_HL, R_λ,B, V̇_max) – kein Unterstrich mehr in den Kopfzeilen, Grundeinstellungen und der Methodik-Variablenliste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="104" t="inlineStr">
+        <is>
+          <t>0.21</t>
+        </is>
+      </c>
+      <c r="B11" s="105" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="C11" s="106" t="inlineStr">
+        <is>
+          <t>• Auslegung jetzt auf A4-Querformat (vorher A3); sichtbare Spalten schmaler, damit das Blatt auf A4 passt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="108" t="n"/>
+      <c r="B12" s="108" t="n"/>
+      <c r="C12" s="106" t="inlineStr">
+        <is>
           <t>• Deckblatt: Titel 'Fußbodenheizung – Auslegung' (Wort 'überschlägige' entfernt); Vereinfachungen bleiben dokumentiert.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="108" t="n"/>
-      <c r="B11" s="108" t="n"/>
-      <c r="C11" s="106" t="inlineStr">
-        <is>
-          <t>• Anleitung: Abschnitt 'Planungstechnische Grundlagen' wieder entfernt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="104" t="inlineStr">
-        <is>
-          <t>0.20</t>
-        </is>
-      </c>
-      <c r="B12" s="105" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="C12" s="106" t="inlineStr">
-        <is>
-          <t>• Grundeinstellungen: Spaltenbreiten optimiert und lange Beschriftungen/Hinweise gekürzt – Texte werden in LibreOffice nicht mehr abgeschnitten.</t>
         </is>
       </c>
     </row>
@@ -2071,33 +2028,33 @@
       <c r="B13" s="107" t="n"/>
       <c r="C13" s="106" t="inlineStr">
         <is>
+          <t>• Anleitung: Abschnitt 'Planungstechnische Grundlagen' wieder entfernt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="104" t="inlineStr">
+        <is>
+          <t>0.20</t>
+        </is>
+      </c>
+      <c r="B14" s="105" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="C14" s="106" t="inlineStr">
+        <is>
+          <t>• Grundeinstellungen: Spaltenbreiten optimiert und lange Beschriftungen/Hinweise gekürzt – Texte werden in LibreOffice nicht mehr abgeschnitten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="108" t="n"/>
+      <c r="B15" s="108" t="n"/>
+      <c r="C15" s="106" t="inlineStr">
+        <is>
           <t>• Verifikation: Untertitel und Hinweise vereinfacht (Modellvergleich-Erläuterung entfernt); klarer Hinweis, dass der Korrekturfaktor f VOR der Raumauslegung kalibriert wird; Diagramm etwas größer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="108" t="n"/>
-      <c r="B14" s="108" t="n"/>
-      <c r="C14" s="106" t="inlineStr">
-        <is>
-          <t>• Anleitung: Schritt-für-Schritt neu geordnet – Verifikation/Kalibrierung des Korrekturfaktors jetzt VOR der Raumauslegung; neuer Abschnitt 'Planungstechnische Grundlagen'; Hinweis zur vorgefertigten Revit-Liste entfernt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="104" t="inlineStr">
-        <is>
-          <t>0.19</t>
-        </is>
-      </c>
-      <c r="B15" s="105" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="C15" s="106" t="inlineStr">
-        <is>
-          <t>• Grundeinstellungen: neuer Grenzwert 'Maximaler Volumenstrom je Kreis' (V̇_max, Default 150 l/h); Abschnitt 'Strömungsgeschwindigkeit' → 'Strömungsgrenzwerte'.</t>
         </is>
       </c>
     </row>
@@ -2106,16 +2063,24 @@
       <c r="B16" s="107" t="n"/>
       <c r="C16" s="106" t="inlineStr">
         <is>
-          <t>• Auslegung: Volumenstrom je Kreis wird gegen V̇_max geprüft und per Ampel eingefärbt (grün ≤ Grenze, rot darüber); zusätzliche Warnung im Blatt 'Kontrolle'.</t>
+          <t>• Anleitung: Schritt-für-Schritt neu geordnet – Verifikation/Kalibrierung des Korrekturfaktors jetzt VOR der Raumauslegung; neuer Abschnitt 'Planungstechnische Grundlagen'; Hinweis zur vorgefertigten Revit-Liste entfernt.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="107" t="n"/>
-      <c r="B17" s="107" t="n"/>
+      <c r="A17" s="104" t="inlineStr">
+        <is>
+          <t>0.19</t>
+        </is>
+      </c>
+      <c r="B17" s="105" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
       <c r="C17" s="106" t="inlineStr">
         <is>
-          <t>• Anleitung: durchgehende Schritt-für-Schritt-Anleitung mit integriertem Revit-Export (vorgefertigte Bauteilliste muss nicht erst angelegt werden); redundanter Abschnitt 'Räume aus Revit' und der Hinweis zum direkten Kopieren entfernt.</t>
+          <t>• Grundeinstellungen: neuer Grenzwert 'Maximaler Volumenstrom je Kreis' (V̇_max, Default 150 l/h); Abschnitt 'Strömungsgeschwindigkeit' → 'Strömungsgrenzwerte'.</t>
         </is>
       </c>
     </row>
@@ -2124,40 +2089,32 @@
       <c r="B18" s="108" t="n"/>
       <c r="C18" s="106" t="inlineStr">
         <is>
+          <t>• Auslegung: Volumenstrom je Kreis wird gegen V̇_max geprüft und per Ampel eingefärbt (grün ≤ Grenze, rot darüber); zusätzliche Warnung im Blatt 'Kontrolle'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="108" t="n"/>
+      <c r="B19" s="108" t="n"/>
+      <c r="C19" s="106" t="inlineStr">
+        <is>
+          <t>• Anleitung: durchgehende Schritt-für-Schritt-Anleitung mit integriertem Revit-Export (vorgefertigte Bauteilliste muss nicht erst angelegt werden); redundanter Abschnitt 'Räume aus Revit' und der Hinweis zum direkten Kopieren entfernt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="107" t="n"/>
+      <c r="B20" s="107" t="n"/>
+      <c r="C20" s="106" t="inlineStr">
+        <is>
           <t>• Deckblatt: Pfeil-Spalten breiter und Pfeilgröße angepasst (optisch sauberer).</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="104" t="inlineStr">
-        <is>
-          <t>0.18</t>
-        </is>
-      </c>
-      <c r="B19" s="105" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="C19" s="106" t="inlineStr">
-        <is>
-          <t>• Auslegung: Eingabespalten neu sortiert – zuerst die Revit-Spalten (A HKV, B Raum-Nr., C Bezeichnung, D Raumfläche, E Raumtemperatur, F Heizlast), dann G spez. Heizlast (berechnet), danach die manuellen Felder (H aktiv. Fläche, I R-Wert, J Verlegeabstand, K Anz. Kreise, L Zuleitung, M Zone).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="108" t="n"/>
-      <c r="B20" s="108" t="n"/>
-      <c r="C20" s="106" t="inlineStr">
-        <is>
-          <t>• Anleitung: Excel-Export aus Revit ist jetzt der Standard-Workflow (direktes Kopieren funktioniert nicht); Spaltenliste an neue Reihenfolge angepasst.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="104" t="inlineStr">
         <is>
-          <t>0.17</t>
+          <t>0.18</t>
         </is>
       </c>
       <c r="B21" s="105" t="inlineStr">
@@ -2167,33 +2124,33 @@
       </c>
       <c r="C21" s="106" t="inlineStr">
         <is>
-          <t>• Neues Blatt 'Anleitung' (2. Blatt): Aufbau der Mappe, Schritt-für-Schritt, Farblegende.</t>
+          <t>• Auslegung: Eingabespalten neu sortiert – zuerst die Revit-Spalten (A HKV, B Raum-Nr., C Bezeichnung, D Raumfläche, E Raumtemperatur, F Heizlast), dann G spez. Heizlast (berechnet), danach die manuellen Felder (H aktiv. Fläche, I R-Wert, J Verlegeabstand, K Anz. Kreise, L Zuleitung, M Zone).</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="108" t="n"/>
-      <c r="B22" s="108" t="n"/>
+      <c r="A22" s="107" t="n"/>
+      <c r="B22" s="107" t="n"/>
       <c r="C22" s="106" t="inlineStr">
         <is>
-          <t>• Anleitung enthält den Workflow zum Übernehmen der Räume aus Revit (Copy &amp; Paste, Schedule, Dynamo/Power Query).</t>
+          <t>• Anleitung: Excel-Export aus Revit ist jetzt der Standard-Workflow (direktes Kopieren funktioniert nicht); Spaltenliste an neue Reihenfolge angepasst.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="104" t="inlineStr">
         <is>
-          <t>0.16</t>
+          <t>0.17</t>
         </is>
       </c>
       <c r="B23" s="105" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="C23" s="106" t="inlineStr">
         <is>
-          <t>• Alle Blätter im A4-Querformat (nur Auslegung A3 quer); einheitlichere Schriftgrößen/Skalierung.</t>
+          <t>• Neues Blatt 'Anleitung' (2. Blatt): Aufbau der Mappe, Schritt-für-Schritt, Farblegende.</t>
         </is>
       </c>
     </row>
@@ -2202,34 +2159,42 @@
       <c r="B24" s="107" t="n"/>
       <c r="C24" s="106" t="inlineStr">
         <is>
+          <t>• Anleitung enthält den Workflow zum Übernehmen der Räume aus Revit (Copy &amp; Paste, Schedule, Dynamo/Power Query).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="104" t="inlineStr">
+        <is>
+          <t>0.16</t>
+        </is>
+      </c>
+      <c r="B25" s="105" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="C25" s="106" t="inlineStr">
+        <is>
+          <t>• Alle Blätter im A4-Querformat (nur Auslegung A3 quer); einheitlichere Schriftgrößen/Skalierung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="108" t="n"/>
+      <c r="B26" s="108" t="n"/>
+      <c r="C26" s="106" t="inlineStr">
+        <is>
           <t>• Grundeinstellungen zweispaltig (Einstellwerte teilweise nebeneinander).</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="107" t="n"/>
-      <c r="B25" s="107" t="n"/>
-      <c r="C25" s="106" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="108" t="n"/>
+      <c r="B27" s="108" t="n"/>
+      <c r="C27" s="106" t="inlineStr">
         <is>
           <t>• Verifikation: Diagramm rechts neben den Tabellen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="107" t="n"/>
-      <c r="B26" s="107" t="n"/>
-      <c r="C26" s="106" t="inlineStr">
-        <is>
-          <t>• Methodik: Formelzeichen links, Berechnungsschritte in zwei Spalten rechts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="107" t="n"/>
-      <c r="B27" s="107" t="n"/>
-      <c r="C27" s="106" t="inlineStr">
-        <is>
-          <t>• Konstanten: Tabellen teilweise nebeneinander.</t>
         </is>
       </c>
     </row>
@@ -2238,24 +2203,16 @@
       <c r="B28" s="108" t="n"/>
       <c r="C28" s="106" t="inlineStr">
         <is>
-          <t>• Auslegung: Spalte Zone mittig/schmaler, Raum-Nr. breiter; Verifikation-Korrekturfaktor vertikal mittig.</t>
+          <t>• Methodik: Formelzeichen links, Berechnungsschritte in zwei Spalten rechts.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="104" t="inlineStr">
-        <is>
-          <t>0.15</t>
-        </is>
-      </c>
-      <c r="B29" s="105" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
+      <c r="A29" s="108" t="n"/>
+      <c r="B29" s="108" t="n"/>
       <c r="C29" s="106" t="inlineStr">
         <is>
-          <t>• Deckblatt-Diagramm aus Excel-Zellen statt Bild – direkt in Excel bearbeitbar.</t>
+          <t>• Konstanten: Tabellen teilweise nebeneinander.</t>
         </is>
       </c>
     </row>
@@ -2264,77 +2221,85 @@
       <c r="B30" s="107" t="n"/>
       <c r="C30" s="106" t="inlineStr">
         <is>
+          <t>• Auslegung: Spalte Zone mittig/schmaler, Raum-Nr. breiter; Verifikation-Korrekturfaktor vertikal mittig.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="104" t="inlineStr">
+        <is>
+          <t>0.15</t>
+        </is>
+      </c>
+      <c r="B31" s="105" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="C31" s="106" t="inlineStr">
+        <is>
+          <t>• Deckblatt-Diagramm aus Excel-Zellen statt Bild – direkt in Excel bearbeitbar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="108" t="n"/>
+      <c r="B32" s="108" t="n"/>
+      <c r="C32" s="106" t="inlineStr">
+        <is>
           <t>• Auslegung: Beispielräume mit gemischter Heizlast (≤ 50 W/m²); Formelzeichen in Zeile 5 ergänzt (Flächen u. a.).</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="108" t="n"/>
-      <c r="B31" s="108" t="n"/>
-      <c r="C31" s="106" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="107" t="n"/>
+      <c r="B33" s="107" t="n"/>
+      <c r="C33" s="106" t="inlineStr">
         <is>
           <t>• Heizkreisverteiler: zusätzliche Spalte Spreizung [K].</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="104" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="104" t="inlineStr">
         <is>
           <t>0.14</t>
         </is>
       </c>
-      <c r="B32" s="105" t="inlineStr">
+      <c r="B34" s="105" t="inlineStr">
         <is>
           <t>2026-06-09</t>
         </is>
       </c>
-      <c r="C32" s="106" t="inlineStr">
+      <c r="C34" s="106" t="inlineStr">
         <is>
           <t>• Deckblatt als erstes Blatt: Übersichtsdiagramm Eingaben → Verarbeitung → Ergebnisse (inkl. Vereinfachungen).</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="104" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="104" t="inlineStr">
         <is>
           <t>0.13</t>
         </is>
       </c>
-      <c r="B33" s="105" t="inlineStr">
+      <c r="B35" s="105" t="inlineStr">
         <is>
           <t>2026-06-08</t>
         </is>
       </c>
-      <c r="C33" s="106" t="inlineStr">
+      <c r="C35" s="106" t="inlineStr">
         <is>
           <t>• Strömungsbereich dreistufig: laminar (Re &lt; 2300), Übergangsbereich (2300–4000), turbulent (Re &gt; 4000).</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="107" t="n"/>
-      <c r="B34" s="107" t="n"/>
-      <c r="C34" s="106" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="108" t="n"/>
+      <c r="B36" s="108" t="n"/>
+      <c r="C36" s="106" t="inlineStr">
         <is>
           <t>• Spalte 'Strömungsbereich' ausgeblendet (für die Auslegung nicht relevant) und ohne Färbung.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="107" t="n"/>
-      <c r="B35" s="107" t="n"/>
-      <c r="C35" s="106" t="inlineStr">
-        <is>
-          <t>• Auslegung schlanker: weitere Zwischenspalten standardmäßig ausgeblendet (jederzeit einblendbar).</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="107" t="n"/>
-      <c r="B36" s="107" t="n"/>
-      <c r="C36" s="106" t="inlineStr">
-        <is>
-          <t>• Verifikation: Korrekturfaktor kleiner dargestellt (passt nun vollständig in die Zelle).</t>
         </is>
       </c>
     </row>
@@ -2343,24 +2308,16 @@
       <c r="B37" s="108" t="n"/>
       <c r="C37" s="106" t="inlineStr">
         <is>
-          <t>• Changelog wieder ausführlich.</t>
+          <t>• Auslegung schlanker: weitere Zwischenspalten standardmäßig ausgeblendet (jederzeit einblendbar).</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="104" t="inlineStr">
-        <is>
-          <t>0.12</t>
-        </is>
-      </c>
-      <c r="B38" s="105" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
+      <c r="A38" s="108" t="n"/>
+      <c r="B38" s="108" t="n"/>
       <c r="C38" s="106" t="inlineStr">
         <is>
-          <t>• Grundeinstellungen: Bezeichnungen ausgeschrieben (keine Abkürzungen).</t>
+          <t>• Verifikation: Korrekturfaktor kleiner dargestellt (passt nun vollständig in die Zelle).</t>
         </is>
       </c>
     </row>
@@ -2369,25 +2326,33 @@
       <c r="B39" s="107" t="n"/>
       <c r="C39" s="106" t="inlineStr">
         <is>
+          <t>• Changelog wieder ausführlich.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="104" t="inlineStr">
+        <is>
+          <t>0.12</t>
+        </is>
+      </c>
+      <c r="B40" s="105" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C40" s="106" t="inlineStr">
+        <is>
+          <t>• Grundeinstellungen: Bezeichnungen ausgeschrieben (keine Abkürzungen).</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="108" t="n"/>
+      <c r="B41" s="108" t="n"/>
+      <c r="C41" s="106" t="inlineStr">
+        <is>
           <t>• Neue Spalte 'spez. Heizlast [W/m²]' (Heizlast bezogen auf die Raumfläche).</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="107" t="n"/>
-      <c r="B40" s="107" t="n"/>
-      <c r="C40" s="106" t="inlineStr">
-        <is>
-          <t>• Massenstrom/Geschwindigkeit/Druckverlust auf Basis min(Leistung; Heizlast) + Verlust nach unten (realer Betriebspunkt).</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="107" t="n"/>
-      <c r="B41" s="107" t="n"/>
-      <c r="C41" s="106" t="inlineStr">
-        <is>
-          <t>• Heizkreisverteiler zusätzlich mit Massenstrom [kg/h]; Zonen-Kürzel (AZ/RZ/BAD).</t>
         </is>
       </c>
     </row>
@@ -2396,24 +2361,16 @@
       <c r="B42" s="108" t="n"/>
       <c r="C42" s="106" t="inlineStr">
         <is>
-          <t>• Kapazität 200 Räume / 50 Verteiler; Auslegung A3 quer, übrige Blätter A4 hoch.</t>
+          <t>• Massenstrom/Geschwindigkeit/Druckverlust auf Basis min(Leistung; Heizlast) + Verlust nach unten (realer Betriebspunkt).</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="104" t="inlineStr">
-        <is>
-          <t>0.11</t>
-        </is>
-      </c>
-      <c r="B43" s="105" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
+      <c r="A43" s="108" t="n"/>
+      <c r="B43" s="108" t="n"/>
       <c r="C43" s="106" t="inlineStr">
         <is>
-          <t>• Bugfixes: Hinweistext wurde als Formel interpretiert (Fehler 501); MAXIFS ersetzt (#NAME? in LibreOffice).</t>
+          <t>• Heizkreisverteiler zusätzlich mit Massenstrom [kg/h]; Zonen-Kürzel (AZ/RZ/BAD).</t>
         </is>
       </c>
     </row>
@@ -2422,16 +2379,24 @@
       <c r="B44" s="107" t="n"/>
       <c r="C44" s="106" t="inlineStr">
         <is>
-          <t>• Verifikation: Korrekturfaktor prominent oben; Hersteller-q direkt neben q berechnet.</t>
+          <t>• Kapazität 200 Räume / 50 Verteiler; Auslegung A3 quer, übrige Blätter A4 hoch.</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="107" t="n"/>
-      <c r="B45" s="107" t="n"/>
+      <c r="A45" s="104" t="inlineStr">
+        <is>
+          <t>0.11</t>
+        </is>
+      </c>
+      <c r="B45" s="105" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
       <c r="C45" s="106" t="inlineStr">
         <is>
-          <t>• Konstanten: alle Tabellen untereinander, mit Leerzeilen für weitere Einträge.</t>
+          <t>• Bugfixes: Hinweistext wurde als Formel interpretiert (Fehler 501); MAXIFS ersetzt (#NAME? in LibreOffice).</t>
         </is>
       </c>
     </row>
@@ -2440,24 +2405,16 @@
       <c r="B46" s="108" t="n"/>
       <c r="C46" s="106" t="inlineStr">
         <is>
-          <t>• Methodik: Variablen zuerst, dann Formeln mit Erklärung je Schritt; weitere Musterräume (Verwaltungsbau).</t>
+          <t>• Verifikation: Korrekturfaktor prominent oben; Hersteller-q direkt neben q berechnet.</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="104" t="inlineStr">
-        <is>
-          <t>0.10</t>
-        </is>
-      </c>
-      <c r="B47" s="105" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
+      <c r="A47" s="108" t="n"/>
+      <c r="B47" s="108" t="n"/>
       <c r="C47" s="106" t="inlineStr">
         <is>
-          <t>• Heizkreisverteiler-Liste und Verifikation ohne dynamische Array-Funktionen → läuft in Excel UND LibreOffice.</t>
+          <t>• Konstanten: alle Tabellen untereinander, mit Leerzeilen für weitere Einträge.</t>
         </is>
       </c>
     </row>
@@ -2466,33 +2423,33 @@
       <c r="B48" s="107" t="n"/>
       <c r="C48" s="106" t="inlineStr">
         <is>
+          <t>• Methodik: Variablen zuerst, dann Formeln mit Erklärung je Schritt; weitere Musterräume (Verwaltungsbau).</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="104" t="inlineStr">
+        <is>
+          <t>0.10</t>
+        </is>
+      </c>
+      <c r="B49" s="105" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C49" s="106" t="inlineStr">
+        <is>
+          <t>• Heizkreisverteiler-Liste und Verifikation ohne dynamische Array-Funktionen → läuft in Excel UND LibreOffice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="108" t="n"/>
+      <c r="B50" s="108" t="n"/>
+      <c r="C50" s="106" t="inlineStr">
+        <is>
           <t>• Verifikation mit Liniendiagramm; Konstanten/Bibliotheken in eigenes Blatt ausgelagert.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="108" t="n"/>
-      <c r="B49" s="108" t="n"/>
-      <c r="C49" s="106" t="inlineStr">
-        <is>
-          <t>• Gewähltes Rohrsystem mit Außen-/Innendurchmesser, Wandstärke und Rauheit im Druckbereich.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="104" t="inlineStr">
-        <is>
-          <t>0.9</t>
-        </is>
-      </c>
-      <c r="B50" s="105" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C50" s="106" t="inlineStr">
-        <is>
-          <t>• Neues Blatt 'Heizkreisverteiler' (Leistung, max. Druckverlust, Volumenstrom je HKV).</t>
         </is>
       </c>
     </row>
@@ -2501,16 +2458,24 @@
       <c r="B51" s="107" t="n"/>
       <c r="C51" s="106" t="inlineStr">
         <is>
-          <t>• Spaltenüberschriften der Auslegung dreizeilig (Name / Formelzeichen / Einheit).</t>
+          <t>• Gewähltes Rohrsystem mit Außen-/Innendurchmesser, Wandstärke und Rauheit im Druckbereich.</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="107" t="n"/>
-      <c r="B52" s="107" t="n"/>
+      <c r="A52" s="104" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="B52" s="105" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
       <c r="C52" s="106" t="inlineStr">
         <is>
-          <t>• Korrekturfaktor f wird auf 'Verifikation' eingegeben (mit Vergleichsdiagramm).</t>
+          <t>• Neues Blatt 'Heizkreisverteiler' (Leistung, max. Druckverlust, Volumenstrom je HKV).</t>
         </is>
       </c>
     </row>
@@ -2519,24 +2484,16 @@
       <c r="B53" s="108" t="n"/>
       <c r="C53" s="106" t="inlineStr">
         <is>
-          <t>• Geschwindigkeits-Grenzwerte v_min/v_max als Grundeinstellung.</t>
+          <t>• Spaltenüberschriften der Auslegung dreizeilig (Name / Formelzeichen / Einheit).</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="104" t="inlineStr">
-        <is>
-          <t>0.8</t>
-        </is>
-      </c>
-      <c r="B54" s="105" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
+      <c r="A54" s="108" t="n"/>
+      <c r="B54" s="108" t="n"/>
       <c r="C54" s="106" t="inlineStr">
         <is>
-          <t>• Grundeinstellungen für A3 quer optimiert (Einstellungen links, Tabellen rechts).</t>
+          <t>• Korrekturfaktor f wird auf 'Verifikation' eingegeben (mit Vergleichsdiagramm).</t>
         </is>
       </c>
     </row>
@@ -2545,16 +2502,24 @@
       <c r="B55" s="107" t="n"/>
       <c r="C55" s="106" t="inlineStr">
         <is>
-          <t>• Auslegung passt auf eine Seite breit; Korrekturfaktor Heizleistung zur Kalibrierung ergänzt.</t>
+          <t>• Geschwindigkeits-Grenzwerte v_min/v_max als Grundeinstellung.</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="107" t="n"/>
-      <c r="B56" s="107" t="n"/>
+      <c r="A56" s="104" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="B56" s="105" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
       <c r="C56" s="106" t="inlineStr">
         <is>
-          <t>• Wärmeabgabe nach unten berücksichtigt (Verlust + Gesamtleistung).</t>
+          <t>• Grundeinstellungen für A3 quer optimiert (Einstellungen links, Tabellen rechts).</t>
         </is>
       </c>
     </row>
@@ -2563,24 +2528,16 @@
       <c r="B57" s="108" t="n"/>
       <c r="C57" s="106" t="inlineStr">
         <is>
-          <t>• Blätter umbenannt: Raumliste → Auslegung, Übersicht → Kontrolle; zusätzliche Kontrollen.</t>
+          <t>• Auslegung passt auf eine Seite breit; Korrekturfaktor Heizleistung zur Kalibrierung ergänzt.</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="104" t="inlineStr">
-        <is>
-          <t>0.7</t>
-        </is>
-      </c>
-      <c r="B58" s="105" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
+      <c r="A58" s="108" t="n"/>
+      <c r="B58" s="108" t="n"/>
       <c r="C58" s="106" t="inlineStr">
         <is>
-          <t>• Deckung-%-Spalte färbt nur noch gefüllte Zellen (leere bleiben farblos).</t>
+          <t>• Wärmeabgabe nach unten berücksichtigt (Verlust + Gesamtleistung).</t>
         </is>
       </c>
     </row>
@@ -2589,66 +2546,66 @@
       <c r="B59" s="107" t="n"/>
       <c r="C59" s="106" t="inlineStr">
         <is>
+          <t>• Blätter umbenannt: Raumliste → Auslegung, Übersicht → Kontrolle; zusätzliche Kontrollen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="104" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="B60" s="105" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="C60" s="106" t="inlineStr">
+        <is>
+          <t>• Deckung-%-Spalte färbt nur noch gefüllte Zellen (leere bleiben farblos).</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="108" t="n"/>
+      <c r="B61" s="108" t="n"/>
+      <c r="C61" s="106" t="inlineStr">
+        <is>
           <t>• Neues Blatt 'Verifikation'; neue Spalte 'Strömungsbereich' (laminar/turbulent).</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="108" t="n"/>
-      <c r="B60" s="108" t="n"/>
-      <c r="C60" s="106" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="107" t="n"/>
+      <c r="B62" s="107" t="n"/>
+      <c r="C62" s="106" t="inlineStr">
         <is>
           <t>• Alle Blätter im A3-Querformat; einheitlicher Kopf je Blatt.</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="104" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="104" t="inlineStr">
         <is>
           <t>0.6</t>
         </is>
       </c>
-      <c r="B61" s="105" t="inlineStr">
+      <c r="B63" s="105" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="C61" s="106" t="inlineStr">
+      <c r="C63" s="106" t="inlineStr">
         <is>
           <t>• Bugfix: Zellfärbung (bedingte Formatierung) wird jetzt auch in Excel angezeigt – dxf-Füllfarbe mit voller Deckkraft.</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="104" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
-      </c>
-      <c r="B62" s="105" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C62" s="106" t="inlineStr">
-        <is>
-          <t>• Versionsnummer und Autor werden nur noch im Changelog angezeigt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="108" t="n"/>
-      <c r="B63" s="108" t="n"/>
-      <c r="C63" s="106" t="inlineStr">
-        <is>
-          <t>• Editierbares Bearbeiter-Kürzel rechts oben unter dem Logo (Grundeinstellungen, Auslegung, Kontrolle, HKV).</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="104" t="inlineStr">
         <is>
-          <t>0.4</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="B64" s="105" t="inlineStr">
@@ -2658,7 +2615,7 @@
       </c>
       <c r="C64" s="106" t="inlineStr">
         <is>
-          <t>• Status-Spalten entfernt – Bewertung erfolgt jetzt direkt als Zellfärbung (grün/rot).</t>
+          <t>• Versionsnummer und Autor werden nur noch im Changelog angezeigt.</t>
         </is>
       </c>
     </row>
@@ -2667,16 +2624,24 @@
       <c r="B65" s="107" t="n"/>
       <c r="C65" s="106" t="inlineStr">
         <is>
-          <t>• Methodik um die Formelzeichen-Legende erweitert.</t>
+          <t>• Editierbares Bearbeiter-Kürzel rechts oben unter dem Logo (Grundeinstellungen, Auslegung, Kontrolle, HKV).</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="107" t="n"/>
-      <c r="B66" s="107" t="n"/>
+      <c r="A66" s="104" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="B66" s="105" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
       <c r="C66" s="106" t="inlineStr">
         <is>
-          <t>• Heizkreisverteiler (HKV) als erste Spalte der Auslegung; Standardwert max. Druckverlust 15.000 Pa.</t>
+          <t>• Status-Spalten entfernt – Bewertung erfolgt jetzt direkt als Zellfärbung (grün/rot).</t>
         </is>
       </c>
     </row>
@@ -2685,24 +2650,16 @@
       <c r="B67" s="108" t="n"/>
       <c r="C67" s="106" t="inlineStr">
         <is>
-          <t>• Versionsschema 0.x eingeführt (1.0 erst nach Test); interner Autor (dh).</t>
+          <t>• Methodik um die Formelzeichen-Legende erweitert.</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="104" t="inlineStr">
-        <is>
-          <t>0.3</t>
-        </is>
-      </c>
-      <c r="B68" s="105" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
+      <c r="A68" s="108" t="n"/>
+      <c r="B68" s="108" t="n"/>
       <c r="C68" s="106" t="inlineStr">
         <is>
-          <t>• Zonentypen (Aufenthalt/Rand/Bad) mit eigener zulässiger Oberflächentemperatur.</t>
+          <t>• Heizkreisverteiler (HKV) als erste Spalte der Auslegung; Standardwert max. Druckverlust 15.000 Pa.</t>
         </is>
       </c>
     </row>
@@ -2711,25 +2668,33 @@
       <c r="B69" s="107" t="n"/>
       <c r="C69" s="106" t="inlineStr">
         <is>
+          <t>• Versionsschema 0.x eingeführt (1.0 erst nach Test); interner Autor (dh).</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="104" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="B70" s="105" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="C70" s="106" t="inlineStr">
+        <is>
+          <t>• Zonentypen (Aufenthalt/Rand/Bad) mit eigener zulässiger Oberflächentemperatur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="108" t="n"/>
+      <c r="B71" s="108" t="n"/>
+      <c r="C71" s="106" t="inlineStr">
+        <is>
           <t>• Einheitlicher Kopf: Titel oben links, agn-Logo oben rechts, Projektkopf darunter.</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="107" t="n"/>
-      <c r="B70" s="107" t="n"/>
-      <c r="C70" s="106" t="inlineStr">
-        <is>
-          <t>• Oberflächentemperatur θF und Volumenstrom eingeblendet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="107" t="n"/>
-      <c r="B71" s="107" t="n"/>
-      <c r="C71" s="106" t="inlineStr">
-        <is>
-          <t>• Neue Spalten 'spez. Druckverlust [Pa/m]' und Eingabespalte 'Verteiler (Anbindung)'.</t>
         </is>
       </c>
     </row>
@@ -2738,24 +2703,16 @@
       <c r="B72" s="108" t="n"/>
       <c r="C72" s="106" t="inlineStr">
         <is>
-          <t>• Warnung (rot), wenn die aktivierbare Fläche größer als die Raumfläche ist.</t>
+          <t>• Oberflächentemperatur θF und Volumenstrom eingeblendet.</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="104" t="inlineStr">
-        <is>
-          <t>0.2</t>
-        </is>
-      </c>
-      <c r="B73" s="105" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
+      <c r="A73" s="108" t="n"/>
+      <c r="B73" s="108" t="n"/>
       <c r="C73" s="106" t="inlineStr">
         <is>
-          <t>• agn-Logo eingebunden und eigenes Changelog-Blatt ergänzt.</t>
+          <t>• Neue Spalten 'spez. Druckverlust [Pa/m]' und Eingabespalte 'Verteiler (Anbindung)'.</t>
         </is>
       </c>
     </row>
@@ -2764,25 +2721,33 @@
       <c r="B74" s="107" t="n"/>
       <c r="C74" s="106" t="inlineStr">
         <is>
+          <t>• Warnung (rot), wenn die aktivierbare Fläche größer als die Raumfläche ist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="104" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="B75" s="105" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="C75" s="106" t="inlineStr">
+        <is>
+          <t>• agn-Logo eingebunden und eigenes Changelog-Blatt ergänzt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="108" t="n"/>
+      <c r="B76" s="108" t="n"/>
+      <c r="C76" s="106" t="inlineStr">
+        <is>
           <t>• Zuschlag Einzelwiderstände (5 %) und fester Verteiler-Aufschlag (500 Pa je Kreis).</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="107" t="n"/>
-      <c r="B75" s="107" t="n"/>
-      <c r="C75" s="106" t="inlineStr">
-        <is>
-          <t>• Einheiten als Zellformat; Projektnummer/Projektname erscheinen im Ausdruck.</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="107" t="n"/>
-      <c r="B76" s="107" t="n"/>
-      <c r="C76" s="106" t="inlineStr">
-        <is>
-          <t>• Richtwert-Tabellen für R-Werte und Verlegeabstand-Faktoren; weitere Musterräume.</t>
         </is>
       </c>
     </row>
@@ -2791,24 +2756,16 @@
       <c r="B77" s="108" t="n"/>
       <c r="C77" s="106" t="inlineStr">
         <is>
-          <t>• Druckaufbereitung für DIN A4.</t>
+          <t>• Einheiten als Zellformat; Projektnummer/Projektname erscheinen im Ausdruck.</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="104" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="B78" s="105" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
+      <c r="A78" s="108" t="n"/>
+      <c r="B78" s="108" t="n"/>
       <c r="C78" s="106" t="inlineStr">
         <is>
-          <t>• Ersterstellung mit den Blättern Grundeinstellungen, Raumliste, Übersicht und Methodik.</t>
+          <t>• Richtwert-Tabellen für R-Werte und Verlegeabstand-Faktoren; weitere Musterräume.</t>
         </is>
       </c>
     </row>
@@ -2817,25 +2774,33 @@
       <c r="B79" s="107" t="n"/>
       <c r="C79" s="106" t="inlineStr">
         <is>
+          <t>• Druckaufbereitung für DIN A4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="104" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="B80" s="105" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="C80" s="106" t="inlineStr">
+        <is>
+          <t>• Ersterstellung mit den Blättern Grundeinstellungen, Raumliste, Übersicht und Methodik.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="108" t="n"/>
+      <c r="B81" s="108" t="n"/>
+      <c r="C81" s="106" t="inlineStr">
+        <is>
           <t>• Heizleistung über die logarithmische Übertemperatur (q = η · K_H · ΔθH).</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="107" t="n"/>
-      <c r="B80" s="107" t="n"/>
-      <c r="C80" s="106" t="inlineStr">
-        <is>
-          <t>• Druckverlustberechnung nach Darcy-Weisbach.</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="107" t="n"/>
-      <c r="B81" s="107" t="n"/>
-      <c r="C81" s="106" t="inlineStr">
-        <is>
-          <t>• Editierbare Rohrbibliothek und Verlegeabstand-Faktoren.</t>
         </is>
       </c>
     </row>
@@ -2844,52 +2809,72 @@
       <c r="B82" s="108" t="n"/>
       <c r="C82" s="106" t="inlineStr">
         <is>
+          <t>• Druckverlustberechnung nach Darcy-Weisbach.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="108" t="n"/>
+      <c r="B83" s="108" t="n"/>
+      <c r="C83" s="106" t="inlineStr">
+        <is>
+          <t>• Editierbare Rohrbibliothek und Verlegeabstand-Faktoren.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="107" t="n"/>
+      <c r="B84" s="107" t="n"/>
+      <c r="C84" s="106" t="inlineStr">
+        <is>
           <t>• Prüfungen: Oberflächentemperatur, Heizlastdeckung, Kreislänge, Druckverlust.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="40">
-    <mergeCell ref="A12:A14"/>
-    <mergeCell ref="B62:B63"/>
-    <mergeCell ref="B78:B82"/>
-    <mergeCell ref="B38:B42"/>
-    <mergeCell ref="B50:B53"/>
-    <mergeCell ref="A64:A67"/>
-    <mergeCell ref="A29:A31"/>
-    <mergeCell ref="A47:A49"/>
-    <mergeCell ref="A33:A37"/>
-    <mergeCell ref="A54:A57"/>
-    <mergeCell ref="A68:A72"/>
-    <mergeCell ref="B43:B46"/>
-    <mergeCell ref="B68:B72"/>
-    <mergeCell ref="A58:A60"/>
-    <mergeCell ref="B33:B37"/>
-    <mergeCell ref="A38:A42"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="B47:B49"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="A9:A11"/>
-    <mergeCell ref="B23:B28"/>
+  <mergeCells count="42">
+    <mergeCell ref="B66:B69"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="B49:B51"/>
+    <mergeCell ref="B56:B59"/>
+    <mergeCell ref="B25:B30"/>
+    <mergeCell ref="A45:A48"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="B40:B44"/>
+    <mergeCell ref="B52:B55"/>
+    <mergeCell ref="A66:A69"/>
+    <mergeCell ref="B17:B20"/>
+    <mergeCell ref="A35:A39"/>
+    <mergeCell ref="A25:A30"/>
+    <mergeCell ref="A56:A59"/>
+    <mergeCell ref="B80:B84"/>
+    <mergeCell ref="A31:A33"/>
+    <mergeCell ref="A49:A51"/>
+    <mergeCell ref="B6:B7"/>
     <mergeCell ref="A21:A22"/>
-    <mergeCell ref="A73:A77"/>
-    <mergeCell ref="B12:B14"/>
-    <mergeCell ref="B15:B18"/>
-    <mergeCell ref="A6:A8"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A23:A28"/>
-    <mergeCell ref="B58:B60"/>
-    <mergeCell ref="A62:A63"/>
-    <mergeCell ref="A78:A82"/>
-    <mergeCell ref="A43:A46"/>
-    <mergeCell ref="B64:B67"/>
-    <mergeCell ref="B73:B77"/>
-    <mergeCell ref="B29:B31"/>
-    <mergeCell ref="B9:B11"/>
-    <mergeCell ref="A15:A18"/>
-    <mergeCell ref="B54:B57"/>
+    <mergeCell ref="B35:B39"/>
+    <mergeCell ref="A40:A44"/>
+    <mergeCell ref="B31:B33"/>
+    <mergeCell ref="A17:A20"/>
+    <mergeCell ref="A60:A62"/>
+    <mergeCell ref="B64:B65"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="B75:B79"/>
+    <mergeCell ref="A70:A74"/>
+    <mergeCell ref="A64:A65"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="B60:B62"/>
+    <mergeCell ref="B45:B48"/>
+    <mergeCell ref="B70:B74"/>
+    <mergeCell ref="A80:A84"/>
+    <mergeCell ref="A75:A79"/>
     <mergeCell ref="B21:B22"/>
-    <mergeCell ref="B6:B8"/>
+    <mergeCell ref="A52:A55"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -2930,116 +2915,116 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>Globale Grundeinstellungen – Fußbodenheizung</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="20" t="inlineStr">
+      <c r="A2" s="18" t="inlineStr">
         <is>
           <t>Projekt-Nr.</t>
         </is>
       </c>
-      <c r="C2" s="21" t="inlineStr"/>
-      <c r="D2" s="22" t="n"/>
-      <c r="L2" s="23" t="inlineStr">
+      <c r="C2" s="19" t="inlineStr"/>
+      <c r="D2" s="20" t="n"/>
+      <c r="L2" s="21" t="inlineStr">
         <is>
           <t>Bearbeiter:</t>
         </is>
       </c>
-      <c r="M2" s="24" t="inlineStr"/>
+      <c r="M2" s="22" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="20" t="inlineStr">
+      <c r="A3" s="18" t="inlineStr">
         <is>
           <t>Projektname</t>
         </is>
       </c>
-      <c r="C3" s="21" t="inlineStr"/>
-      <c r="D3" s="22" t="n"/>
+      <c r="C3" s="19" t="inlineStr"/>
+      <c r="D3" s="20" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="25" t="inlineStr">
+      <c r="A5" s="23" t="inlineStr">
         <is>
           <t>Heizmedium / Temperaturen</t>
         </is>
       </c>
-      <c r="B5" s="26" t="n"/>
-      <c r="C5" s="26" t="n"/>
-      <c r="D5" s="26" t="n"/>
-      <c r="E5" s="26" t="n"/>
-      <c r="F5" s="26" t="n"/>
-      <c r="H5" s="25" t="inlineStr">
+      <c r="B5" s="24" t="n"/>
+      <c r="C5" s="24" t="n"/>
+      <c r="D5" s="24" t="n"/>
+      <c r="E5" s="24" t="n"/>
+      <c r="F5" s="24" t="n"/>
+      <c r="H5" s="23" t="inlineStr">
         <is>
           <t>Wärmeübergang / Fußbodenaufbau</t>
         </is>
       </c>
-      <c r="I5" s="26" t="n"/>
-      <c r="J5" s="26" t="n"/>
-      <c r="K5" s="26" t="n"/>
-      <c r="L5" s="26" t="n"/>
-      <c r="M5" s="26" t="n"/>
+      <c r="I5" s="24" t="n"/>
+      <c r="J5" s="24" t="n"/>
+      <c r="K5" s="24" t="n"/>
+      <c r="L5" s="24" t="n"/>
+      <c r="M5" s="24" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="27" t="inlineStr">
+      <c r="A6" s="25" t="inlineStr">
         <is>
           <t>Vorlauftemperatur  θV</t>
         </is>
       </c>
-      <c r="C6" s="28" t="n">
+      <c r="C6" s="26" t="n">
         <v>35</v>
       </c>
-      <c r="D6" s="29" t="inlineStr">
+      <c r="D6" s="27" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="E6" s="30" t="inlineStr">
+      <c r="E6" s="28" t="inlineStr">
         <is>
           <t>Auslegungs-Vorlauf</t>
         </is>
       </c>
-      <c r="H6" s="27" t="inlineStr">
+      <c r="H6" s="25" t="inlineStr">
         <is>
           <t>Wärmeübergang Oberfläche  α</t>
         </is>
       </c>
-      <c r="J6" s="31" t="n">
+      <c r="J6" s="29" t="n">
         <v>10.8</v>
       </c>
-      <c r="K6" s="29" t="inlineStr">
+      <c r="K6" s="27" t="inlineStr">
         <is>
           <t>W/m²K</t>
         </is>
       </c>
-      <c r="L6" s="30" t="inlineStr">
+      <c r="L6" s="28" t="inlineStr">
         <is>
           <t>Boden → Raum (EN 1264)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="27" t="inlineStr">
+      <c r="A7" s="25" t="inlineStr">
         <is>
           <t>Rücklauftemperatur  θR</t>
         </is>
       </c>
-      <c r="C7" s="28" t="n">
+      <c r="C7" s="26" t="n">
         <v>28</v>
       </c>
-      <c r="D7" s="29" t="inlineStr">
+      <c r="D7" s="27" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="E7" s="30" t="inlineStr">
+      <c r="E7" s="28" t="inlineStr">
         <is>
           <t>Auslegungs-Rücklauf</t>
         </is>
       </c>
-      <c r="H7" s="27" t="inlineStr">
+      <c r="H7" s="25" t="inlineStr">
         <is>
           <r>
             <t>Estrichüberdeckung über Rohr  s</t>
@@ -3055,41 +3040,41 @@
           </r>
         </is>
       </c>
-      <c r="J7" s="32" t="n">
+      <c r="J7" s="30" t="n">
         <v>0.045</v>
       </c>
-      <c r="K7" s="29" t="inlineStr">
+      <c r="K7" s="27" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="L7" s="30" t="inlineStr">
+      <c r="L7" s="28" t="inlineStr">
         <is>
           <t>Estrich über den Rohren</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="27" t="inlineStr">
+      <c r="A8" s="25" t="inlineStr">
         <is>
           <t>Spreizung  θV − θR</t>
         </is>
       </c>
-      <c r="C8" s="33">
+      <c r="C8" s="31">
         <f>C6-C7</f>
         <v/>
       </c>
-      <c r="D8" s="29" t="inlineStr">
+      <c r="D8" s="27" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="E8" s="30" t="inlineStr">
+      <c r="E8" s="28" t="inlineStr">
         <is>
           <t>berechnet</t>
         </is>
       </c>
-      <c r="H8" s="27" t="inlineStr">
+      <c r="H8" s="25" t="inlineStr">
         <is>
           <r>
             <t>Wärmeleitfähigkeit Estrich  λ</t>
@@ -3105,62 +3090,62 @@
           </r>
         </is>
       </c>
-      <c r="J8" s="34" t="n">
+      <c r="J8" s="32" t="n">
         <v>1.2</v>
       </c>
-      <c r="K8" s="29" t="inlineStr">
+      <c r="K8" s="27" t="inlineStr">
         <is>
           <t>W/mK</t>
         </is>
       </c>
-      <c r="L8" s="30" t="inlineStr">
+      <c r="L8" s="28" t="inlineStr">
         <is>
           <t>Zementestrich typ. 1,2</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="25" t="inlineStr">
+      <c r="A10" s="23" t="inlineStr">
         <is>
           <t>Grenzwerte</t>
         </is>
       </c>
-      <c r="B10" s="26" t="n"/>
-      <c r="C10" s="26" t="n"/>
-      <c r="D10" s="26" t="n"/>
-      <c r="E10" s="26" t="n"/>
-      <c r="F10" s="26" t="n"/>
-      <c r="H10" s="25" t="inlineStr">
+      <c r="B10" s="24" t="n"/>
+      <c r="C10" s="24" t="n"/>
+      <c r="D10" s="24" t="n"/>
+      <c r="E10" s="24" t="n"/>
+      <c r="F10" s="24" t="n"/>
+      <c r="H10" s="23" t="inlineStr">
         <is>
           <t>Wärmeabgabe nach unten (Dämmung, global)</t>
         </is>
       </c>
-      <c r="I10" s="26" t="n"/>
-      <c r="J10" s="26" t="n"/>
-      <c r="K10" s="26" t="n"/>
-      <c r="L10" s="26" t="n"/>
-      <c r="M10" s="26" t="n"/>
+      <c r="I10" s="24" t="n"/>
+      <c r="J10" s="24" t="n"/>
+      <c r="K10" s="24" t="n"/>
+      <c r="L10" s="24" t="n"/>
+      <c r="M10" s="24" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="27" t="inlineStr">
+      <c r="A11" s="25" t="inlineStr">
         <is>
           <t>Maximale zulässige Kreislänge</t>
         </is>
       </c>
-      <c r="C11" s="35" t="n">
+      <c r="C11" s="33" t="n">
         <v>120</v>
       </c>
-      <c r="D11" s="29" t="inlineStr">
+      <c r="D11" s="27" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="E11" s="30" t="inlineStr">
+      <c r="E11" s="28" t="inlineStr">
         <is>
           <t>Obergrenze je Heizkreis</t>
         </is>
       </c>
-      <c r="H11" s="27" t="inlineStr">
+      <c r="H11" s="25" t="inlineStr">
         <is>
           <r>
             <t>Wärmedurchlasswiderstand  R</t>
@@ -3176,40 +3161,40 @@
           </r>
         </is>
       </c>
-      <c r="J11" s="34" t="n">
+      <c r="J11" s="32" t="n">
         <v>2</v>
       </c>
-      <c r="K11" s="29" t="inlineStr">
+      <c r="K11" s="27" t="inlineStr">
         <is>
           <t>m²K/W</t>
         </is>
       </c>
-      <c r="L11" s="30" t="inlineStr">
+      <c r="L11" s="28" t="inlineStr">
         <is>
           <t>Dämmung unter den Rohren</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="27" t="inlineStr">
+      <c r="A12" s="25" t="inlineStr">
         <is>
           <t>Maximaler Druckverlust je Kreis</t>
         </is>
       </c>
-      <c r="C12" s="36" t="n">
+      <c r="C12" s="34" t="n">
         <v>15000</v>
       </c>
-      <c r="D12" s="29" t="inlineStr">
+      <c r="D12" s="27" t="inlineStr">
         <is>
           <t>Pa</t>
         </is>
       </c>
-      <c r="E12" s="30" t="inlineStr">
+      <c r="E12" s="28" t="inlineStr">
         <is>
           <t>Warnschwelle</t>
         </is>
       </c>
-      <c r="H12" s="27" t="inlineStr">
+      <c r="H12" s="25" t="inlineStr">
         <is>
           <r>
             <t>Temperatur unter der Decke  θ</t>
@@ -3225,22 +3210,22 @@
           </r>
         </is>
       </c>
-      <c r="J12" s="28" t="n">
+      <c r="J12" s="26" t="n">
         <v>10</v>
       </c>
-      <c r="K12" s="29" t="inlineStr">
+      <c r="K12" s="27" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
-      <c r="L12" s="30" t="inlineStr">
+      <c r="L12" s="28" t="inlineStr">
         <is>
           <t>Raum/Erdreich unter FBH</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="H13" s="27" t="inlineStr">
+      <c r="H13" s="25" t="inlineStr">
         <is>
           <r>
             <t>Wärmestrom nach unten  q</t>
@@ -3256,65 +3241,65 @@
           </r>
         </is>
       </c>
-      <c r="J13" s="37">
+      <c r="J13" s="35">
         <f>((C6+C7)/2-J12)/J11</f>
         <v/>
       </c>
-      <c r="K13" s="29" t="inlineStr">
+      <c r="K13" s="27" t="inlineStr">
         <is>
           <t>W/m²</t>
         </is>
       </c>
-      <c r="L13" s="30" t="inlineStr">
+      <c r="L13" s="28" t="inlineStr">
         <is>
           <t>Mittel θm = (θV+θR)/2</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="25" t="inlineStr">
+      <c r="A14" s="23" t="inlineStr">
         <is>
           <t>Stoffwerte Heizmedium (Wasser ~30 °C)</t>
         </is>
       </c>
-      <c r="B14" s="26" t="n"/>
-      <c r="C14" s="26" t="n"/>
-      <c r="D14" s="26" t="n"/>
-      <c r="E14" s="26" t="n"/>
-      <c r="F14" s="26" t="n"/>
+      <c r="B14" s="24" t="n"/>
+      <c r="C14" s="24" t="n"/>
+      <c r="D14" s="24" t="n"/>
+      <c r="E14" s="24" t="n"/>
+      <c r="F14" s="24" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="27" t="inlineStr">
+      <c r="A15" s="25" t="inlineStr">
         <is>
           <t>Dichte  ρ</t>
         </is>
       </c>
-      <c r="C15" s="31" t="n">
+      <c r="C15" s="29" t="n">
         <v>995.7</v>
       </c>
-      <c r="D15" s="29" t="inlineStr">
+      <c r="D15" s="27" t="inlineStr">
         <is>
           <t>kg/m³</t>
         </is>
       </c>
-      <c r="E15" s="30" t="inlineStr">
+      <c r="E15" s="28" t="inlineStr">
         <is>
           <t>Dichte des Mediums</t>
         </is>
       </c>
-      <c r="H15" s="25" t="inlineStr">
+      <c r="H15" s="23" t="inlineStr">
         <is>
           <t>Rohrsystem-Auswahl (Werte aus Konstanten)</t>
         </is>
       </c>
-      <c r="I15" s="26" t="n"/>
-      <c r="J15" s="26" t="n"/>
-      <c r="K15" s="26" t="n"/>
-      <c r="L15" s="26" t="n"/>
-      <c r="M15" s="26" t="n"/>
+      <c r="I15" s="24" t="n"/>
+      <c r="J15" s="24" t="n"/>
+      <c r="K15" s="24" t="n"/>
+      <c r="L15" s="24" t="n"/>
+      <c r="M15" s="24" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="27" t="inlineStr">
+      <c r="A16" s="25" t="inlineStr">
         <is>
           <r>
             <t>spezifische Wärmekapazität  c</t>
@@ -3330,129 +3315,129 @@
           </r>
         </is>
       </c>
-      <c r="C16" s="38" t="n">
+      <c r="C16" s="36" t="n">
         <v>4180</v>
       </c>
-      <c r="D16" s="29" t="inlineStr">
+      <c r="D16" s="27" t="inlineStr">
         <is>
           <t>J/(kg·K)</t>
         </is>
       </c>
-      <c r="E16" s="30" t="inlineStr">
+      <c r="E16" s="28" t="inlineStr">
         <is>
           <t>spez. Wärmekapazität</t>
         </is>
       </c>
-      <c r="H16" s="27" t="inlineStr">
+      <c r="H16" s="25" t="inlineStr">
         <is>
           <t>Gewähltes Rohrsystem</t>
         </is>
       </c>
-      <c r="J16" s="24" t="inlineStr">
+      <c r="J16" s="22" t="inlineStr">
         <is>
           <t>PE-Xa 17x2</t>
         </is>
       </c>
-      <c r="K16" s="22" t="n"/>
-      <c r="L16" s="30" t="inlineStr">
+      <c r="K16" s="20" t="n"/>
+      <c r="L16" s="28" t="inlineStr">
         <is>
           <t>Dropdown</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="27" t="inlineStr">
+      <c r="A17" s="25" t="inlineStr">
         <is>
           <t>kinematische Viskosität  ν</t>
         </is>
       </c>
-      <c r="C17" s="39" t="n">
+      <c r="C17" s="37" t="n">
         <v>8.01e-07</v>
       </c>
-      <c r="D17" s="29" t="inlineStr">
+      <c r="D17" s="27" t="inlineStr">
         <is>
           <t>m²/s</t>
         </is>
       </c>
-      <c r="E17" s="30" t="inlineStr">
+      <c r="E17" s="28" t="inlineStr">
         <is>
           <t>für die Reynolds-Zahl</t>
         </is>
       </c>
-      <c r="H17" s="27" t="inlineStr">
+      <c r="H17" s="25" t="inlineStr">
         <is>
           <t>→ Außendurchmesser  da</t>
         </is>
       </c>
-      <c r="J17" s="40">
+      <c r="J17" s="38">
         <f>VLOOKUP($J$16,'Konstanten'!$A$18:$E$25,2,FALSE)</f>
         <v/>
       </c>
-      <c r="K17" s="29" t="inlineStr">
+      <c r="K17" s="27" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="L17" s="30" t="inlineStr">
+      <c r="L17" s="28" t="inlineStr">
         <is>
           <t>aus Rohrbibliothek</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="H18" s="27" t="inlineStr">
+      <c r="H18" s="25" t="inlineStr">
         <is>
           <t>→ Wandstärke  s</t>
         </is>
       </c>
-      <c r="J18" s="40">
+      <c r="J18" s="38">
         <f>VLOOKUP($J$16,'Konstanten'!$A$18:$E$25,3,FALSE)</f>
         <v/>
       </c>
-      <c r="K18" s="29" t="inlineStr">
+      <c r="K18" s="27" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="L18" s="30" t="inlineStr">
+      <c r="L18" s="28" t="inlineStr">
         <is>
           <t>aus Rohrbibliothek</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="25" t="inlineStr">
+      <c r="A19" s="23" t="inlineStr">
         <is>
           <t>Strömungsgrenzwerte</t>
         </is>
       </c>
-      <c r="B19" s="26" t="n"/>
-      <c r="C19" s="26" t="n"/>
-      <c r="D19" s="26" t="n"/>
-      <c r="E19" s="26" t="n"/>
-      <c r="F19" s="26" t="n"/>
-      <c r="H19" s="27" t="inlineStr">
+      <c r="B19" s="24" t="n"/>
+      <c r="C19" s="24" t="n"/>
+      <c r="D19" s="24" t="n"/>
+      <c r="E19" s="24" t="n"/>
+      <c r="F19" s="24" t="n"/>
+      <c r="H19" s="25" t="inlineStr">
         <is>
           <t>→ Innendurchmesser  di</t>
         </is>
       </c>
-      <c r="J19" s="40">
+      <c r="J19" s="38">
         <f>VLOOKUP($J$16,'Konstanten'!$A$18:$E$25,4,FALSE)</f>
         <v/>
       </c>
-      <c r="K19" s="29" t="inlineStr">
+      <c r="K19" s="27" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="L19" s="30" t="inlineStr">
+      <c r="L19" s="28" t="inlineStr">
         <is>
           <t>di = da − 2·s</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="27" t="inlineStr">
+      <c r="A20" s="25" t="inlineStr">
         <is>
           <r>
             <t>Minimale Geschwindigkeit  v</t>
@@ -3468,41 +3453,41 @@
           </r>
         </is>
       </c>
-      <c r="C20" s="41" t="n">
+      <c r="C20" s="39" t="n">
         <v>0.1</v>
       </c>
-      <c r="D20" s="29" t="inlineStr">
+      <c r="D20" s="27" t="inlineStr">
         <is>
           <t>m/s</t>
         </is>
       </c>
-      <c r="E20" s="30" t="inlineStr">
+      <c r="E20" s="28" t="inlineStr">
         <is>
           <t>untere empfohlene Grenze</t>
         </is>
       </c>
-      <c r="H20" s="27" t="inlineStr">
+      <c r="H20" s="25" t="inlineStr">
         <is>
           <t>→ Rauheit  k</t>
         </is>
       </c>
-      <c r="J20" s="42">
+      <c r="J20" s="40">
         <f>VLOOKUP($J$16,'Konstanten'!$A$18:$E$25,5,FALSE)</f>
         <v/>
       </c>
-      <c r="K20" s="29" t="inlineStr">
+      <c r="K20" s="27" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
       </c>
-      <c r="L20" s="30" t="inlineStr">
+      <c r="L20" s="28" t="inlineStr">
         <is>
           <t>aus Rohrbibliothek</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="27" t="inlineStr">
+      <c r="A21" s="25" t="inlineStr">
         <is>
           <r>
             <t>Maximale Geschwindigkeit  v</t>
@@ -3518,41 +3503,41 @@
           </r>
         </is>
       </c>
-      <c r="C21" s="41" t="n">
+      <c r="C21" s="39" t="n">
         <v>0.5</v>
       </c>
-      <c r="D21" s="29" t="inlineStr">
+      <c r="D21" s="27" t="inlineStr">
         <is>
           <t>m/s</t>
         </is>
       </c>
-      <c r="E21" s="30" t="inlineStr">
+      <c r="E21" s="28" t="inlineStr">
         <is>
           <t>obere empfohlene Grenze</t>
         </is>
       </c>
-      <c r="H21" s="27" t="inlineStr">
+      <c r="H21" s="25" t="inlineStr">
         <is>
           <t>→ Innendurchmesser  di</t>
         </is>
       </c>
-      <c r="J21" s="43">
+      <c r="J21" s="41">
         <f>J19/1000</f>
         <v/>
       </c>
-      <c r="K21" s="29" t="inlineStr">
+      <c r="K21" s="27" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="L21" s="30" t="inlineStr">
+      <c r="L21" s="28" t="inlineStr">
         <is>
           <t>für die Berechnung</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="27" t="inlineStr">
+      <c r="A22" s="25" t="inlineStr">
         <is>
           <r>
             <t>Max. Volumenstrom je Kreis  V̇</t>
@@ -3568,20 +3553,20 @@
           </r>
         </is>
       </c>
-      <c r="C22" s="44" t="n">
+      <c r="C22" s="42" t="n">
         <v>150</v>
       </c>
-      <c r="D22" s="29" t="inlineStr">
+      <c r="D22" s="27" t="inlineStr">
         <is>
           <t>l/h</t>
         </is>
       </c>
-      <c r="E22" s="30" t="inlineStr">
+      <c r="E22" s="28" t="inlineStr">
         <is>
           <t>Warnschwelle je Heizkreis</t>
         </is>
       </c>
-      <c r="H22" s="27" t="inlineStr">
+      <c r="H22" s="25" t="inlineStr">
         <is>
           <r>
             <t>→ Innenquerschnitt  A</t>
@@ -3597,68 +3582,68 @@
           </r>
         </is>
       </c>
-      <c r="J22" s="45">
+      <c r="J22" s="43">
         <f>PI()/4*J21^2</f>
         <v/>
       </c>
-      <c r="K22" s="29" t="inlineStr">
+      <c r="K22" s="27" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="L22" s="30" t="inlineStr">
+      <c r="L22" s="28" t="inlineStr">
         <is>
           <t>für die Berechnung</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="25" t="inlineStr">
+      <c r="A23" s="23" t="inlineStr">
         <is>
           <t>Druckverlust-Zuschläge</t>
         </is>
       </c>
-      <c r="B23" s="26" t="n"/>
-      <c r="C23" s="26" t="n"/>
-      <c r="D23" s="26" t="n"/>
-      <c r="E23" s="26" t="n"/>
-      <c r="F23" s="26" t="n"/>
+      <c r="B23" s="24" t="n"/>
+      <c r="C23" s="24" t="n"/>
+      <c r="D23" s="24" t="n"/>
+      <c r="E23" s="24" t="n"/>
+      <c r="F23" s="24" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="27" t="inlineStr">
+      <c r="A24" s="25" t="inlineStr">
         <is>
           <t>Zuschlag Einzelwiderstände</t>
         </is>
       </c>
-      <c r="C24" s="46" t="n">
+      <c r="C24" s="44" t="n">
         <v>0.05</v>
       </c>
-      <c r="D24" s="29" t="inlineStr">
+      <c r="D24" s="27" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E24" s="30" t="inlineStr">
+      <c r="E24" s="28" t="inlineStr">
         <is>
           <t>Formstücke (5 %)</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="27" t="inlineStr">
+      <c r="A25" s="25" t="inlineStr">
         <is>
           <t>Aufschlag Verteiler je Kreis</t>
         </is>
       </c>
-      <c r="C25" s="36" t="n">
+      <c r="C25" s="34" t="n">
         <v>500</v>
       </c>
-      <c r="D25" s="29" t="inlineStr">
+      <c r="D25" s="27" t="inlineStr">
         <is>
           <t>Pa</t>
         </is>
       </c>
-      <c r="E25" s="30" t="inlineStr">
+      <c r="E25" s="28" t="inlineStr">
         <is>
           <t>fester Wert je Verteiler</t>
         </is>
@@ -3756,20 +3741,20 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
     <col width="9" customWidth="1" min="10" max="10"/>
     <col width="7" customWidth="1" min="11" max="11"/>
-    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
     <col width="6" customWidth="1" min="13" max="13"/>
     <col hidden="1" width="12" customWidth="1" min="14" max="14"/>
     <col hidden="1" width="11" customWidth="1" min="15" max="15"/>
     <col hidden="1" width="11" customWidth="1" min="16" max="16"/>
-    <col width="10" customWidth="1" min="17" max="17"/>
-    <col width="9" customWidth="1" min="18" max="18"/>
+    <col width="11" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="18" max="18"/>
     <col hidden="1" width="11" customWidth="1" min="19" max="19"/>
     <col hidden="1" width="12" customWidth="1" min="20" max="20"/>
     <col hidden="1" width="12" customWidth="1" min="21" max="21"/>
@@ -3792,217 +3777,227 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>Auslegung – Fußbodenheizung</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="47">
+      <c r="A2" s="45">
         <f>"Projekt-Nr.: "&amp;'Grundeinstellungen'!$C$2</f>
         <v/>
       </c>
-      <c r="AJ2" s="48">
+      <c r="AJ2" s="46">
         <f>"Bearbeiter: "&amp;'Grundeinstellungen'!$M$2</f>
         <v/>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="47">
+      <c r="A3" s="45">
         <f>"Projekt: "&amp;'Grundeinstellungen'!$C$3</f>
         <v/>
       </c>
     </row>
     <row r="4" ht="46" customHeight="1">
-      <c r="A4" s="49" t="inlineStr">
-        <is>
-          <t>Heizkreisverteiler</t>
-        </is>
-      </c>
-      <c r="B4" s="49" t="inlineStr">
+      <c r="A4" s="47" t="inlineStr">
+        <is>
+          <t>Heizkreis-
+verteiler</t>
+        </is>
+      </c>
+      <c r="B4" s="47" t="inlineStr">
         <is>
           <t>Raum-Nr.</t>
         </is>
       </c>
-      <c r="C4" s="49" t="inlineStr">
-        <is>
-          <t>Raumbezeichnung</t>
-        </is>
-      </c>
-      <c r="D4" s="49" t="inlineStr">
+      <c r="C4" s="47" t="inlineStr">
+        <is>
+          <t>Raum-
+bezeichnung</t>
+        </is>
+      </c>
+      <c r="D4" s="47" t="inlineStr">
         <is>
           <t>Raum-fläche</t>
         </is>
       </c>
-      <c r="E4" s="49" t="inlineStr">
-        <is>
-          <t>Raumtemperatur</t>
-        </is>
-      </c>
-      <c r="F4" s="49" t="inlineStr">
+      <c r="E4" s="47" t="inlineStr">
+        <is>
+          <t>Raum-
+temperatur</t>
+        </is>
+      </c>
+      <c r="F4" s="47" t="inlineStr">
         <is>
           <t>Heizlast</t>
         </is>
       </c>
-      <c r="G4" s="49" t="inlineStr">
+      <c r="G4" s="47" t="inlineStr">
         <is>
           <t>spez. Heizlast</t>
         </is>
       </c>
-      <c r="H4" s="49" t="inlineStr">
-        <is>
-          <t>aktivierbare Fläche</t>
-        </is>
-      </c>
-      <c r="I4" s="49" t="inlineStr">
-        <is>
-          <t>R-Wert Bodenbelag</t>
-        </is>
-      </c>
-      <c r="J4" s="49" t="inlineStr">
+      <c r="H4" s="47" t="inlineStr">
+        <is>
+          <t>aktivier-
+bare Fläche</t>
+        </is>
+      </c>
+      <c r="I4" s="47" t="inlineStr">
+        <is>
+          <t>R-Wert
+Bodenbelag</t>
+        </is>
+      </c>
+      <c r="J4" s="47" t="inlineStr">
         <is>
           <t>Verlege–abstand</t>
         </is>
       </c>
-      <c r="K4" s="49" t="inlineStr">
+      <c r="K4" s="47" t="inlineStr">
         <is>
           <t>Anz.
 HK</t>
         </is>
       </c>
-      <c r="L4" s="49" t="inlineStr">
-        <is>
-          <t>Zuleitungslänge</t>
-        </is>
-      </c>
-      <c r="M4" s="49" t="inlineStr">
+      <c r="L4" s="47" t="inlineStr">
+        <is>
+          <t>Zuleitungs-
+länge</t>
+        </is>
+      </c>
+      <c r="M4" s="47" t="inlineStr">
         <is>
           <t>Zone</t>
         </is>
       </c>
-      <c r="N4" s="50" t="inlineStr">
+      <c r="N4" s="48" t="inlineStr">
         <is>
           <t>log. Übertemperatur</t>
         </is>
       </c>
-      <c r="O4" s="50" t="inlineStr">
+      <c r="O4" s="48" t="inlineStr">
         <is>
           <t>Wärmedurchgang</t>
         </is>
       </c>
-      <c r="P4" s="50" t="inlineStr">
+      <c r="P4" s="48" t="inlineStr">
         <is>
           <t>Verlegeabstand-Faktor</t>
         </is>
       </c>
-      <c r="Q4" s="50" t="inlineStr">
-        <is>
-          <t>spez. Heizleistung</t>
-        </is>
-      </c>
-      <c r="R4" s="50" t="inlineStr">
-        <is>
-          <t>Oberflächentemperatur</t>
-        </is>
-      </c>
-      <c r="S4" s="50" t="inlineStr">
+      <c r="Q4" s="48" t="inlineStr">
+        <is>
+          <t>spez. Heiz-
+leistung</t>
+        </is>
+      </c>
+      <c r="R4" s="48" t="inlineStr">
+        <is>
+          <t>Ober-
+flächen-
+temperatur</t>
+        </is>
+      </c>
+      <c r="S4" s="48" t="inlineStr">
         <is>
           <t>max. Oberflächentemp.</t>
         </is>
       </c>
-      <c r="T4" s="50" t="inlineStr">
+      <c r="T4" s="48" t="inlineStr">
         <is>
           <t>Leistung FBH nach oben</t>
         </is>
       </c>
-      <c r="U4" s="50" t="inlineStr">
+      <c r="U4" s="48" t="inlineStr">
         <is>
           <t>Deckung absolut</t>
         </is>
       </c>
-      <c r="V4" s="50" t="inlineStr">
+      <c r="V4" s="48" t="inlineStr">
         <is>
           <t>Deckung</t>
         </is>
       </c>
-      <c r="W4" s="50" t="inlineStr">
+      <c r="W4" s="48" t="inlineStr">
         <is>
           <t>Verlust nach unten</t>
         </is>
       </c>
-      <c r="X4" s="50" t="inlineStr">
+      <c r="X4" s="48" t="inlineStr">
         <is>
           <t>maßgebl. Leistung</t>
         </is>
       </c>
-      <c r="Y4" s="50" t="inlineStr">
+      <c r="Y4" s="48" t="inlineStr">
         <is>
           <t>Rohrlänge Fläche</t>
         </is>
       </c>
-      <c r="Z4" s="50" t="inlineStr">
+      <c r="Z4" s="48" t="inlineStr">
         <is>
           <t>Rohrlänge Zuleitung</t>
         </is>
       </c>
-      <c r="AA4" s="50" t="inlineStr">
+      <c r="AA4" s="48" t="inlineStr">
         <is>
           <t>Rohrlänge gesamt</t>
         </is>
       </c>
-      <c r="AB4" s="50" t="inlineStr">
+      <c r="AB4" s="48" t="inlineStr">
         <is>
           <t>Rohrlänge je Kreis</t>
         </is>
       </c>
-      <c r="AC4" s="50" t="inlineStr">
+      <c r="AC4" s="48" t="inlineStr">
         <is>
           <t>Massenstrom je Kreis</t>
         </is>
       </c>
-      <c r="AD4" s="50" t="inlineStr">
+      <c r="AD4" s="48" t="inlineStr">
         <is>
           <t>Volumen-strom je Kreis</t>
         </is>
       </c>
-      <c r="AE4" s="50" t="inlineStr">
+      <c r="AE4" s="48" t="inlineStr">
         <is>
           <t>Geschwin-digkeit</t>
         </is>
       </c>
-      <c r="AF4" s="50" t="inlineStr">
+      <c r="AF4" s="48" t="inlineStr">
         <is>
           <t>Reynolds-Zahl</t>
         </is>
       </c>
-      <c r="AG4" s="50" t="inlineStr">
+      <c r="AG4" s="48" t="inlineStr">
         <is>
           <t>Strömungsbereich</t>
         </is>
       </c>
-      <c r="AH4" s="50" t="inlineStr">
+      <c r="AH4" s="48" t="inlineStr">
         <is>
           <t>Rohrreibungszahl</t>
         </is>
       </c>
-      <c r="AI4" s="50" t="inlineStr">
+      <c r="AI4" s="48" t="inlineStr">
         <is>
           <t>Δp Reibung</t>
         </is>
       </c>
-      <c r="AJ4" s="50" t="inlineStr">
+      <c r="AJ4" s="48" t="inlineStr">
         <is>
           <t>spez. Druckverlust</t>
         </is>
       </c>
-      <c r="AK4" s="50" t="inlineStr">
-        <is>
-          <t>Druckverlust</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="14" customHeight="1">
+      <c r="AK4" s="48" t="inlineStr">
+        <is>
+          <t>Druck-
+verlust</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
       <c r="A5" s="49" t="inlineStr">
         <is>
           <t>HKV</t>
@@ -4020,7 +4015,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="001F4E78"/>
-              <sz val="10"/>
+              <sz val="13"/>
               <vertAlign val="subscript"/>
             </rPr>
             <t>R</t>
@@ -4047,7 +4042,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="001F4E78"/>
-              <sz val="10"/>
+              <sz val="13"/>
               <vertAlign val="subscript"/>
             </rPr>
             <t>HL</t>
@@ -4064,7 +4059,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="001F4E78"/>
-              <sz val="10"/>
+              <sz val="13"/>
               <vertAlign val="subscript"/>
             </rPr>
             <t>F</t>
@@ -4081,7 +4076,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="001F4E78"/>
-              <sz val="10"/>
+              <sz val="13"/>
               <vertAlign val="subscript"/>
             </rPr>
             <t>λ,B</t>
@@ -4108,7 +4103,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="001F4E78"/>
-              <sz val="10"/>
+              <sz val="13"/>
               <vertAlign val="subscript"/>
             </rPr>
             <t>zu</t>
@@ -4131,7 +4126,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="00FFFFFF"/>
-              <sz val="10"/>
+              <sz val="13"/>
               <vertAlign val="subscript"/>
             </rPr>
             <t>H</t>
@@ -4168,7 +4163,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="00FFFFFF"/>
-              <sz val="10"/>
+              <sz val="13"/>
               <vertAlign val="subscript"/>
             </rPr>
             <t>o</t>
@@ -4191,7 +4186,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="00FFFFFF"/>
-              <sz val="10"/>
+              <sz val="13"/>
               <vertAlign val="subscript"/>
             </rPr>
             <t>u</t>
@@ -4208,7 +4203,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="00FFFFFF"/>
-              <sz val="10"/>
+              <sz val="13"/>
               <vertAlign val="subscript"/>
             </rPr>
             <t>m</t>
@@ -4225,7 +4220,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="00FFFFFF"/>
-              <sz val="10"/>
+              <sz val="13"/>
               <vertAlign val="subscript"/>
             </rPr>
             <t>F</t>
@@ -4242,7 +4237,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="00FFFFFF"/>
-              <sz val="10"/>
+              <sz val="13"/>
               <vertAlign val="subscript"/>
             </rPr>
             <t>Z</t>
@@ -4259,7 +4254,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="00FFFFFF"/>
-              <sz val="10"/>
+              <sz val="13"/>
               <vertAlign val="subscript"/>
             </rPr>
             <t>ges</t>
@@ -4276,7 +4271,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="00FFFFFF"/>
-              <sz val="10"/>
+              <sz val="13"/>
               <vertAlign val="subscript"/>
             </rPr>
             <t>K</t>
@@ -4319,7 +4314,7 @@
               <rFont val="Arial"/>
               <b val="1"/>
               <color rgb="00FFFFFF"/>
-              <sz val="10"/>
+              <sz val="13"/>
               <vertAlign val="subscript"/>
             </rPr>
             <t>R</t>
@@ -27691,40 +27686,40 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>Kontrolle / Auswertung</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="47">
+      <c r="A2" s="45">
         <f>"Projekt-Nr.: "&amp;'Grundeinstellungen'!$C$2</f>
         <v/>
       </c>
-      <c r="D2" s="48">
+      <c r="D2" s="46">
         <f>"Bearbeiter: "&amp;'Grundeinstellungen'!$M$2</f>
         <v/>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="47">
+      <c r="A3" s="45">
         <f>"Projekt: "&amp;'Grundeinstellungen'!$C$3</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="25" t="inlineStr">
+      <c r="A5" s="23" t="inlineStr">
         <is>
           <t>Summen / Kennzahlen</t>
         </is>
       </c>
-      <c r="B5" s="26" t="n"/>
-      <c r="C5" s="26" t="n"/>
-      <c r="D5" s="26" t="n"/>
+      <c r="B5" s="24" t="n"/>
+      <c r="C5" s="24" t="n"/>
+      <c r="D5" s="24" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="27" t="inlineStr">
+      <c r="A6" s="25" t="inlineStr">
         <is>
           <t>Anzahl Räume</t>
         </is>
@@ -27733,14 +27728,14 @@
         <f>COUNTA('Auslegung'!B7:B206)</f>
         <v/>
       </c>
-      <c r="C6" s="29" t="inlineStr">
+      <c r="C6" s="27" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="27" t="inlineStr">
+      <c r="A7" s="25" t="inlineStr">
         <is>
           <t>Gesamte Heizlast</t>
         </is>
@@ -27749,14 +27744,14 @@
         <f>SUM('Auslegung'!F7:F206)</f>
         <v/>
       </c>
-      <c r="C7" s="29" t="inlineStr">
+      <c r="C7" s="27" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="27" t="inlineStr">
+      <c r="A8" s="25" t="inlineStr">
         <is>
           <t>Gesamte FBH-Leistung (nach oben)</t>
         </is>
@@ -27765,14 +27760,14 @@
         <f>SUM('Auslegung'!T7:T206)</f>
         <v/>
       </c>
-      <c r="C8" s="29" t="inlineStr">
+      <c r="C8" s="27" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="27" t="inlineStr">
+      <c r="A9" s="25" t="inlineStr">
         <is>
           <t>Verlustleistung nach unten</t>
         </is>
@@ -27781,14 +27776,14 @@
         <f>SUM('Auslegung'!W7:W206)</f>
         <v/>
       </c>
-      <c r="C9" s="29" t="inlineStr">
+      <c r="C9" s="27" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="27" t="inlineStr">
+      <c r="A10" s="25" t="inlineStr">
         <is>
           <t>Maßgebliche Gesamtleistung (Hydraulik)</t>
         </is>
@@ -27797,14 +27792,14 @@
         <f>SUM('Auslegung'!X7:X206)</f>
         <v/>
       </c>
-      <c r="C10" s="29" t="inlineStr">
+      <c r="C10" s="27" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="27" t="inlineStr">
+      <c r="A11" s="25" t="inlineStr">
         <is>
           <t>Deckungsgrad gesamt</t>
         </is>
@@ -27813,14 +27808,14 @@
         <f>IFERROR(B8/B7,0)</f>
         <v/>
       </c>
-      <c r="C11" s="29" t="inlineStr">
+      <c r="C11" s="27" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="27" t="inlineStr">
+      <c r="A12" s="25" t="inlineStr">
         <is>
           <t>Gesamte Rohrlänge</t>
         </is>
@@ -27829,14 +27824,14 @@
         <f>SUM('Auslegung'!AA7:AA206)</f>
         <v/>
       </c>
-      <c r="C12" s="29" t="inlineStr">
+      <c r="C12" s="27" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="27" t="inlineStr">
+      <c r="A13" s="25" t="inlineStr">
         <is>
           <t>Anzahl Heizkreise gesamt</t>
         </is>
@@ -27845,14 +27840,14 @@
         <f>SUM('Auslegung'!K7:K206)</f>
         <v/>
       </c>
-      <c r="C13" s="29" t="inlineStr">
+      <c r="C13" s="27" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="27" t="inlineStr">
+      <c r="A14" s="25" t="inlineStr">
         <is>
           <t>Gesamtmassenstrom (Pumpe)</t>
         </is>
@@ -27861,14 +27856,14 @@
         <f>SUM('Auslegung'!AC7:AC206)</f>
         <v/>
       </c>
-      <c r="C14" s="29" t="inlineStr">
+      <c r="C14" s="27" t="inlineStr">
         <is>
           <t>kg/h</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="27" t="inlineStr">
+      <c r="A15" s="25" t="inlineStr">
         <is>
           <t>Gesamtvolumenstrom (Pumpe)</t>
         </is>
@@ -27877,14 +27872,14 @@
         <f>SUM('Auslegung'!AD7:AD206)</f>
         <v/>
       </c>
-      <c r="C15" s="29" t="inlineStr">
+      <c r="C15" s="27" t="inlineStr">
         <is>
           <t>l/h</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="27" t="inlineStr">
+      <c r="A16" s="25" t="inlineStr">
         <is>
           <t>Max. Druckverlust eines Kreises</t>
         </is>
@@ -27893,14 +27888,14 @@
         <f>IFERROR(MAX('Auslegung'!AK7:AK206),0)</f>
         <v/>
       </c>
-      <c r="C16" s="29" t="inlineStr">
+      <c r="C16" s="27" t="inlineStr">
         <is>
           <t>Pa</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="27" t="inlineStr">
+      <c r="A17" s="25" t="inlineStr">
         <is>
           <t>Max. Strömungsgeschwindigkeit</t>
         </is>
@@ -27909,24 +27904,24 @@
         <f>IFERROR(MAX('Auslegung'!AE7:AE206),0)</f>
         <v/>
       </c>
-      <c r="C17" s="29" t="inlineStr">
+      <c r="C17" s="27" t="inlineStr">
         <is>
           <t>m/s</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="25" t="inlineStr">
+      <c r="A19" s="23" t="inlineStr">
         <is>
           <t>Warnungen</t>
         </is>
       </c>
-      <c r="B19" s="26" t="n"/>
-      <c r="C19" s="26" t="n"/>
-      <c r="D19" s="26" t="n"/>
+      <c r="B19" s="24" t="n"/>
+      <c r="C19" s="24" t="n"/>
+      <c r="D19" s="24" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="27" t="inlineStr">
+      <c r="A20" s="25" t="inlineStr">
         <is>
           <t>Räume unterdeckt</t>
         </is>
@@ -27935,19 +27930,19 @@
         <f>COUNTIF('Auslegung'!V7:V206,"&lt;1")</f>
         <v/>
       </c>
-      <c r="C20" s="29" t="inlineStr">
+      <c r="C20" s="27" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D20" s="30" t="inlineStr">
+      <c r="D20" s="28" t="inlineStr">
         <is>
           <t>Heizlast nicht gedeckt</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="27" t="inlineStr">
+      <c r="A21" s="25" t="inlineStr">
         <is>
           <t>Kreise zu lang</t>
         </is>
@@ -27956,19 +27951,19 @@
         <f>COUNTIF('Auslegung'!AB7:AB206,"&gt;"&amp;'Grundeinstellungen'!$C$11)</f>
         <v/>
       </c>
-      <c r="C21" s="29" t="inlineStr">
+      <c r="C21" s="27" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D21" s="30" t="inlineStr">
+      <c r="D21" s="28" t="inlineStr">
         <is>
           <t>&gt; max. Kreislänge</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="27" t="inlineStr">
+      <c r="A22" s="25" t="inlineStr">
         <is>
           <t>Druckverlust über Warnschwelle</t>
         </is>
@@ -27977,14 +27972,14 @@
         <f>COUNTIF('Auslegung'!AK7:AK206,"&gt;"&amp;'Grundeinstellungen'!$C$12)</f>
         <v/>
       </c>
-      <c r="C22" s="29" t="inlineStr">
+      <c r="C22" s="27" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="27" t="inlineStr">
+      <c r="A23" s="25" t="inlineStr">
         <is>
           <t>Oberflächentemperatur zu hoch</t>
         </is>
@@ -27993,14 +27988,14 @@
         <f>SUMPRODUCT(('Auslegung'!R7:R206&lt;&gt;"")*('Auslegung'!R7:R206&gt;'Auslegung'!S7:S206))</f>
         <v/>
       </c>
-      <c r="C23" s="29" t="inlineStr">
+      <c r="C23" s="27" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="27" t="inlineStr">
+      <c r="A24" s="25" t="inlineStr">
         <is>
           <t>Geschwindigkeit außerhalb v_min–v_max</t>
         </is>
@@ -28009,19 +28004,19 @@
         <f>SUMPRODUCT(('Auslegung'!AE7:AE206&lt;&gt;"")*(('Auslegung'!AE7:AE206&lt;'Grundeinstellungen'!$C$20)+('Auslegung'!AE7:AE206&gt;'Grundeinstellungen'!$C$21)))</f>
         <v/>
       </c>
-      <c r="C24" s="29" t="inlineStr">
+      <c r="C24" s="27" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D24" s="30" t="inlineStr">
+      <c r="D24" s="28" t="inlineStr">
         <is>
           <t>Kreise</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="27" t="inlineStr">
+      <c r="A25" s="25" t="inlineStr">
         <is>
           <t>Volumenstrom je Kreis zu hoch</t>
         </is>
@@ -28030,12 +28025,12 @@
         <f>COUNTIF('Auslegung'!AD7:AD206,"&gt;"&amp;'Grundeinstellungen'!$C$22)</f>
         <v/>
       </c>
-      <c r="C25" s="29" t="inlineStr">
+      <c r="C25" s="27" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D25" s="30" t="inlineStr">
+      <c r="D25" s="28" t="inlineStr">
         <is>
           <t>&gt; max. Volumenstrom</t>
         </is>
@@ -28123,60 +28118,60 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>Heizkreisverteiler – Übersicht je HKV</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="47">
+      <c r="A2" s="45">
         <f>"Projekt-Nr.: "&amp;'Grundeinstellungen'!$C$2</f>
         <v/>
       </c>
-      <c r="F2" s="48">
+      <c r="F2" s="46">
         <f>"Bearbeiter: "&amp;'Grundeinstellungen'!$M$2</f>
         <v/>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="47">
+      <c r="A3" s="45">
         <f>"Projekt: "&amp;'Grundeinstellungen'!$C$3</f>
         <v/>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="50" t="inlineStr">
+      <c r="A4" s="48" t="inlineStr">
         <is>
           <t>Heizkreisverteiler (HKV)</t>
         </is>
       </c>
-      <c r="B4" s="50" t="inlineStr">
+      <c r="B4" s="48" t="inlineStr">
         <is>
           <t>Anzahl Kreise</t>
         </is>
       </c>
-      <c r="C4" s="50" t="inlineStr">
+      <c r="C4" s="48" t="inlineStr">
         <is>
           <t>Spreizung [K]</t>
         </is>
       </c>
-      <c r="D4" s="50" t="inlineStr">
+      <c r="D4" s="48" t="inlineStr">
         <is>
           <t>maßgebl. Leistung [W]</t>
         </is>
       </c>
-      <c r="E4" s="50" t="inlineStr">
+      <c r="E4" s="48" t="inlineStr">
         <is>
           <t>Massenstrom [kg/h]</t>
         </is>
       </c>
-      <c r="F4" s="50" t="inlineStr">
+      <c r="F4" s="48" t="inlineStr">
         <is>
           <t>Volumenstrom [l/h]</t>
         </is>
       </c>
-      <c r="G4" s="50" t="inlineStr">
+      <c r="G4" s="48" t="inlineStr">
         <is>
           <t>max. Druckverlust [Pa]</t>
         </is>
@@ -29683,7 +29678,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="30" t="inlineStr">
+      <c r="A56" s="28" t="inlineStr">
         <is>
           <t>Baut sich automatisch aus der Auslegung auf (Array-Formeln, Excel &amp; LibreOffice).</t>
         </is>
@@ -29735,20 +29730,20 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>Verifikation – Abgleich mit Herstellerdaten</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="47">
+      <c r="A2" s="45">
         <f>"Projekt-Nr.: "&amp;'Grundeinstellungen'!$C$2</f>
         <v/>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="47">
+      <c r="A3" s="45">
         <f>"Projekt: "&amp;'Grundeinstellungen'!$C$3</f>
         <v/>
       </c>
@@ -29763,125 +29758,125 @@
       <c r="C5" s="89" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="30" t="inlineStr">
+      <c r="D5" s="28" t="inlineStr">
         <is>
           <t>← an Herstellerdaten anpassen</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="25" t="inlineStr">
+      <c r="A7" s="23" t="inlineStr">
         <is>
           <t>Vergleichsbedingungen (fix)</t>
         </is>
       </c>
-      <c r="B7" s="26" t="n"/>
-      <c r="C7" s="26" t="n"/>
+      <c r="B7" s="24" t="n"/>
+      <c r="C7" s="24" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="27" t="inlineStr">
+      <c r="A8" s="25" t="inlineStr">
         <is>
           <t>Vorlauftemperatur  θV</t>
         </is>
       </c>
-      <c r="B8" s="28" t="n">
+      <c r="B8" s="26" t="n">
         <v>35</v>
       </c>
-      <c r="C8" s="29" t="inlineStr">
+      <c r="C8" s="27" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="27" t="inlineStr">
+      <c r="A9" s="25" t="inlineStr">
         <is>
           <t>Rücklauftemperatur  θR</t>
         </is>
       </c>
-      <c r="B9" s="28" t="n">
+      <c r="B9" s="26" t="n">
         <v>28</v>
       </c>
-      <c r="C9" s="29" t="inlineStr">
+      <c r="C9" s="27" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="27" t="inlineStr">
+      <c r="A10" s="25" t="inlineStr">
         <is>
           <t>Raumtemperatur  θi</t>
         </is>
       </c>
-      <c r="B10" s="28" t="n">
+      <c r="B10" s="26" t="n">
         <v>20</v>
       </c>
-      <c r="C10" s="29" t="inlineStr">
+      <c r="C10" s="27" t="inlineStr">
         <is>
           <t>°C</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="27" t="inlineStr">
+      <c r="A11" s="25" t="inlineStr">
         <is>
           <t>R-Wert Bodenbelag</t>
         </is>
       </c>
-      <c r="B11" s="32" t="n">
+      <c r="B11" s="30" t="n">
         <v>0.1</v>
       </c>
-      <c r="C11" s="29" t="inlineStr">
+      <c r="C11" s="27" t="inlineStr">
         <is>
           <t>m²K/W</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="30" t="inlineStr">
+      <c r="A12" s="28" t="inlineStr">
         <is>
           <t>q berechnet = f · η(VA) · K_H · ΔθH</t>
         </is>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1">
-      <c r="A14" s="50" t="inlineStr">
+      <c r="A14" s="48" t="inlineStr">
         <is>
           <t>Verlegeabstand [mm]</t>
         </is>
       </c>
-      <c r="B14" s="50" t="inlineStr">
+      <c r="B14" s="48" t="inlineStr">
         <is>
           <t>q berechnet [W/m²]</t>
         </is>
       </c>
-      <c r="C14" s="49" t="inlineStr">
+      <c r="C14" s="47" t="inlineStr">
         <is>
           <t>Hersteller q [W/m²]</t>
         </is>
       </c>
-      <c r="D14" s="50" t="inlineStr">
+      <c r="D14" s="48" t="inlineStr">
         <is>
           <t>Abweichung [W/m²]</t>
         </is>
       </c>
-      <c r="E14" s="50" t="inlineStr">
+      <c r="E14" s="48" t="inlineStr">
         <is>
           <t>Abweichung [%]</t>
         </is>
       </c>
-      <c r="F14" s="50" t="inlineStr">
+      <c r="F14" s="48" t="inlineStr">
         <is>
           <t>ΔθH [K]</t>
         </is>
       </c>
-      <c r="G14" s="50" t="inlineStr">
+      <c r="G14" s="48" t="inlineStr">
         <is>
           <t>K_H [W/m²K]</t>
         </is>
       </c>
-      <c r="H14" s="50" t="inlineStr">
+      <c r="H14" s="48" t="inlineStr">
         <is>
           <t>η [-]</t>
         </is>
@@ -30151,35 +30146,35 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="27" t="inlineStr">
+      <c r="A25" s="25" t="inlineStr">
         <is>
           <t>• Hersteller-q je Verlegeabstand aus dem Datenblatt in Spalte C eintragen.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="27" t="inlineStr">
+      <c r="A26" s="25" t="inlineStr">
         <is>
           <t>• Korrekturfaktor f oben so einstellen, dass berechnetes q und Hersteller-q</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="27" t="inlineStr">
+      <c r="A27" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">   möglichst übereinstimmen (Abweichung grün).</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="30" t="inlineStr">
+      <c r="A28" s="28" t="inlineStr">
         <is>
           <t>• Der so kalibrierte Faktor f gilt für die gesamte Auslegung – daher VOR</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="30" t="inlineStr">
+      <c r="A29" s="28" t="inlineStr">
         <is>
           <t xml:space="preserve">   der Raumauslegung kalibrieren.</t>
         </is>
@@ -30228,7 +30223,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>Anleitung / Bedienung</t>
         </is>
@@ -30594,7 +30589,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>Methodik &amp; Annahmen</t>
         </is>
@@ -31076,14 +31071,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>Konstanten / Bibliotheken</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="30" t="inlineStr">
+      <c r="A3" s="28" t="inlineStr">
         <is>
           <t>Nachschlage-Tabellen (editierbar). Leerzeilen = Platz für weitere Einträge.</t>
         </is>

</xml_diff>

<commit_message>
FBH-Auslegung v0.24 - Verifikation mit echten DIN-EN-1264-Referenzwerten
Verifikation: Referenzspalte (vormals Beispielwerte) mit echten Waermestromdichten nach DIN EN 1264 vorbelegt - Nasssystem/Tacker, Standardestrich, VL 40 / RL 30 C, Raumtemp. 20 C, Bodenbelag R=0,10 m2K/W (Quelle: Leistungstabelle fussbodenheizung24.de). Vergleichsbedingungen entsprechend auf 40/30 C gesetzt.

Verifikation: Korrekturfaktor f auf 0,85 vorkalibriert (Best-Fit, alle Abweichungen <=7,2 Prozent, komplett gruen). Spalte C bleibt editierbar fuer herstellereigene Datenblattwerte (Rehau, Uponor, Buderus, Kermi).

Spaltentitel 'Hersteller q' -> 'Referenz q EN 1264'; Hinweise mit Quelle und Bedingungen.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FBH_Auslegung.xlsx
+++ b/FBH_Auslegung.xlsx
@@ -29,7 +29,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="6">'Anleitung'!$A$1:$D$32</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">'Methodik'!$A$1:$F$26</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="8">'Konstanten'!$A$1:$I$26</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="9">'Changelog'!$A$1:$C$84</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="9">'Changelog'!$A$1:$C$86</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1897,7 +1897,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C84"/>
+  <dimension ref="A1:C86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1915,7 +1915,7 @@
     <row r="3">
       <c r="C3" s="21" t="inlineStr">
         <is>
-          <t>Version 0.23 · dh</t>
+          <t>Version 0.24 · dh</t>
         </is>
       </c>
     </row>
@@ -1939,17 +1939,17 @@
     <row r="6">
       <c r="A6" s="104" t="inlineStr">
         <is>
-          <t>0.23</t>
+          <t>0.24</t>
         </is>
       </c>
       <c r="B6" s="105" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="C6" s="106" t="inlineStr">
         <is>
-          <t>• Auslegung: Formelzeichen größer (besser lesbare Tiefstellungen); Kopfzeilen-Umbrüche optimiert – keine Trennung mehr mitten im Wort.</t>
+          <t>• Verifikation: Referenzspalte mit echten Werten nach DIN EN 1264 vorbelegt (Nasssystem/Tacker, VL 40 / RL 30 °C, θi 20 °C, R = 0,10 m²K/W); Vergleichsbedingungen entsprechend auf 40/30 °C gesetzt.</t>
         </is>
       </c>
     </row>
@@ -1958,173 +1958,173 @@
       <c r="B7" s="107" t="n"/>
       <c r="C7" s="106" t="inlineStr">
         <is>
-          <t>• Deckblatt: Druck-Hinweis wieder entfernt.</t>
+          <t>• Verifikation: Korrekturfaktor f auf 0,85 vorkalibriert (Best-Fit zu den EN-1264-Werten); Spalte C bleibt editierbar für herstellereigene Datenblattwerte (Rehau, Uponor, Buderus, Kermi …).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="104" t="inlineStr">
         <is>
+          <t>0.23</t>
+        </is>
+      </c>
+      <c r="B8" s="105" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="C8" s="106" t="inlineStr">
+        <is>
+          <t>• Auslegung: Formelzeichen größer (besser lesbare Tiefstellungen); Kopfzeilen-Umbrüche optimiert – keine Trennung mehr mitten im Wort.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="107" t="n"/>
+      <c r="B9" s="107" t="n"/>
+      <c r="C9" s="106" t="inlineStr">
+        <is>
+          <t>• Deckblatt: Druck-Hinweis wieder entfernt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="104" t="inlineStr">
+        <is>
           <t>0.22</t>
         </is>
       </c>
-      <c r="B8" s="105" t="inlineStr">
+      <c r="B10" s="105" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="C8" s="106" t="inlineStr">
+      <c r="C10" s="106" t="inlineStr">
         <is>
           <t>• Anleitung: neue Ampel-Legende (warum ist eine Zelle rot?) und Hinweis zur Auslegung mehrerer Verteiler/Geschosse; Blatt nach hinten verschoben (jetzt vor der Methodik).</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="108" t="n"/>
-      <c r="B9" s="108" t="n"/>
-      <c r="C9" s="106" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="108" t="n"/>
+      <c r="B11" s="108" t="n"/>
+      <c r="C11" s="106" t="inlineStr">
         <is>
           <t>• Deckblatt: Druck-Hinweis ergänzt – nur die relevanten Blätter (Deckblatt, Grundeinstellungen, Auslegung, Kontrolle, HKV, Anleitung) gemeinsam als 'Aktive Blätter' drucken.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="107" t="n"/>
-      <c r="B10" s="107" t="n"/>
-      <c r="C10" s="106" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="107" t="n"/>
+      <c r="B12" s="107" t="n"/>
+      <c r="C12" s="106" t="inlineStr">
         <is>
           <t>• Formelzeichen mit echten Tiefstellungen dargestellt (z. B. q_HL, R_λ,B, V̇_max) – kein Unterstrich mehr in den Kopfzeilen, Grundeinstellungen und der Methodik-Variablenliste.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="104" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="104" t="inlineStr">
         <is>
           <t>0.21</t>
         </is>
       </c>
-      <c r="B11" s="105" t="inlineStr">
+      <c r="B13" s="105" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="C11" s="106" t="inlineStr">
+      <c r="C13" s="106" t="inlineStr">
         <is>
           <t>• Auslegung jetzt auf A4-Querformat (vorher A3); sichtbare Spalten schmaler, damit das Blatt auf A4 passt.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="108" t="n"/>
-      <c r="B12" s="108" t="n"/>
-      <c r="C12" s="106" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="108" t="n"/>
+      <c r="B14" s="108" t="n"/>
+      <c r="C14" s="106" t="inlineStr">
         <is>
           <t>• Deckblatt: Titel 'Fußbodenheizung – Auslegung' (Wort 'überschlägige' entfernt); Vereinfachungen bleiben dokumentiert.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="107" t="n"/>
-      <c r="B13" s="107" t="n"/>
-      <c r="C13" s="106" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="107" t="n"/>
+      <c r="B15" s="107" t="n"/>
+      <c r="C15" s="106" t="inlineStr">
         <is>
           <t>• Anleitung: Abschnitt 'Planungstechnische Grundlagen' wieder entfernt.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="104" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="104" t="inlineStr">
         <is>
           <t>0.20</t>
         </is>
       </c>
-      <c r="B14" s="105" t="inlineStr">
+      <c r="B16" s="105" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="C14" s="106" t="inlineStr">
+      <c r="C16" s="106" t="inlineStr">
         <is>
           <t>• Grundeinstellungen: Spaltenbreiten optimiert und lange Beschriftungen/Hinweise gekürzt – Texte werden in LibreOffice nicht mehr abgeschnitten.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="108" t="n"/>
-      <c r="B15" s="108" t="n"/>
-      <c r="C15" s="106" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="108" t="n"/>
+      <c r="B17" s="108" t="n"/>
+      <c r="C17" s="106" t="inlineStr">
         <is>
           <t>• Verifikation: Untertitel und Hinweise vereinfacht (Modellvergleich-Erläuterung entfernt); klarer Hinweis, dass der Korrekturfaktor f VOR der Raumauslegung kalibriert wird; Diagramm etwas größer.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="107" t="n"/>
-      <c r="B16" s="107" t="n"/>
-      <c r="C16" s="106" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="107" t="n"/>
+      <c r="B18" s="107" t="n"/>
+      <c r="C18" s="106" t="inlineStr">
         <is>
           <t>• Anleitung: Schritt-für-Schritt neu geordnet – Verifikation/Kalibrierung des Korrekturfaktors jetzt VOR der Raumauslegung; neuer Abschnitt 'Planungstechnische Grundlagen'; Hinweis zur vorgefertigten Revit-Liste entfernt.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="104" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="104" t="inlineStr">
         <is>
           <t>0.19</t>
         </is>
       </c>
-      <c r="B17" s="105" t="inlineStr">
+      <c r="B19" s="105" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="C17" s="106" t="inlineStr">
+      <c r="C19" s="106" t="inlineStr">
         <is>
           <t>• Grundeinstellungen: neuer Grenzwert 'Maximaler Volumenstrom je Kreis' (V̇_max, Default 150 l/h); Abschnitt 'Strömungsgeschwindigkeit' → 'Strömungsgrenzwerte'.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="108" t="n"/>
-      <c r="B18" s="108" t="n"/>
-      <c r="C18" s="106" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="108" t="n"/>
+      <c r="B20" s="108" t="n"/>
+      <c r="C20" s="106" t="inlineStr">
         <is>
           <t>• Auslegung: Volumenstrom je Kreis wird gegen V̇_max geprüft und per Ampel eingefärbt (grün ≤ Grenze, rot darüber); zusätzliche Warnung im Blatt 'Kontrolle'.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="108" t="n"/>
-      <c r="B19" s="108" t="n"/>
-      <c r="C19" s="106" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="108" t="n"/>
+      <c r="B21" s="108" t="n"/>
+      <c r="C21" s="106" t="inlineStr">
         <is>
           <t>• Anleitung: durchgehende Schritt-für-Schritt-Anleitung mit integriertem Revit-Export (vorgefertigte Bauteilliste muss nicht erst angelegt werden); redundanter Abschnitt 'Räume aus Revit' und der Hinweis zum direkten Kopieren entfernt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="107" t="n"/>
-      <c r="B20" s="107" t="n"/>
-      <c r="C20" s="106" t="inlineStr">
-        <is>
-          <t>• Deckblatt: Pfeil-Spalten breiter und Pfeilgröße angepasst (optisch sauberer).</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="104" t="inlineStr">
-        <is>
-          <t>0.18</t>
-        </is>
-      </c>
-      <c r="B21" s="105" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="C21" s="106" t="inlineStr">
-        <is>
-          <t>• Auslegung: Eingabespalten neu sortiert – zuerst die Revit-Spalten (A HKV, B Raum-Nr., C Bezeichnung, D Raumfläche, E Raumtemperatur, F Heizlast), dann G spez. Heizlast (berechnet), danach die manuellen Felder (H aktiv. Fläche, I R-Wert, J Verlegeabstand, K Anz. Kreise, L Zuleitung, M Zone).</t>
         </is>
       </c>
     </row>
@@ -2133,14 +2133,14 @@
       <c r="B22" s="107" t="n"/>
       <c r="C22" s="106" t="inlineStr">
         <is>
-          <t>• Anleitung: Excel-Export aus Revit ist jetzt der Standard-Workflow (direktes Kopieren funktioniert nicht); Spaltenliste an neue Reihenfolge angepasst.</t>
+          <t>• Deckblatt: Pfeil-Spalten breiter und Pfeilgröße angepasst (optisch sauberer).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="104" t="inlineStr">
         <is>
-          <t>0.17</t>
+          <t>0.18</t>
         </is>
       </c>
       <c r="B23" s="105" t="inlineStr">
@@ -2150,7 +2150,7 @@
       </c>
       <c r="C23" s="106" t="inlineStr">
         <is>
-          <t>• Neues Blatt 'Anleitung' (2. Blatt): Aufbau der Mappe, Schritt-für-Schritt, Farblegende.</t>
+          <t>• Auslegung: Eingabespalten neu sortiert – zuerst die Revit-Spalten (A HKV, B Raum-Nr., C Bezeichnung, D Raumfläche, E Raumtemperatur, F Heizlast), dann G spez. Heizlast (berechnet), danach die manuellen Felder (H aktiv. Fläche, I R-Wert, J Verlegeabstand, K Anz. Kreise, L Zuleitung, M Zone).</t>
         </is>
       </c>
     </row>
@@ -2159,42 +2159,50 @@
       <c r="B24" s="107" t="n"/>
       <c r="C24" s="106" t="inlineStr">
         <is>
-          <t>• Anleitung enthält den Workflow zum Übernehmen der Räume aus Revit (Copy &amp; Paste, Schedule, Dynamo/Power Query).</t>
+          <t>• Anleitung: Excel-Export aus Revit ist jetzt der Standard-Workflow (direktes Kopieren funktioniert nicht); Spaltenliste an neue Reihenfolge angepasst.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="104" t="inlineStr">
         <is>
+          <t>0.17</t>
+        </is>
+      </c>
+      <c r="B25" s="105" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="C25" s="106" t="inlineStr">
+        <is>
+          <t>• Neues Blatt 'Anleitung' (2. Blatt): Aufbau der Mappe, Schritt-für-Schritt, Farblegende.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="107" t="n"/>
+      <c r="B26" s="107" t="n"/>
+      <c r="C26" s="106" t="inlineStr">
+        <is>
+          <t>• Anleitung enthält den Workflow zum Übernehmen der Räume aus Revit (Copy &amp; Paste, Schedule, Dynamo/Power Query).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="104" t="inlineStr">
+        <is>
           <t>0.16</t>
         </is>
       </c>
-      <c r="B25" s="105" t="inlineStr">
+      <c r="B27" s="105" t="inlineStr">
         <is>
           <t>2026-06-09</t>
         </is>
       </c>
-      <c r="C25" s="106" t="inlineStr">
+      <c r="C27" s="106" t="inlineStr">
         <is>
           <t>• Alle Blätter im A4-Querformat (nur Auslegung A3 quer); einheitlichere Schriftgrößen/Skalierung.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="108" t="n"/>
-      <c r="B26" s="108" t="n"/>
-      <c r="C26" s="106" t="inlineStr">
-        <is>
-          <t>• Grundeinstellungen zweispaltig (Einstellwerte teilweise nebeneinander).</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="108" t="n"/>
-      <c r="B27" s="108" t="n"/>
-      <c r="C27" s="106" t="inlineStr">
-        <is>
-          <t>• Verifikation: Diagramm rechts neben den Tabellen.</t>
         </is>
       </c>
     </row>
@@ -2203,7 +2211,7 @@
       <c r="B28" s="108" t="n"/>
       <c r="C28" s="106" t="inlineStr">
         <is>
-          <t>• Methodik: Formelzeichen links, Berechnungsschritte in zwei Spalten rechts.</t>
+          <t>• Grundeinstellungen zweispaltig (Einstellwerte teilweise nebeneinander).</t>
         </is>
       </c>
     </row>
@@ -2212,103 +2220,103 @@
       <c r="B29" s="108" t="n"/>
       <c r="C29" s="106" t="inlineStr">
         <is>
+          <t>• Verifikation: Diagramm rechts neben den Tabellen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="108" t="n"/>
+      <c r="B30" s="108" t="n"/>
+      <c r="C30" s="106" t="inlineStr">
+        <is>
+          <t>• Methodik: Formelzeichen links, Berechnungsschritte in zwei Spalten rechts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="108" t="n"/>
+      <c r="B31" s="108" t="n"/>
+      <c r="C31" s="106" t="inlineStr">
+        <is>
           <t>• Konstanten: Tabellen teilweise nebeneinander.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="107" t="n"/>
-      <c r="B30" s="107" t="n"/>
-      <c r="C30" s="106" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="107" t="n"/>
+      <c r="B32" s="107" t="n"/>
+      <c r="C32" s="106" t="inlineStr">
         <is>
           <t>• Auslegung: Spalte Zone mittig/schmaler, Raum-Nr. breiter; Verifikation-Korrekturfaktor vertikal mittig.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="104" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="104" t="inlineStr">
         <is>
           <t>0.15</t>
         </is>
       </c>
-      <c r="B31" s="105" t="inlineStr">
+      <c r="B33" s="105" t="inlineStr">
         <is>
           <t>2026-06-09</t>
         </is>
       </c>
-      <c r="C31" s="106" t="inlineStr">
+      <c r="C33" s="106" t="inlineStr">
         <is>
           <t>• Deckblatt-Diagramm aus Excel-Zellen statt Bild – direkt in Excel bearbeitbar.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="108" t="n"/>
-      <c r="B32" s="108" t="n"/>
-      <c r="C32" s="106" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="108" t="n"/>
+      <c r="B34" s="108" t="n"/>
+      <c r="C34" s="106" t="inlineStr">
         <is>
           <t>• Auslegung: Beispielräume mit gemischter Heizlast (≤ 50 W/m²); Formelzeichen in Zeile 5 ergänzt (Flächen u. a.).</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="107" t="n"/>
-      <c r="B33" s="107" t="n"/>
-      <c r="C33" s="106" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="107" t="n"/>
+      <c r="B35" s="107" t="n"/>
+      <c r="C35" s="106" t="inlineStr">
         <is>
           <t>• Heizkreisverteiler: zusätzliche Spalte Spreizung [K].</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="104" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="104" t="inlineStr">
         <is>
           <t>0.14</t>
         </is>
       </c>
-      <c r="B34" s="105" t="inlineStr">
+      <c r="B36" s="105" t="inlineStr">
         <is>
           <t>2026-06-09</t>
         </is>
       </c>
-      <c r="C34" s="106" t="inlineStr">
+      <c r="C36" s="106" t="inlineStr">
         <is>
           <t>• Deckblatt als erstes Blatt: Übersichtsdiagramm Eingaben → Verarbeitung → Ergebnisse (inkl. Vereinfachungen).</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="104" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="104" t="inlineStr">
         <is>
           <t>0.13</t>
         </is>
       </c>
-      <c r="B35" s="105" t="inlineStr">
+      <c r="B37" s="105" t="inlineStr">
         <is>
           <t>2026-06-08</t>
         </is>
       </c>
-      <c r="C35" s="106" t="inlineStr">
+      <c r="C37" s="106" t="inlineStr">
         <is>
           <t>• Strömungsbereich dreistufig: laminar (Re &lt; 2300), Übergangsbereich (2300–4000), turbulent (Re &gt; 4000).</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="108" t="n"/>
-      <c r="B36" s="108" t="n"/>
-      <c r="C36" s="106" t="inlineStr">
-        <is>
-          <t>• Spalte 'Strömungsbereich' ausgeblendet (für die Auslegung nicht relevant) und ohne Färbung.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="108" t="n"/>
-      <c r="B37" s="108" t="n"/>
-      <c r="C37" s="106" t="inlineStr">
-        <is>
-          <t>• Auslegung schlanker: weitere Zwischenspalten standardmäßig ausgeblendet (jederzeit einblendbar).</t>
         </is>
       </c>
     </row>
@@ -2317,51 +2325,51 @@
       <c r="B38" s="108" t="n"/>
       <c r="C38" s="106" t="inlineStr">
         <is>
+          <t>• Spalte 'Strömungsbereich' ausgeblendet (für die Auslegung nicht relevant) und ohne Färbung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="108" t="n"/>
+      <c r="B39" s="108" t="n"/>
+      <c r="C39" s="106" t="inlineStr">
+        <is>
+          <t>• Auslegung schlanker: weitere Zwischenspalten standardmäßig ausgeblendet (jederzeit einblendbar).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="108" t="n"/>
+      <c r="B40" s="108" t="n"/>
+      <c r="C40" s="106" t="inlineStr">
+        <is>
           <t>• Verifikation: Korrekturfaktor kleiner dargestellt (passt nun vollständig in die Zelle).</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="107" t="n"/>
-      <c r="B39" s="107" t="n"/>
-      <c r="C39" s="106" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="107" t="n"/>
+      <c r="B41" s="107" t="n"/>
+      <c r="C41" s="106" t="inlineStr">
         <is>
           <t>• Changelog wieder ausführlich.</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="104" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="104" t="inlineStr">
         <is>
           <t>0.12</t>
         </is>
       </c>
-      <c r="B40" s="105" t="inlineStr">
+      <c r="B42" s="105" t="inlineStr">
         <is>
           <t>2026-06-08</t>
         </is>
       </c>
-      <c r="C40" s="106" t="inlineStr">
+      <c r="C42" s="106" t="inlineStr">
         <is>
           <t>• Grundeinstellungen: Bezeichnungen ausgeschrieben (keine Abkürzungen).</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="108" t="n"/>
-      <c r="B41" s="108" t="n"/>
-      <c r="C41" s="106" t="inlineStr">
-        <is>
-          <t>• Neue Spalte 'spez. Heizlast [W/m²]' (Heizlast bezogen auf die Raumfläche).</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="108" t="n"/>
-      <c r="B42" s="108" t="n"/>
-      <c r="C42" s="106" t="inlineStr">
-        <is>
-          <t>• Massenstrom/Geschwindigkeit/Druckverlust auf Basis min(Leistung; Heizlast) + Verlust nach unten (realer Betriebspunkt).</t>
         </is>
       </c>
     </row>
@@ -2370,340 +2378,340 @@
       <c r="B43" s="108" t="n"/>
       <c r="C43" s="106" t="inlineStr">
         <is>
+          <t>• Neue Spalte 'spez. Heizlast [W/m²]' (Heizlast bezogen auf die Raumfläche).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="108" t="n"/>
+      <c r="B44" s="108" t="n"/>
+      <c r="C44" s="106" t="inlineStr">
+        <is>
+          <t>• Massenstrom/Geschwindigkeit/Druckverlust auf Basis min(Leistung; Heizlast) + Verlust nach unten (realer Betriebspunkt).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="108" t="n"/>
+      <c r="B45" s="108" t="n"/>
+      <c r="C45" s="106" t="inlineStr">
+        <is>
           <t>• Heizkreisverteiler zusätzlich mit Massenstrom [kg/h]; Zonen-Kürzel (AZ/RZ/BAD).</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="107" t="n"/>
-      <c r="B44" s="107" t="n"/>
-      <c r="C44" s="106" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="107" t="n"/>
+      <c r="B46" s="107" t="n"/>
+      <c r="C46" s="106" t="inlineStr">
         <is>
           <t>• Kapazität 200 Räume / 50 Verteiler; Auslegung A3 quer, übrige Blätter A4 hoch.</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="104" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="104" t="inlineStr">
         <is>
           <t>0.11</t>
         </is>
       </c>
-      <c r="B45" s="105" t="inlineStr">
+      <c r="B47" s="105" t="inlineStr">
         <is>
           <t>2026-06-08</t>
         </is>
       </c>
-      <c r="C45" s="106" t="inlineStr">
+      <c r="C47" s="106" t="inlineStr">
         <is>
           <t>• Bugfixes: Hinweistext wurde als Formel interpretiert (Fehler 501); MAXIFS ersetzt (#NAME? in LibreOffice).</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="108" t="n"/>
-      <c r="B46" s="108" t="n"/>
-      <c r="C46" s="106" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="108" t="n"/>
+      <c r="B48" s="108" t="n"/>
+      <c r="C48" s="106" t="inlineStr">
         <is>
           <t>• Verifikation: Korrekturfaktor prominent oben; Hersteller-q direkt neben q berechnet.</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="108" t="n"/>
-      <c r="B47" s="108" t="n"/>
-      <c r="C47" s="106" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="108" t="n"/>
+      <c r="B49" s="108" t="n"/>
+      <c r="C49" s="106" t="inlineStr">
         <is>
           <t>• Konstanten: alle Tabellen untereinander, mit Leerzeilen für weitere Einträge.</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="107" t="n"/>
-      <c r="B48" s="107" t="n"/>
-      <c r="C48" s="106" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="107" t="n"/>
+      <c r="B50" s="107" t="n"/>
+      <c r="C50" s="106" t="inlineStr">
         <is>
           <t>• Methodik: Variablen zuerst, dann Formeln mit Erklärung je Schritt; weitere Musterräume (Verwaltungsbau).</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="104" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="104" t="inlineStr">
         <is>
           <t>0.10</t>
         </is>
       </c>
-      <c r="B49" s="105" t="inlineStr">
+      <c r="B51" s="105" t="inlineStr">
         <is>
           <t>2026-06-08</t>
         </is>
       </c>
-      <c r="C49" s="106" t="inlineStr">
+      <c r="C51" s="106" t="inlineStr">
         <is>
           <t>• Heizkreisverteiler-Liste und Verifikation ohne dynamische Array-Funktionen → läuft in Excel UND LibreOffice.</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="108" t="n"/>
-      <c r="B50" s="108" t="n"/>
-      <c r="C50" s="106" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="108" t="n"/>
+      <c r="B52" s="108" t="n"/>
+      <c r="C52" s="106" t="inlineStr">
         <is>
           <t>• Verifikation mit Liniendiagramm; Konstanten/Bibliotheken in eigenes Blatt ausgelagert.</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="107" t="n"/>
-      <c r="B51" s="107" t="n"/>
-      <c r="C51" s="106" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="107" t="n"/>
+      <c r="B53" s="107" t="n"/>
+      <c r="C53" s="106" t="inlineStr">
         <is>
           <t>• Gewähltes Rohrsystem mit Außen-/Innendurchmesser, Wandstärke und Rauheit im Druckbereich.</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="104" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="104" t="inlineStr">
         <is>
           <t>0.9</t>
         </is>
       </c>
-      <c r="B52" s="105" t="inlineStr">
+      <c r="B54" s="105" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="C52" s="106" t="inlineStr">
+      <c r="C54" s="106" t="inlineStr">
         <is>
           <t>• Neues Blatt 'Heizkreisverteiler' (Leistung, max. Druckverlust, Volumenstrom je HKV).</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="108" t="n"/>
-      <c r="B53" s="108" t="n"/>
-      <c r="C53" s="106" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="108" t="n"/>
+      <c r="B55" s="108" t="n"/>
+      <c r="C55" s="106" t="inlineStr">
         <is>
           <t>• Spaltenüberschriften der Auslegung dreizeilig (Name / Formelzeichen / Einheit).</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="108" t="n"/>
-      <c r="B54" s="108" t="n"/>
-      <c r="C54" s="106" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="108" t="n"/>
+      <c r="B56" s="108" t="n"/>
+      <c r="C56" s="106" t="inlineStr">
         <is>
           <t>• Korrekturfaktor f wird auf 'Verifikation' eingegeben (mit Vergleichsdiagramm).</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="107" t="n"/>
-      <c r="B55" s="107" t="n"/>
-      <c r="C55" s="106" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="107" t="n"/>
+      <c r="B57" s="107" t="n"/>
+      <c r="C57" s="106" t="inlineStr">
         <is>
           <t>• Geschwindigkeits-Grenzwerte v_min/v_max als Grundeinstellung.</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="104" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="104" t="inlineStr">
         <is>
           <t>0.8</t>
         </is>
       </c>
-      <c r="B56" s="105" t="inlineStr">
+      <c r="B58" s="105" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="C56" s="106" t="inlineStr">
+      <c r="C58" s="106" t="inlineStr">
         <is>
           <t>• Grundeinstellungen für A3 quer optimiert (Einstellungen links, Tabellen rechts).</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="108" t="n"/>
-      <c r="B57" s="108" t="n"/>
-      <c r="C57" s="106" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="108" t="n"/>
+      <c r="B59" s="108" t="n"/>
+      <c r="C59" s="106" t="inlineStr">
         <is>
           <t>• Auslegung passt auf eine Seite breit; Korrekturfaktor Heizleistung zur Kalibrierung ergänzt.</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="108" t="n"/>
-      <c r="B58" s="108" t="n"/>
-      <c r="C58" s="106" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="108" t="n"/>
+      <c r="B60" s="108" t="n"/>
+      <c r="C60" s="106" t="inlineStr">
         <is>
           <t>• Wärmeabgabe nach unten berücksichtigt (Verlust + Gesamtleistung).</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="107" t="n"/>
-      <c r="B59" s="107" t="n"/>
-      <c r="C59" s="106" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="107" t="n"/>
+      <c r="B61" s="107" t="n"/>
+      <c r="C61" s="106" t="inlineStr">
         <is>
           <t>• Blätter umbenannt: Raumliste → Auslegung, Übersicht → Kontrolle; zusätzliche Kontrollen.</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="104" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="104" t="inlineStr">
         <is>
           <t>0.7</t>
         </is>
       </c>
-      <c r="B60" s="105" t="inlineStr">
+      <c r="B62" s="105" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="C60" s="106" t="inlineStr">
+      <c r="C62" s="106" t="inlineStr">
         <is>
           <t>• Deckung-%-Spalte färbt nur noch gefüllte Zellen (leere bleiben farblos).</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="108" t="n"/>
-      <c r="B61" s="108" t="n"/>
-      <c r="C61" s="106" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="108" t="n"/>
+      <c r="B63" s="108" t="n"/>
+      <c r="C63" s="106" t="inlineStr">
         <is>
           <t>• Neues Blatt 'Verifikation'; neue Spalte 'Strömungsbereich' (laminar/turbulent).</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="107" t="n"/>
-      <c r="B62" s="107" t="n"/>
-      <c r="C62" s="106" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="107" t="n"/>
+      <c r="B64" s="107" t="n"/>
+      <c r="C64" s="106" t="inlineStr">
         <is>
           <t>• Alle Blätter im A3-Querformat; einheitlicher Kopf je Blatt.</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="104" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="104" t="inlineStr">
         <is>
           <t>0.6</t>
         </is>
       </c>
-      <c r="B63" s="105" t="inlineStr">
+      <c r="B65" s="105" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="C63" s="106" t="inlineStr">
+      <c r="C65" s="106" t="inlineStr">
         <is>
           <t>• Bugfix: Zellfärbung (bedingte Formatierung) wird jetzt auch in Excel angezeigt – dxf-Füllfarbe mit voller Deckkraft.</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="104" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
-      </c>
-      <c r="B64" s="105" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C64" s="106" t="inlineStr">
-        <is>
-          <t>• Versionsnummer und Autor werden nur noch im Changelog angezeigt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="107" t="n"/>
-      <c r="B65" s="107" t="n"/>
-      <c r="C65" s="106" t="inlineStr">
-        <is>
-          <t>• Editierbares Bearbeiter-Kürzel rechts oben unter dem Logo (Grundeinstellungen, Auslegung, Kontrolle, HKV).</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="104" t="inlineStr">
         <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="B66" s="105" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="C66" s="106" t="inlineStr">
+        <is>
+          <t>• Versionsnummer und Autor werden nur noch im Changelog angezeigt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="107" t="n"/>
+      <c r="B67" s="107" t="n"/>
+      <c r="C67" s="106" t="inlineStr">
+        <is>
+          <t>• Editierbares Bearbeiter-Kürzel rechts oben unter dem Logo (Grundeinstellungen, Auslegung, Kontrolle, HKV).</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="104" t="inlineStr">
+        <is>
           <t>0.4</t>
         </is>
       </c>
-      <c r="B66" s="105" t="inlineStr">
+      <c r="B68" s="105" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="C66" s="106" t="inlineStr">
+      <c r="C68" s="106" t="inlineStr">
         <is>
           <t>• Status-Spalten entfernt – Bewertung erfolgt jetzt direkt als Zellfärbung (grün/rot).</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="108" t="n"/>
-      <c r="B67" s="108" t="n"/>
-      <c r="C67" s="106" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="108" t="n"/>
+      <c r="B69" s="108" t="n"/>
+      <c r="C69" s="106" t="inlineStr">
         <is>
           <t>• Methodik um die Formelzeichen-Legende erweitert.</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="108" t="n"/>
-      <c r="B68" s="108" t="n"/>
-      <c r="C68" s="106" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="108" t="n"/>
+      <c r="B70" s="108" t="n"/>
+      <c r="C70" s="106" t="inlineStr">
         <is>
           <t>• Heizkreisverteiler (HKV) als erste Spalte der Auslegung; Standardwert max. Druckverlust 15.000 Pa.</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="107" t="n"/>
-      <c r="B69" s="107" t="n"/>
-      <c r="C69" s="106" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="107" t="n"/>
+      <c r="B71" s="107" t="n"/>
+      <c r="C71" s="106" t="inlineStr">
         <is>
           <t>• Versionsschema 0.x eingeführt (1.0 erst nach Test); interner Autor (dh).</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="104" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="104" t="inlineStr">
         <is>
           <t>0.3</t>
         </is>
       </c>
-      <c r="B70" s="105" t="inlineStr">
+      <c r="B72" s="105" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="C70" s="106" t="inlineStr">
+      <c r="C72" s="106" t="inlineStr">
         <is>
           <t>• Zonentypen (Aufenthalt/Rand/Bad) mit eigener zulässiger Oberflächentemperatur.</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="108" t="n"/>
-      <c r="B71" s="108" t="n"/>
-      <c r="C71" s="106" t="inlineStr">
-        <is>
-          <t>• Einheitlicher Kopf: Titel oben links, agn-Logo oben rechts, Projektkopf darunter.</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="108" t="n"/>
-      <c r="B72" s="108" t="n"/>
-      <c r="C72" s="106" t="inlineStr">
-        <is>
-          <t>• Oberflächentemperatur θF und Volumenstrom eingeblendet.</t>
         </is>
       </c>
     </row>
@@ -2712,51 +2720,51 @@
       <c r="B73" s="108" t="n"/>
       <c r="C73" s="106" t="inlineStr">
         <is>
+          <t>• Einheitlicher Kopf: Titel oben links, agn-Logo oben rechts, Projektkopf darunter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="108" t="n"/>
+      <c r="B74" s="108" t="n"/>
+      <c r="C74" s="106" t="inlineStr">
+        <is>
+          <t>• Oberflächentemperatur θF und Volumenstrom eingeblendet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="108" t="n"/>
+      <c r="B75" s="108" t="n"/>
+      <c r="C75" s="106" t="inlineStr">
+        <is>
           <t>• Neue Spalten 'spez. Druckverlust [Pa/m]' und Eingabespalte 'Verteiler (Anbindung)'.</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="107" t="n"/>
-      <c r="B74" s="107" t="n"/>
-      <c r="C74" s="106" t="inlineStr">
+    <row r="76">
+      <c r="A76" s="107" t="n"/>
+      <c r="B76" s="107" t="n"/>
+      <c r="C76" s="106" t="inlineStr">
         <is>
           <t>• Warnung (rot), wenn die aktivierbare Fläche größer als die Raumfläche ist.</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="104" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="104" t="inlineStr">
         <is>
           <t>0.2</t>
         </is>
       </c>
-      <c r="B75" s="105" t="inlineStr">
+      <c r="B77" s="105" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="C75" s="106" t="inlineStr">
+      <c r="C77" s="106" t="inlineStr">
         <is>
           <t>• agn-Logo eingebunden und eigenes Changelog-Blatt ergänzt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="108" t="n"/>
-      <c r="B76" s="108" t="n"/>
-      <c r="C76" s="106" t="inlineStr">
-        <is>
-          <t>• Zuschlag Einzelwiderstände (5 %) und fester Verteiler-Aufschlag (500 Pa je Kreis).</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="108" t="n"/>
-      <c r="B77" s="108" t="n"/>
-      <c r="C77" s="106" t="inlineStr">
-        <is>
-          <t>• Einheiten als Zellformat; Projektnummer/Projektname erscheinen im Ausdruck.</t>
         </is>
       </c>
     </row>
@@ -2765,51 +2773,51 @@
       <c r="B78" s="108" t="n"/>
       <c r="C78" s="106" t="inlineStr">
         <is>
+          <t>• Zuschlag Einzelwiderstände (5 %) und fester Verteiler-Aufschlag (500 Pa je Kreis).</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="108" t="n"/>
+      <c r="B79" s="108" t="n"/>
+      <c r="C79" s="106" t="inlineStr">
+        <is>
+          <t>• Einheiten als Zellformat; Projektnummer/Projektname erscheinen im Ausdruck.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="108" t="n"/>
+      <c r="B80" s="108" t="n"/>
+      <c r="C80" s="106" t="inlineStr">
+        <is>
           <t>• Richtwert-Tabellen für R-Werte und Verlegeabstand-Faktoren; weitere Musterräume.</t>
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="107" t="n"/>
-      <c r="B79" s="107" t="n"/>
-      <c r="C79" s="106" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="107" t="n"/>
+      <c r="B81" s="107" t="n"/>
+      <c r="C81" s="106" t="inlineStr">
         <is>
           <t>• Druckaufbereitung für DIN A4.</t>
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" s="104" t="inlineStr">
+    <row r="82">
+      <c r="A82" s="104" t="inlineStr">
         <is>
           <t>0.1</t>
         </is>
       </c>
-      <c r="B80" s="105" t="inlineStr">
+      <c r="B82" s="105" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="C80" s="106" t="inlineStr">
+      <c r="C82" s="106" t="inlineStr">
         <is>
           <t>• Ersterstellung mit den Blättern Grundeinstellungen, Raumliste, Übersicht und Methodik.</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="108" t="n"/>
-      <c r="B81" s="108" t="n"/>
-      <c r="C81" s="106" t="inlineStr">
-        <is>
-          <t>• Heizleistung über die logarithmische Übertemperatur (q = η · K_H · ΔθH).</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="108" t="n"/>
-      <c r="B82" s="108" t="n"/>
-      <c r="C82" s="106" t="inlineStr">
-        <is>
-          <t>• Druckverlustberechnung nach Darcy-Weisbach.</t>
         </is>
       </c>
     </row>
@@ -2818,63 +2826,83 @@
       <c r="B83" s="108" t="n"/>
       <c r="C83" s="106" t="inlineStr">
         <is>
+          <t>• Heizleistung über die logarithmische Übertemperatur (q = η · K_H · ΔθH).</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="108" t="n"/>
+      <c r="B84" s="108" t="n"/>
+      <c r="C84" s="106" t="inlineStr">
+        <is>
+          <t>• Druckverlustberechnung nach Darcy-Weisbach.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="108" t="n"/>
+      <c r="B85" s="108" t="n"/>
+      <c r="C85" s="106" t="inlineStr">
+        <is>
           <t>• Editierbare Rohrbibliothek und Verlegeabstand-Faktoren.</t>
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="107" t="n"/>
-      <c r="B84" s="107" t="n"/>
-      <c r="C84" s="106" t="inlineStr">
+    <row r="86">
+      <c r="A86" s="107" t="n"/>
+      <c r="B86" s="107" t="n"/>
+      <c r="C86" s="106" t="inlineStr">
         <is>
           <t>• Prüfungen: Oberflächentemperatur, Heizlastdeckung, Kreislänge, Druckverlust.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="42">
-    <mergeCell ref="B66:B69"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="B49:B51"/>
-    <mergeCell ref="B56:B59"/>
-    <mergeCell ref="B25:B30"/>
-    <mergeCell ref="A45:A48"/>
+  <mergeCells count="44">
+    <mergeCell ref="B82:B86"/>
+    <mergeCell ref="B47:B50"/>
+    <mergeCell ref="A33:A35"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="B33:B35"/>
+    <mergeCell ref="A42:A46"/>
+    <mergeCell ref="B37:B41"/>
     <mergeCell ref="A6:A7"/>
-    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="A72:A76"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="A66:A67"/>
+    <mergeCell ref="B27:B32"/>
+    <mergeCell ref="A13:A15"/>
+    <mergeCell ref="A62:A64"/>
     <mergeCell ref="B23:B24"/>
-    <mergeCell ref="B40:B44"/>
-    <mergeCell ref="B52:B55"/>
-    <mergeCell ref="A66:A69"/>
-    <mergeCell ref="B17:B20"/>
-    <mergeCell ref="A35:A39"/>
-    <mergeCell ref="A25:A30"/>
-    <mergeCell ref="A56:A59"/>
-    <mergeCell ref="B80:B84"/>
-    <mergeCell ref="A31:A33"/>
-    <mergeCell ref="A49:A51"/>
+    <mergeCell ref="B51:B53"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="B58:B61"/>
+    <mergeCell ref="A77:A81"/>
+    <mergeCell ref="B16:B18"/>
+    <mergeCell ref="B19:B22"/>
     <mergeCell ref="B6:B7"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="B35:B39"/>
-    <mergeCell ref="A40:A44"/>
-    <mergeCell ref="B31:B33"/>
-    <mergeCell ref="A17:A20"/>
-    <mergeCell ref="A60:A62"/>
-    <mergeCell ref="B64:B65"/>
-    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="B54:B57"/>
+    <mergeCell ref="B72:B76"/>
+    <mergeCell ref="A27:A32"/>
+    <mergeCell ref="B62:B64"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A51:A53"/>
+    <mergeCell ref="A82:A86"/>
     <mergeCell ref="A23:A24"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="B75:B79"/>
-    <mergeCell ref="A70:A74"/>
-    <mergeCell ref="A64:A65"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="B60:B62"/>
-    <mergeCell ref="B45:B48"/>
-    <mergeCell ref="B70:B74"/>
-    <mergeCell ref="A80:A84"/>
-    <mergeCell ref="A75:A79"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="A52:A55"/>
+    <mergeCell ref="B68:B71"/>
+    <mergeCell ref="A19:A22"/>
+    <mergeCell ref="A47:A50"/>
+    <mergeCell ref="B10:B12"/>
+    <mergeCell ref="A16:A18"/>
+    <mergeCell ref="B66:B67"/>
+    <mergeCell ref="B77:B81"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="B42:B46"/>
+    <mergeCell ref="A68:A71"/>
+    <mergeCell ref="A37:A41"/>
+    <mergeCell ref="A58:A61"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -29708,7 +29736,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -29756,7 +29784,7 @@
       </c>
       <c r="B5" s="88" t="n"/>
       <c r="C5" s="89" t="n">
-        <v>1</v>
+        <v>0.85</v>
       </c>
       <c r="D5" s="28" t="inlineStr">
         <is>
@@ -29780,7 +29808,7 @@
         </is>
       </c>
       <c r="B8" s="26" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C8" s="27" t="inlineStr">
         <is>
@@ -29795,7 +29823,7 @@
         </is>
       </c>
       <c r="B9" s="26" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C9" s="27" t="inlineStr">
         <is>
@@ -29853,7 +29881,8 @@
       </c>
       <c r="C14" s="47" t="inlineStr">
         <is>
-          <t>Hersteller q [W/m²]</t>
+          <t>Referenz q
+EN 1264 [W/m²]</t>
         </is>
       </c>
       <c r="D14" s="48" t="inlineStr">
@@ -29891,7 +29920,7 @@
         <v/>
       </c>
       <c r="C15" s="90" t="n">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="D15" s="65">
         <f>IF(OR($B15="",$C15=""),"",$C15-$B15)</f>
@@ -29923,7 +29952,7 @@
         <v/>
       </c>
       <c r="C16" s="90" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="D16" s="65">
         <f>IF(OR($B16="",$C16=""),"",$C16-$B16)</f>
@@ -29955,7 +29984,7 @@
         <v/>
       </c>
       <c r="C17" s="90" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="D17" s="65">
         <f>IF(OR($B17="",$C17=""),"",$C17-$B17)</f>
@@ -29987,7 +30016,7 @@
         <v/>
       </c>
       <c r="C18" s="90" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D18" s="65">
         <f>IF(OR($B18="",$C18=""),"",$C18-$B18)</f>
@@ -30019,7 +30048,7 @@
         <v/>
       </c>
       <c r="C19" s="90" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D19" s="65">
         <f>IF(OR($B19="",$C19=""),"",$C19-$B19)</f>
@@ -30051,7 +30080,7 @@
         <v/>
       </c>
       <c r="C20" s="90" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D20" s="65">
         <f>IF(OR($B20="",$C20=""),"",$C20-$B20)</f>
@@ -30115,7 +30144,7 @@
         <v/>
       </c>
       <c r="C22" s="90" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D22" s="65">
         <f>IF(OR($B22="",$C22=""),"",$C22-$B22)</f>
@@ -30148,35 +30177,56 @@
     <row r="25">
       <c r="A25" s="25" t="inlineStr">
         <is>
-          <t>• Hersteller-q je Verlegeabstand aus dem Datenblatt in Spalte C eintragen.</t>
+          <t>• Referenzwerte (Spalte C) nach DIN EN 1264 – Nasssystem/Tacker, Standardestrich,</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="25" t="inlineStr">
         <is>
-          <t>• Korrekturfaktor f oben so einstellen, dass berechnetes q und Hersteller-q</t>
+          <t xml:space="preserve">   VL 40 / RL 30 °C, θi 20 °C, Bodenbelag R = 0,10 m²K/W. Quelle: fussbodenheizung24.de.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">   möglichst übereinstimmen (Abweichung grün).</t>
+          <t>• Alle nach EN 1264 zertifizierten Systeme (Rehau, Uponor, Buderus, Kermi …) liegen</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="28" t="inlineStr">
-        <is>
-          <t>• Der so kalibrierte Faktor f gilt für die gesamte Auslegung – daher VOR</t>
+      <c r="A28" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   nah an diesen Werten – herstellereigene Datenblattwerte einfach in Spalte C eintragen.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   der Raumauslegung kalibrieren.</t>
+      <c r="A29" s="25" t="inlineStr">
+        <is>
+          <t>• Korrekturfaktor f oben so einstellen, dass berechnetes q und Referenz-q übereinstimmen</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   (Abweichung grün). f ≈ 0,85 passt zu den EN-1264-Werten oben.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="28" t="inlineStr">
+        <is>
+          <t>• Der kalibrierte Faktor f gilt für die gesamte Auslegung – daher VOR der Raumauslegung</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   kalibrieren.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
FBH-Auslegung v0.25 - 'Korrekturfaktor' -> 'Systemfaktor (EN-1264-Kalibrierung)'
Begriff umbenannt in Verifikation (Label + Hinweise), Methodik-Variablenliste, Deckblatt (Input + Vereinfachungen) und Anleitung. f ist die bewusste Kalibrierung des ueberschlaegigen Modells an EN 1264 (buendelt Rohrwand- und Estrichspreizungs-Widerstand), kein Fehlerfaktor - daher neutralerer Name. Changelog-Historie unveraendert.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FBH_Auslegung.xlsx
+++ b/FBH_Auslegung.xlsx
@@ -25,11 +25,11 @@
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Auslegung'!$A$1:$AK$206</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'Kontrolle'!$A$1:$D$25</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'HKV'!$A$1:$G$56</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="5">'Verifikation'!$A$1:$Q$28</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'Verifikation'!$A$1:$Q$34</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="6">'Anleitung'!$A$1:$D$32</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">'Methodik'!$A$1:$F$26</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="8">'Konstanten'!$A$1:$I$26</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="9">'Changelog'!$A$1:$C$86</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="9">'Changelog'!$A$1:$C$87</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1563,7 +1563,7 @@
 • R-Wert Belag, Verlegeabstand
 • Anzahl Kreise, Zuleitung, Zone, HKV
 Kalibrierung
-• Korrekturfaktor f</t>
+• Systemfaktor f (EN 1264)</t>
         </is>
       </c>
       <c r="B6" s="11" t="n"/>
@@ -1829,7 +1829,7 @@
     <row r="27">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>Vereinfachtes K_H + Verlegeabstand-Faktor statt vollständigem EN 1264   ·   Rohrwandwiderstand nicht enthalten (→ Korrekturfaktor f)   ·   Wärmeabgabe nach unten global (gleiche Dämmung)   ·   pauschaler Druckverlust-Zuschlag + fester Verteiler-Aufschlag</t>
+          <t>Vereinfachtes K_H + Verlegeabstand-Faktor statt vollständigem EN 1264   ·   Rohrwandwiderstand nicht enthalten (→ Systemfaktor f)   ·   Wärmeabgabe nach unten global (gleiche Dämmung)   ·   pauschaler Druckverlust-Zuschlag + fester Verteiler-Aufschlag</t>
         </is>
       </c>
       <c r="B27" s="16" t="n"/>
@@ -1897,7 +1897,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C86"/>
+  <dimension ref="A1:C87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1915,7 +1915,7 @@
     <row r="3">
       <c r="C3" s="21" t="inlineStr">
         <is>
-          <t>Version 0.24 · dh</t>
+          <t>Version 0.25 · dh</t>
         </is>
       </c>
     </row>
@@ -1939,183 +1939,191 @@
     <row r="6">
       <c r="A6" s="104" t="inlineStr">
         <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="B6" s="105" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="C6" s="106" t="inlineStr">
+        <is>
+          <t>• Begriff 'Korrekturfaktor' in 'Systemfaktor (EN-1264-Kalibrierung)' umbenannt (Verifikation, Methodik, Deckblatt, Anleitung) – f ist die bewusste Kalibrierung des überschlägigen Modells an EN 1264, kein Fehlerfaktor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="104" t="inlineStr">
+        <is>
           <t>0.24</t>
         </is>
       </c>
-      <c r="B6" s="105" t="inlineStr">
+      <c r="B7" s="105" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="C6" s="106" t="inlineStr">
+      <c r="C7" s="106" t="inlineStr">
         <is>
           <t>• Verifikation: Referenzspalte mit echten Werten nach DIN EN 1264 vorbelegt (Nasssystem/Tacker, VL 40 / RL 30 °C, θi 20 °C, R = 0,10 m²K/W); Vergleichsbedingungen entsprechend auf 40/30 °C gesetzt.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="107" t="n"/>
-      <c r="B7" s="107" t="n"/>
-      <c r="C7" s="106" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="107" t="n"/>
+      <c r="B8" s="107" t="n"/>
+      <c r="C8" s="106" t="inlineStr">
         <is>
           <t>• Verifikation: Korrekturfaktor f auf 0,85 vorkalibriert (Best-Fit zu den EN-1264-Werten); Spalte C bleibt editierbar für herstellereigene Datenblattwerte (Rehau, Uponor, Buderus, Kermi …).</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="104" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="104" t="inlineStr">
         <is>
           <t>0.23</t>
         </is>
       </c>
-      <c r="B8" s="105" t="inlineStr">
+      <c r="B9" s="105" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="C8" s="106" t="inlineStr">
+      <c r="C9" s="106" t="inlineStr">
         <is>
           <t>• Auslegung: Formelzeichen größer (besser lesbare Tiefstellungen); Kopfzeilen-Umbrüche optimiert – keine Trennung mehr mitten im Wort.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="107" t="n"/>
-      <c r="B9" s="107" t="n"/>
-      <c r="C9" s="106" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="107" t="n"/>
+      <c r="B10" s="107" t="n"/>
+      <c r="C10" s="106" t="inlineStr">
         <is>
           <t>• Deckblatt: Druck-Hinweis wieder entfernt.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="104" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="104" t="inlineStr">
         <is>
           <t>0.22</t>
         </is>
       </c>
-      <c r="B10" s="105" t="inlineStr">
+      <c r="B11" s="105" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="C10" s="106" t="inlineStr">
+      <c r="C11" s="106" t="inlineStr">
         <is>
           <t>• Anleitung: neue Ampel-Legende (warum ist eine Zelle rot?) und Hinweis zur Auslegung mehrerer Verteiler/Geschosse; Blatt nach hinten verschoben (jetzt vor der Methodik).</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="108" t="n"/>
-      <c r="B11" s="108" t="n"/>
-      <c r="C11" s="106" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="108" t="n"/>
+      <c r="B12" s="108" t="n"/>
+      <c r="C12" s="106" t="inlineStr">
         <is>
           <t>• Deckblatt: Druck-Hinweis ergänzt – nur die relevanten Blätter (Deckblatt, Grundeinstellungen, Auslegung, Kontrolle, HKV, Anleitung) gemeinsam als 'Aktive Blätter' drucken.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="107" t="n"/>
-      <c r="B12" s="107" t="n"/>
-      <c r="C12" s="106" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="107" t="n"/>
+      <c r="B13" s="107" t="n"/>
+      <c r="C13" s="106" t="inlineStr">
         <is>
           <t>• Formelzeichen mit echten Tiefstellungen dargestellt (z. B. q_HL, R_λ,B, V̇_max) – kein Unterstrich mehr in den Kopfzeilen, Grundeinstellungen und der Methodik-Variablenliste.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="104" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="104" t="inlineStr">
         <is>
           <t>0.21</t>
         </is>
       </c>
-      <c r="B13" s="105" t="inlineStr">
+      <c r="B14" s="105" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="C13" s="106" t="inlineStr">
+      <c r="C14" s="106" t="inlineStr">
         <is>
           <t>• Auslegung jetzt auf A4-Querformat (vorher A3); sichtbare Spalten schmaler, damit das Blatt auf A4 passt.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="108" t="n"/>
-      <c r="B14" s="108" t="n"/>
-      <c r="C14" s="106" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="108" t="n"/>
+      <c r="B15" s="108" t="n"/>
+      <c r="C15" s="106" t="inlineStr">
         <is>
           <t>• Deckblatt: Titel 'Fußbodenheizung – Auslegung' (Wort 'überschlägige' entfernt); Vereinfachungen bleiben dokumentiert.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="107" t="n"/>
-      <c r="B15" s="107" t="n"/>
-      <c r="C15" s="106" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="107" t="n"/>
+      <c r="B16" s="107" t="n"/>
+      <c r="C16" s="106" t="inlineStr">
         <is>
           <t>• Anleitung: Abschnitt 'Planungstechnische Grundlagen' wieder entfernt.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="104" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="104" t="inlineStr">
         <is>
           <t>0.20</t>
         </is>
       </c>
-      <c r="B16" s="105" t="inlineStr">
+      <c r="B17" s="105" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="C16" s="106" t="inlineStr">
+      <c r="C17" s="106" t="inlineStr">
         <is>
           <t>• Grundeinstellungen: Spaltenbreiten optimiert und lange Beschriftungen/Hinweise gekürzt – Texte werden in LibreOffice nicht mehr abgeschnitten.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="108" t="n"/>
-      <c r="B17" s="108" t="n"/>
-      <c r="C17" s="106" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="108" t="n"/>
+      <c r="B18" s="108" t="n"/>
+      <c r="C18" s="106" t="inlineStr">
         <is>
           <t>• Verifikation: Untertitel und Hinweise vereinfacht (Modellvergleich-Erläuterung entfernt); klarer Hinweis, dass der Korrekturfaktor f VOR der Raumauslegung kalibriert wird; Diagramm etwas größer.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="107" t="n"/>
-      <c r="B18" s="107" t="n"/>
-      <c r="C18" s="106" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="107" t="n"/>
+      <c r="B19" s="107" t="n"/>
+      <c r="C19" s="106" t="inlineStr">
         <is>
           <t>• Anleitung: Schritt-für-Schritt neu geordnet – Verifikation/Kalibrierung des Korrekturfaktors jetzt VOR der Raumauslegung; neuer Abschnitt 'Planungstechnische Grundlagen'; Hinweis zur vorgefertigten Revit-Liste entfernt.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="104" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="104" t="inlineStr">
         <is>
           <t>0.19</t>
         </is>
       </c>
-      <c r="B19" s="105" t="inlineStr">
+      <c r="B20" s="105" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="C19" s="106" t="inlineStr">
+      <c r="C20" s="106" t="inlineStr">
         <is>
           <t>• Grundeinstellungen: neuer Grenzwert 'Maximaler Volumenstrom je Kreis' (V̇_max, Default 150 l/h); Abschnitt 'Strömungsgeschwindigkeit' → 'Strömungsgrenzwerte'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="108" t="n"/>
-      <c r="B20" s="108" t="n"/>
-      <c r="C20" s="106" t="inlineStr">
-        <is>
-          <t>• Auslegung: Volumenstrom je Kreis wird gegen V̇_max geprüft und per Ampel eingefärbt (grün ≤ Grenze, rot darüber); zusätzliche Warnung im Blatt 'Kontrolle'.</t>
         </is>
       </c>
     </row>
@@ -2124,94 +2132,94 @@
       <c r="B21" s="108" t="n"/>
       <c r="C21" s="106" t="inlineStr">
         <is>
+          <t>• Auslegung: Volumenstrom je Kreis wird gegen V̇_max geprüft und per Ampel eingefärbt (grün ≤ Grenze, rot darüber); zusätzliche Warnung im Blatt 'Kontrolle'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="108" t="n"/>
+      <c r="B22" s="108" t="n"/>
+      <c r="C22" s="106" t="inlineStr">
+        <is>
           <t>• Anleitung: durchgehende Schritt-für-Schritt-Anleitung mit integriertem Revit-Export (vorgefertigte Bauteilliste muss nicht erst angelegt werden); redundanter Abschnitt 'Räume aus Revit' und der Hinweis zum direkten Kopieren entfernt.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="107" t="n"/>
-      <c r="B22" s="107" t="n"/>
-      <c r="C22" s="106" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="107" t="n"/>
+      <c r="B23" s="107" t="n"/>
+      <c r="C23" s="106" t="inlineStr">
         <is>
           <t>• Deckblatt: Pfeil-Spalten breiter und Pfeilgröße angepasst (optisch sauberer).</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="104" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="104" t="inlineStr">
         <is>
           <t>0.18</t>
         </is>
       </c>
-      <c r="B23" s="105" t="inlineStr">
+      <c r="B24" s="105" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="C23" s="106" t="inlineStr">
+      <c r="C24" s="106" t="inlineStr">
         <is>
           <t>• Auslegung: Eingabespalten neu sortiert – zuerst die Revit-Spalten (A HKV, B Raum-Nr., C Bezeichnung, D Raumfläche, E Raumtemperatur, F Heizlast), dann G spez. Heizlast (berechnet), danach die manuellen Felder (H aktiv. Fläche, I R-Wert, J Verlegeabstand, K Anz. Kreise, L Zuleitung, M Zone).</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="107" t="n"/>
-      <c r="B24" s="107" t="n"/>
-      <c r="C24" s="106" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="107" t="n"/>
+      <c r="B25" s="107" t="n"/>
+      <c r="C25" s="106" t="inlineStr">
         <is>
           <t>• Anleitung: Excel-Export aus Revit ist jetzt der Standard-Workflow (direktes Kopieren funktioniert nicht); Spaltenliste an neue Reihenfolge angepasst.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="104" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="104" t="inlineStr">
         <is>
           <t>0.17</t>
         </is>
       </c>
-      <c r="B25" s="105" t="inlineStr">
+      <c r="B26" s="105" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="C25" s="106" t="inlineStr">
+      <c r="C26" s="106" t="inlineStr">
         <is>
           <t>• Neues Blatt 'Anleitung' (2. Blatt): Aufbau der Mappe, Schritt-für-Schritt, Farblegende.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="107" t="n"/>
-      <c r="B26" s="107" t="n"/>
-      <c r="C26" s="106" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="107" t="n"/>
+      <c r="B27" s="107" t="n"/>
+      <c r="C27" s="106" t="inlineStr">
         <is>
           <t>• Anleitung enthält den Workflow zum Übernehmen der Räume aus Revit (Copy &amp; Paste, Schedule, Dynamo/Power Query).</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="104" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="104" t="inlineStr">
         <is>
           <t>0.16</t>
         </is>
       </c>
-      <c r="B27" s="105" t="inlineStr">
+      <c r="B28" s="105" t="inlineStr">
         <is>
           <t>2026-06-09</t>
         </is>
       </c>
-      <c r="C27" s="106" t="inlineStr">
+      <c r="C28" s="106" t="inlineStr">
         <is>
           <t>• Alle Blätter im A4-Querformat (nur Auslegung A3 quer); einheitlichere Schriftgrößen/Skalierung.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="108" t="n"/>
-      <c r="B28" s="108" t="n"/>
-      <c r="C28" s="106" t="inlineStr">
-        <is>
-          <t>• Grundeinstellungen zweispaltig (Einstellwerte teilweise nebeneinander).</t>
         </is>
       </c>
     </row>
@@ -2220,7 +2228,7 @@
       <c r="B29" s="108" t="n"/>
       <c r="C29" s="106" t="inlineStr">
         <is>
-          <t>• Verifikation: Diagramm rechts neben den Tabellen.</t>
+          <t>• Grundeinstellungen zweispaltig (Einstellwerte teilweise nebeneinander).</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2237,7 @@
       <c r="B30" s="108" t="n"/>
       <c r="C30" s="106" t="inlineStr">
         <is>
-          <t>• Methodik: Formelzeichen links, Berechnungsschritte in zwei Spalten rechts.</t>
+          <t>• Verifikation: Diagramm rechts neben den Tabellen.</t>
         </is>
       </c>
     </row>
@@ -2238,94 +2246,94 @@
       <c r="B31" s="108" t="n"/>
       <c r="C31" s="106" t="inlineStr">
         <is>
+          <t>• Methodik: Formelzeichen links, Berechnungsschritte in zwei Spalten rechts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="108" t="n"/>
+      <c r="B32" s="108" t="n"/>
+      <c r="C32" s="106" t="inlineStr">
+        <is>
           <t>• Konstanten: Tabellen teilweise nebeneinander.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="107" t="n"/>
-      <c r="B32" s="107" t="n"/>
-      <c r="C32" s="106" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="107" t="n"/>
+      <c r="B33" s="107" t="n"/>
+      <c r="C33" s="106" t="inlineStr">
         <is>
           <t>• Auslegung: Spalte Zone mittig/schmaler, Raum-Nr. breiter; Verifikation-Korrekturfaktor vertikal mittig.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="104" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="104" t="inlineStr">
         <is>
           <t>0.15</t>
         </is>
       </c>
-      <c r="B33" s="105" t="inlineStr">
+      <c r="B34" s="105" t="inlineStr">
         <is>
           <t>2026-06-09</t>
         </is>
       </c>
-      <c r="C33" s="106" t="inlineStr">
+      <c r="C34" s="106" t="inlineStr">
         <is>
           <t>• Deckblatt-Diagramm aus Excel-Zellen statt Bild – direkt in Excel bearbeitbar.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="108" t="n"/>
-      <c r="B34" s="108" t="n"/>
-      <c r="C34" s="106" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="108" t="n"/>
+      <c r="B35" s="108" t="n"/>
+      <c r="C35" s="106" t="inlineStr">
         <is>
           <t>• Auslegung: Beispielräume mit gemischter Heizlast (≤ 50 W/m²); Formelzeichen in Zeile 5 ergänzt (Flächen u. a.).</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="107" t="n"/>
-      <c r="B35" s="107" t="n"/>
-      <c r="C35" s="106" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="107" t="n"/>
+      <c r="B36" s="107" t="n"/>
+      <c r="C36" s="106" t="inlineStr">
         <is>
           <t>• Heizkreisverteiler: zusätzliche Spalte Spreizung [K].</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="104" t="inlineStr">
-        <is>
-          <t>0.14</t>
-        </is>
-      </c>
-      <c r="B36" s="105" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="C36" s="106" t="inlineStr">
-        <is>
-          <t>• Deckblatt als erstes Blatt: Übersichtsdiagramm Eingaben → Verarbeitung → Ergebnisse (inkl. Vereinfachungen).</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="104" t="inlineStr">
         <is>
+          <t>0.14</t>
+        </is>
+      </c>
+      <c r="B37" s="105" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="C37" s="106" t="inlineStr">
+        <is>
+          <t>• Deckblatt als erstes Blatt: Übersichtsdiagramm Eingaben → Verarbeitung → Ergebnisse (inkl. Vereinfachungen).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="104" t="inlineStr">
+        <is>
           <t>0.13</t>
         </is>
       </c>
-      <c r="B37" s="105" t="inlineStr">
+      <c r="B38" s="105" t="inlineStr">
         <is>
           <t>2026-06-08</t>
         </is>
       </c>
-      <c r="C37" s="106" t="inlineStr">
+      <c r="C38" s="106" t="inlineStr">
         <is>
           <t>• Strömungsbereich dreistufig: laminar (Re &lt; 2300), Übergangsbereich (2300–4000), turbulent (Re &gt; 4000).</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="108" t="n"/>
-      <c r="B38" s="108" t="n"/>
-      <c r="C38" s="106" t="inlineStr">
-        <is>
-          <t>• Spalte 'Strömungsbereich' ausgeblendet (für die Auslegung nicht relevant) und ohne Färbung.</t>
         </is>
       </c>
     </row>
@@ -2334,7 +2342,7 @@
       <c r="B39" s="108" t="n"/>
       <c r="C39" s="106" t="inlineStr">
         <is>
-          <t>• Auslegung schlanker: weitere Zwischenspalten standardmäßig ausgeblendet (jederzeit einblendbar).</t>
+          <t>• Spalte 'Strömungsbereich' ausgeblendet (für die Auslegung nicht relevant) und ohne Färbung.</t>
         </is>
       </c>
     </row>
@@ -2343,42 +2351,42 @@
       <c r="B40" s="108" t="n"/>
       <c r="C40" s="106" t="inlineStr">
         <is>
+          <t>• Auslegung schlanker: weitere Zwischenspalten standardmäßig ausgeblendet (jederzeit einblendbar).</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="108" t="n"/>
+      <c r="B41" s="108" t="n"/>
+      <c r="C41" s="106" t="inlineStr">
+        <is>
           <t>• Verifikation: Korrekturfaktor kleiner dargestellt (passt nun vollständig in die Zelle).</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="107" t="n"/>
-      <c r="B41" s="107" t="n"/>
-      <c r="C41" s="106" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="107" t="n"/>
+      <c r="B42" s="107" t="n"/>
+      <c r="C42" s="106" t="inlineStr">
         <is>
           <t>• Changelog wieder ausführlich.</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="104" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="104" t="inlineStr">
         <is>
           <t>0.12</t>
         </is>
       </c>
-      <c r="B42" s="105" t="inlineStr">
+      <c r="B43" s="105" t="inlineStr">
         <is>
           <t>2026-06-08</t>
         </is>
       </c>
-      <c r="C42" s="106" t="inlineStr">
+      <c r="C43" s="106" t="inlineStr">
         <is>
           <t>• Grundeinstellungen: Bezeichnungen ausgeschrieben (keine Abkürzungen).</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="108" t="n"/>
-      <c r="B43" s="108" t="n"/>
-      <c r="C43" s="106" t="inlineStr">
-        <is>
-          <t>• Neue Spalte 'spez. Heizlast [W/m²]' (Heizlast bezogen auf die Raumfläche).</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2395,7 @@
       <c r="B44" s="108" t="n"/>
       <c r="C44" s="106" t="inlineStr">
         <is>
-          <t>• Massenstrom/Geschwindigkeit/Druckverlust auf Basis min(Leistung; Heizlast) + Verlust nach unten (realer Betriebspunkt).</t>
+          <t>• Neue Spalte 'spez. Heizlast [W/m²]' (Heizlast bezogen auf die Raumfläche).</t>
         </is>
       </c>
     </row>
@@ -2396,42 +2404,42 @@
       <c r="B45" s="108" t="n"/>
       <c r="C45" s="106" t="inlineStr">
         <is>
+          <t>• Massenstrom/Geschwindigkeit/Druckverlust auf Basis min(Leistung; Heizlast) + Verlust nach unten (realer Betriebspunkt).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="108" t="n"/>
+      <c r="B46" s="108" t="n"/>
+      <c r="C46" s="106" t="inlineStr">
+        <is>
           <t>• Heizkreisverteiler zusätzlich mit Massenstrom [kg/h]; Zonen-Kürzel (AZ/RZ/BAD).</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="107" t="n"/>
-      <c r="B46" s="107" t="n"/>
-      <c r="C46" s="106" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="107" t="n"/>
+      <c r="B47" s="107" t="n"/>
+      <c r="C47" s="106" t="inlineStr">
         <is>
           <t>• Kapazität 200 Räume / 50 Verteiler; Auslegung A3 quer, übrige Blätter A4 hoch.</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="104" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="104" t="inlineStr">
         <is>
           <t>0.11</t>
         </is>
       </c>
-      <c r="B47" s="105" t="inlineStr">
+      <c r="B48" s="105" t="inlineStr">
         <is>
           <t>2026-06-08</t>
         </is>
       </c>
-      <c r="C47" s="106" t="inlineStr">
+      <c r="C48" s="106" t="inlineStr">
         <is>
           <t>• Bugfixes: Hinweistext wurde als Formel interpretiert (Fehler 501); MAXIFS ersetzt (#NAME? in LibreOffice).</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="108" t="n"/>
-      <c r="B48" s="108" t="n"/>
-      <c r="C48" s="106" t="inlineStr">
-        <is>
-          <t>• Verifikation: Korrekturfaktor prominent oben; Hersteller-q direkt neben q berechnet.</t>
         </is>
       </c>
     </row>
@@ -2440,77 +2448,77 @@
       <c r="B49" s="108" t="n"/>
       <c r="C49" s="106" t="inlineStr">
         <is>
+          <t>• Verifikation: Korrekturfaktor prominent oben; Hersteller-q direkt neben q berechnet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="108" t="n"/>
+      <c r="B50" s="108" t="n"/>
+      <c r="C50" s="106" t="inlineStr">
+        <is>
           <t>• Konstanten: alle Tabellen untereinander, mit Leerzeilen für weitere Einträge.</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="107" t="n"/>
-      <c r="B50" s="107" t="n"/>
-      <c r="C50" s="106" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="107" t="n"/>
+      <c r="B51" s="107" t="n"/>
+      <c r="C51" s="106" t="inlineStr">
         <is>
           <t>• Methodik: Variablen zuerst, dann Formeln mit Erklärung je Schritt; weitere Musterräume (Verwaltungsbau).</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="104" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="104" t="inlineStr">
         <is>
           <t>0.10</t>
         </is>
       </c>
-      <c r="B51" s="105" t="inlineStr">
+      <c r="B52" s="105" t="inlineStr">
         <is>
           <t>2026-06-08</t>
         </is>
       </c>
-      <c r="C51" s="106" t="inlineStr">
+      <c r="C52" s="106" t="inlineStr">
         <is>
           <t>• Heizkreisverteiler-Liste und Verifikation ohne dynamische Array-Funktionen → läuft in Excel UND LibreOffice.</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="108" t="n"/>
-      <c r="B52" s="108" t="n"/>
-      <c r="C52" s="106" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="108" t="n"/>
+      <c r="B53" s="108" t="n"/>
+      <c r="C53" s="106" t="inlineStr">
         <is>
           <t>• Verifikation mit Liniendiagramm; Konstanten/Bibliotheken in eigenes Blatt ausgelagert.</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="107" t="n"/>
-      <c r="B53" s="107" t="n"/>
-      <c r="C53" s="106" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="107" t="n"/>
+      <c r="B54" s="107" t="n"/>
+      <c r="C54" s="106" t="inlineStr">
         <is>
           <t>• Gewähltes Rohrsystem mit Außen-/Innendurchmesser, Wandstärke und Rauheit im Druckbereich.</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="104" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="104" t="inlineStr">
         <is>
           <t>0.9</t>
         </is>
       </c>
-      <c r="B54" s="105" t="inlineStr">
+      <c r="B55" s="105" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="C54" s="106" t="inlineStr">
+      <c r="C55" s="106" t="inlineStr">
         <is>
           <t>• Neues Blatt 'Heizkreisverteiler' (Leistung, max. Druckverlust, Volumenstrom je HKV).</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="108" t="n"/>
-      <c r="B55" s="108" t="n"/>
-      <c r="C55" s="106" t="inlineStr">
-        <is>
-          <t>• Spaltenüberschriften der Auslegung dreizeilig (Name / Formelzeichen / Einheit).</t>
         </is>
       </c>
     </row>
@@ -2519,42 +2527,42 @@
       <c r="B56" s="108" t="n"/>
       <c r="C56" s="106" t="inlineStr">
         <is>
+          <t>• Spaltenüberschriften der Auslegung dreizeilig (Name / Formelzeichen / Einheit).</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="108" t="n"/>
+      <c r="B57" s="108" t="n"/>
+      <c r="C57" s="106" t="inlineStr">
+        <is>
           <t>• Korrekturfaktor f wird auf 'Verifikation' eingegeben (mit Vergleichsdiagramm).</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="107" t="n"/>
-      <c r="B57" s="107" t="n"/>
-      <c r="C57" s="106" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="107" t="n"/>
+      <c r="B58" s="107" t="n"/>
+      <c r="C58" s="106" t="inlineStr">
         <is>
           <t>• Geschwindigkeits-Grenzwerte v_min/v_max als Grundeinstellung.</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="104" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="104" t="inlineStr">
         <is>
           <t>0.8</t>
         </is>
       </c>
-      <c r="B58" s="105" t="inlineStr">
+      <c r="B59" s="105" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="C58" s="106" t="inlineStr">
+      <c r="C59" s="106" t="inlineStr">
         <is>
           <t>• Grundeinstellungen für A3 quer optimiert (Einstellungen links, Tabellen rechts).</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="108" t="n"/>
-      <c r="B59" s="108" t="n"/>
-      <c r="C59" s="106" t="inlineStr">
-        <is>
-          <t>• Auslegung passt auf eine Seite breit; Korrekturfaktor Heizleistung zur Kalibrierung ergänzt.</t>
         </is>
       </c>
     </row>
@@ -2563,120 +2571,120 @@
       <c r="B60" s="108" t="n"/>
       <c r="C60" s="106" t="inlineStr">
         <is>
+          <t>• Auslegung passt auf eine Seite breit; Korrekturfaktor Heizleistung zur Kalibrierung ergänzt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="108" t="n"/>
+      <c r="B61" s="108" t="n"/>
+      <c r="C61" s="106" t="inlineStr">
+        <is>
           <t>• Wärmeabgabe nach unten berücksichtigt (Verlust + Gesamtleistung).</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="107" t="n"/>
-      <c r="B61" s="107" t="n"/>
-      <c r="C61" s="106" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="107" t="n"/>
+      <c r="B62" s="107" t="n"/>
+      <c r="C62" s="106" t="inlineStr">
         <is>
           <t>• Blätter umbenannt: Raumliste → Auslegung, Übersicht → Kontrolle; zusätzliche Kontrollen.</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="104" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="104" t="inlineStr">
         <is>
           <t>0.7</t>
         </is>
       </c>
-      <c r="B62" s="105" t="inlineStr">
+      <c r="B63" s="105" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="C62" s="106" t="inlineStr">
+      <c r="C63" s="106" t="inlineStr">
         <is>
           <t>• Deckung-%-Spalte färbt nur noch gefüllte Zellen (leere bleiben farblos).</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="108" t="n"/>
-      <c r="B63" s="108" t="n"/>
-      <c r="C63" s="106" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="108" t="n"/>
+      <c r="B64" s="108" t="n"/>
+      <c r="C64" s="106" t="inlineStr">
         <is>
           <t>• Neues Blatt 'Verifikation'; neue Spalte 'Strömungsbereich' (laminar/turbulent).</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="107" t="n"/>
-      <c r="B64" s="107" t="n"/>
-      <c r="C64" s="106" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="107" t="n"/>
+      <c r="B65" s="107" t="n"/>
+      <c r="C65" s="106" t="inlineStr">
         <is>
           <t>• Alle Blätter im A3-Querformat; einheitlicher Kopf je Blatt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="104" t="inlineStr">
-        <is>
-          <t>0.6</t>
-        </is>
-      </c>
-      <c r="B65" s="105" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C65" s="106" t="inlineStr">
-        <is>
-          <t>• Bugfix: Zellfärbung (bedingte Formatierung) wird jetzt auch in Excel angezeigt – dxf-Füllfarbe mit voller Deckkraft.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="104" t="inlineStr">
         <is>
+          <t>0.6</t>
+        </is>
+      </c>
+      <c r="B66" s="105" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="C66" s="106" t="inlineStr">
+        <is>
+          <t>• Bugfix: Zellfärbung (bedingte Formatierung) wird jetzt auch in Excel angezeigt – dxf-Füllfarbe mit voller Deckkraft.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="104" t="inlineStr">
+        <is>
           <t>0.5</t>
         </is>
       </c>
-      <c r="B66" s="105" t="inlineStr">
+      <c r="B67" s="105" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="C66" s="106" t="inlineStr">
+      <c r="C67" s="106" t="inlineStr">
         <is>
           <t>• Versionsnummer und Autor werden nur noch im Changelog angezeigt.</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="107" t="n"/>
-      <c r="B67" s="107" t="n"/>
-      <c r="C67" s="106" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="107" t="n"/>
+      <c r="B68" s="107" t="n"/>
+      <c r="C68" s="106" t="inlineStr">
         <is>
           <t>• Editierbares Bearbeiter-Kürzel rechts oben unter dem Logo (Grundeinstellungen, Auslegung, Kontrolle, HKV).</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="104" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="104" t="inlineStr">
         <is>
           <t>0.4</t>
         </is>
       </c>
-      <c r="B68" s="105" t="inlineStr">
+      <c r="B69" s="105" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="C68" s="106" t="inlineStr">
+      <c r="C69" s="106" t="inlineStr">
         <is>
           <t>• Status-Spalten entfernt – Bewertung erfolgt jetzt direkt als Zellfärbung (grün/rot).</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="108" t="n"/>
-      <c r="B69" s="108" t="n"/>
-      <c r="C69" s="106" t="inlineStr">
-        <is>
-          <t>• Methodik um die Formelzeichen-Legende erweitert.</t>
         </is>
       </c>
     </row>
@@ -2685,42 +2693,42 @@
       <c r="B70" s="108" t="n"/>
       <c r="C70" s="106" t="inlineStr">
         <is>
+          <t>• Methodik um die Formelzeichen-Legende erweitert.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="108" t="n"/>
+      <c r="B71" s="108" t="n"/>
+      <c r="C71" s="106" t="inlineStr">
+        <is>
           <t>• Heizkreisverteiler (HKV) als erste Spalte der Auslegung; Standardwert max. Druckverlust 15.000 Pa.</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="107" t="n"/>
-      <c r="B71" s="107" t="n"/>
-      <c r="C71" s="106" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="107" t="n"/>
+      <c r="B72" s="107" t="n"/>
+      <c r="C72" s="106" t="inlineStr">
         <is>
           <t>• Versionsschema 0.x eingeführt (1.0 erst nach Test); interner Autor (dh).</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="104" t="inlineStr">
+    <row r="73">
+      <c r="A73" s="104" t="inlineStr">
         <is>
           <t>0.3</t>
         </is>
       </c>
-      <c r="B72" s="105" t="inlineStr">
+      <c r="B73" s="105" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="C72" s="106" t="inlineStr">
+      <c r="C73" s="106" t="inlineStr">
         <is>
           <t>• Zonentypen (Aufenthalt/Rand/Bad) mit eigener zulässiger Oberflächentemperatur.</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="108" t="n"/>
-      <c r="B73" s="108" t="n"/>
-      <c r="C73" s="106" t="inlineStr">
-        <is>
-          <t>• Einheitlicher Kopf: Titel oben links, agn-Logo oben rechts, Projektkopf darunter.</t>
         </is>
       </c>
     </row>
@@ -2729,7 +2737,7 @@
       <c r="B74" s="108" t="n"/>
       <c r="C74" s="106" t="inlineStr">
         <is>
-          <t>• Oberflächentemperatur θF und Volumenstrom eingeblendet.</t>
+          <t>• Einheitlicher Kopf: Titel oben links, agn-Logo oben rechts, Projektkopf darunter.</t>
         </is>
       </c>
     </row>
@@ -2738,42 +2746,42 @@
       <c r="B75" s="108" t="n"/>
       <c r="C75" s="106" t="inlineStr">
         <is>
+          <t>• Oberflächentemperatur θF und Volumenstrom eingeblendet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="108" t="n"/>
+      <c r="B76" s="108" t="n"/>
+      <c r="C76" s="106" t="inlineStr">
+        <is>
           <t>• Neue Spalten 'spez. Druckverlust [Pa/m]' und Eingabespalte 'Verteiler (Anbindung)'.</t>
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="107" t="n"/>
-      <c r="B76" s="107" t="n"/>
-      <c r="C76" s="106" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="107" t="n"/>
+      <c r="B77" s="107" t="n"/>
+      <c r="C77" s="106" t="inlineStr">
         <is>
           <t>• Warnung (rot), wenn die aktivierbare Fläche größer als die Raumfläche ist.</t>
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="104" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="104" t="inlineStr">
         <is>
           <t>0.2</t>
         </is>
       </c>
-      <c r="B77" s="105" t="inlineStr">
+      <c r="B78" s="105" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="C77" s="106" t="inlineStr">
+      <c r="C78" s="106" t="inlineStr">
         <is>
           <t>• agn-Logo eingebunden und eigenes Changelog-Blatt ergänzt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="108" t="n"/>
-      <c r="B78" s="108" t="n"/>
-      <c r="C78" s="106" t="inlineStr">
-        <is>
-          <t>• Zuschlag Einzelwiderstände (5 %) und fester Verteiler-Aufschlag (500 Pa je Kreis).</t>
         </is>
       </c>
     </row>
@@ -2782,7 +2790,7 @@
       <c r="B79" s="108" t="n"/>
       <c r="C79" s="106" t="inlineStr">
         <is>
-          <t>• Einheiten als Zellformat; Projektnummer/Projektname erscheinen im Ausdruck.</t>
+          <t>• Zuschlag Einzelwiderstände (5 %) und fester Verteiler-Aufschlag (500 Pa je Kreis).</t>
         </is>
       </c>
     </row>
@@ -2791,42 +2799,42 @@
       <c r="B80" s="108" t="n"/>
       <c r="C80" s="106" t="inlineStr">
         <is>
+          <t>• Einheiten als Zellformat; Projektnummer/Projektname erscheinen im Ausdruck.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="108" t="n"/>
+      <c r="B81" s="108" t="n"/>
+      <c r="C81" s="106" t="inlineStr">
+        <is>
           <t>• Richtwert-Tabellen für R-Werte und Verlegeabstand-Faktoren; weitere Musterräume.</t>
         </is>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" s="107" t="n"/>
-      <c r="B81" s="107" t="n"/>
-      <c r="C81" s="106" t="inlineStr">
+    <row r="82">
+      <c r="A82" s="107" t="n"/>
+      <c r="B82" s="107" t="n"/>
+      <c r="C82" s="106" t="inlineStr">
         <is>
           <t>• Druckaufbereitung für DIN A4.</t>
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" s="104" t="inlineStr">
+    <row r="83">
+      <c r="A83" s="104" t="inlineStr">
         <is>
           <t>0.1</t>
         </is>
       </c>
-      <c r="B82" s="105" t="inlineStr">
+      <c r="B83" s="105" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="C82" s="106" t="inlineStr">
+      <c r="C83" s="106" t="inlineStr">
         <is>
           <t>• Ersterstellung mit den Blättern Grundeinstellungen, Raumliste, Übersicht und Methodik.</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="108" t="n"/>
-      <c r="B83" s="108" t="n"/>
-      <c r="C83" s="106" t="inlineStr">
-        <is>
-          <t>• Heizleistung über die logarithmische Übertemperatur (q = η · K_H · ΔθH).</t>
         </is>
       </c>
     </row>
@@ -2835,7 +2843,7 @@
       <c r="B84" s="108" t="n"/>
       <c r="C84" s="106" t="inlineStr">
         <is>
-          <t>• Druckverlustberechnung nach Darcy-Weisbach.</t>
+          <t>• Heizleistung über die logarithmische Übertemperatur (q = η · K_H · ΔθH).</t>
         </is>
       </c>
     </row>
@@ -2844,14 +2852,23 @@
       <c r="B85" s="108" t="n"/>
       <c r="C85" s="106" t="inlineStr">
         <is>
+          <t>• Druckverlustberechnung nach Darcy-Weisbach.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="108" t="n"/>
+      <c r="B86" s="108" t="n"/>
+      <c r="C86" s="106" t="inlineStr">
+        <is>
           <t>• Editierbare Rohrbibliothek und Verlegeabstand-Faktoren.</t>
         </is>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" s="107" t="n"/>
-      <c r="B86" s="107" t="n"/>
-      <c r="C86" s="106" t="inlineStr">
+    <row r="87">
+      <c r="A87" s="107" t="n"/>
+      <c r="B87" s="107" t="n"/>
+      <c r="C87" s="106" t="inlineStr">
         <is>
           <t>• Prüfungen: Oberflächentemperatur, Heizlastdeckung, Kreislänge, Druckverlust.</t>
         </is>
@@ -2859,50 +2876,50 @@
     </row>
   </sheetData>
   <mergeCells count="44">
-    <mergeCell ref="B82:B86"/>
-    <mergeCell ref="B47:B50"/>
-    <mergeCell ref="A33:A35"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="B33:B35"/>
-    <mergeCell ref="A42:A46"/>
-    <mergeCell ref="B37:B41"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="A72:A76"/>
-    <mergeCell ref="A54:A57"/>
-    <mergeCell ref="A66:A67"/>
-    <mergeCell ref="B27:B32"/>
-    <mergeCell ref="A13:A15"/>
-    <mergeCell ref="A62:A64"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="B51:B53"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="A10:A12"/>
-    <mergeCell ref="B58:B61"/>
-    <mergeCell ref="A77:A81"/>
-    <mergeCell ref="B16:B18"/>
-    <mergeCell ref="B19:B22"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="B54:B57"/>
-    <mergeCell ref="B72:B76"/>
-    <mergeCell ref="A27:A32"/>
-    <mergeCell ref="B62:B64"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="A51:A53"/>
-    <mergeCell ref="A82:A86"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="B68:B71"/>
-    <mergeCell ref="A19:A22"/>
-    <mergeCell ref="A47:A50"/>
-    <mergeCell ref="B10:B12"/>
-    <mergeCell ref="A16:A18"/>
-    <mergeCell ref="B66:B67"/>
-    <mergeCell ref="B77:B81"/>
-    <mergeCell ref="B13:B15"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="B42:B46"/>
-    <mergeCell ref="A68:A71"/>
-    <mergeCell ref="A37:A41"/>
-    <mergeCell ref="A58:A61"/>
+    <mergeCell ref="A48:A51"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="B78:B82"/>
+    <mergeCell ref="A17:A19"/>
+    <mergeCell ref="B34:B36"/>
+    <mergeCell ref="B38:B42"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="B59:B62"/>
+    <mergeCell ref="A69:A72"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="A63:A65"/>
+    <mergeCell ref="B67:B68"/>
+    <mergeCell ref="B83:B87"/>
+    <mergeCell ref="A34:A36"/>
+    <mergeCell ref="A52:A54"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="A38:A42"/>
+    <mergeCell ref="A43:A47"/>
+    <mergeCell ref="A83:A87"/>
+    <mergeCell ref="A55:A58"/>
+    <mergeCell ref="B63:B65"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="A73:A77"/>
+    <mergeCell ref="B48:B51"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="B69:B72"/>
+    <mergeCell ref="B52:B54"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="A20:A23"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="B28:B33"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="A78:A82"/>
+    <mergeCell ref="B43:B47"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B55:B58"/>
+    <mergeCell ref="B20:B23"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="B73:B77"/>
+    <mergeCell ref="A28:A33"/>
+    <mergeCell ref="A59:A62"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="A67:A68"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -29736,7 +29753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -29779,7 +29796,7 @@
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="87" t="inlineStr">
         <is>
-          <t>Korrekturfaktor Heizleistung  f =</t>
+          <t>Systemfaktor (EN 1264)  f =</t>
         </is>
       </c>
       <c r="B5" s="88" t="n"/>
@@ -30205,7 +30222,7 @@
     <row r="29">
       <c r="A29" s="25" t="inlineStr">
         <is>
-          <t>• Korrekturfaktor f oben so einstellen, dass berechnetes q und Referenz-q übereinstimmen</t>
+          <t>• Systemfaktor f oben so einstellen, dass berechnetes q und Referenz-q übereinstimmen</t>
         </is>
       </c>
     </row>
@@ -30219,12 +30236,19 @@
     <row r="31">
       <c r="A31" s="28" t="inlineStr">
         <is>
-          <t>• Der kalibrierte Faktor f gilt für die gesamte Auslegung – daher VOR der Raumauslegung</t>
+          <t>• f bündelt die im überschlägigen Modell vereinfachten Effekte (Rohrwand-, Estrich-</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   spreizungs-Widerstand). Gilt für die gesamte Auslegung – daher VOR der Raumauslegung</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="28" t="inlineStr">
         <is>
           <t xml:space="preserve">   kalibrieren.</t>
         </is>
@@ -30335,7 +30359,7 @@
       </c>
       <c r="D7" s="92" t="inlineStr">
         <is>
-          <t>3. Verifikation: Korrekturfaktor f kalibrieren – VOR der</t>
+          <t>3. Verifikation: Systemfaktor f kalibrieren – VOR der</t>
         </is>
       </c>
     </row>
@@ -30897,7 +30921,7 @@
     <row r="16">
       <c r="B16" s="94" t="inlineStr">
         <is>
-          <t>f — Korrekturfaktor Heizleistung [-]</t>
+          <t>f — Systemfaktor (EN-1264-Kalibrierung) [-]</t>
         </is>
       </c>
       <c r="D16" s="96" t="inlineStr">

</xml_diff>

<commit_message>
FBH-Auslegung v0.27 - Leistung-FBH-Ampel, R-Werte erweitert, HKV-Raumspalte breiter, A4-Feinschliff
Auslegung: 'Ueber-/Unterdeckung' (U) wieder ausgeblendet; 'Leistung FBH' (T) gruen/rot je nach Heizlastdeckung (T>=Heizlast gruen, sonst rot). Raum-Nr. breiter (8->11). Anzahl HK mit Einheit 'HK' je Zelle (Format '0" HK"'). Auslegung-Seitenraender schmaler (L/R 0.2, O/U 0.3) fuer besseren A4-Sitz.

HKV-Liste: Spalte 'angebundene Raeume' auf Breite 50 (Rebalance der uebrigen Spalten); lange/viele Raumnummern werden vollstaendig dargestellt (wrap + Auto-Zeilenhoehe).

Konstanten: R-Werte Bodenbelaege von 5 auf 11 Eintraege erweitert (Keramik/Naturstein/PVC/Designboden/Linoleum/Laminat/Parkett/Kork/Holzdielen/Teppich duenn+dick) und nach rechts (G/H) gestellt; Zonen-Tabelle nach links (D/E/F). Referenzen RW_RANGE=H6:H19, ZONE_RANGE=E6:F10 angepasst.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FBH_Auslegung.xlsx
+++ b/FBH_Auslegung.xlsx
@@ -28,8 +28,8 @@
     <definedName name="_xlnm.Print_Area" localSheetId="5">'Verifikation'!$A$1:$L$26</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="6">'Anleitung'!$A$1:$D$32</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">'Methodik'!$A$1:$F$26</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="8">'Konstanten'!$A$1:$I$26</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="9">'Changelog'!$A$1:$C$92</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="8">'Konstanten'!$A$1:$H$26</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="9">'Changelog'!$A$1:$C$95</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -37,7 +37,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="28">
+  <numFmts count="29">
     <numFmt numFmtId="164" formatCode="0.0&quot; °C&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0&quot; K&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; m&quot;"/>
@@ -54,18 +54,19 @@
     <numFmt numFmtId="177" formatCode="0.0&quot; m²&quot;"/>
     <numFmt numFmtId="178" formatCode="#,##0&quot; W&quot;"/>
     <numFmt numFmtId="179" formatCode="0&quot; mm&quot;"/>
-    <numFmt numFmtId="180" formatCode="0.0&quot; m&quot;"/>
-    <numFmt numFmtId="181" formatCode="0.00&quot; K&quot;"/>
-    <numFmt numFmtId="182" formatCode="&quot;+&quot;#,##0&quot; W&quot;;&quot;-&quot;#,##0&quot; W&quot;;0&quot; W&quot;"/>
-    <numFmt numFmtId="183" formatCode="0.0%"/>
-    <numFmt numFmtId="184" formatCode="0.0&quot; kg/h&quot;"/>
-    <numFmt numFmtId="185" formatCode="0.0&quot; l/h&quot;"/>
-    <numFmt numFmtId="186" formatCode="0.000&quot; m/s&quot;"/>
-    <numFmt numFmtId="187" formatCode="0.0000"/>
-    <numFmt numFmtId="188" formatCode="#,##0&quot; Pa/m&quot;"/>
-    <numFmt numFmtId="189" formatCode="#,##0&quot; kg/h&quot;"/>
-    <numFmt numFmtId="190" formatCode="#,##0&quot; l/h&quot;"/>
-    <numFmt numFmtId="191" formatCode="0&quot; °C&quot;"/>
+    <numFmt numFmtId="180" formatCode="0&quot; HK&quot;"/>
+    <numFmt numFmtId="181" formatCode="0.0&quot; m&quot;"/>
+    <numFmt numFmtId="182" formatCode="0.00&quot; K&quot;"/>
+    <numFmt numFmtId="183" formatCode="&quot;+&quot;#,##0&quot; W&quot;;&quot;-&quot;#,##0&quot; W&quot;;0&quot; W&quot;"/>
+    <numFmt numFmtId="184" formatCode="0.0%"/>
+    <numFmt numFmtId="185" formatCode="0.0&quot; kg/h&quot;"/>
+    <numFmt numFmtId="186" formatCode="0.0&quot; l/h&quot;"/>
+    <numFmt numFmtId="187" formatCode="0.000&quot; m/s&quot;"/>
+    <numFmt numFmtId="188" formatCode="0.0000"/>
+    <numFmt numFmtId="189" formatCode="#,##0&quot; Pa/m&quot;"/>
+    <numFmt numFmtId="190" formatCode="#,##0&quot; kg/h&quot;"/>
+    <numFmt numFmtId="191" formatCode="#,##0&quot; l/h&quot;"/>
+    <numFmt numFmtId="192" formatCode="0&quot; °C&quot;"/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -560,11 +561,11 @@
       <alignment horizontal="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="1" fontId="13" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="180" fontId="13" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="180" fontId="13" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="181" fontId="13" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -572,7 +573,7 @@
       <alignment horizontal="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="181" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="182" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="171" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -587,16 +588,13 @@
     <xf numFmtId="178" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="182" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="183" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="180" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="184" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="184" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="181" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="185" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -605,19 +603,22 @@
     <xf numFmtId="186" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="187" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="187" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="188" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="167" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="188" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="189" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -626,7 +627,7 @@
     <xf numFmtId="3" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="183" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="184" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="171" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -641,10 +642,10 @@
     <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="189" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="190" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="190" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="191" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -701,7 +702,7 @@
       <alignment horizontal="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="191" fontId="13" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="192" fontId="13" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -979,7 +980,7 @@
   <oneCellAnchor>
     <from>
       <col>7</col>
-      <colOff>1200150</colOff>
+      <colOff>2266950</colOff>
       <row>0</row>
       <rowOff>9525</rowOff>
     </from>
@@ -1098,8 +1099,8 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>7</col>
-      <colOff>247650</colOff>
+      <col>6</col>
+      <colOff>1447800</colOff>
       <row>0</row>
       <rowOff>9525</rowOff>
     </from>
@@ -1855,7 +1856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C92"/>
+  <dimension ref="A1:C95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1882,7 +1883,7 @@
       <c r="B3" s="2" t="n"/>
       <c r="C3" s="23" t="inlineStr">
         <is>
-          <t>Version 0.26 · dh</t>
+          <t>Version 0.27 · dh</t>
         </is>
       </c>
     </row>
@@ -1911,7 +1912,7 @@
     <row r="6">
       <c r="A6" s="109" t="inlineStr">
         <is>
-          <t>0.26</t>
+          <t>0.27</t>
         </is>
       </c>
       <c r="B6" s="110" t="inlineStr">
@@ -1921,7 +1922,7 @@
       </c>
       <c r="C6" s="111" t="inlineStr">
         <is>
-          <t>• HKV-Liste: neue Spalte 'angebundene Räume (Raum-Nr.)' – listet je Verteiler automatisch die zugehörigen Raumnummern (TEXTJOIN-Array, Excel &amp; LibreOffice).</t>
+          <t>• Auslegung: 'Über-/Unterdeckung' wieder ausgeblendet; stattdessen wird die 'Leistung FBH' eingefärbt (grün = Heizlast gedeckt, rot = nicht gedeckt). Raum-Nr. breiter; Anzahl Heizkreise mit Einheit 'HK' je Zelle; schmalere Seitenränder für besseren A4-Sitz.</t>
         </is>
       </c>
     </row>
@@ -1930,68 +1931,60 @@
       <c r="B7" s="112" t="n"/>
       <c r="C7" s="111" t="inlineStr">
         <is>
+          <t>• HKV-Liste: Spalte 'angebundene Räume' deutlich breiter (lange/viele Raumnummern werden vollständig dargestellt).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="113" t="n"/>
+      <c r="B8" s="113" t="n"/>
+      <c r="C8" s="111" t="inlineStr">
+        <is>
+          <t>• Konstanten: R-Werte-Tabelle der Bodenbeläge erweitert (11 Beläge statt 5) und nach rechts gestellt; Zonen-Tabelle nach links – so kann die R-Werte-Tabelle höher werden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="109" t="inlineStr">
+        <is>
+          <t>0.26</t>
+        </is>
+      </c>
+      <c r="B9" s="110" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="C9" s="111" t="inlineStr">
+        <is>
+          <t>• HKV-Liste: neue Spalte 'angebundene Räume (Raum-Nr.)' – listet je Verteiler automatisch die zugehörigen Raumnummern (TEXTJOIN-Array, Excel &amp; LibreOffice).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="112" t="n"/>
+      <c r="B10" s="112" t="n"/>
+      <c r="C10" s="111" t="inlineStr">
+        <is>
           <t>• Auslegung: Spalten 'Leistung FBH' und 'Über-/Unterdeckung' eingeblendet; Über-/Unterdeckung mit Vorzeichen (+/–) und Ampel (grün = Überdeckung, rot = Unterdeckung).</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="112" t="n"/>
-      <c r="B8" s="112" t="n"/>
-      <c r="C8" s="111" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="112" t="n"/>
+      <c r="B11" s="112" t="n"/>
+      <c r="C11" s="111" t="inlineStr">
         <is>
           <t>• Grundeinstellungen: Eingabefelder Projekt-Nr./Projektname breiter; Spalte J (Rohrsystem-Werte) breiter.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="112" t="n"/>
-      <c r="B9" s="112" t="n"/>
-      <c r="C9" s="111" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="112" t="n"/>
+      <c r="B12" s="112" t="n"/>
+      <c r="C12" s="111" t="inlineStr">
         <is>
           <t>• Verifikation: kein fixer Vergleichspunkt mehr – jede Zeile ist ein eigener Auslegungspunkt (VL/RL, θi, R, Verlegeabstand) mit eigener Abweichung; Diagramm entfernt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="113" t="n"/>
-      <c r="B10" s="113" t="n"/>
-      <c r="C10" s="111" t="inlineStr">
-        <is>
-          <t>• Blattschutz: Zellen mit Formeln sind gesperrt (vor versehentlichem Überschreiben geschützt), Eingabezellen bleiben editierbar; Schutz ohne Passwort.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="109" t="inlineStr">
-        <is>
-          <t>0.25</t>
-        </is>
-      </c>
-      <c r="B11" s="110" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="C11" s="111" t="inlineStr">
-        <is>
-          <t>• Begriff 'Korrekturfaktor' in 'Systemfaktor (EN-1264-Kalibrierung)' umbenannt (Verifikation, Methodik, Deckblatt, Anleitung) – f ist die bewusste Kalibrierung des überschlägigen Modells an EN 1264, kein Fehlerfaktor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="109" t="inlineStr">
-        <is>
-          <t>0.24</t>
-        </is>
-      </c>
-      <c r="B12" s="110" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="C12" s="111" t="inlineStr">
-        <is>
-          <t>• Verifikation: Referenzspalte mit echten Werten nach DIN EN 1264 vorbelegt (Nasssystem/Tacker, VL 40 / RL 30 °C, θi 20 °C, R = 0,10 m²K/W); Vergleichsbedingungen entsprechend auf 40/30 °C gesetzt.</t>
         </is>
       </c>
     </row>
@@ -2000,59 +1993,67 @@
       <c r="B13" s="113" t="n"/>
       <c r="C13" s="111" t="inlineStr">
         <is>
-          <t>• Verifikation: Korrekturfaktor f auf 0,85 vorkalibriert (Best-Fit zu den EN-1264-Werten); Spalte C bleibt editierbar für herstellereigene Datenblattwerte (Rehau, Uponor, Buderus, Kermi …).</t>
+          <t>• Blattschutz: Zellen mit Formeln sind gesperrt (vor versehentlichem Überschreiben geschützt), Eingabezellen bleiben editierbar; Schutz ohne Passwort.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="109" t="inlineStr">
         <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="B14" s="110" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="C14" s="111" t="inlineStr">
+        <is>
+          <t>• Begriff 'Korrekturfaktor' in 'Systemfaktor (EN-1264-Kalibrierung)' umbenannt (Verifikation, Methodik, Deckblatt, Anleitung) – f ist die bewusste Kalibrierung des überschlägigen Modells an EN 1264, kein Fehlerfaktor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="109" t="inlineStr">
+        <is>
+          <t>0.24</t>
+        </is>
+      </c>
+      <c r="B15" s="110" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="C15" s="111" t="inlineStr">
+        <is>
+          <t>• Verifikation: Referenzspalte mit echten Werten nach DIN EN 1264 vorbelegt (Nasssystem/Tacker, VL 40 / RL 30 °C, θi 20 °C, R = 0,10 m²K/W); Vergleichsbedingungen entsprechend auf 40/30 °C gesetzt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="113" t="n"/>
+      <c r="B16" s="113" t="n"/>
+      <c r="C16" s="111" t="inlineStr">
+        <is>
+          <t>• Verifikation: Korrekturfaktor f auf 0,85 vorkalibriert (Best-Fit zu den EN-1264-Werten); Spalte C bleibt editierbar für herstellereigene Datenblattwerte (Rehau, Uponor, Buderus, Kermi …).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="109" t="inlineStr">
+        <is>
           <t>0.23</t>
         </is>
       </c>
-      <c r="B14" s="110" t="inlineStr">
+      <c r="B17" s="110" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="C14" s="111" t="inlineStr">
+      <c r="C17" s="111" t="inlineStr">
         <is>
           <t>• Auslegung: Formelzeichen größer (besser lesbare Tiefstellungen); Kopfzeilen-Umbrüche optimiert – keine Trennung mehr mitten im Wort.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="113" t="n"/>
-      <c r="B15" s="113" t="n"/>
-      <c r="C15" s="111" t="inlineStr">
-        <is>
-          <t>• Deckblatt: Druck-Hinweis wieder entfernt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="109" t="inlineStr">
-        <is>
-          <t>0.22</t>
-        </is>
-      </c>
-      <c r="B16" s="110" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="C16" s="111" t="inlineStr">
-        <is>
-          <t>• Anleitung: neue Ampel-Legende (warum ist eine Zelle rot?) und Hinweis zur Auslegung mehrerer Verteiler/Geschosse; Blatt nach hinten verschoben (jetzt vor der Methodik).</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="112" t="n"/>
-      <c r="B17" s="112" t="n"/>
-      <c r="C17" s="111" t="inlineStr">
-        <is>
-          <t>• Deckblatt: Druck-Hinweis ergänzt – nur die relevanten Blätter (Deckblatt, Grundeinstellungen, Auslegung, Kontrolle, HKV, Anleitung) gemeinsam als 'Aktive Blätter' drucken.</t>
         </is>
       </c>
     </row>
@@ -2061,14 +2062,14 @@
       <c r="B18" s="113" t="n"/>
       <c r="C18" s="111" t="inlineStr">
         <is>
-          <t>• Formelzeichen mit echten Tiefstellungen dargestellt (z. B. q_HL, R_λ,B, V̇_max) – kein Unterstrich mehr in den Kopfzeilen, Grundeinstellungen und der Methodik-Variablenliste.</t>
+          <t>• Deckblatt: Druck-Hinweis wieder entfernt.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="109" t="inlineStr">
         <is>
-          <t>0.21</t>
+          <t>0.22</t>
         </is>
       </c>
       <c r="B19" s="110" t="inlineStr">
@@ -2078,7 +2079,7 @@
       </c>
       <c r="C19" s="111" t="inlineStr">
         <is>
-          <t>• Auslegung jetzt auf A4-Querformat (vorher A3); sichtbare Spalten schmaler, damit das Blatt auf A4 passt.</t>
+          <t>• Anleitung: neue Ampel-Legende (warum ist eine Zelle rot?) und Hinweis zur Auslegung mehrerer Verteiler/Geschosse; Blatt nach hinten verschoben (jetzt vor der Methodik).</t>
         </is>
       </c>
     </row>
@@ -2087,7 +2088,7 @@
       <c r="B20" s="112" t="n"/>
       <c r="C20" s="111" t="inlineStr">
         <is>
-          <t>• Deckblatt: Titel 'Fußbodenheizung – Auslegung' (Wort 'überschlägige' entfernt); Vereinfachungen bleiben dokumentiert.</t>
+          <t>• Deckblatt: Druck-Hinweis ergänzt – nur die relevanten Blätter (Deckblatt, Grundeinstellungen, Auslegung, Kontrolle, HKV, Anleitung) gemeinsam als 'Aktive Blätter' drucken.</t>
         </is>
       </c>
     </row>
@@ -2096,14 +2097,14 @@
       <c r="B21" s="113" t="n"/>
       <c r="C21" s="111" t="inlineStr">
         <is>
-          <t>• Anleitung: Abschnitt 'Planungstechnische Grundlagen' wieder entfernt.</t>
+          <t>• Formelzeichen mit echten Tiefstellungen dargestellt (z. B. q_HL, R_λ,B, V̇_max) – kein Unterstrich mehr in den Kopfzeilen, Grundeinstellungen und der Methodik-Variablenliste.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="109" t="inlineStr">
         <is>
-          <t>0.20</t>
+          <t>0.21</t>
         </is>
       </c>
       <c r="B22" s="110" t="inlineStr">
@@ -2113,7 +2114,7 @@
       </c>
       <c r="C22" s="111" t="inlineStr">
         <is>
-          <t>• Grundeinstellungen: Spaltenbreiten optimiert und lange Beschriftungen/Hinweise gekürzt – Texte werden in LibreOffice nicht mehr abgeschnitten.</t>
+          <t>• Auslegung jetzt auf A4-Querformat (vorher A3); sichtbare Spalten schmaler, damit das Blatt auf A4 passt.</t>
         </is>
       </c>
     </row>
@@ -2122,7 +2123,7 @@
       <c r="B23" s="112" t="n"/>
       <c r="C23" s="111" t="inlineStr">
         <is>
-          <t>• Verifikation: Untertitel und Hinweise vereinfacht (Modellvergleich-Erläuterung entfernt); klarer Hinweis, dass der Korrekturfaktor f VOR der Raumauslegung kalibriert wird; Diagramm etwas größer.</t>
+          <t>• Deckblatt: Titel 'Fußbodenheizung – Auslegung' (Wort 'überschlägige' entfernt); Vereinfachungen bleiben dokumentiert.</t>
         </is>
       </c>
     </row>
@@ -2131,14 +2132,14 @@
       <c r="B24" s="113" t="n"/>
       <c r="C24" s="111" t="inlineStr">
         <is>
-          <t>• Anleitung: Schritt-für-Schritt neu geordnet – Verifikation/Kalibrierung des Korrekturfaktors jetzt VOR der Raumauslegung; neuer Abschnitt 'Planungstechnische Grundlagen'; Hinweis zur vorgefertigten Revit-Liste entfernt.</t>
+          <t>• Anleitung: Abschnitt 'Planungstechnische Grundlagen' wieder entfernt.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="109" t="inlineStr">
         <is>
-          <t>0.19</t>
+          <t>0.20</t>
         </is>
       </c>
       <c r="B25" s="110" t="inlineStr">
@@ -2148,7 +2149,7 @@
       </c>
       <c r="C25" s="111" t="inlineStr">
         <is>
-          <t>• Grundeinstellungen: neuer Grenzwert 'Maximaler Volumenstrom je Kreis' (V̇_max, Default 150 l/h); Abschnitt 'Strömungsgeschwindigkeit' → 'Strömungsgrenzwerte'.</t>
+          <t>• Grundeinstellungen: Spaltenbreiten optimiert und lange Beschriftungen/Hinweise gekürzt – Texte werden in LibreOffice nicht mehr abgeschnitten.</t>
         </is>
       </c>
     </row>
@@ -2157,121 +2158,129 @@
       <c r="B26" s="112" t="n"/>
       <c r="C26" s="111" t="inlineStr">
         <is>
+          <t>• Verifikation: Untertitel und Hinweise vereinfacht (Modellvergleich-Erläuterung entfernt); klarer Hinweis, dass der Korrekturfaktor f VOR der Raumauslegung kalibriert wird; Diagramm etwas größer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="113" t="n"/>
+      <c r="B27" s="113" t="n"/>
+      <c r="C27" s="111" t="inlineStr">
+        <is>
+          <t>• Anleitung: Schritt-für-Schritt neu geordnet – Verifikation/Kalibrierung des Korrekturfaktors jetzt VOR der Raumauslegung; neuer Abschnitt 'Planungstechnische Grundlagen'; Hinweis zur vorgefertigten Revit-Liste entfernt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="109" t="inlineStr">
+        <is>
+          <t>0.19</t>
+        </is>
+      </c>
+      <c r="B28" s="110" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="C28" s="111" t="inlineStr">
+        <is>
+          <t>• Grundeinstellungen: neuer Grenzwert 'Maximaler Volumenstrom je Kreis' (V̇_max, Default 150 l/h); Abschnitt 'Strömungsgeschwindigkeit' → 'Strömungsgrenzwerte'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="112" t="n"/>
+      <c r="B29" s="112" t="n"/>
+      <c r="C29" s="111" t="inlineStr">
+        <is>
           <t>• Auslegung: Volumenstrom je Kreis wird gegen V̇_max geprüft und per Ampel eingefärbt (grün ≤ Grenze, rot darüber); zusätzliche Warnung im Blatt 'Kontrolle'.</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="112" t="n"/>
-      <c r="B27" s="112" t="n"/>
-      <c r="C27" s="111" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="112" t="n"/>
+      <c r="B30" s="112" t="n"/>
+      <c r="C30" s="111" t="inlineStr">
         <is>
           <t>• Anleitung: durchgehende Schritt-für-Schritt-Anleitung mit integriertem Revit-Export (vorgefertigte Bauteilliste muss nicht erst angelegt werden); redundanter Abschnitt 'Räume aus Revit' und der Hinweis zum direkten Kopieren entfernt.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="113" t="n"/>
-      <c r="B28" s="113" t="n"/>
-      <c r="C28" s="111" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="113" t="n"/>
+      <c r="B31" s="113" t="n"/>
+      <c r="C31" s="111" t="inlineStr">
         <is>
           <t>• Deckblatt: Pfeil-Spalten breiter und Pfeilgröße angepasst (optisch sauberer).</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="109" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="109" t="inlineStr">
         <is>
           <t>0.18</t>
         </is>
       </c>
-      <c r="B29" s="110" t="inlineStr">
+      <c r="B32" s="110" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="C29" s="111" t="inlineStr">
+      <c r="C32" s="111" t="inlineStr">
         <is>
           <t>• Auslegung: Eingabespalten neu sortiert – zuerst die Revit-Spalten (A HKV, B Raum-Nr., C Bezeichnung, D Raumfläche, E Raumtemperatur, F Heizlast), dann G spez. Heizlast (berechnet), danach die manuellen Felder (H aktiv. Fläche, I R-Wert, J Verlegeabstand, K Anz. Kreise, L Zuleitung, M Zone).</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="113" t="n"/>
-      <c r="B30" s="113" t="n"/>
-      <c r="C30" s="111" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="113" t="n"/>
+      <c r="B33" s="113" t="n"/>
+      <c r="C33" s="111" t="inlineStr">
         <is>
           <t>• Anleitung: Excel-Export aus Revit ist jetzt der Standard-Workflow (direktes Kopieren funktioniert nicht); Spaltenliste an neue Reihenfolge angepasst.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="109" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="109" t="inlineStr">
         <is>
           <t>0.17</t>
         </is>
       </c>
-      <c r="B31" s="110" t="inlineStr">
+      <c r="B34" s="110" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="C31" s="111" t="inlineStr">
+      <c r="C34" s="111" t="inlineStr">
         <is>
           <t>• Neues Blatt 'Anleitung' (2. Blatt): Aufbau der Mappe, Schritt-für-Schritt, Farblegende.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="113" t="n"/>
-      <c r="B32" s="113" t="n"/>
-      <c r="C32" s="111" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="113" t="n"/>
+      <c r="B35" s="113" t="n"/>
+      <c r="C35" s="111" t="inlineStr">
         <is>
           <t>• Anleitung enthält den Workflow zum Übernehmen der Räume aus Revit (Copy &amp; Paste, Schedule, Dynamo/Power Query).</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="109" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="109" t="inlineStr">
         <is>
           <t>0.16</t>
         </is>
       </c>
-      <c r="B33" s="110" t="inlineStr">
+      <c r="B36" s="110" t="inlineStr">
         <is>
           <t>2026-06-09</t>
         </is>
       </c>
-      <c r="C33" s="111" t="inlineStr">
+      <c r="C36" s="111" t="inlineStr">
         <is>
           <t>• Alle Blätter im A4-Querformat (nur Auslegung A3 quer); einheitlichere Schriftgrößen/Skalierung.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="112" t="n"/>
-      <c r="B34" s="112" t="n"/>
-      <c r="C34" s="111" t="inlineStr">
-        <is>
-          <t>• Grundeinstellungen zweispaltig (Einstellwerte teilweise nebeneinander).</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="112" t="n"/>
-      <c r="B35" s="112" t="n"/>
-      <c r="C35" s="111" t="inlineStr">
-        <is>
-          <t>• Verifikation: Diagramm rechts neben den Tabellen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="112" t="n"/>
-      <c r="B36" s="112" t="n"/>
-      <c r="C36" s="111" t="inlineStr">
-        <is>
-          <t>• Methodik: Formelzeichen links, Berechnungsschritte in zwei Spalten rechts.</t>
         </is>
       </c>
     </row>
@@ -2280,33 +2289,25 @@
       <c r="B37" s="112" t="n"/>
       <c r="C37" s="111" t="inlineStr">
         <is>
-          <t>• Konstanten: Tabellen teilweise nebeneinander.</t>
+          <t>• Grundeinstellungen zweispaltig (Einstellwerte teilweise nebeneinander).</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="113" t="n"/>
-      <c r="B38" s="113" t="n"/>
+      <c r="A38" s="112" t="n"/>
+      <c r="B38" s="112" t="n"/>
       <c r="C38" s="111" t="inlineStr">
         <is>
-          <t>• Auslegung: Spalte Zone mittig/schmaler, Raum-Nr. breiter; Verifikation-Korrekturfaktor vertikal mittig.</t>
+          <t>• Verifikation: Diagramm rechts neben den Tabellen.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="109" t="inlineStr">
-        <is>
-          <t>0.15</t>
-        </is>
-      </c>
-      <c r="B39" s="110" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
+      <c r="A39" s="112" t="n"/>
+      <c r="B39" s="112" t="n"/>
       <c r="C39" s="111" t="inlineStr">
         <is>
-          <t>• Deckblatt-Diagramm aus Excel-Zellen statt Bild – direkt in Excel bearbeitbar.</t>
+          <t>• Methodik: Formelzeichen links, Berechnungsschritte in zwei Spalten rechts.</t>
         </is>
       </c>
     </row>
@@ -2315,7 +2316,7 @@
       <c r="B40" s="112" t="n"/>
       <c r="C40" s="111" t="inlineStr">
         <is>
-          <t>• Auslegung: Beispielräume mit gemischter Heizlast (≤ 50 W/m²); Formelzeichen in Zeile 5 ergänzt (Flächen u. a.).</t>
+          <t>• Konstanten: Tabellen teilweise nebeneinander.</t>
         </is>
       </c>
     </row>
@@ -2324,94 +2325,94 @@
       <c r="B41" s="113" t="n"/>
       <c r="C41" s="111" t="inlineStr">
         <is>
-          <t>• Heizkreisverteiler: zusätzliche Spalte Spreizung [K].</t>
+          <t>• Auslegung: Spalte Zone mittig/schmaler, Raum-Nr. breiter; Verifikation-Korrekturfaktor vertikal mittig.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="109" t="inlineStr">
         <is>
+          <t>0.15</t>
+        </is>
+      </c>
+      <c r="B42" s="110" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="C42" s="111" t="inlineStr">
+        <is>
+          <t>• Deckblatt-Diagramm aus Excel-Zellen statt Bild – direkt in Excel bearbeitbar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="112" t="n"/>
+      <c r="B43" s="112" t="n"/>
+      <c r="C43" s="111" t="inlineStr">
+        <is>
+          <t>• Auslegung: Beispielräume mit gemischter Heizlast (≤ 50 W/m²); Formelzeichen in Zeile 5 ergänzt (Flächen u. a.).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="113" t="n"/>
+      <c r="B44" s="113" t="n"/>
+      <c r="C44" s="111" t="inlineStr">
+        <is>
+          <t>• Heizkreisverteiler: zusätzliche Spalte Spreizung [K].</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="109" t="inlineStr">
+        <is>
           <t>0.14</t>
         </is>
       </c>
-      <c r="B42" s="110" t="inlineStr">
+      <c r="B45" s="110" t="inlineStr">
         <is>
           <t>2026-06-09</t>
         </is>
       </c>
-      <c r="C42" s="111" t="inlineStr">
+      <c r="C45" s="111" t="inlineStr">
         <is>
           <t>• Deckblatt als erstes Blatt: Übersichtsdiagramm Eingaben → Verarbeitung → Ergebnisse (inkl. Vereinfachungen).</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="109" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="109" t="inlineStr">
         <is>
           <t>0.13</t>
         </is>
       </c>
-      <c r="B43" s="110" t="inlineStr">
+      <c r="B46" s="110" t="inlineStr">
         <is>
           <t>2026-06-08</t>
         </is>
       </c>
-      <c r="C43" s="111" t="inlineStr">
+      <c r="C46" s="111" t="inlineStr">
         <is>
           <t>• Strömungsbereich dreistufig: laminar (Re &lt; 2300), Übergangsbereich (2300–4000), turbulent (Re &gt; 4000).</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="112" t="n"/>
-      <c r="B44" s="112" t="n"/>
-      <c r="C44" s="111" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="112" t="n"/>
+      <c r="B47" s="112" t="n"/>
+      <c r="C47" s="111" t="inlineStr">
         <is>
           <t>• Spalte 'Strömungsbereich' ausgeblendet (für die Auslegung nicht relevant) und ohne Färbung.</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="112" t="n"/>
-      <c r="B45" s="112" t="n"/>
-      <c r="C45" s="111" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="112" t="n"/>
+      <c r="B48" s="112" t="n"/>
+      <c r="C48" s="111" t="inlineStr">
         <is>
           <t>• Auslegung schlanker: weitere Zwischenspalten standardmäßig ausgeblendet (jederzeit einblendbar).</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="112" t="n"/>
-      <c r="B46" s="112" t="n"/>
-      <c r="C46" s="111" t="inlineStr">
-        <is>
-          <t>• Verifikation: Korrekturfaktor kleiner dargestellt (passt nun vollständig in die Zelle).</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="113" t="n"/>
-      <c r="B47" s="113" t="n"/>
-      <c r="C47" s="111" t="inlineStr">
-        <is>
-          <t>• Changelog wieder ausführlich.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="109" t="inlineStr">
-        <is>
-          <t>0.12</t>
-        </is>
-      </c>
-      <c r="B48" s="110" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="C48" s="111" t="inlineStr">
-        <is>
-          <t>• Grundeinstellungen: Bezeichnungen ausgeschrieben (keine Abkürzungen).</t>
         </is>
       </c>
     </row>
@@ -2420,51 +2421,51 @@
       <c r="B49" s="112" t="n"/>
       <c r="C49" s="111" t="inlineStr">
         <is>
+          <t>• Verifikation: Korrekturfaktor kleiner dargestellt (passt nun vollständig in die Zelle).</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="113" t="n"/>
+      <c r="B50" s="113" t="n"/>
+      <c r="C50" s="111" t="inlineStr">
+        <is>
+          <t>• Changelog wieder ausführlich.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="109" t="inlineStr">
+        <is>
+          <t>0.12</t>
+        </is>
+      </c>
+      <c r="B51" s="110" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C51" s="111" t="inlineStr">
+        <is>
+          <t>• Grundeinstellungen: Bezeichnungen ausgeschrieben (keine Abkürzungen).</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="112" t="n"/>
+      <c r="B52" s="112" t="n"/>
+      <c r="C52" s="111" t="inlineStr">
+        <is>
           <t>• Neue Spalte 'spez. Heizlast [W/m²]' (Heizlast bezogen auf die Raumfläche).</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="112" t="n"/>
-      <c r="B50" s="112" t="n"/>
-      <c r="C50" s="111" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="112" t="n"/>
+      <c r="B53" s="112" t="n"/>
+      <c r="C53" s="111" t="inlineStr">
         <is>
           <t>• Massenstrom/Geschwindigkeit/Druckverlust auf Basis min(Leistung; Heizlast) + Verlust nach unten (realer Betriebspunkt).</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="112" t="n"/>
-      <c r="B51" s="112" t="n"/>
-      <c r="C51" s="111" t="inlineStr">
-        <is>
-          <t>• Heizkreisverteiler zusätzlich mit Massenstrom [kg/h]; Zonen-Kürzel (AZ/RZ/BAD).</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="113" t="n"/>
-      <c r="B52" s="113" t="n"/>
-      <c r="C52" s="111" t="inlineStr">
-        <is>
-          <t>• Kapazität 200 Räume / 50 Verteiler; Auslegung A3 quer, übrige Blätter A4 hoch.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="109" t="inlineStr">
-        <is>
-          <t>0.11</t>
-        </is>
-      </c>
-      <c r="B53" s="110" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="C53" s="111" t="inlineStr">
-        <is>
-          <t>• Bugfixes: Hinweistext wurde als Formel interpretiert (Fehler 501); MAXIFS ersetzt (#NAME? in LibreOffice).</t>
         </is>
       </c>
     </row>
@@ -2473,42 +2474,42 @@
       <c r="B54" s="112" t="n"/>
       <c r="C54" s="111" t="inlineStr">
         <is>
+          <t>• Heizkreisverteiler zusätzlich mit Massenstrom [kg/h]; Zonen-Kürzel (AZ/RZ/BAD).</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="113" t="n"/>
+      <c r="B55" s="113" t="n"/>
+      <c r="C55" s="111" t="inlineStr">
+        <is>
+          <t>• Kapazität 200 Räume / 50 Verteiler; Auslegung A3 quer, übrige Blätter A4 hoch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="109" t="inlineStr">
+        <is>
+          <t>0.11</t>
+        </is>
+      </c>
+      <c r="B56" s="110" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C56" s="111" t="inlineStr">
+        <is>
+          <t>• Bugfixes: Hinweistext wurde als Formel interpretiert (Fehler 501); MAXIFS ersetzt (#NAME? in LibreOffice).</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="112" t="n"/>
+      <c r="B57" s="112" t="n"/>
+      <c r="C57" s="111" t="inlineStr">
+        <is>
           <t>• Verifikation: Korrekturfaktor prominent oben; Hersteller-q direkt neben q berechnet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="112" t="n"/>
-      <c r="B55" s="112" t="n"/>
-      <c r="C55" s="111" t="inlineStr">
-        <is>
-          <t>• Konstanten: alle Tabellen untereinander, mit Leerzeilen für weitere Einträge.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="113" t="n"/>
-      <c r="B56" s="113" t="n"/>
-      <c r="C56" s="111" t="inlineStr">
-        <is>
-          <t>• Methodik: Variablen zuerst, dann Formeln mit Erklärung je Schritt; weitere Musterräume (Verwaltungsbau).</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="109" t="inlineStr">
-        <is>
-          <t>0.10</t>
-        </is>
-      </c>
-      <c r="B57" s="110" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="C57" s="111" t="inlineStr">
-        <is>
-          <t>• Heizkreisverteiler-Liste und Verifikation ohne dynamische Array-Funktionen → läuft in Excel UND LibreOffice.</t>
         </is>
       </c>
     </row>
@@ -2517,7 +2518,7 @@
       <c r="B58" s="112" t="n"/>
       <c r="C58" s="111" t="inlineStr">
         <is>
-          <t>• Verifikation mit Liniendiagramm; Konstanten/Bibliotheken in eigenes Blatt ausgelagert.</t>
+          <t>• Konstanten: alle Tabellen untereinander, mit Leerzeilen für weitere Einträge.</t>
         </is>
       </c>
     </row>
@@ -2526,24 +2527,24 @@
       <c r="B59" s="113" t="n"/>
       <c r="C59" s="111" t="inlineStr">
         <is>
-          <t>• Gewähltes Rohrsystem mit Außen-/Innendurchmesser, Wandstärke und Rauheit im Druckbereich.</t>
+          <t>• Methodik: Variablen zuerst, dann Formeln mit Erklärung je Schritt; weitere Musterräume (Verwaltungsbau).</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="109" t="inlineStr">
         <is>
-          <t>0.9</t>
+          <t>0.10</t>
         </is>
       </c>
       <c r="B60" s="110" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C60" s="111" t="inlineStr">
         <is>
-          <t>• Neues Blatt 'Heizkreisverteiler' (Leistung, max. Druckverlust, Volumenstrom je HKV).</t>
+          <t>• Heizkreisverteiler-Liste und Verifikation ohne dynamische Array-Funktionen → läuft in Excel UND LibreOffice.</t>
         </is>
       </c>
     </row>
@@ -2552,42 +2553,42 @@
       <c r="B61" s="112" t="n"/>
       <c r="C61" s="111" t="inlineStr">
         <is>
+          <t>• Verifikation mit Liniendiagramm; Konstanten/Bibliotheken in eigenes Blatt ausgelagert.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="113" t="n"/>
+      <c r="B62" s="113" t="n"/>
+      <c r="C62" s="111" t="inlineStr">
+        <is>
+          <t>• Gewähltes Rohrsystem mit Außen-/Innendurchmesser, Wandstärke und Rauheit im Druckbereich.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="109" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="B63" s="110" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="C63" s="111" t="inlineStr">
+        <is>
+          <t>• Neues Blatt 'Heizkreisverteiler' (Leistung, max. Druckverlust, Volumenstrom je HKV).</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="112" t="n"/>
+      <c r="B64" s="112" t="n"/>
+      <c r="C64" s="111" t="inlineStr">
+        <is>
           <t>• Spaltenüberschriften der Auslegung dreizeilig (Name / Formelzeichen / Einheit).</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="112" t="n"/>
-      <c r="B62" s="112" t="n"/>
-      <c r="C62" s="111" t="inlineStr">
-        <is>
-          <t>• Korrekturfaktor f wird auf 'Verifikation' eingegeben (mit Vergleichsdiagramm).</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="113" t="n"/>
-      <c r="B63" s="113" t="n"/>
-      <c r="C63" s="111" t="inlineStr">
-        <is>
-          <t>• Geschwindigkeits-Grenzwerte v_min/v_max als Grundeinstellung.</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="109" t="inlineStr">
-        <is>
-          <t>0.8</t>
-        </is>
-      </c>
-      <c r="B64" s="110" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C64" s="111" t="inlineStr">
-        <is>
-          <t>• Grundeinstellungen für A3 quer optimiert (Einstellungen links, Tabellen rechts).</t>
         </is>
       </c>
     </row>
@@ -2596,42 +2597,42 @@
       <c r="B65" s="112" t="n"/>
       <c r="C65" s="111" t="inlineStr">
         <is>
+          <t>• Korrekturfaktor f wird auf 'Verifikation' eingegeben (mit Vergleichsdiagramm).</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="113" t="n"/>
+      <c r="B66" s="113" t="n"/>
+      <c r="C66" s="111" t="inlineStr">
+        <is>
+          <t>• Geschwindigkeits-Grenzwerte v_min/v_max als Grundeinstellung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="109" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="B67" s="110" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="C67" s="111" t="inlineStr">
+        <is>
+          <t>• Grundeinstellungen für A3 quer optimiert (Einstellungen links, Tabellen rechts).</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="112" t="n"/>
+      <c r="B68" s="112" t="n"/>
+      <c r="C68" s="111" t="inlineStr">
+        <is>
           <t>• Auslegung passt auf eine Seite breit; Korrekturfaktor Heizleistung zur Kalibrierung ergänzt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="112" t="n"/>
-      <c r="B66" s="112" t="n"/>
-      <c r="C66" s="111" t="inlineStr">
-        <is>
-          <t>• Wärmeabgabe nach unten berücksichtigt (Verlust + Gesamtleistung).</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="113" t="n"/>
-      <c r="B67" s="113" t="n"/>
-      <c r="C67" s="111" t="inlineStr">
-        <is>
-          <t>• Blätter umbenannt: Raumliste → Auslegung, Übersicht → Kontrolle; zusätzliche Kontrollen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="109" t="inlineStr">
-        <is>
-          <t>0.7</t>
-        </is>
-      </c>
-      <c r="B68" s="110" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C68" s="111" t="inlineStr">
-        <is>
-          <t>• Deckung-%-Spalte färbt nur noch gefüllte Zellen (leere bleiben farblos).</t>
         </is>
       </c>
     </row>
@@ -2640,7 +2641,7 @@
       <c r="B69" s="112" t="n"/>
       <c r="C69" s="111" t="inlineStr">
         <is>
-          <t>• Neues Blatt 'Verifikation'; neue Spalte 'Strömungsbereich' (laminar/turbulent).</t>
+          <t>• Wärmeabgabe nach unten berücksichtigt (Verlust + Gesamtleistung).</t>
         </is>
       </c>
     </row>
@@ -2649,14 +2650,14 @@
       <c r="B70" s="113" t="n"/>
       <c r="C70" s="111" t="inlineStr">
         <is>
-          <t>• Alle Blätter im A3-Querformat; einheitlicher Kopf je Blatt.</t>
+          <t>• Blätter umbenannt: Raumliste → Auslegung, Übersicht → Kontrolle; zusätzliche Kontrollen.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="109" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>0.7</t>
         </is>
       </c>
       <c r="B71" s="110" t="inlineStr">
@@ -2666,24 +2667,16 @@
       </c>
       <c r="C71" s="111" t="inlineStr">
         <is>
-          <t>• Bugfix: Zellfärbung (bedingte Formatierung) wird jetzt auch in Excel angezeigt – dxf-Füllfarbe mit voller Deckkraft.</t>
+          <t>• Deckung-%-Spalte färbt nur noch gefüllte Zellen (leere bleiben farblos).</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="109" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
-      </c>
-      <c r="B72" s="110" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
+      <c r="A72" s="112" t="n"/>
+      <c r="B72" s="112" t="n"/>
       <c r="C72" s="111" t="inlineStr">
         <is>
-          <t>• Versionsnummer und Autor werden nur noch im Changelog angezeigt.</t>
+          <t>• Neues Blatt 'Verifikation'; neue Spalte 'Strömungsbereich' (laminar/turbulent).</t>
         </is>
       </c>
     </row>
@@ -2692,68 +2685,76 @@
       <c r="B73" s="113" t="n"/>
       <c r="C73" s="111" t="inlineStr">
         <is>
-          <t>• Editierbares Bearbeiter-Kürzel rechts oben unter dem Logo (Grundeinstellungen, Auslegung, Kontrolle, HKV).</t>
+          <t>• Alle Blätter im A3-Querformat; einheitlicher Kopf je Blatt.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="109" t="inlineStr">
         <is>
+          <t>0.6</t>
+        </is>
+      </c>
+      <c r="B74" s="110" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="C74" s="111" t="inlineStr">
+        <is>
+          <t>• Bugfix: Zellfärbung (bedingte Formatierung) wird jetzt auch in Excel angezeigt – dxf-Füllfarbe mit voller Deckkraft.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="109" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="B75" s="110" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="C75" s="111" t="inlineStr">
+        <is>
+          <t>• Versionsnummer und Autor werden nur noch im Changelog angezeigt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="113" t="n"/>
+      <c r="B76" s="113" t="n"/>
+      <c r="C76" s="111" t="inlineStr">
+        <is>
+          <t>• Editierbares Bearbeiter-Kürzel rechts oben unter dem Logo (Grundeinstellungen, Auslegung, Kontrolle, HKV).</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="109" t="inlineStr">
+        <is>
           <t>0.4</t>
         </is>
       </c>
-      <c r="B74" s="110" t="inlineStr">
+      <c r="B77" s="110" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="C74" s="111" t="inlineStr">
+      <c r="C77" s="111" t="inlineStr">
         <is>
           <t>• Status-Spalten entfernt – Bewertung erfolgt jetzt direkt als Zellfärbung (grün/rot).</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="112" t="n"/>
-      <c r="B75" s="112" t="n"/>
-      <c r="C75" s="111" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="112" t="n"/>
+      <c r="B78" s="112" t="n"/>
+      <c r="C78" s="111" t="inlineStr">
         <is>
           <t>• Methodik um die Formelzeichen-Legende erweitert.</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="112" t="n"/>
-      <c r="B76" s="112" t="n"/>
-      <c r="C76" s="111" t="inlineStr">
-        <is>
-          <t>• Heizkreisverteiler (HKV) als erste Spalte der Auslegung; Standardwert max. Druckverlust 15.000 Pa.</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="113" t="n"/>
-      <c r="B77" s="113" t="n"/>
-      <c r="C77" s="111" t="inlineStr">
-        <is>
-          <t>• Versionsschema 0.x eingeführt (1.0 erst nach Test); interner Autor (dh).</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="109" t="inlineStr">
-        <is>
-          <t>0.3</t>
-        </is>
-      </c>
-      <c r="B78" s="110" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C78" s="111" t="inlineStr">
-        <is>
-          <t>• Zonentypen (Aufenthalt/Rand/Bad) mit eigener zulässiger Oberflächentemperatur.</t>
         </is>
       </c>
     </row>
@@ -2762,51 +2763,51 @@
       <c r="B79" s="112" t="n"/>
       <c r="C79" s="111" t="inlineStr">
         <is>
+          <t>• Heizkreisverteiler (HKV) als erste Spalte der Auslegung; Standardwert max. Druckverlust 15.000 Pa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="113" t="n"/>
+      <c r="B80" s="113" t="n"/>
+      <c r="C80" s="111" t="inlineStr">
+        <is>
+          <t>• Versionsschema 0.x eingeführt (1.0 erst nach Test); interner Autor (dh).</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="109" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="B81" s="110" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="C81" s="111" t="inlineStr">
+        <is>
+          <t>• Zonentypen (Aufenthalt/Rand/Bad) mit eigener zulässiger Oberflächentemperatur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="112" t="n"/>
+      <c r="B82" s="112" t="n"/>
+      <c r="C82" s="111" t="inlineStr">
+        <is>
           <t>• Einheitlicher Kopf: Titel oben links, agn-Logo oben rechts, Projektkopf darunter.</t>
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" s="112" t="n"/>
-      <c r="B80" s="112" t="n"/>
-      <c r="C80" s="111" t="inlineStr">
+    <row r="83">
+      <c r="A83" s="112" t="n"/>
+      <c r="B83" s="112" t="n"/>
+      <c r="C83" s="111" t="inlineStr">
         <is>
           <t>• Oberflächentemperatur θF und Volumenstrom eingeblendet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="112" t="n"/>
-      <c r="B81" s="112" t="n"/>
-      <c r="C81" s="111" t="inlineStr">
-        <is>
-          <t>• Neue Spalten 'spez. Druckverlust [Pa/m]' und Eingabespalte 'Verteiler (Anbindung)'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="113" t="n"/>
-      <c r="B82" s="113" t="n"/>
-      <c r="C82" s="111" t="inlineStr">
-        <is>
-          <t>• Warnung (rot), wenn die aktivierbare Fläche größer als die Raumfläche ist.</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="109" t="inlineStr">
-        <is>
-          <t>0.2</t>
-        </is>
-      </c>
-      <c r="B83" s="110" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C83" s="111" t="inlineStr">
-        <is>
-          <t>• agn-Logo eingebunden und eigenes Changelog-Blatt ergänzt.</t>
         </is>
       </c>
     </row>
@@ -2815,51 +2816,51 @@
       <c r="B84" s="112" t="n"/>
       <c r="C84" s="111" t="inlineStr">
         <is>
+          <t>• Neue Spalten 'spez. Druckverlust [Pa/m]' und Eingabespalte 'Verteiler (Anbindung)'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="113" t="n"/>
+      <c r="B85" s="113" t="n"/>
+      <c r="C85" s="111" t="inlineStr">
+        <is>
+          <t>• Warnung (rot), wenn die aktivierbare Fläche größer als die Raumfläche ist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="109" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="B86" s="110" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="C86" s="111" t="inlineStr">
+        <is>
+          <t>• agn-Logo eingebunden und eigenes Changelog-Blatt ergänzt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="112" t="n"/>
+      <c r="B87" s="112" t="n"/>
+      <c r="C87" s="111" t="inlineStr">
+        <is>
           <t>• Zuschlag Einzelwiderstände (5 %) und fester Verteiler-Aufschlag (500 Pa je Kreis).</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" s="112" t="n"/>
-      <c r="B85" s="112" t="n"/>
-      <c r="C85" s="111" t="inlineStr">
+    <row r="88">
+      <c r="A88" s="112" t="n"/>
+      <c r="B88" s="112" t="n"/>
+      <c r="C88" s="111" t="inlineStr">
         <is>
           <t>• Einheiten als Zellformat; Projektnummer/Projektname erscheinen im Ausdruck.</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="112" t="n"/>
-      <c r="B86" s="112" t="n"/>
-      <c r="C86" s="111" t="inlineStr">
-        <is>
-          <t>• Richtwert-Tabellen für R-Werte und Verlegeabstand-Faktoren; weitere Musterräume.</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="113" t="n"/>
-      <c r="B87" s="113" t="n"/>
-      <c r="C87" s="111" t="inlineStr">
-        <is>
-          <t>• Druckaufbereitung für DIN A4.</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="109" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="B88" s="110" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C88" s="111" t="inlineStr">
-        <is>
-          <t>• Ersterstellung mit den Blättern Grundeinstellungen, Raumliste, Übersicht und Methodik.</t>
         </is>
       </c>
     </row>
@@ -2868,32 +2869,67 @@
       <c r="B89" s="112" t="n"/>
       <c r="C89" s="111" t="inlineStr">
         <is>
+          <t>• Richtwert-Tabellen für R-Werte und Verlegeabstand-Faktoren; weitere Musterräume.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="113" t="n"/>
+      <c r="B90" s="113" t="n"/>
+      <c r="C90" s="111" t="inlineStr">
+        <is>
+          <t>• Druckaufbereitung für DIN A4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="109" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="B91" s="110" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="C91" s="111" t="inlineStr">
+        <is>
+          <t>• Ersterstellung mit den Blättern Grundeinstellungen, Raumliste, Übersicht und Methodik.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="112" t="n"/>
+      <c r="B92" s="112" t="n"/>
+      <c r="C92" s="111" t="inlineStr">
+        <is>
           <t>• Heizleistung über die logarithmische Übertemperatur (q = η · K_H · ΔθH).</t>
         </is>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" s="112" t="n"/>
-      <c r="B90" s="112" t="n"/>
-      <c r="C90" s="111" t="inlineStr">
+    <row r="93">
+      <c r="A93" s="112" t="n"/>
+      <c r="B93" s="112" t="n"/>
+      <c r="C93" s="111" t="inlineStr">
         <is>
           <t>• Druckverlustberechnung nach Darcy-Weisbach.</t>
         </is>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" s="112" t="n"/>
-      <c r="B91" s="112" t="n"/>
-      <c r="C91" s="111" t="inlineStr">
+    <row r="94">
+      <c r="A94" s="112" t="n"/>
+      <c r="B94" s="112" t="n"/>
+      <c r="C94" s="111" t="inlineStr">
         <is>
           <t>• Editierbare Rohrbibliothek und Verlegeabstand-Faktoren.</t>
         </is>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" s="113" t="n"/>
-      <c r="B92" s="113" t="n"/>
-      <c r="C92" s="111" t="inlineStr">
+    <row r="95">
+      <c r="A95" s="113" t="n"/>
+      <c r="B95" s="113" t="n"/>
+      <c r="C95" s="111" t="inlineStr">
         <is>
           <t>• Prüfungen: Oberflächentemperatur, Heizlastdeckung, Kreislänge, Druckverlust.</t>
         </is>
@@ -2901,53 +2937,55 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <mergeCells count="46">
-    <mergeCell ref="B88:B92"/>
-    <mergeCell ref="A57:A59"/>
-    <mergeCell ref="B78:B82"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="A64:A67"/>
-    <mergeCell ref="B68:B70"/>
-    <mergeCell ref="A60:A63"/>
-    <mergeCell ref="B6:B10"/>
-    <mergeCell ref="A25:A28"/>
+  <mergeCells count="48">
+    <mergeCell ref="A67:A70"/>
+    <mergeCell ref="B56:B59"/>
+    <mergeCell ref="A86:A90"/>
+    <mergeCell ref="B9:B13"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="B77:B80"/>
+    <mergeCell ref="A36:A41"/>
     <mergeCell ref="A22:A24"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="A68:A70"/>
-    <mergeCell ref="B83:B87"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="A43:A47"/>
-    <mergeCell ref="A74:A77"/>
+    <mergeCell ref="A71:A73"/>
+    <mergeCell ref="A75:A76"/>
+    <mergeCell ref="B67:B70"/>
+    <mergeCell ref="A91:A95"/>
+    <mergeCell ref="A9:A13"/>
+    <mergeCell ref="A81:A85"/>
+    <mergeCell ref="B51:B55"/>
+    <mergeCell ref="A56:A59"/>
+    <mergeCell ref="A19:A21"/>
+    <mergeCell ref="B25:B27"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="B63:B66"/>
+    <mergeCell ref="B28:B31"/>
+    <mergeCell ref="B22:B24"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="B91:B95"/>
+    <mergeCell ref="A60:A62"/>
+    <mergeCell ref="A51:A55"/>
+    <mergeCell ref="B81:B85"/>
+    <mergeCell ref="B71:B73"/>
+    <mergeCell ref="A6:A8"/>
+    <mergeCell ref="B42:B44"/>
+    <mergeCell ref="B46:B50"/>
+    <mergeCell ref="A63:A66"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="B36:B41"/>
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="B75:B76"/>
+    <mergeCell ref="B86:B90"/>
+    <mergeCell ref="A25:A27"/>
+    <mergeCell ref="A28:A31"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="B60:B62"/>
+    <mergeCell ref="A77:A80"/>
     <mergeCell ref="B19:B21"/>
-    <mergeCell ref="A19:A21"/>
-    <mergeCell ref="A83:A87"/>
-    <mergeCell ref="B16:B18"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="B22:B24"/>
-    <mergeCell ref="A39:A41"/>
-    <mergeCell ref="B53:B56"/>
-    <mergeCell ref="A48:A52"/>
-    <mergeCell ref="B60:B63"/>
-    <mergeCell ref="A72:A73"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="B74:B77"/>
-    <mergeCell ref="A88:A92"/>
-    <mergeCell ref="A53:A56"/>
-    <mergeCell ref="A33:A38"/>
-    <mergeCell ref="B33:B38"/>
-    <mergeCell ref="A6:A10"/>
-    <mergeCell ref="B39:B41"/>
-    <mergeCell ref="B57:B59"/>
-    <mergeCell ref="B48:B52"/>
-    <mergeCell ref="B43:B47"/>
-    <mergeCell ref="A16:A18"/>
-    <mergeCell ref="A78:A82"/>
-    <mergeCell ref="B64:B67"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="B25:B28"/>
-    <mergeCell ref="B72:B73"/>
-    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="A46:A50"/>
+    <mergeCell ref="A42:A44"/>
+    <mergeCell ref="B6:B8"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -3926,7 +3964,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
@@ -3935,7 +3973,7 @@
     <col width="9" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
     <col width="11" customWidth="1" min="12" max="12"/>
     <col width="6" customWidth="1" min="13" max="13"/>
     <col hidden="1" width="12" customWidth="1" min="14" max="14"/>
@@ -3945,7 +3983,7 @@
     <col width="11" customWidth="1" min="18" max="18"/>
     <col hidden="1" width="11" customWidth="1" min="19" max="19"/>
     <col width="9" customWidth="1" min="20" max="20"/>
-    <col width="13" customWidth="1" min="21" max="21"/>
+    <col hidden="1" width="12" customWidth="1" min="21" max="21"/>
     <col width="8" customWidth="1" min="22" max="22"/>
     <col hidden="1" width="11" customWidth="1" min="23" max="23"/>
     <col hidden="1" width="12" customWidth="1" min="24" max="24"/>
@@ -4869,7 +4907,7 @@
         <v/>
       </c>
       <c r="S7" s="68">
-        <f>IF($B7="","",IFERROR(VLOOKUP($M7,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B7="","",IFERROR(VLOOKUP($M7,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T7" s="69">
@@ -5015,7 +5053,7 @@
         <v/>
       </c>
       <c r="S8" s="68">
-        <f>IF($B8="","",IFERROR(VLOOKUP($M8,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B8="","",IFERROR(VLOOKUP($M8,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T8" s="69">
@@ -5161,7 +5199,7 @@
         <v/>
       </c>
       <c r="S9" s="68">
-        <f>IF($B9="","",IFERROR(VLOOKUP($M9,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B9="","",IFERROR(VLOOKUP($M9,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T9" s="69">
@@ -5307,7 +5345,7 @@
         <v/>
       </c>
       <c r="S10" s="68">
-        <f>IF($B10="","",IFERROR(VLOOKUP($M10,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B10="","",IFERROR(VLOOKUP($M10,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T10" s="69">
@@ -5453,7 +5491,7 @@
         <v/>
       </c>
       <c r="S11" s="68">
-        <f>IF($B11="","",IFERROR(VLOOKUP($M11,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B11="","",IFERROR(VLOOKUP($M11,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T11" s="69">
@@ -5599,7 +5637,7 @@
         <v/>
       </c>
       <c r="S12" s="68">
-        <f>IF($B12="","",IFERROR(VLOOKUP($M12,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B12="","",IFERROR(VLOOKUP($M12,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T12" s="69">
@@ -5745,7 +5783,7 @@
         <v/>
       </c>
       <c r="S13" s="68">
-        <f>IF($B13="","",IFERROR(VLOOKUP($M13,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B13="","",IFERROR(VLOOKUP($M13,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T13" s="69">
@@ -5891,7 +5929,7 @@
         <v/>
       </c>
       <c r="S14" s="68">
-        <f>IF($B14="","",IFERROR(VLOOKUP($M14,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B14="","",IFERROR(VLOOKUP($M14,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T14" s="69">
@@ -6037,7 +6075,7 @@
         <v/>
       </c>
       <c r="S15" s="68">
-        <f>IF($B15="","",IFERROR(VLOOKUP($M15,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B15="","",IFERROR(VLOOKUP($M15,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T15" s="69">
@@ -6151,7 +6189,7 @@
         <v/>
       </c>
       <c r="S16" s="68">
-        <f>IF($B16="","",IFERROR(VLOOKUP($M16,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B16="","",IFERROR(VLOOKUP($M16,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T16" s="69">
@@ -6265,7 +6303,7 @@
         <v/>
       </c>
       <c r="S17" s="68">
-        <f>IF($B17="","",IFERROR(VLOOKUP($M17,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B17="","",IFERROR(VLOOKUP($M17,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T17" s="69">
@@ -6379,7 +6417,7 @@
         <v/>
       </c>
       <c r="S18" s="68">
-        <f>IF($B18="","",IFERROR(VLOOKUP($M18,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B18="","",IFERROR(VLOOKUP($M18,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T18" s="69">
@@ -6493,7 +6531,7 @@
         <v/>
       </c>
       <c r="S19" s="68">
-        <f>IF($B19="","",IFERROR(VLOOKUP($M19,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B19="","",IFERROR(VLOOKUP($M19,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T19" s="69">
@@ -6607,7 +6645,7 @@
         <v/>
       </c>
       <c r="S20" s="68">
-        <f>IF($B20="","",IFERROR(VLOOKUP($M20,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B20="","",IFERROR(VLOOKUP($M20,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T20" s="69">
@@ -6721,7 +6759,7 @@
         <v/>
       </c>
       <c r="S21" s="68">
-        <f>IF($B21="","",IFERROR(VLOOKUP($M21,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B21="","",IFERROR(VLOOKUP($M21,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T21" s="69">
@@ -6835,7 +6873,7 @@
         <v/>
       </c>
       <c r="S22" s="68">
-        <f>IF($B22="","",IFERROR(VLOOKUP($M22,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B22="","",IFERROR(VLOOKUP($M22,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T22" s="69">
@@ -6949,7 +6987,7 @@
         <v/>
       </c>
       <c r="S23" s="68">
-        <f>IF($B23="","",IFERROR(VLOOKUP($M23,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B23="","",IFERROR(VLOOKUP($M23,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T23" s="69">
@@ -7063,7 +7101,7 @@
         <v/>
       </c>
       <c r="S24" s="68">
-        <f>IF($B24="","",IFERROR(VLOOKUP($M24,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B24="","",IFERROR(VLOOKUP($M24,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T24" s="69">
@@ -7177,7 +7215,7 @@
         <v/>
       </c>
       <c r="S25" s="68">
-        <f>IF($B25="","",IFERROR(VLOOKUP($M25,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B25="","",IFERROR(VLOOKUP($M25,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T25" s="69">
@@ -7291,7 +7329,7 @@
         <v/>
       </c>
       <c r="S26" s="68">
-        <f>IF($B26="","",IFERROR(VLOOKUP($M26,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B26="","",IFERROR(VLOOKUP($M26,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T26" s="69">
@@ -7405,7 +7443,7 @@
         <v/>
       </c>
       <c r="S27" s="68">
-        <f>IF($B27="","",IFERROR(VLOOKUP($M27,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B27="","",IFERROR(VLOOKUP($M27,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T27" s="69">
@@ -7519,7 +7557,7 @@
         <v/>
       </c>
       <c r="S28" s="68">
-        <f>IF($B28="","",IFERROR(VLOOKUP($M28,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B28="","",IFERROR(VLOOKUP($M28,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T28" s="69">
@@ -7633,7 +7671,7 @@
         <v/>
       </c>
       <c r="S29" s="68">
-        <f>IF($B29="","",IFERROR(VLOOKUP($M29,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B29="","",IFERROR(VLOOKUP($M29,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T29" s="69">
@@ -7747,7 +7785,7 @@
         <v/>
       </c>
       <c r="S30" s="68">
-        <f>IF($B30="","",IFERROR(VLOOKUP($M30,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B30="","",IFERROR(VLOOKUP($M30,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T30" s="69">
@@ -7861,7 +7899,7 @@
         <v/>
       </c>
       <c r="S31" s="68">
-        <f>IF($B31="","",IFERROR(VLOOKUP($M31,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B31="","",IFERROR(VLOOKUP($M31,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T31" s="69">
@@ -7975,7 +8013,7 @@
         <v/>
       </c>
       <c r="S32" s="68">
-        <f>IF($B32="","",IFERROR(VLOOKUP($M32,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B32="","",IFERROR(VLOOKUP($M32,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T32" s="69">
@@ -8089,7 +8127,7 @@
         <v/>
       </c>
       <c r="S33" s="68">
-        <f>IF($B33="","",IFERROR(VLOOKUP($M33,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B33="","",IFERROR(VLOOKUP($M33,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T33" s="69">
@@ -8203,7 +8241,7 @@
         <v/>
       </c>
       <c r="S34" s="68">
-        <f>IF($B34="","",IFERROR(VLOOKUP($M34,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B34="","",IFERROR(VLOOKUP($M34,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T34" s="69">
@@ -8317,7 +8355,7 @@
         <v/>
       </c>
       <c r="S35" s="68">
-        <f>IF($B35="","",IFERROR(VLOOKUP($M35,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B35="","",IFERROR(VLOOKUP($M35,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T35" s="69">
@@ -8431,7 +8469,7 @@
         <v/>
       </c>
       <c r="S36" s="68">
-        <f>IF($B36="","",IFERROR(VLOOKUP($M36,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B36="","",IFERROR(VLOOKUP($M36,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T36" s="69">
@@ -8545,7 +8583,7 @@
         <v/>
       </c>
       <c r="S37" s="68">
-        <f>IF($B37="","",IFERROR(VLOOKUP($M37,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B37="","",IFERROR(VLOOKUP($M37,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T37" s="69">
@@ -8659,7 +8697,7 @@
         <v/>
       </c>
       <c r="S38" s="68">
-        <f>IF($B38="","",IFERROR(VLOOKUP($M38,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B38="","",IFERROR(VLOOKUP($M38,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T38" s="69">
@@ -8773,7 +8811,7 @@
         <v/>
       </c>
       <c r="S39" s="68">
-        <f>IF($B39="","",IFERROR(VLOOKUP($M39,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B39="","",IFERROR(VLOOKUP($M39,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T39" s="69">
@@ -8887,7 +8925,7 @@
         <v/>
       </c>
       <c r="S40" s="68">
-        <f>IF($B40="","",IFERROR(VLOOKUP($M40,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B40="","",IFERROR(VLOOKUP($M40,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T40" s="69">
@@ -9001,7 +9039,7 @@
         <v/>
       </c>
       <c r="S41" s="68">
-        <f>IF($B41="","",IFERROR(VLOOKUP($M41,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B41="","",IFERROR(VLOOKUP($M41,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T41" s="69">
@@ -9115,7 +9153,7 @@
         <v/>
       </c>
       <c r="S42" s="68">
-        <f>IF($B42="","",IFERROR(VLOOKUP($M42,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B42="","",IFERROR(VLOOKUP($M42,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T42" s="69">
@@ -9229,7 +9267,7 @@
         <v/>
       </c>
       <c r="S43" s="68">
-        <f>IF($B43="","",IFERROR(VLOOKUP($M43,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B43="","",IFERROR(VLOOKUP($M43,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T43" s="69">
@@ -9343,7 +9381,7 @@
         <v/>
       </c>
       <c r="S44" s="68">
-        <f>IF($B44="","",IFERROR(VLOOKUP($M44,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B44="","",IFERROR(VLOOKUP($M44,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T44" s="69">
@@ -9457,7 +9495,7 @@
         <v/>
       </c>
       <c r="S45" s="68">
-        <f>IF($B45="","",IFERROR(VLOOKUP($M45,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B45="","",IFERROR(VLOOKUP($M45,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T45" s="69">
@@ -9571,7 +9609,7 @@
         <v/>
       </c>
       <c r="S46" s="68">
-        <f>IF($B46="","",IFERROR(VLOOKUP($M46,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B46="","",IFERROR(VLOOKUP($M46,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T46" s="69">
@@ -9685,7 +9723,7 @@
         <v/>
       </c>
       <c r="S47" s="68">
-        <f>IF($B47="","",IFERROR(VLOOKUP($M47,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B47="","",IFERROR(VLOOKUP($M47,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T47" s="69">
@@ -9799,7 +9837,7 @@
         <v/>
       </c>
       <c r="S48" s="68">
-        <f>IF($B48="","",IFERROR(VLOOKUP($M48,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B48="","",IFERROR(VLOOKUP($M48,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T48" s="69">
@@ -9913,7 +9951,7 @@
         <v/>
       </c>
       <c r="S49" s="68">
-        <f>IF($B49="","",IFERROR(VLOOKUP($M49,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B49="","",IFERROR(VLOOKUP($M49,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T49" s="69">
@@ -10027,7 +10065,7 @@
         <v/>
       </c>
       <c r="S50" s="68">
-        <f>IF($B50="","",IFERROR(VLOOKUP($M50,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B50="","",IFERROR(VLOOKUP($M50,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T50" s="69">
@@ -10141,7 +10179,7 @@
         <v/>
       </c>
       <c r="S51" s="68">
-        <f>IF($B51="","",IFERROR(VLOOKUP($M51,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B51="","",IFERROR(VLOOKUP($M51,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T51" s="69">
@@ -10255,7 +10293,7 @@
         <v/>
       </c>
       <c r="S52" s="68">
-        <f>IF($B52="","",IFERROR(VLOOKUP($M52,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B52="","",IFERROR(VLOOKUP($M52,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T52" s="69">
@@ -10369,7 +10407,7 @@
         <v/>
       </c>
       <c r="S53" s="68">
-        <f>IF($B53="","",IFERROR(VLOOKUP($M53,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B53="","",IFERROR(VLOOKUP($M53,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T53" s="69">
@@ -10483,7 +10521,7 @@
         <v/>
       </c>
       <c r="S54" s="68">
-        <f>IF($B54="","",IFERROR(VLOOKUP($M54,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B54="","",IFERROR(VLOOKUP($M54,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T54" s="69">
@@ -10597,7 +10635,7 @@
         <v/>
       </c>
       <c r="S55" s="68">
-        <f>IF($B55="","",IFERROR(VLOOKUP($M55,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B55="","",IFERROR(VLOOKUP($M55,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T55" s="69">
@@ -10711,7 +10749,7 @@
         <v/>
       </c>
       <c r="S56" s="68">
-        <f>IF($B56="","",IFERROR(VLOOKUP($M56,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B56="","",IFERROR(VLOOKUP($M56,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T56" s="69">
@@ -10825,7 +10863,7 @@
         <v/>
       </c>
       <c r="S57" s="68">
-        <f>IF($B57="","",IFERROR(VLOOKUP($M57,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B57="","",IFERROR(VLOOKUP($M57,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T57" s="69">
@@ -10939,7 +10977,7 @@
         <v/>
       </c>
       <c r="S58" s="68">
-        <f>IF($B58="","",IFERROR(VLOOKUP($M58,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B58="","",IFERROR(VLOOKUP($M58,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T58" s="69">
@@ -11053,7 +11091,7 @@
         <v/>
       </c>
       <c r="S59" s="68">
-        <f>IF($B59="","",IFERROR(VLOOKUP($M59,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B59="","",IFERROR(VLOOKUP($M59,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T59" s="69">
@@ -11167,7 +11205,7 @@
         <v/>
       </c>
       <c r="S60" s="68">
-        <f>IF($B60="","",IFERROR(VLOOKUP($M60,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B60="","",IFERROR(VLOOKUP($M60,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T60" s="69">
@@ -11281,7 +11319,7 @@
         <v/>
       </c>
       <c r="S61" s="68">
-        <f>IF($B61="","",IFERROR(VLOOKUP($M61,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B61="","",IFERROR(VLOOKUP($M61,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T61" s="69">
@@ -11395,7 +11433,7 @@
         <v/>
       </c>
       <c r="S62" s="68">
-        <f>IF($B62="","",IFERROR(VLOOKUP($M62,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B62="","",IFERROR(VLOOKUP($M62,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T62" s="69">
@@ -11509,7 +11547,7 @@
         <v/>
       </c>
       <c r="S63" s="68">
-        <f>IF($B63="","",IFERROR(VLOOKUP($M63,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B63="","",IFERROR(VLOOKUP($M63,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T63" s="69">
@@ -11623,7 +11661,7 @@
         <v/>
       </c>
       <c r="S64" s="68">
-        <f>IF($B64="","",IFERROR(VLOOKUP($M64,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B64="","",IFERROR(VLOOKUP($M64,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T64" s="69">
@@ -11737,7 +11775,7 @@
         <v/>
       </c>
       <c r="S65" s="68">
-        <f>IF($B65="","",IFERROR(VLOOKUP($M65,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B65="","",IFERROR(VLOOKUP($M65,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T65" s="69">
@@ -11851,7 +11889,7 @@
         <v/>
       </c>
       <c r="S66" s="68">
-        <f>IF($B66="","",IFERROR(VLOOKUP($M66,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B66="","",IFERROR(VLOOKUP($M66,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T66" s="69">
@@ -11965,7 +12003,7 @@
         <v/>
       </c>
       <c r="S67" s="68">
-        <f>IF($B67="","",IFERROR(VLOOKUP($M67,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B67="","",IFERROR(VLOOKUP($M67,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T67" s="69">
@@ -12079,7 +12117,7 @@
         <v/>
       </c>
       <c r="S68" s="68">
-        <f>IF($B68="","",IFERROR(VLOOKUP($M68,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B68="","",IFERROR(VLOOKUP($M68,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T68" s="69">
@@ -12193,7 +12231,7 @@
         <v/>
       </c>
       <c r="S69" s="68">
-        <f>IF($B69="","",IFERROR(VLOOKUP($M69,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B69="","",IFERROR(VLOOKUP($M69,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T69" s="69">
@@ -12307,7 +12345,7 @@
         <v/>
       </c>
       <c r="S70" s="68">
-        <f>IF($B70="","",IFERROR(VLOOKUP($M70,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B70="","",IFERROR(VLOOKUP($M70,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T70" s="69">
@@ -12421,7 +12459,7 @@
         <v/>
       </c>
       <c r="S71" s="68">
-        <f>IF($B71="","",IFERROR(VLOOKUP($M71,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B71="","",IFERROR(VLOOKUP($M71,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T71" s="69">
@@ -12535,7 +12573,7 @@
         <v/>
       </c>
       <c r="S72" s="68">
-        <f>IF($B72="","",IFERROR(VLOOKUP($M72,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B72="","",IFERROR(VLOOKUP($M72,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T72" s="69">
@@ -12649,7 +12687,7 @@
         <v/>
       </c>
       <c r="S73" s="68">
-        <f>IF($B73="","",IFERROR(VLOOKUP($M73,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B73="","",IFERROR(VLOOKUP($M73,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T73" s="69">
@@ -12763,7 +12801,7 @@
         <v/>
       </c>
       <c r="S74" s="68">
-        <f>IF($B74="","",IFERROR(VLOOKUP($M74,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B74="","",IFERROR(VLOOKUP($M74,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T74" s="69">
@@ -12877,7 +12915,7 @@
         <v/>
       </c>
       <c r="S75" s="68">
-        <f>IF($B75="","",IFERROR(VLOOKUP($M75,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B75="","",IFERROR(VLOOKUP($M75,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T75" s="69">
@@ -12991,7 +13029,7 @@
         <v/>
       </c>
       <c r="S76" s="68">
-        <f>IF($B76="","",IFERROR(VLOOKUP($M76,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B76="","",IFERROR(VLOOKUP($M76,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T76" s="69">
@@ -13105,7 +13143,7 @@
         <v/>
       </c>
       <c r="S77" s="68">
-        <f>IF($B77="","",IFERROR(VLOOKUP($M77,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B77="","",IFERROR(VLOOKUP($M77,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T77" s="69">
@@ -13219,7 +13257,7 @@
         <v/>
       </c>
       <c r="S78" s="68">
-        <f>IF($B78="","",IFERROR(VLOOKUP($M78,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B78="","",IFERROR(VLOOKUP($M78,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T78" s="69">
@@ -13333,7 +13371,7 @@
         <v/>
       </c>
       <c r="S79" s="68">
-        <f>IF($B79="","",IFERROR(VLOOKUP($M79,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B79="","",IFERROR(VLOOKUP($M79,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T79" s="69">
@@ -13447,7 +13485,7 @@
         <v/>
       </c>
       <c r="S80" s="68">
-        <f>IF($B80="","",IFERROR(VLOOKUP($M80,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B80="","",IFERROR(VLOOKUP($M80,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T80" s="69">
@@ -13561,7 +13599,7 @@
         <v/>
       </c>
       <c r="S81" s="68">
-        <f>IF($B81="","",IFERROR(VLOOKUP($M81,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B81="","",IFERROR(VLOOKUP($M81,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T81" s="69">
@@ -13675,7 +13713,7 @@
         <v/>
       </c>
       <c r="S82" s="68">
-        <f>IF($B82="","",IFERROR(VLOOKUP($M82,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B82="","",IFERROR(VLOOKUP($M82,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T82" s="69">
@@ -13789,7 +13827,7 @@
         <v/>
       </c>
       <c r="S83" s="68">
-        <f>IF($B83="","",IFERROR(VLOOKUP($M83,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B83="","",IFERROR(VLOOKUP($M83,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T83" s="69">
@@ -13903,7 +13941,7 @@
         <v/>
       </c>
       <c r="S84" s="68">
-        <f>IF($B84="","",IFERROR(VLOOKUP($M84,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B84="","",IFERROR(VLOOKUP($M84,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T84" s="69">
@@ -14017,7 +14055,7 @@
         <v/>
       </c>
       <c r="S85" s="68">
-        <f>IF($B85="","",IFERROR(VLOOKUP($M85,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B85="","",IFERROR(VLOOKUP($M85,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T85" s="69">
@@ -14131,7 +14169,7 @@
         <v/>
       </c>
       <c r="S86" s="68">
-        <f>IF($B86="","",IFERROR(VLOOKUP($M86,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B86="","",IFERROR(VLOOKUP($M86,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T86" s="69">
@@ -14245,7 +14283,7 @@
         <v/>
       </c>
       <c r="S87" s="68">
-        <f>IF($B87="","",IFERROR(VLOOKUP($M87,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B87="","",IFERROR(VLOOKUP($M87,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T87" s="69">
@@ -14359,7 +14397,7 @@
         <v/>
       </c>
       <c r="S88" s="68">
-        <f>IF($B88="","",IFERROR(VLOOKUP($M88,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B88="","",IFERROR(VLOOKUP($M88,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T88" s="69">
@@ -14473,7 +14511,7 @@
         <v/>
       </c>
       <c r="S89" s="68">
-        <f>IF($B89="","",IFERROR(VLOOKUP($M89,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B89="","",IFERROR(VLOOKUP($M89,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T89" s="69">
@@ -14587,7 +14625,7 @@
         <v/>
       </c>
       <c r="S90" s="68">
-        <f>IF($B90="","",IFERROR(VLOOKUP($M90,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B90="","",IFERROR(VLOOKUP($M90,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T90" s="69">
@@ -14701,7 +14739,7 @@
         <v/>
       </c>
       <c r="S91" s="68">
-        <f>IF($B91="","",IFERROR(VLOOKUP($M91,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B91="","",IFERROR(VLOOKUP($M91,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T91" s="69">
@@ -14815,7 +14853,7 @@
         <v/>
       </c>
       <c r="S92" s="68">
-        <f>IF($B92="","",IFERROR(VLOOKUP($M92,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B92="","",IFERROR(VLOOKUP($M92,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T92" s="69">
@@ -14929,7 +14967,7 @@
         <v/>
       </c>
       <c r="S93" s="68">
-        <f>IF($B93="","",IFERROR(VLOOKUP($M93,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B93="","",IFERROR(VLOOKUP($M93,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T93" s="69">
@@ -15043,7 +15081,7 @@
         <v/>
       </c>
       <c r="S94" s="68">
-        <f>IF($B94="","",IFERROR(VLOOKUP($M94,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B94="","",IFERROR(VLOOKUP($M94,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T94" s="69">
@@ -15157,7 +15195,7 @@
         <v/>
       </c>
       <c r="S95" s="68">
-        <f>IF($B95="","",IFERROR(VLOOKUP($M95,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B95="","",IFERROR(VLOOKUP($M95,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T95" s="69">
@@ -15271,7 +15309,7 @@
         <v/>
       </c>
       <c r="S96" s="68">
-        <f>IF($B96="","",IFERROR(VLOOKUP($M96,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B96="","",IFERROR(VLOOKUP($M96,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T96" s="69">
@@ -15385,7 +15423,7 @@
         <v/>
       </c>
       <c r="S97" s="68">
-        <f>IF($B97="","",IFERROR(VLOOKUP($M97,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B97="","",IFERROR(VLOOKUP($M97,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T97" s="69">
@@ -15499,7 +15537,7 @@
         <v/>
       </c>
       <c r="S98" s="68">
-        <f>IF($B98="","",IFERROR(VLOOKUP($M98,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B98="","",IFERROR(VLOOKUP($M98,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T98" s="69">
@@ -15613,7 +15651,7 @@
         <v/>
       </c>
       <c r="S99" s="68">
-        <f>IF($B99="","",IFERROR(VLOOKUP($M99,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B99="","",IFERROR(VLOOKUP($M99,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T99" s="69">
@@ -15727,7 +15765,7 @@
         <v/>
       </c>
       <c r="S100" s="68">
-        <f>IF($B100="","",IFERROR(VLOOKUP($M100,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B100="","",IFERROR(VLOOKUP($M100,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T100" s="69">
@@ -15841,7 +15879,7 @@
         <v/>
       </c>
       <c r="S101" s="68">
-        <f>IF($B101="","",IFERROR(VLOOKUP($M101,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B101="","",IFERROR(VLOOKUP($M101,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T101" s="69">
@@ -15955,7 +15993,7 @@
         <v/>
       </c>
       <c r="S102" s="68">
-        <f>IF($B102="","",IFERROR(VLOOKUP($M102,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B102="","",IFERROR(VLOOKUP($M102,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T102" s="69">
@@ -16069,7 +16107,7 @@
         <v/>
       </c>
       <c r="S103" s="68">
-        <f>IF($B103="","",IFERROR(VLOOKUP($M103,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B103="","",IFERROR(VLOOKUP($M103,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T103" s="69">
@@ -16183,7 +16221,7 @@
         <v/>
       </c>
       <c r="S104" s="68">
-        <f>IF($B104="","",IFERROR(VLOOKUP($M104,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B104="","",IFERROR(VLOOKUP($M104,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T104" s="69">
@@ -16297,7 +16335,7 @@
         <v/>
       </c>
       <c r="S105" s="68">
-        <f>IF($B105="","",IFERROR(VLOOKUP($M105,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B105="","",IFERROR(VLOOKUP($M105,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T105" s="69">
@@ -16411,7 +16449,7 @@
         <v/>
       </c>
       <c r="S106" s="68">
-        <f>IF($B106="","",IFERROR(VLOOKUP($M106,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B106="","",IFERROR(VLOOKUP($M106,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T106" s="69">
@@ -16525,7 +16563,7 @@
         <v/>
       </c>
       <c r="S107" s="68">
-        <f>IF($B107="","",IFERROR(VLOOKUP($M107,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B107="","",IFERROR(VLOOKUP($M107,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T107" s="69">
@@ -16639,7 +16677,7 @@
         <v/>
       </c>
       <c r="S108" s="68">
-        <f>IF($B108="","",IFERROR(VLOOKUP($M108,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B108="","",IFERROR(VLOOKUP($M108,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T108" s="69">
@@ -16753,7 +16791,7 @@
         <v/>
       </c>
       <c r="S109" s="68">
-        <f>IF($B109="","",IFERROR(VLOOKUP($M109,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B109="","",IFERROR(VLOOKUP($M109,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T109" s="69">
@@ -16867,7 +16905,7 @@
         <v/>
       </c>
       <c r="S110" s="68">
-        <f>IF($B110="","",IFERROR(VLOOKUP($M110,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B110="","",IFERROR(VLOOKUP($M110,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T110" s="69">
@@ -16981,7 +17019,7 @@
         <v/>
       </c>
       <c r="S111" s="68">
-        <f>IF($B111="","",IFERROR(VLOOKUP($M111,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B111="","",IFERROR(VLOOKUP($M111,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T111" s="69">
@@ -17095,7 +17133,7 @@
         <v/>
       </c>
       <c r="S112" s="68">
-        <f>IF($B112="","",IFERROR(VLOOKUP($M112,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B112="","",IFERROR(VLOOKUP($M112,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T112" s="69">
@@ -17209,7 +17247,7 @@
         <v/>
       </c>
       <c r="S113" s="68">
-        <f>IF($B113="","",IFERROR(VLOOKUP($M113,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B113="","",IFERROR(VLOOKUP($M113,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T113" s="69">
@@ -17323,7 +17361,7 @@
         <v/>
       </c>
       <c r="S114" s="68">
-        <f>IF($B114="","",IFERROR(VLOOKUP($M114,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B114="","",IFERROR(VLOOKUP($M114,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T114" s="69">
@@ -17437,7 +17475,7 @@
         <v/>
       </c>
       <c r="S115" s="68">
-        <f>IF($B115="","",IFERROR(VLOOKUP($M115,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B115="","",IFERROR(VLOOKUP($M115,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T115" s="69">
@@ -17551,7 +17589,7 @@
         <v/>
       </c>
       <c r="S116" s="68">
-        <f>IF($B116="","",IFERROR(VLOOKUP($M116,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B116="","",IFERROR(VLOOKUP($M116,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T116" s="69">
@@ -17665,7 +17703,7 @@
         <v/>
       </c>
       <c r="S117" s="68">
-        <f>IF($B117="","",IFERROR(VLOOKUP($M117,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B117="","",IFERROR(VLOOKUP($M117,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T117" s="69">
@@ -17779,7 +17817,7 @@
         <v/>
       </c>
       <c r="S118" s="68">
-        <f>IF($B118="","",IFERROR(VLOOKUP($M118,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B118="","",IFERROR(VLOOKUP($M118,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T118" s="69">
@@ -17893,7 +17931,7 @@
         <v/>
       </c>
       <c r="S119" s="68">
-        <f>IF($B119="","",IFERROR(VLOOKUP($M119,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B119="","",IFERROR(VLOOKUP($M119,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T119" s="69">
@@ -18007,7 +18045,7 @@
         <v/>
       </c>
       <c r="S120" s="68">
-        <f>IF($B120="","",IFERROR(VLOOKUP($M120,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B120="","",IFERROR(VLOOKUP($M120,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T120" s="69">
@@ -18121,7 +18159,7 @@
         <v/>
       </c>
       <c r="S121" s="68">
-        <f>IF($B121="","",IFERROR(VLOOKUP($M121,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B121="","",IFERROR(VLOOKUP($M121,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T121" s="69">
@@ -18235,7 +18273,7 @@
         <v/>
       </c>
       <c r="S122" s="68">
-        <f>IF($B122="","",IFERROR(VLOOKUP($M122,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B122="","",IFERROR(VLOOKUP($M122,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T122" s="69">
@@ -18349,7 +18387,7 @@
         <v/>
       </c>
       <c r="S123" s="68">
-        <f>IF($B123="","",IFERROR(VLOOKUP($M123,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B123="","",IFERROR(VLOOKUP($M123,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T123" s="69">
@@ -18463,7 +18501,7 @@
         <v/>
       </c>
       <c r="S124" s="68">
-        <f>IF($B124="","",IFERROR(VLOOKUP($M124,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B124="","",IFERROR(VLOOKUP($M124,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T124" s="69">
@@ -18577,7 +18615,7 @@
         <v/>
       </c>
       <c r="S125" s="68">
-        <f>IF($B125="","",IFERROR(VLOOKUP($M125,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B125="","",IFERROR(VLOOKUP($M125,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T125" s="69">
@@ -18691,7 +18729,7 @@
         <v/>
       </c>
       <c r="S126" s="68">
-        <f>IF($B126="","",IFERROR(VLOOKUP($M126,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B126="","",IFERROR(VLOOKUP($M126,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T126" s="69">
@@ -18805,7 +18843,7 @@
         <v/>
       </c>
       <c r="S127" s="68">
-        <f>IF($B127="","",IFERROR(VLOOKUP($M127,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B127="","",IFERROR(VLOOKUP($M127,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T127" s="69">
@@ -18919,7 +18957,7 @@
         <v/>
       </c>
       <c r="S128" s="68">
-        <f>IF($B128="","",IFERROR(VLOOKUP($M128,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B128="","",IFERROR(VLOOKUP($M128,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T128" s="69">
@@ -19033,7 +19071,7 @@
         <v/>
       </c>
       <c r="S129" s="68">
-        <f>IF($B129="","",IFERROR(VLOOKUP($M129,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B129="","",IFERROR(VLOOKUP($M129,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T129" s="69">
@@ -19147,7 +19185,7 @@
         <v/>
       </c>
       <c r="S130" s="68">
-        <f>IF($B130="","",IFERROR(VLOOKUP($M130,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B130="","",IFERROR(VLOOKUP($M130,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T130" s="69">
@@ -19261,7 +19299,7 @@
         <v/>
       </c>
       <c r="S131" s="68">
-        <f>IF($B131="","",IFERROR(VLOOKUP($M131,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B131="","",IFERROR(VLOOKUP($M131,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T131" s="69">
@@ -19375,7 +19413,7 @@
         <v/>
       </c>
       <c r="S132" s="68">
-        <f>IF($B132="","",IFERROR(VLOOKUP($M132,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B132="","",IFERROR(VLOOKUP($M132,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T132" s="69">
@@ -19489,7 +19527,7 @@
         <v/>
       </c>
       <c r="S133" s="68">
-        <f>IF($B133="","",IFERROR(VLOOKUP($M133,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B133="","",IFERROR(VLOOKUP($M133,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T133" s="69">
@@ -19603,7 +19641,7 @@
         <v/>
       </c>
       <c r="S134" s="68">
-        <f>IF($B134="","",IFERROR(VLOOKUP($M134,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B134="","",IFERROR(VLOOKUP($M134,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T134" s="69">
@@ -19717,7 +19755,7 @@
         <v/>
       </c>
       <c r="S135" s="68">
-        <f>IF($B135="","",IFERROR(VLOOKUP($M135,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B135="","",IFERROR(VLOOKUP($M135,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T135" s="69">
@@ -19831,7 +19869,7 @@
         <v/>
       </c>
       <c r="S136" s="68">
-        <f>IF($B136="","",IFERROR(VLOOKUP($M136,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B136="","",IFERROR(VLOOKUP($M136,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T136" s="69">
@@ -19945,7 +19983,7 @@
         <v/>
       </c>
       <c r="S137" s="68">
-        <f>IF($B137="","",IFERROR(VLOOKUP($M137,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B137="","",IFERROR(VLOOKUP($M137,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T137" s="69">
@@ -20059,7 +20097,7 @@
         <v/>
       </c>
       <c r="S138" s="68">
-        <f>IF($B138="","",IFERROR(VLOOKUP($M138,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B138="","",IFERROR(VLOOKUP($M138,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T138" s="69">
@@ -20173,7 +20211,7 @@
         <v/>
       </c>
       <c r="S139" s="68">
-        <f>IF($B139="","",IFERROR(VLOOKUP($M139,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B139="","",IFERROR(VLOOKUP($M139,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T139" s="69">
@@ -20287,7 +20325,7 @@
         <v/>
       </c>
       <c r="S140" s="68">
-        <f>IF($B140="","",IFERROR(VLOOKUP($M140,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B140="","",IFERROR(VLOOKUP($M140,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T140" s="69">
@@ -20401,7 +20439,7 @@
         <v/>
       </c>
       <c r="S141" s="68">
-        <f>IF($B141="","",IFERROR(VLOOKUP($M141,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B141="","",IFERROR(VLOOKUP($M141,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T141" s="69">
@@ -20515,7 +20553,7 @@
         <v/>
       </c>
       <c r="S142" s="68">
-        <f>IF($B142="","",IFERROR(VLOOKUP($M142,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B142="","",IFERROR(VLOOKUP($M142,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T142" s="69">
@@ -20629,7 +20667,7 @@
         <v/>
       </c>
       <c r="S143" s="68">
-        <f>IF($B143="","",IFERROR(VLOOKUP($M143,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B143="","",IFERROR(VLOOKUP($M143,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T143" s="69">
@@ -20743,7 +20781,7 @@
         <v/>
       </c>
       <c r="S144" s="68">
-        <f>IF($B144="","",IFERROR(VLOOKUP($M144,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B144="","",IFERROR(VLOOKUP($M144,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T144" s="69">
@@ -20857,7 +20895,7 @@
         <v/>
       </c>
       <c r="S145" s="68">
-        <f>IF($B145="","",IFERROR(VLOOKUP($M145,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B145="","",IFERROR(VLOOKUP($M145,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T145" s="69">
@@ -20971,7 +21009,7 @@
         <v/>
       </c>
       <c r="S146" s="68">
-        <f>IF($B146="","",IFERROR(VLOOKUP($M146,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B146="","",IFERROR(VLOOKUP($M146,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T146" s="69">
@@ -21085,7 +21123,7 @@
         <v/>
       </c>
       <c r="S147" s="68">
-        <f>IF($B147="","",IFERROR(VLOOKUP($M147,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B147="","",IFERROR(VLOOKUP($M147,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T147" s="69">
@@ -21199,7 +21237,7 @@
         <v/>
       </c>
       <c r="S148" s="68">
-        <f>IF($B148="","",IFERROR(VLOOKUP($M148,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B148="","",IFERROR(VLOOKUP($M148,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T148" s="69">
@@ -21313,7 +21351,7 @@
         <v/>
       </c>
       <c r="S149" s="68">
-        <f>IF($B149="","",IFERROR(VLOOKUP($M149,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B149="","",IFERROR(VLOOKUP($M149,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T149" s="69">
@@ -21427,7 +21465,7 @@
         <v/>
       </c>
       <c r="S150" s="68">
-        <f>IF($B150="","",IFERROR(VLOOKUP($M150,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B150="","",IFERROR(VLOOKUP($M150,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T150" s="69">
@@ -21541,7 +21579,7 @@
         <v/>
       </c>
       <c r="S151" s="68">
-        <f>IF($B151="","",IFERROR(VLOOKUP($M151,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B151="","",IFERROR(VLOOKUP($M151,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T151" s="69">
@@ -21655,7 +21693,7 @@
         <v/>
       </c>
       <c r="S152" s="68">
-        <f>IF($B152="","",IFERROR(VLOOKUP($M152,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B152="","",IFERROR(VLOOKUP($M152,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T152" s="69">
@@ -21769,7 +21807,7 @@
         <v/>
       </c>
       <c r="S153" s="68">
-        <f>IF($B153="","",IFERROR(VLOOKUP($M153,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B153="","",IFERROR(VLOOKUP($M153,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T153" s="69">
@@ -21883,7 +21921,7 @@
         <v/>
       </c>
       <c r="S154" s="68">
-        <f>IF($B154="","",IFERROR(VLOOKUP($M154,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B154="","",IFERROR(VLOOKUP($M154,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T154" s="69">
@@ -21997,7 +22035,7 @@
         <v/>
       </c>
       <c r="S155" s="68">
-        <f>IF($B155="","",IFERROR(VLOOKUP($M155,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B155="","",IFERROR(VLOOKUP($M155,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T155" s="69">
@@ -22111,7 +22149,7 @@
         <v/>
       </c>
       <c r="S156" s="68">
-        <f>IF($B156="","",IFERROR(VLOOKUP($M156,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B156="","",IFERROR(VLOOKUP($M156,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T156" s="69">
@@ -22225,7 +22263,7 @@
         <v/>
       </c>
       <c r="S157" s="68">
-        <f>IF($B157="","",IFERROR(VLOOKUP($M157,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B157="","",IFERROR(VLOOKUP($M157,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T157" s="69">
@@ -22339,7 +22377,7 @@
         <v/>
       </c>
       <c r="S158" s="68">
-        <f>IF($B158="","",IFERROR(VLOOKUP($M158,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B158="","",IFERROR(VLOOKUP($M158,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T158" s="69">
@@ -22453,7 +22491,7 @@
         <v/>
       </c>
       <c r="S159" s="68">
-        <f>IF($B159="","",IFERROR(VLOOKUP($M159,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B159="","",IFERROR(VLOOKUP($M159,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T159" s="69">
@@ -22567,7 +22605,7 @@
         <v/>
       </c>
       <c r="S160" s="68">
-        <f>IF($B160="","",IFERROR(VLOOKUP($M160,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B160="","",IFERROR(VLOOKUP($M160,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T160" s="69">
@@ -22681,7 +22719,7 @@
         <v/>
       </c>
       <c r="S161" s="68">
-        <f>IF($B161="","",IFERROR(VLOOKUP($M161,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B161="","",IFERROR(VLOOKUP($M161,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T161" s="69">
@@ -22795,7 +22833,7 @@
         <v/>
       </c>
       <c r="S162" s="68">
-        <f>IF($B162="","",IFERROR(VLOOKUP($M162,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B162="","",IFERROR(VLOOKUP($M162,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T162" s="69">
@@ -22909,7 +22947,7 @@
         <v/>
       </c>
       <c r="S163" s="68">
-        <f>IF($B163="","",IFERROR(VLOOKUP($M163,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B163="","",IFERROR(VLOOKUP($M163,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T163" s="69">
@@ -23023,7 +23061,7 @@
         <v/>
       </c>
       <c r="S164" s="68">
-        <f>IF($B164="","",IFERROR(VLOOKUP($M164,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B164="","",IFERROR(VLOOKUP($M164,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T164" s="69">
@@ -23137,7 +23175,7 @@
         <v/>
       </c>
       <c r="S165" s="68">
-        <f>IF($B165="","",IFERROR(VLOOKUP($M165,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B165="","",IFERROR(VLOOKUP($M165,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T165" s="69">
@@ -23251,7 +23289,7 @@
         <v/>
       </c>
       <c r="S166" s="68">
-        <f>IF($B166="","",IFERROR(VLOOKUP($M166,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B166="","",IFERROR(VLOOKUP($M166,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T166" s="69">
@@ -23365,7 +23403,7 @@
         <v/>
       </c>
       <c r="S167" s="68">
-        <f>IF($B167="","",IFERROR(VLOOKUP($M167,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B167="","",IFERROR(VLOOKUP($M167,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T167" s="69">
@@ -23479,7 +23517,7 @@
         <v/>
       </c>
       <c r="S168" s="68">
-        <f>IF($B168="","",IFERROR(VLOOKUP($M168,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B168="","",IFERROR(VLOOKUP($M168,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T168" s="69">
@@ -23593,7 +23631,7 @@
         <v/>
       </c>
       <c r="S169" s="68">
-        <f>IF($B169="","",IFERROR(VLOOKUP($M169,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B169="","",IFERROR(VLOOKUP($M169,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T169" s="69">
@@ -23707,7 +23745,7 @@
         <v/>
       </c>
       <c r="S170" s="68">
-        <f>IF($B170="","",IFERROR(VLOOKUP($M170,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B170="","",IFERROR(VLOOKUP($M170,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T170" s="69">
@@ -23821,7 +23859,7 @@
         <v/>
       </c>
       <c r="S171" s="68">
-        <f>IF($B171="","",IFERROR(VLOOKUP($M171,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B171="","",IFERROR(VLOOKUP($M171,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T171" s="69">
@@ -23935,7 +23973,7 @@
         <v/>
       </c>
       <c r="S172" s="68">
-        <f>IF($B172="","",IFERROR(VLOOKUP($M172,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B172="","",IFERROR(VLOOKUP($M172,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T172" s="69">
@@ -24049,7 +24087,7 @@
         <v/>
       </c>
       <c r="S173" s="68">
-        <f>IF($B173="","",IFERROR(VLOOKUP($M173,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B173="","",IFERROR(VLOOKUP($M173,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T173" s="69">
@@ -24163,7 +24201,7 @@
         <v/>
       </c>
       <c r="S174" s="68">
-        <f>IF($B174="","",IFERROR(VLOOKUP($M174,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B174="","",IFERROR(VLOOKUP($M174,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T174" s="69">
@@ -24277,7 +24315,7 @@
         <v/>
       </c>
       <c r="S175" s="68">
-        <f>IF($B175="","",IFERROR(VLOOKUP($M175,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B175="","",IFERROR(VLOOKUP($M175,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T175" s="69">
@@ -24391,7 +24429,7 @@
         <v/>
       </c>
       <c r="S176" s="68">
-        <f>IF($B176="","",IFERROR(VLOOKUP($M176,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B176="","",IFERROR(VLOOKUP($M176,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T176" s="69">
@@ -24505,7 +24543,7 @@
         <v/>
       </c>
       <c r="S177" s="68">
-        <f>IF($B177="","",IFERROR(VLOOKUP($M177,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B177="","",IFERROR(VLOOKUP($M177,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T177" s="69">
@@ -24619,7 +24657,7 @@
         <v/>
       </c>
       <c r="S178" s="68">
-        <f>IF($B178="","",IFERROR(VLOOKUP($M178,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B178="","",IFERROR(VLOOKUP($M178,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T178" s="69">
@@ -24733,7 +24771,7 @@
         <v/>
       </c>
       <c r="S179" s="68">
-        <f>IF($B179="","",IFERROR(VLOOKUP($M179,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B179="","",IFERROR(VLOOKUP($M179,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T179" s="69">
@@ -24847,7 +24885,7 @@
         <v/>
       </c>
       <c r="S180" s="68">
-        <f>IF($B180="","",IFERROR(VLOOKUP($M180,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B180="","",IFERROR(VLOOKUP($M180,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T180" s="69">
@@ -24961,7 +24999,7 @@
         <v/>
       </c>
       <c r="S181" s="68">
-        <f>IF($B181="","",IFERROR(VLOOKUP($M181,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B181="","",IFERROR(VLOOKUP($M181,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T181" s="69">
@@ -25075,7 +25113,7 @@
         <v/>
       </c>
       <c r="S182" s="68">
-        <f>IF($B182="","",IFERROR(VLOOKUP($M182,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B182="","",IFERROR(VLOOKUP($M182,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T182" s="69">
@@ -25189,7 +25227,7 @@
         <v/>
       </c>
       <c r="S183" s="68">
-        <f>IF($B183="","",IFERROR(VLOOKUP($M183,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B183="","",IFERROR(VLOOKUP($M183,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T183" s="69">
@@ -25303,7 +25341,7 @@
         <v/>
       </c>
       <c r="S184" s="68">
-        <f>IF($B184="","",IFERROR(VLOOKUP($M184,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B184="","",IFERROR(VLOOKUP($M184,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T184" s="69">
@@ -25417,7 +25455,7 @@
         <v/>
       </c>
       <c r="S185" s="68">
-        <f>IF($B185="","",IFERROR(VLOOKUP($M185,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B185="","",IFERROR(VLOOKUP($M185,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T185" s="69">
@@ -25531,7 +25569,7 @@
         <v/>
       </c>
       <c r="S186" s="68">
-        <f>IF($B186="","",IFERROR(VLOOKUP($M186,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B186="","",IFERROR(VLOOKUP($M186,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T186" s="69">
@@ -25645,7 +25683,7 @@
         <v/>
       </c>
       <c r="S187" s="68">
-        <f>IF($B187="","",IFERROR(VLOOKUP($M187,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B187="","",IFERROR(VLOOKUP($M187,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T187" s="69">
@@ -25759,7 +25797,7 @@
         <v/>
       </c>
       <c r="S188" s="68">
-        <f>IF($B188="","",IFERROR(VLOOKUP($M188,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B188="","",IFERROR(VLOOKUP($M188,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T188" s="69">
@@ -25873,7 +25911,7 @@
         <v/>
       </c>
       <c r="S189" s="68">
-        <f>IF($B189="","",IFERROR(VLOOKUP($M189,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B189="","",IFERROR(VLOOKUP($M189,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T189" s="69">
@@ -25987,7 +26025,7 @@
         <v/>
       </c>
       <c r="S190" s="68">
-        <f>IF($B190="","",IFERROR(VLOOKUP($M190,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B190="","",IFERROR(VLOOKUP($M190,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T190" s="69">
@@ -26101,7 +26139,7 @@
         <v/>
       </c>
       <c r="S191" s="68">
-        <f>IF($B191="","",IFERROR(VLOOKUP($M191,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B191="","",IFERROR(VLOOKUP($M191,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T191" s="69">
@@ -26215,7 +26253,7 @@
         <v/>
       </c>
       <c r="S192" s="68">
-        <f>IF($B192="","",IFERROR(VLOOKUP($M192,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B192="","",IFERROR(VLOOKUP($M192,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T192" s="69">
@@ -26329,7 +26367,7 @@
         <v/>
       </c>
       <c r="S193" s="68">
-        <f>IF($B193="","",IFERROR(VLOOKUP($M193,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B193="","",IFERROR(VLOOKUP($M193,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T193" s="69">
@@ -26443,7 +26481,7 @@
         <v/>
       </c>
       <c r="S194" s="68">
-        <f>IF($B194="","",IFERROR(VLOOKUP($M194,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B194="","",IFERROR(VLOOKUP($M194,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T194" s="69">
@@ -26557,7 +26595,7 @@
         <v/>
       </c>
       <c r="S195" s="68">
-        <f>IF($B195="","",IFERROR(VLOOKUP($M195,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B195="","",IFERROR(VLOOKUP($M195,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T195" s="69">
@@ -26671,7 +26709,7 @@
         <v/>
       </c>
       <c r="S196" s="68">
-        <f>IF($B196="","",IFERROR(VLOOKUP($M196,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B196="","",IFERROR(VLOOKUP($M196,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T196" s="69">
@@ -26785,7 +26823,7 @@
         <v/>
       </c>
       <c r="S197" s="68">
-        <f>IF($B197="","",IFERROR(VLOOKUP($M197,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B197="","",IFERROR(VLOOKUP($M197,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T197" s="69">
@@ -26899,7 +26937,7 @@
         <v/>
       </c>
       <c r="S198" s="68">
-        <f>IF($B198="","",IFERROR(VLOOKUP($M198,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B198="","",IFERROR(VLOOKUP($M198,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T198" s="69">
@@ -27013,7 +27051,7 @@
         <v/>
       </c>
       <c r="S199" s="68">
-        <f>IF($B199="","",IFERROR(VLOOKUP($M199,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B199="","",IFERROR(VLOOKUP($M199,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T199" s="69">
@@ -27127,7 +27165,7 @@
         <v/>
       </c>
       <c r="S200" s="68">
-        <f>IF($B200="","",IFERROR(VLOOKUP($M200,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B200="","",IFERROR(VLOOKUP($M200,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T200" s="69">
@@ -27241,7 +27279,7 @@
         <v/>
       </c>
       <c r="S201" s="68">
-        <f>IF($B201="","",IFERROR(VLOOKUP($M201,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B201="","",IFERROR(VLOOKUP($M201,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T201" s="69">
@@ -27355,7 +27393,7 @@
         <v/>
       </c>
       <c r="S202" s="68">
-        <f>IF($B202="","",IFERROR(VLOOKUP($M202,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B202="","",IFERROR(VLOOKUP($M202,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T202" s="69">
@@ -27469,7 +27507,7 @@
         <v/>
       </c>
       <c r="S203" s="68">
-        <f>IF($B203="","",IFERROR(VLOOKUP($M203,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B203="","",IFERROR(VLOOKUP($M203,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T203" s="69">
@@ -27583,7 +27621,7 @@
         <v/>
       </c>
       <c r="S204" s="68">
-        <f>IF($B204="","",IFERROR(VLOOKUP($M204,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B204="","",IFERROR(VLOOKUP($M204,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T204" s="69">
@@ -27697,7 +27735,7 @@
         <v/>
       </c>
       <c r="S205" s="68">
-        <f>IF($B205="","",IFERROR(VLOOKUP($M205,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B205="","",IFERROR(VLOOKUP($M205,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T205" s="69">
@@ -27811,7 +27849,7 @@
         <v/>
       </c>
       <c r="S206" s="68">
-        <f>IF($B206="","",IFERROR(VLOOKUP($M206,'Konstanten'!$H$6:$I$10,2,FALSE),29))</f>
+        <f>IF($B206="","",IFERROR(VLOOKUP($M206,'Konstanten'!$E$6:$F$10,2,FALSE),29))</f>
         <v/>
       </c>
       <c r="T206" s="69">
@@ -27900,12 +27938,12 @@
       <formula>AND($R7&lt;&gt;"",$R7&lt;=$S7)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U7:U206">
+  <conditionalFormatting sqref="T7:T206">
     <cfRule type="expression" priority="3" dxfId="0">
-      <formula>AND($U7&lt;&gt;"",$U7&lt;0)</formula>
+      <formula>AND($T7&lt;&gt;"",$F7&lt;&gt;"",$T7&lt;$F7)</formula>
     </cfRule>
     <cfRule type="expression" priority="4" dxfId="1">
-      <formula>AND($U7&lt;&gt;"",$U7&gt;=0)</formula>
+      <formula>AND($T7&lt;&gt;"",$F7&lt;&gt;"",$T7&gt;=$F7)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V7:V206">
@@ -27955,13 +27993,13 @@
   </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation sqref="M7:M206" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>='Konstanten'!$H$6:$H$10</formula1>
+      <formula1>='Konstanten'!$E$6:$E$10</formula1>
     </dataValidation>
     <dataValidation sqref="I7:I206" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>='Konstanten'!$E$6:$E$13</formula1>
+      <formula1>='Konstanten'!$H$6:$H$19</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageMargins left="0.2" right="0.2" top="0.3" bottom="0.3" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
@@ -28448,14 +28486,14 @@
   <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -32028,18 +32066,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="2" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="2" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -32055,7 +32093,6 @@
       <c r="F1" s="2" t="n"/>
       <c r="G1" s="2" t="n"/>
       <c r="H1" s="2" t="n"/>
-      <c r="I1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n"/>
@@ -32066,7 +32103,6 @@
       <c r="F2" s="2" t="n"/>
       <c r="G2" s="2" t="n"/>
       <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="30" t="inlineStr">
@@ -32081,7 +32117,6 @@
       <c r="F3" s="2" t="n"/>
       <c r="G3" s="2" t="n"/>
       <c r="H3" s="2" t="n"/>
-      <c r="I3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="103" t="inlineStr">
@@ -32092,13 +32127,12 @@
       <c r="C4" s="2" t="n"/>
       <c r="D4" s="103" t="inlineStr">
         <is>
+          <t>Zonen / max. Oberflächentemp.</t>
+        </is>
+      </c>
+      <c r="G4" s="103" t="inlineStr">
+        <is>
           <t>R-Werte Bodenbeläge</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="n"/>
-      <c r="G4" s="103" t="inlineStr">
-        <is>
-          <t>Zonen / max. Oberflächentemp.</t>
         </is>
       </c>
     </row>
@@ -32116,28 +32150,27 @@
       <c r="C5" s="2" t="n"/>
       <c r="D5" s="104" t="inlineStr">
         <is>
+          <t>Zone</t>
+        </is>
+      </c>
+      <c r="E5" s="104" t="inlineStr">
+        <is>
+          <t>Kürzel</t>
+        </is>
+      </c>
+      <c r="F5" s="104" t="inlineStr">
+        <is>
+          <t>θF,max [°C]</t>
+        </is>
+      </c>
+      <c r="G5" s="104" t="inlineStr">
+        <is>
           <t>Bodenbelag</t>
         </is>
       </c>
-      <c r="E5" s="104" t="inlineStr">
+      <c r="H5" s="104" t="inlineStr">
         <is>
           <t>R [m²·K/W]</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="n"/>
-      <c r="G5" s="104" t="inlineStr">
-        <is>
-          <t>Zone</t>
-        </is>
-      </c>
-      <c r="H5" s="104" t="inlineStr">
-        <is>
-          <t>Kürzel</t>
-        </is>
-      </c>
-      <c r="I5" s="104" t="inlineStr">
-        <is>
-          <t>θF,max [°C]</t>
         </is>
       </c>
     </row>
@@ -32151,25 +32184,24 @@
       <c r="C6" s="2" t="n"/>
       <c r="D6" s="55" t="inlineStr">
         <is>
-          <t>Fliesen / Naturstein</t>
-        </is>
-      </c>
-      <c r="E6" s="60" t="n">
+          <t>Aufenthaltszone</t>
+        </is>
+      </c>
+      <c r="E6" s="55" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="F6" s="105" t="n">
+        <v>29</v>
+      </c>
+      <c r="G6" s="55" t="inlineStr">
+        <is>
+          <t>Keramik / Feinsteinzeug</t>
+        </is>
+      </c>
+      <c r="H6" s="60" t="n">
         <v>0.01</v>
-      </c>
-      <c r="F6" s="2" t="n"/>
-      <c r="G6" s="55" t="inlineStr">
-        <is>
-          <t>Aufenthaltszone</t>
-        </is>
-      </c>
-      <c r="H6" s="55" t="inlineStr">
-        <is>
-          <t>AZ</t>
-        </is>
-      </c>
-      <c r="I6" s="105" t="n">
-        <v>29</v>
       </c>
     </row>
     <row r="7">
@@ -32182,25 +32214,24 @@
       <c r="C7" s="2" t="n"/>
       <c r="D7" s="55" t="inlineStr">
         <is>
-          <t>Linoleum / PVC</t>
-        </is>
-      </c>
-      <c r="E7" s="60" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="F7" s="2" t="n"/>
+          <t>Randzone</t>
+        </is>
+      </c>
+      <c r="E7" s="55" t="inlineStr">
+        <is>
+          <t>RZ</t>
+        </is>
+      </c>
+      <c r="F7" s="105" t="n">
+        <v>35</v>
+      </c>
       <c r="G7" s="55" t="inlineStr">
         <is>
-          <t>Randzone</t>
-        </is>
-      </c>
-      <c r="H7" s="55" t="inlineStr">
-        <is>
-          <t>RZ</t>
-        </is>
-      </c>
-      <c r="I7" s="105" t="n">
-        <v>35</v>
+          <t>Naturstein / Marmor</t>
+        </is>
+      </c>
+      <c r="H7" s="60" t="n">
+        <v>0.015</v>
       </c>
     </row>
     <row r="8">
@@ -32213,25 +32244,24 @@
       <c r="C8" s="2" t="n"/>
       <c r="D8" s="55" t="inlineStr">
         <is>
-          <t>Parkett / Laminat</t>
-        </is>
-      </c>
-      <c r="E8" s="60" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F8" s="2" t="n"/>
+          <t>Badezimmer</t>
+        </is>
+      </c>
+      <c r="E8" s="55" t="inlineStr">
+        <is>
+          <t>BAD</t>
+        </is>
+      </c>
+      <c r="F8" s="105" t="n">
+        <v>33</v>
+      </c>
       <c r="G8" s="55" t="inlineStr">
         <is>
-          <t>Badezimmer</t>
-        </is>
-      </c>
-      <c r="H8" s="55" t="inlineStr">
-        <is>
-          <t>BAD</t>
-        </is>
-      </c>
-      <c r="I8" s="105" t="n">
-        <v>33</v>
+          <t>PVC / Vinyl (verklebt)</t>
+        </is>
+      </c>
+      <c r="H8" s="60" t="n">
+        <v>0.02</v>
       </c>
     </row>
     <row r="9">
@@ -32242,18 +32272,17 @@
         <v>0.97</v>
       </c>
       <c r="C9" s="2" t="n"/>
-      <c r="D9" s="55" t="inlineStr">
-        <is>
-          <t>Holzdielen</t>
-        </is>
-      </c>
-      <c r="E9" s="60" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F9" s="2" t="n"/>
-      <c r="G9" s="55" t="n"/>
-      <c r="H9" s="55" t="n"/>
-      <c r="I9" s="105" t="n"/>
+      <c r="D9" s="55" t="n"/>
+      <c r="E9" s="55" t="n"/>
+      <c r="F9" s="105" t="n"/>
+      <c r="G9" s="55" t="inlineStr">
+        <is>
+          <t>Designboden (Klick)</t>
+        </is>
+      </c>
+      <c r="H9" s="60" t="n">
+        <v>0.04</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="64" t="n">
@@ -32263,18 +32292,17 @@
         <v>0.93</v>
       </c>
       <c r="C10" s="2" t="n"/>
-      <c r="D10" s="55" t="inlineStr">
-        <is>
-          <t>Teppich</t>
-        </is>
-      </c>
-      <c r="E10" s="60" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="F10" s="2" t="n"/>
-      <c r="G10" s="55" t="n"/>
-      <c r="H10" s="55" t="n"/>
-      <c r="I10" s="105" t="n"/>
+      <c r="D10" s="55" t="n"/>
+      <c r="E10" s="55" t="n"/>
+      <c r="F10" s="105" t="n"/>
+      <c r="G10" s="55" t="inlineStr">
+        <is>
+          <t>Linoleum 2,5 mm</t>
+        </is>
+      </c>
+      <c r="H10" s="60" t="n">
+        <v>0.05</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="64" t="n">
@@ -32284,12 +32312,17 @@
         <v>0.85</v>
       </c>
       <c r="C11" s="2" t="n"/>
-      <c r="D11" s="55" t="n"/>
-      <c r="E11" s="60" t="n"/>
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="2" t="n"/>
       <c r="F11" s="2" t="n"/>
-      <c r="G11" s="2" t="n"/>
-      <c r="H11" s="2" t="n"/>
-      <c r="I11" s="2" t="n"/>
+      <c r="G11" s="55" t="inlineStr">
+        <is>
+          <t>Laminat + Trittschall</t>
+        </is>
+      </c>
+      <c r="H11" s="60" t="n">
+        <v>0.06</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="64" t="n">
@@ -32299,12 +32332,17 @@
         <v>0.78</v>
       </c>
       <c r="C12" s="2" t="n"/>
-      <c r="D12" s="55" t="n"/>
-      <c r="E12" s="60" t="n"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n"/>
       <c r="F12" s="2" t="n"/>
-      <c r="G12" s="2" t="n"/>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="n"/>
+      <c r="G12" s="55" t="inlineStr">
+        <is>
+          <t>Parkett / Fertigparkett</t>
+        </is>
+      </c>
+      <c r="H12" s="60" t="n">
+        <v>0.075</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="64" t="n">
@@ -32314,12 +32352,17 @@
         <v>0.72</v>
       </c>
       <c r="C13" s="2" t="n"/>
-      <c r="D13" s="55" t="n"/>
-      <c r="E13" s="60" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
       <c r="F13" s="2" t="n"/>
-      <c r="G13" s="2" t="n"/>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="n"/>
+      <c r="G13" s="55" t="inlineStr">
+        <is>
+          <t>Kork</t>
+        </is>
+      </c>
+      <c r="H13" s="60" t="n">
+        <v>0.1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n"/>
@@ -32328,9 +32371,14 @@
       <c r="D14" s="2" t="n"/>
       <c r="E14" s="2" t="n"/>
       <c r="F14" s="2" t="n"/>
-      <c r="G14" s="2" t="n"/>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="n"/>
+      <c r="G14" s="55" t="inlineStr">
+        <is>
+          <t>Holzdielen</t>
+        </is>
+      </c>
+      <c r="H14" s="60" t="n">
+        <v>0.11</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n"/>
@@ -32339,9 +32387,14 @@
       <c r="D15" s="2" t="n"/>
       <c r="E15" s="2" t="n"/>
       <c r="F15" s="2" t="n"/>
-      <c r="G15" s="2" t="n"/>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="n"/>
+      <c r="G15" s="55" t="inlineStr">
+        <is>
+          <t>Teppich (dünn)</t>
+        </is>
+      </c>
+      <c r="H15" s="60" t="n">
+        <v>0.1</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="103" t="inlineStr">
@@ -32354,9 +32407,14 @@
       <c r="D16" s="2" t="n"/>
       <c r="E16" s="2" t="n"/>
       <c r="F16" s="2" t="n"/>
-      <c r="G16" s="2" t="n"/>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="n"/>
+      <c r="G16" s="55" t="inlineStr">
+        <is>
+          <t>Teppich (dick)</t>
+        </is>
+      </c>
+      <c r="H16" s="60" t="n">
+        <v>0.17</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="104" t="inlineStr">
@@ -32385,9 +32443,8 @@
         </is>
       </c>
       <c r="F17" s="2" t="n"/>
-      <c r="G17" s="2" t="n"/>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="n"/>
+      <c r="G17" s="55" t="n"/>
+      <c r="H17" s="60" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="55" t="inlineStr">
@@ -32409,9 +32466,8 @@
         <v>0.007</v>
       </c>
       <c r="F18" s="2" t="n"/>
-      <c r="G18" s="2" t="n"/>
-      <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="n"/>
+      <c r="G18" s="55" t="n"/>
+      <c r="H18" s="60" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="55" t="inlineStr">
@@ -32433,9 +32489,8 @@
         <v>0.007</v>
       </c>
       <c r="F19" s="2" t="n"/>
-      <c r="G19" s="2" t="n"/>
-      <c r="H19" s="2" t="n"/>
-      <c r="I19" s="2" t="n"/>
+      <c r="G19" s="55" t="n"/>
+      <c r="H19" s="60" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="55" t="inlineStr">
@@ -32459,7 +32514,6 @@
       <c r="F20" s="2" t="n"/>
       <c r="G20" s="2" t="n"/>
       <c r="H20" s="2" t="n"/>
-      <c r="I20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="55" t="inlineStr">
@@ -32483,7 +32537,6 @@
       <c r="F21" s="2" t="n"/>
       <c r="G21" s="2" t="n"/>
       <c r="H21" s="2" t="n"/>
-      <c r="I21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="55" t="n"/>
@@ -32497,7 +32550,6 @@
       <c r="F22" s="2" t="n"/>
       <c r="G22" s="2" t="n"/>
       <c r="H22" s="2" t="n"/>
-      <c r="I22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="55" t="n"/>
@@ -32511,7 +32563,6 @@
       <c r="F23" s="2" t="n"/>
       <c r="G23" s="2" t="n"/>
       <c r="H23" s="2" t="n"/>
-      <c r="I23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="55" t="n"/>
@@ -32525,7 +32576,6 @@
       <c r="F24" s="2" t="n"/>
       <c r="G24" s="2" t="n"/>
       <c r="H24" s="2" t="n"/>
-      <c r="I24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="55" t="n"/>
@@ -32539,14 +32589,13 @@
       <c r="F25" s="2" t="n"/>
       <c r="G25" s="2" t="n"/>
       <c r="H25" s="2" t="n"/>
-      <c r="I25" s="2" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <mergeCells count="3">
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="G4:I4"/>
-    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="D4:F4"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
FBH-Auslegung v0.34 - Auslegung-Design auf Graustufen + Zebra + Filter
- Rot zurueckgenommen: Graustufen-Design, Schrift durchgehend schwarz (auch Einheiten)
- Eingabe-/editierbare Zellen grau hinterlegt statt farbig; Farbe nur Logo + Ampel
- Rote Linien raus; schwarze Linie unter dem Tabellenkopf + duenne Briefkopflinie
- Zebra-Streifen je zweiter sichtbarer Zeile via CF/SUBTOTAL (filterfest)
- AutoFilter auf der Tabelle; Filtern trotz Blattschutz erlaubt

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FBH_Auslegung.xlsx
+++ b/FBH_Auslegung.xlsx
@@ -21,6 +21,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Deckblatt'!$A$1:$K$22</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Grundeinstellungen'!$A$1:$M$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Auslegung'!$A$6:$AK$206</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Auslegung'!$1:$6</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Auslegung'!$A$1:$AK$206</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'Kontrolle'!$A$1:$D$25</definedName>
@@ -29,7 +30,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="6">'Anleitung'!$A$1:$D$32</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">'Methodik'!$A$1:$F$26</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="8">'Konstanten'!$A$1:$I$27</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="9">'Changelog'!$A$1:$C$115</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="9">'Changelog'!$A$1:$C$119</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -70,7 +71,7 @@
     <numFmt numFmtId="193" formatCode="&quot;+&quot;0.0%;&quot;-&quot;0.0%;0.0%"/>
     <numFmt numFmtId="194" formatCode="0&quot; °C&quot;"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="24">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -121,40 +122,29 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="001A1A1A"/>
-      <sz val="10"/>
+      <color rgb="00000000"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00000000"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="001A1A1A"/>
-      <sz val="13"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="008A8A82"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="001A1A1A"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="001A1A1A"/>
+      <color rgb="00000000"/>
       <sz val="16"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="008A8A82"/>
+      <color rgb="00000000"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
       <i val="1"/>
-      <color rgb="008A8A82"/>
+      <color rgb="00000000"/>
       <sz val="9"/>
     </font>
     <font>
@@ -239,7 +229,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCF1F0"/>
+        <fgColor rgb="00E9E9E9"/>
       </patternFill>
     </fill>
     <fill>
@@ -273,7 +263,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -341,40 +331,35 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00E0DED7"/>
+        <color rgb="00C9C9C9"/>
       </left>
       <right style="thin">
-        <color rgb="00E0DED7"/>
+        <color rgb="00C9C9C9"/>
       </right>
       <top style="thin">
-        <color rgb="00E0DED7"/>
+        <color rgb="00C9C9C9"/>
       </top>
       <bottom style="thin">
-        <color rgb="00E0DED7"/>
+        <color rgb="00C9C9C9"/>
       </bottom>
     </border>
     <border>
       <left style="thin">
-        <color rgb="00E0DED7"/>
+        <color rgb="00C9C9C9"/>
       </left>
       <right style="thin">
-        <color rgb="00E0DED7"/>
+        <color rgb="00C9C9C9"/>
       </right>
       <top style="thin">
-        <color rgb="00E0DED7"/>
+        <color rgb="00C9C9C9"/>
       </top>
       <bottom style="medium">
-        <color rgb="00E2001A"/>
+        <color rgb="00000000"/>
       </bottom>
     </border>
     <border>
-      <left style="thick">
-        <color rgb="00E2001A"/>
-      </left>
-    </border>
-    <border>
-      <top style="medium">
-        <color rgb="00E2001A"/>
+      <top style="thin">
+        <color rgb="00000000"/>
       </top>
     </border>
     <border>
@@ -416,38 +401,38 @@
   </cellStyleXfs>
   <cellXfs count="137">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="7" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -456,7 +441,7 @@
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -567,17 +552,25 @@
       <alignment horizontal="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -588,110 +581,102 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="7" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="7" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="7" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="7" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="177" fontId="11" fillId="4" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="177" fontId="6" fillId="4" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="178" fontId="11" fillId="4" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="178" fontId="6" fillId="4" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="172" fontId="11" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="172" fontId="6" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="171" fontId="11" fillId="4" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="6" fillId="4" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="179" fontId="11" fillId="4" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="179" fontId="6" fillId="4" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="180" fontId="11" fillId="4" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="180" fontId="6" fillId="4" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="181" fontId="11" fillId="4" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="181" fontId="6" fillId="4" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="182" fontId="11" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="182" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="171" fontId="11" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="172" fontId="11" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="172" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="178" fontId="11" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="178" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="183" fontId="11" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="183" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="184" fontId="11" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="184" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="181" fontId="11" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="181" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="185" fontId="11" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="185" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="186" fontId="11" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="186" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="187" fontId="11" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="187" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="11" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="188" fontId="11" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="188" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="189" fontId="11" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="189" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -737,32 +722,32 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="171" fontId="17" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="15" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="179" fontId="18" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="179" fontId="16" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="16" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="171" fontId="18" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="16" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="172" fontId="18" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="172" fontId="16" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -778,7 +763,7 @@
     <xf numFmtId="171" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -789,14 +774,14 @@
     <xf numFmtId="193" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -804,7 +789,7 @@
       <alignment vertical="top"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -816,30 +801,30 @@
       <alignment vertical="top" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="194" fontId="18" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="194" fontId="16" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="168" fontId="18" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="16" fillId="2" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -862,13 +847,13 @@
       <alignment vertical="top" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="6">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -882,6 +867,22 @@
         <patternFill patternType="solid">
           <fgColor rgb="FFEAF3DE"/>
           <bgColor rgb="FFEAF3DE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDBDBDB"/>
+          <bgColor rgb="FFDBDBDB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF3F3F3"/>
+          <bgColor rgb="FFF3F3F3"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2277,7 +2278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C115"/>
+  <dimension ref="A1:C119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2304,7 +2305,7 @@
       <c r="B3" s="2" t="n"/>
       <c r="C3" s="25" t="inlineStr">
         <is>
-          <t>Version 0.33 · dh</t>
+          <t>Version 0.34 · dh</t>
         </is>
       </c>
     </row>
@@ -2333,7 +2334,7 @@
     <row r="6">
       <c r="A6" s="132" t="inlineStr">
         <is>
-          <t>0.33</t>
+          <t>0.34</t>
         </is>
       </c>
       <c r="B6" s="133" t="inlineStr">
@@ -2343,7 +2344,7 @@
       </c>
       <c r="C6" s="134" t="inlineStr">
         <is>
-          <t>• Neues, cleanes Druck-Design (Pilot auf dem Blatt 'Auslegung'): weißer Hintergrund mit agn-rotem Akzent (Kopflinie, Spaltenkopf-Unterstrich, Logo-Quadrat, roter Akzentbalken am Titel) statt dunkler Navy-Flächen.</t>
+          <t>• Auslegung-Design auf Graustufen umgestellt: Schrift durchgehend schwarz (auch Einheiten), Eingabe-/editierbare Zellen grau hinterlegt statt farbig; Farbe nur noch im Logo und in der Ampel-Bewertung.</t>
         </is>
       </c>
     </row>
@@ -2352,77 +2353,77 @@
       <c r="B7" s="135" t="n"/>
       <c r="C7" s="134" t="inlineStr">
         <is>
+          <t>• Rote Trennlinien entfernt – schwarze Linie unter dem Tabellenkopf, dünne schwarze Briefkopflinie.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="135" t="n"/>
+      <c r="B8" s="135" t="n"/>
+      <c r="C8" s="134" t="inlineStr">
+        <is>
+          <t>• Zebra-Streifen: jede zweite (sichtbare) Datenzeile leicht grau – über bedingte Formatierung mit SUBTOTAL, daher filterfest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="136" t="n"/>
+      <c r="B9" s="136" t="n"/>
+      <c r="C9" s="134" t="inlineStr">
+        <is>
+          <t>• Neue Filterfunktion (AutoFilter) auf der Auslegungstabelle; Filtern ist trotz Blattschutz möglich.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="132" t="inlineStr">
+        <is>
+          <t>0.33</t>
+        </is>
+      </c>
+      <c r="B10" s="133" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="C10" s="134" t="inlineStr">
+        <is>
+          <t>• Neues, cleanes Druck-Design (Pilot auf dem Blatt 'Auslegung'): weißer Hintergrund mit agn-rotem Akzent (Kopflinie, Spaltenkopf-Unterstrich, Logo-Quadrat, roter Akzentbalken am Titel) statt dunkler Navy-Flächen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="135" t="n"/>
+      <c r="B11" s="135" t="n"/>
+      <c r="C11" s="134" t="inlineStr">
+        <is>
           <t>• Auslegung: Eingabespalten zart rot getönt statt kräftig gelb; weiche Haarlinien statt Vollgitter; Ampel-Farben dezenter (sanftes Grün/Rot).</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="136" t="n"/>
-      <c r="B8" s="136" t="n"/>
-      <c r="C8" s="134" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="136" t="n"/>
+      <c r="B12" s="136" t="n"/>
+      <c r="C12" s="134" t="inlineStr">
         <is>
           <t>• Die übrigen Blätter sind noch im bisherigen Stil – das Design wird nach Freigabe übertragen.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="132" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="132" t="inlineStr">
         <is>
           <t>0.32</t>
         </is>
       </c>
-      <c r="B9" s="133" t="inlineStr">
+      <c r="B13" s="133" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="C9" s="134" t="inlineStr">
+      <c r="C13" s="134" t="inlineStr">
         <is>
           <t>• Deckblatt neu strukturiert: jede Information in einer eigenen Zelle (keine Mehrzeilen-Blöcke mehr, keine Fehl-Umbrüche); die wichtigsten Formeln stehen jetzt direkt in der Spalte 'BERECHNUNG'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="135" t="n"/>
-      <c r="B10" s="135" t="n"/>
-      <c r="C10" s="134" t="inlineStr">
-        <is>
-          <t>• Deckblatt: Bauart-A-Hinweis entfernt; steht stattdessen bei den Grundeinstellungen unter 'Gewähltes Rohrsystem'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="136" t="n"/>
-      <c r="B11" s="136" t="n"/>
-      <c r="C11" s="134" t="inlineStr">
-        <is>
-          <t>• Verifikation: Systemfaktor-Feld vergrößert (Spalte breiter, Beschriftung etwas kleiner) – der Wert ist jetzt vollständig lesbar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="132" t="inlineStr">
-        <is>
-          <t>0.31</t>
-        </is>
-      </c>
-      <c r="B12" s="133" t="inlineStr">
-        <is>
-          <t>2026-06-16</t>
-        </is>
-      </c>
-      <c r="C12" s="134" t="inlineStr">
-        <is>
-          <t>• Verifikation: Spaltenköpfe und Hinweis klargestellt – verglichen wird die spez. Heizleistung NACH OBEN (Wärmestrom zur Raumseite); die Wärmeabgabe nach unten ist hier bewusst nicht enthalten.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="135" t="n"/>
-      <c r="B13" s="135" t="n"/>
-      <c r="C13" s="134" t="inlineStr">
-        <is>
-          <t>• Deckblatt überarbeitet: Inhalte über die volle A4-quer-Höhe verteilt, fette Überschriften, ausgeschriebene Begriffe (keine Abkürzungen), neuer Block 'Die wichtigsten Berechnungsformeln' mit Formelzeichen-Legende.</t>
         </is>
       </c>
     </row>
@@ -2431,7 +2432,7 @@
       <c r="B14" s="135" t="n"/>
       <c r="C14" s="134" t="inlineStr">
         <is>
-          <t>• Deckblatt/Methodik: Hinweis ergänzt, dass das Tool nur für Bauart A nach DIN EN 1264 (Heizrohre im Estrich) gilt.</t>
+          <t>• Deckblatt: Bauart-A-Hinweis entfernt; steht stattdessen bei den Grundeinstellungen unter 'Gewähltes Rohrsystem'.</t>
         </is>
       </c>
     </row>
@@ -2440,14 +2441,14 @@
       <c r="B15" s="136" t="n"/>
       <c r="C15" s="134" t="inlineStr">
         <is>
-          <t>• Auslegung: Hinweis-/Kommentartext (Tooltip) an der R-Wert-Spalte wieder entfernt (er aktualisiert sich nicht mit den Konstanten).</t>
+          <t>• Verifikation: Systemfaktor-Feld vergrößert (Spalte breiter, Beschriftung etwas kleiner) – der Wert ist jetzt vollständig lesbar.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="132" t="inlineStr">
         <is>
-          <t>0.30</t>
+          <t>0.31</t>
         </is>
       </c>
       <c r="B16" s="133" t="inlineStr">
@@ -2457,7 +2458,7 @@
       </c>
       <c r="C16" s="134" t="inlineStr">
         <is>
-          <t>• Verifikation: Beispielwerte durch 12 reale Herstellerpunkte ersetzt (Rehau 17×2, Estrichüberdeckung s_ü 45 mm; zwei Belag-/Temperaturfälle, Verlegeabstand 50–300 mm).</t>
+          <t>• Verifikation: Spaltenköpfe und Hinweis klargestellt – verglichen wird die spez. Heizleistung NACH OBEN (Wärmestrom zur Raumseite); die Wärmeabgabe nach unten ist hier bewusst nicht enthalten.</t>
         </is>
       </c>
     </row>
@@ -2466,112 +2467,112 @@
       <c r="B17" s="135" t="n"/>
       <c r="C17" s="134" t="inlineStr">
         <is>
+          <t>• Deckblatt überarbeitet: Inhalte über die volle A4-quer-Höhe verteilt, fette Überschriften, ausgeschriebene Begriffe (keine Abkürzungen), neuer Block 'Die wichtigsten Berechnungsformeln' mit Formelzeichen-Legende.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="135" t="n"/>
+      <c r="B18" s="135" t="n"/>
+      <c r="C18" s="134" t="inlineStr">
+        <is>
+          <t>• Deckblatt/Methodik: Hinweis ergänzt, dass das Tool nur für Bauart A nach DIN EN 1264 (Heizrohre im Estrich) gilt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="136" t="n"/>
+      <c r="B19" s="136" t="n"/>
+      <c r="C19" s="134" t="inlineStr">
+        <is>
+          <t>• Auslegung: Hinweis-/Kommentartext (Tooltip) an der R-Wert-Spalte wieder entfernt (er aktualisiert sich nicht mit den Konstanten).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="132" t="inlineStr">
+        <is>
+          <t>0.30</t>
+        </is>
+      </c>
+      <c r="B20" s="133" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C20" s="134" t="inlineStr">
+        <is>
+          <t>• Verifikation: Beispielwerte durch 12 reale Herstellerpunkte ersetzt (Rehau 17×2, Estrichüberdeckung s_ü 45 mm; zwei Belag-/Temperaturfälle, Verlegeabstand 50–300 mm).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="135" t="n"/>
+      <c r="B21" s="135" t="n"/>
+      <c r="C21" s="134" t="inlineStr">
+        <is>
           <t>• Verifikation: neue Summenzeile 'Gesamtabweichung (Σ über alle Punkte)' in W/m² und % – zeigt, wie gut der Systemfaktor f insgesamt passt (nahe 0 ⇒ gut kalibriert; bei Rehau ≈ −0,2 %).</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="136" t="n"/>
-      <c r="B18" s="136" t="n"/>
-      <c r="C18" s="134" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="136" t="n"/>
+      <c r="B22" s="136" t="n"/>
+      <c r="C22" s="134" t="inlineStr">
         <is>
           <t>• Deckblatt: Hinweis-Kasten 'Vereinfachungen' entfernt (die Vereinfachungen sind weiterhin im Blatt 'Methodik' dokumentiert).</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="132" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="132" t="inlineStr">
         <is>
           <t>0.29</t>
         </is>
       </c>
-      <c r="B19" s="133" t="inlineStr">
+      <c r="B23" s="133" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="C19" s="134" t="inlineStr">
+      <c r="C23" s="134" t="inlineStr">
         <is>
           <t>• Auslegung: in der Spalte wird wieder direkt der R-Wert ausgewählt (Spalte bleibt schmal). Die Zuordnung R-Wert ↔ Bodenbelag erscheint als Hinweis (Tooltip), sobald man die Zelle anklickt – ohne die Spalte zu verbreitern.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="136" t="n"/>
-      <c r="B20" s="136" t="n"/>
-      <c r="C20" s="134" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="136" t="n"/>
+      <c r="B24" s="136" t="n"/>
+      <c r="C24" s="134" t="inlineStr">
         <is>
           <t>• Auslegung: Bearbeiter-Feld wieder aus den Grundeinstellungen referenziert (nur dort einmal eingeben) – daher ungefärbt; auf sichtbaren Spalten, damit der Eintrag nicht abgeschnitten wird.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="132" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="132" t="inlineStr">
         <is>
           <t>0.28</t>
         </is>
       </c>
-      <c r="B21" s="133" t="inlineStr">
+      <c r="B25" s="133" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="C21" s="134" t="inlineStr">
+      <c r="C25" s="134" t="inlineStr">
         <is>
           <t>• Blattschutz: Zeilenhöhe und Spaltenbreite bleiben trotz Schutz änderbar – in der HKV-Liste lässt sich die Zeilenhöhe für lange Raumlisten jetzt wieder anpassen (optimale Höhe).</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="135" t="n"/>
-      <c r="B22" s="135" t="n"/>
-      <c r="C22" s="134" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="135" t="n"/>
+      <c r="B26" s="135" t="n"/>
+      <c r="C26" s="134" t="inlineStr">
         <is>
           <t>• Auslegung: Spalte 'R-Wert Bodenbelag' → Auswahl jetzt über den Bodenbelag-Namen (Dropdown), der R-Wert wird automatisch aus den Konstanten gezogen – man sieht den Belag statt nur die Zahl.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="135" t="n"/>
-      <c r="B23" s="135" t="n"/>
-      <c r="C23" s="134" t="inlineStr">
-        <is>
-          <t>• Auslegung: Bearbeiter-Feld oben rechts als zwei Zellen (Label + eigenes Eingabefeld) und auf sichtbaren Spalten – der Eintrag wird nicht mehr abgeschnitten.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="135" t="n"/>
-      <c r="B24" s="135" t="n"/>
-      <c r="C24" s="134" t="inlineStr">
-        <is>
-          <t>• Verifikation: 15 statt 8 Referenzpunkte nach DIN EN 1264 (mehr Prüfstellen: Verlegeabstand 100–300 mm, VL 40/45/50 °C, R 0,00–0,15 m²K/W).</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="136" t="n"/>
-      <c r="B25" s="136" t="n"/>
-      <c r="C25" s="134" t="inlineStr">
-        <is>
-          <t>• Konstanten: R-Werte-Tabelle auf 17 Beläge erweitert (inkl. 'ohne Belag'); Zonen-Tabelle auf gleiche Höhe wie Verlegeabstand-Tabelle; Leerspalte zwischen Zonen und R-Werten.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="132" t="inlineStr">
-        <is>
-          <t>0.27</t>
-        </is>
-      </c>
-      <c r="B26" s="133" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="C26" s="134" t="inlineStr">
-        <is>
-          <t>• Auslegung: 'Über-/Unterdeckung' wieder ausgeblendet; stattdessen wird die 'Leistung FBH' eingefärbt (grün = Heizlast gedeckt, rot = nicht gedeckt). Raum-Nr. breiter; Anzahl Heizkreise mit Einheit 'HK' je Zelle; schmalere Seitenränder für besseren A4-Sitz.</t>
         </is>
       </c>
     </row>
@@ -2580,42 +2581,42 @@
       <c r="B27" s="135" t="n"/>
       <c r="C27" s="134" t="inlineStr">
         <is>
-          <t>• HKV-Liste: Spalte 'angebundene Räume' deutlich breiter (lange/viele Raumnummern werden vollständig dargestellt).</t>
+          <t>• Auslegung: Bearbeiter-Feld oben rechts als zwei Zellen (Label + eigenes Eingabefeld) und auf sichtbaren Spalten – der Eintrag wird nicht mehr abgeschnitten.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="136" t="n"/>
-      <c r="B28" s="136" t="n"/>
+      <c r="A28" s="135" t="n"/>
+      <c r="B28" s="135" t="n"/>
       <c r="C28" s="134" t="inlineStr">
         <is>
-          <t>• Konstanten: R-Werte-Tabelle der Bodenbeläge erweitert (11 Beläge statt 5) und nach rechts gestellt; Zonen-Tabelle nach links – so kann die R-Werte-Tabelle höher werden.</t>
+          <t>• Verifikation: 15 statt 8 Referenzpunkte nach DIN EN 1264 (mehr Prüfstellen: Verlegeabstand 100–300 mm, VL 40/45/50 °C, R 0,00–0,15 m²K/W).</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="132" t="inlineStr">
-        <is>
-          <t>0.26</t>
-        </is>
-      </c>
-      <c r="B29" s="133" t="inlineStr">
+      <c r="A29" s="136" t="n"/>
+      <c r="B29" s="136" t="n"/>
+      <c r="C29" s="134" t="inlineStr">
+        <is>
+          <t>• Konstanten: R-Werte-Tabelle auf 17 Beläge erweitert (inkl. 'ohne Belag'); Zonen-Tabelle auf gleiche Höhe wie Verlegeabstand-Tabelle; Leerspalte zwischen Zonen und R-Werten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="132" t="inlineStr">
+        <is>
+          <t>0.27</t>
+        </is>
+      </c>
+      <c r="B30" s="133" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="C29" s="134" t="inlineStr">
-        <is>
-          <t>• HKV-Liste: neue Spalte 'angebundene Räume (Raum-Nr.)' – listet je Verteiler automatisch die zugehörigen Raumnummern (TEXTJOIN-Array, Excel &amp; LibreOffice).</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="135" t="n"/>
-      <c r="B30" s="135" t="n"/>
       <c r="C30" s="134" t="inlineStr">
         <is>
-          <t>• Auslegung: Spalten 'Leistung FBH' und 'Über-/Unterdeckung' eingeblendet; Über-/Unterdeckung mit Vorzeichen (+/–) und Ampel (grün = Überdeckung, rot = Unterdeckung).</t>
+          <t>• Auslegung: 'Über-/Unterdeckung' wieder ausgeblendet; stattdessen wird die 'Leistung FBH' eingefärbt (grün = Heizlast gedeckt, rot = nicht gedeckt). Raum-Nr. breiter; Anzahl Heizkreise mit Einheit 'HK' je Zelle; schmalere Seitenränder für besseren A4-Sitz.</t>
         </is>
       </c>
     </row>
@@ -2624,225 +2625,225 @@
       <c r="B31" s="135" t="n"/>
       <c r="C31" s="134" t="inlineStr">
         <is>
+          <t>• HKV-Liste: Spalte 'angebundene Räume' deutlich breiter (lange/viele Raumnummern werden vollständig dargestellt).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="136" t="n"/>
+      <c r="B32" s="136" t="n"/>
+      <c r="C32" s="134" t="inlineStr">
+        <is>
+          <t>• Konstanten: R-Werte-Tabelle der Bodenbeläge erweitert (11 Beläge statt 5) und nach rechts gestellt; Zonen-Tabelle nach links – so kann die R-Werte-Tabelle höher werden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="132" t="inlineStr">
+        <is>
+          <t>0.26</t>
+        </is>
+      </c>
+      <c r="B33" s="133" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="C33" s="134" t="inlineStr">
+        <is>
+          <t>• HKV-Liste: neue Spalte 'angebundene Räume (Raum-Nr.)' – listet je Verteiler automatisch die zugehörigen Raumnummern (TEXTJOIN-Array, Excel &amp; LibreOffice).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="135" t="n"/>
+      <c r="B34" s="135" t="n"/>
+      <c r="C34" s="134" t="inlineStr">
+        <is>
+          <t>• Auslegung: Spalten 'Leistung FBH' und 'Über-/Unterdeckung' eingeblendet; Über-/Unterdeckung mit Vorzeichen (+/–) und Ampel (grün = Überdeckung, rot = Unterdeckung).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="135" t="n"/>
+      <c r="B35" s="135" t="n"/>
+      <c r="C35" s="134" t="inlineStr">
+        <is>
           <t>• Grundeinstellungen: Eingabefelder Projekt-Nr./Projektname breiter; Spalte J (Rohrsystem-Werte) breiter.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="135" t="n"/>
-      <c r="B32" s="135" t="n"/>
-      <c r="C32" s="134" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="135" t="n"/>
+      <c r="B36" s="135" t="n"/>
+      <c r="C36" s="134" t="inlineStr">
         <is>
           <t>• Verifikation: kein fixer Vergleichspunkt mehr – jede Zeile ist ein eigener Auslegungspunkt (VL/RL, θi, R, Verlegeabstand) mit eigener Abweichung; Diagramm entfernt.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="136" t="n"/>
-      <c r="B33" s="136" t="n"/>
-      <c r="C33" s="134" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="136" t="n"/>
+      <c r="B37" s="136" t="n"/>
+      <c r="C37" s="134" t="inlineStr">
         <is>
           <t>• Blattschutz: Zellen mit Formeln sind gesperrt (vor versehentlichem Überschreiben geschützt), Eingabezellen bleiben editierbar; Schutz ohne Passwort.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="132" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="132" t="inlineStr">
         <is>
           <t>0.25</t>
         </is>
       </c>
-      <c r="B34" s="133" t="inlineStr">
+      <c r="B38" s="133" t="inlineStr">
         <is>
           <t>2026-06-14</t>
         </is>
       </c>
-      <c r="C34" s="134" t="inlineStr">
+      <c r="C38" s="134" t="inlineStr">
         <is>
           <t>• Begriff 'Korrekturfaktor' in 'Systemfaktor (EN-1264-Kalibrierung)' umbenannt (Verifikation, Methodik, Deckblatt, Anleitung) – f ist die bewusste Kalibrierung des überschlägigen Modells an EN 1264, kein Fehlerfaktor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="132" t="inlineStr">
-        <is>
-          <t>0.24</t>
-        </is>
-      </c>
-      <c r="B35" s="133" t="inlineStr">
-        <is>
-          <t>2026-06-14</t>
-        </is>
-      </c>
-      <c r="C35" s="134" t="inlineStr">
-        <is>
-          <t>• Verifikation: Referenzspalte mit echten Werten nach DIN EN 1264 vorbelegt (Nasssystem/Tacker, VL 40 / RL 30 °C, θi 20 °C, R = 0,10 m²K/W); Vergleichsbedingungen entsprechend auf 40/30 °C gesetzt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="136" t="n"/>
-      <c r="B36" s="136" t="n"/>
-      <c r="C36" s="134" t="inlineStr">
-        <is>
-          <t>• Verifikation: Korrekturfaktor f auf 0,85 vorkalibriert (Best-Fit zu den EN-1264-Werten); Spalte C bleibt editierbar für herstellereigene Datenblattwerte (Rehau, Uponor, Buderus, Kermi …).</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="132" t="inlineStr">
-        <is>
-          <t>0.23</t>
-        </is>
-      </c>
-      <c r="B37" s="133" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="C37" s="134" t="inlineStr">
-        <is>
-          <t>• Auslegung: Formelzeichen größer (besser lesbare Tiefstellungen); Kopfzeilen-Umbrüche optimiert – keine Trennung mehr mitten im Wort.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="136" t="n"/>
-      <c r="B38" s="136" t="n"/>
-      <c r="C38" s="134" t="inlineStr">
-        <is>
-          <t>• Deckblatt: Druck-Hinweis wieder entfernt.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="132" t="inlineStr">
         <is>
+          <t>0.24</t>
+        </is>
+      </c>
+      <c r="B39" s="133" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="C39" s="134" t="inlineStr">
+        <is>
+          <t>• Verifikation: Referenzspalte mit echten Werten nach DIN EN 1264 vorbelegt (Nasssystem/Tacker, VL 40 / RL 30 °C, θi 20 °C, R = 0,10 m²K/W); Vergleichsbedingungen entsprechend auf 40/30 °C gesetzt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="136" t="n"/>
+      <c r="B40" s="136" t="n"/>
+      <c r="C40" s="134" t="inlineStr">
+        <is>
+          <t>• Verifikation: Korrekturfaktor f auf 0,85 vorkalibriert (Best-Fit zu den EN-1264-Werten); Spalte C bleibt editierbar für herstellereigene Datenblattwerte (Rehau, Uponor, Buderus, Kermi …).</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="132" t="inlineStr">
+        <is>
+          <t>0.23</t>
+        </is>
+      </c>
+      <c r="B41" s="133" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="C41" s="134" t="inlineStr">
+        <is>
+          <t>• Auslegung: Formelzeichen größer (besser lesbare Tiefstellungen); Kopfzeilen-Umbrüche optimiert – keine Trennung mehr mitten im Wort.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="136" t="n"/>
+      <c r="B42" s="136" t="n"/>
+      <c r="C42" s="134" t="inlineStr">
+        <is>
+          <t>• Deckblatt: Druck-Hinweis wieder entfernt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="132" t="inlineStr">
+        <is>
           <t>0.22</t>
         </is>
       </c>
-      <c r="B39" s="133" t="inlineStr">
+      <c r="B43" s="133" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="C39" s="134" t="inlineStr">
+      <c r="C43" s="134" t="inlineStr">
         <is>
           <t>• Anleitung: neue Ampel-Legende (warum ist eine Zelle rot?) und Hinweis zur Auslegung mehrerer Verteiler/Geschosse; Blatt nach hinten verschoben (jetzt vor der Methodik).</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="135" t="n"/>
-      <c r="B40" s="135" t="n"/>
-      <c r="C40" s="134" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="135" t="n"/>
+      <c r="B44" s="135" t="n"/>
+      <c r="C44" s="134" t="inlineStr">
         <is>
           <t>• Deckblatt: Druck-Hinweis ergänzt – nur die relevanten Blätter (Deckblatt, Grundeinstellungen, Auslegung, Kontrolle, HKV, Anleitung) gemeinsam als 'Aktive Blätter' drucken.</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="136" t="n"/>
-      <c r="B41" s="136" t="n"/>
-      <c r="C41" s="134" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="136" t="n"/>
+      <c r="B45" s="136" t="n"/>
+      <c r="C45" s="134" t="inlineStr">
         <is>
           <t>• Formelzeichen mit echten Tiefstellungen dargestellt (z. B. q_HL, R_λ,B, V̇_max) – kein Unterstrich mehr in den Kopfzeilen, Grundeinstellungen und der Methodik-Variablenliste.</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="132" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="132" t="inlineStr">
         <is>
           <t>0.21</t>
         </is>
       </c>
-      <c r="B42" s="133" t="inlineStr">
+      <c r="B46" s="133" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="C42" s="134" t="inlineStr">
+      <c r="C46" s="134" t="inlineStr">
         <is>
           <t>• Auslegung jetzt auf A4-Querformat (vorher A3); sichtbare Spalten schmaler, damit das Blatt auf A4 passt.</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="135" t="n"/>
-      <c r="B43" s="135" t="n"/>
-      <c r="C43" s="134" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="135" t="n"/>
+      <c r="B47" s="135" t="n"/>
+      <c r="C47" s="134" t="inlineStr">
         <is>
           <t>• Deckblatt: Titel 'Fußbodenheizung – Auslegung' (Wort 'überschlägige' entfernt); Vereinfachungen bleiben dokumentiert.</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="136" t="n"/>
-      <c r="B44" s="136" t="n"/>
-      <c r="C44" s="134" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="136" t="n"/>
+      <c r="B48" s="136" t="n"/>
+      <c r="C48" s="134" t="inlineStr">
         <is>
           <t>• Anleitung: Abschnitt 'Planungstechnische Grundlagen' wieder entfernt.</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="132" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="132" t="inlineStr">
         <is>
           <t>0.20</t>
         </is>
       </c>
-      <c r="B45" s="133" t="inlineStr">
+      <c r="B49" s="133" t="inlineStr">
         <is>
           <t>2026-06-13</t>
         </is>
       </c>
-      <c r="C45" s="134" t="inlineStr">
+      <c r="C49" s="134" t="inlineStr">
         <is>
           <t>• Grundeinstellungen: Spaltenbreiten optimiert und lange Beschriftungen/Hinweise gekürzt – Texte werden in LibreOffice nicht mehr abgeschnitten.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="135" t="n"/>
-      <c r="B46" s="135" t="n"/>
-      <c r="C46" s="134" t="inlineStr">
-        <is>
-          <t>• Verifikation: Untertitel und Hinweise vereinfacht (Modellvergleich-Erläuterung entfernt); klarer Hinweis, dass der Korrekturfaktor f VOR der Raumauslegung kalibriert wird; Diagramm etwas größer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="136" t="n"/>
-      <c r="B47" s="136" t="n"/>
-      <c r="C47" s="134" t="inlineStr">
-        <is>
-          <t>• Anleitung: Schritt-für-Schritt neu geordnet – Verifikation/Kalibrierung des Korrekturfaktors jetzt VOR der Raumauslegung; neuer Abschnitt 'Planungstechnische Grundlagen'; Hinweis zur vorgefertigten Revit-Liste entfernt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="132" t="inlineStr">
-        <is>
-          <t>0.19</t>
-        </is>
-      </c>
-      <c r="B48" s="133" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
-      <c r="C48" s="134" t="inlineStr">
-        <is>
-          <t>• Grundeinstellungen: neuer Grenzwert 'Maximaler Volumenstrom je Kreis' (V̇_max, Default 150 l/h); Abschnitt 'Strömungsgeschwindigkeit' → 'Strömungsgrenzwerte'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="135" t="n"/>
-      <c r="B49" s="135" t="n"/>
-      <c r="C49" s="134" t="inlineStr">
-        <is>
-          <t>• Auslegung: Volumenstrom je Kreis wird gegen V̇_max geprüft und per Ampel eingefärbt (grün ≤ Grenze, rot darüber); zusätzliche Warnung im Blatt 'Kontrolle'.</t>
         </is>
       </c>
     </row>
@@ -2851,7 +2852,7 @@
       <c r="B50" s="135" t="n"/>
       <c r="C50" s="134" t="inlineStr">
         <is>
-          <t>• Anleitung: durchgehende Schritt-für-Schritt-Anleitung mit integriertem Revit-Export (vorgefertigte Bauteilliste muss nicht erst angelegt werden); redundanter Abschnitt 'Räume aus Revit' und der Hinweis zum direkten Kopieren entfernt.</t>
+          <t>• Verifikation: Untertitel und Hinweise vereinfacht (Modellvergleich-Erläuterung entfernt); klarer Hinweis, dass der Korrekturfaktor f VOR der Raumauslegung kalibriert wird; Diagramm etwas größer.</t>
         </is>
       </c>
     </row>
@@ -2860,14 +2861,14 @@
       <c r="B51" s="136" t="n"/>
       <c r="C51" s="134" t="inlineStr">
         <is>
-          <t>• Deckblatt: Pfeil-Spalten breiter und Pfeilgröße angepasst (optisch sauberer).</t>
+          <t>• Anleitung: Schritt-für-Schritt neu geordnet – Verifikation/Kalibrierung des Korrekturfaktors jetzt VOR der Raumauslegung; neuer Abschnitt 'Planungstechnische Grundlagen'; Hinweis zur vorgefertigten Revit-Liste entfernt.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="132" t="inlineStr">
         <is>
-          <t>0.18</t>
+          <t>0.19</t>
         </is>
       </c>
       <c r="B52" s="133" t="inlineStr">
@@ -2877,33 +2878,25 @@
       </c>
       <c r="C52" s="134" t="inlineStr">
         <is>
-          <t>• Auslegung: Eingabespalten neu sortiert – zuerst die Revit-Spalten (A HKV, B Raum-Nr., C Bezeichnung, D Raumfläche, E Raumtemperatur, F Heizlast), dann G spez. Heizlast (berechnet), danach die manuellen Felder (H aktiv. Fläche, I R-Wert, J Verlegeabstand, K Anz. Kreise, L Zuleitung, M Zone).</t>
+          <t>• Grundeinstellungen: neuer Grenzwert 'Maximaler Volumenstrom je Kreis' (V̇_max, Default 150 l/h); Abschnitt 'Strömungsgeschwindigkeit' → 'Strömungsgrenzwerte'.</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="136" t="n"/>
-      <c r="B53" s="136" t="n"/>
+      <c r="A53" s="135" t="n"/>
+      <c r="B53" s="135" t="n"/>
       <c r="C53" s="134" t="inlineStr">
         <is>
-          <t>• Anleitung: Excel-Export aus Revit ist jetzt der Standard-Workflow (direktes Kopieren funktioniert nicht); Spaltenliste an neue Reihenfolge angepasst.</t>
+          <t>• Auslegung: Volumenstrom je Kreis wird gegen V̇_max geprüft und per Ampel eingefärbt (grün ≤ Grenze, rot darüber); zusätzliche Warnung im Blatt 'Kontrolle'.</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="132" t="inlineStr">
-        <is>
-          <t>0.17</t>
-        </is>
-      </c>
-      <c r="B54" s="133" t="inlineStr">
-        <is>
-          <t>2026-06-13</t>
-        </is>
-      </c>
+      <c r="A54" s="135" t="n"/>
+      <c r="B54" s="135" t="n"/>
       <c r="C54" s="134" t="inlineStr">
         <is>
-          <t>• Neues Blatt 'Anleitung' (2. Blatt): Aufbau der Mappe, Schritt-für-Schritt, Farblegende.</t>
+          <t>• Anleitung: durchgehende Schritt-für-Schritt-Anleitung mit integriertem Revit-Export (vorgefertigte Bauteilliste muss nicht erst angelegt werden); redundanter Abschnitt 'Räume aus Revit' und der Hinweis zum direkten Kopieren entfernt.</t>
         </is>
       </c>
     </row>
@@ -2912,86 +2905,94 @@
       <c r="B55" s="136" t="n"/>
       <c r="C55" s="134" t="inlineStr">
         <is>
-          <t>• Anleitung enthält den Workflow zum Übernehmen der Räume aus Revit (Copy &amp; Paste, Schedule, Dynamo/Power Query).</t>
+          <t>• Deckblatt: Pfeil-Spalten breiter und Pfeilgröße angepasst (optisch sauberer).</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="132" t="inlineStr">
         <is>
+          <t>0.18</t>
+        </is>
+      </c>
+      <c r="B56" s="133" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="C56" s="134" t="inlineStr">
+        <is>
+          <t>• Auslegung: Eingabespalten neu sortiert – zuerst die Revit-Spalten (A HKV, B Raum-Nr., C Bezeichnung, D Raumfläche, E Raumtemperatur, F Heizlast), dann G spez. Heizlast (berechnet), danach die manuellen Felder (H aktiv. Fläche, I R-Wert, J Verlegeabstand, K Anz. Kreise, L Zuleitung, M Zone).</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="136" t="n"/>
+      <c r="B57" s="136" t="n"/>
+      <c r="C57" s="134" t="inlineStr">
+        <is>
+          <t>• Anleitung: Excel-Export aus Revit ist jetzt der Standard-Workflow (direktes Kopieren funktioniert nicht); Spaltenliste an neue Reihenfolge angepasst.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="132" t="inlineStr">
+        <is>
+          <t>0.17</t>
+        </is>
+      </c>
+      <c r="B58" s="133" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="C58" s="134" t="inlineStr">
+        <is>
+          <t>• Neues Blatt 'Anleitung' (2. Blatt): Aufbau der Mappe, Schritt-für-Schritt, Farblegende.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="136" t="n"/>
+      <c r="B59" s="136" t="n"/>
+      <c r="C59" s="134" t="inlineStr">
+        <is>
+          <t>• Anleitung enthält den Workflow zum Übernehmen der Räume aus Revit (Copy &amp; Paste, Schedule, Dynamo/Power Query).</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="132" t="inlineStr">
+        <is>
           <t>0.16</t>
         </is>
       </c>
-      <c r="B56" s="133" t="inlineStr">
+      <c r="B60" s="133" t="inlineStr">
         <is>
           <t>2026-06-09</t>
         </is>
       </c>
-      <c r="C56" s="134" t="inlineStr">
+      <c r="C60" s="134" t="inlineStr">
         <is>
           <t>• Alle Blätter im A4-Querformat (nur Auslegung A3 quer); einheitlichere Schriftgrößen/Skalierung.</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="135" t="n"/>
-      <c r="B57" s="135" t="n"/>
-      <c r="C57" s="134" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="135" t="n"/>
+      <c r="B61" s="135" t="n"/>
+      <c r="C61" s="134" t="inlineStr">
         <is>
           <t>• Grundeinstellungen zweispaltig (Einstellwerte teilweise nebeneinander).</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="135" t="n"/>
-      <c r="B58" s="135" t="n"/>
-      <c r="C58" s="134" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="135" t="n"/>
+      <c r="B62" s="135" t="n"/>
+      <c r="C62" s="134" t="inlineStr">
         <is>
           <t>• Verifikation: Diagramm rechts neben den Tabellen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="135" t="n"/>
-      <c r="B59" s="135" t="n"/>
-      <c r="C59" s="134" t="inlineStr">
-        <is>
-          <t>• Methodik: Formelzeichen links, Berechnungsschritte in zwei Spalten rechts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="135" t="n"/>
-      <c r="B60" s="135" t="n"/>
-      <c r="C60" s="134" t="inlineStr">
-        <is>
-          <t>• Konstanten: Tabellen teilweise nebeneinander.</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="136" t="n"/>
-      <c r="B61" s="136" t="n"/>
-      <c r="C61" s="134" t="inlineStr">
-        <is>
-          <t>• Auslegung: Spalte Zone mittig/schmaler, Raum-Nr. breiter; Verifikation-Korrekturfaktor vertikal mittig.</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="132" t="inlineStr">
-        <is>
-          <t>0.15</t>
-        </is>
-      </c>
-      <c r="B62" s="133" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="C62" s="134" t="inlineStr">
-        <is>
-          <t>• Deckblatt-Diagramm aus Excel-Zellen statt Bild – direkt in Excel bearbeitbar.</t>
         </is>
       </c>
     </row>
@@ -3000,50 +3001,42 @@
       <c r="B63" s="135" t="n"/>
       <c r="C63" s="134" t="inlineStr">
         <is>
-          <t>• Auslegung: Beispielräume mit gemischter Heizlast (≤ 50 W/m²); Formelzeichen in Zeile 5 ergänzt (Flächen u. a.).</t>
+          <t>• Methodik: Formelzeichen links, Berechnungsschritte in zwei Spalten rechts.</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="136" t="n"/>
-      <c r="B64" s="136" t="n"/>
+      <c r="A64" s="135" t="n"/>
+      <c r="B64" s="135" t="n"/>
       <c r="C64" s="134" t="inlineStr">
         <is>
-          <t>• Heizkreisverteiler: zusätzliche Spalte Spreizung [K].</t>
+          <t>• Konstanten: Tabellen teilweise nebeneinander.</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="132" t="inlineStr">
-        <is>
-          <t>0.14</t>
-        </is>
-      </c>
-      <c r="B65" s="133" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
+      <c r="A65" s="136" t="n"/>
+      <c r="B65" s="136" t="n"/>
       <c r="C65" s="134" t="inlineStr">
         <is>
-          <t>• Deckblatt als erstes Blatt: Übersichtsdiagramm Eingaben → Verarbeitung → Ergebnisse (inkl. Vereinfachungen).</t>
+          <t>• Auslegung: Spalte Zone mittig/schmaler, Raum-Nr. breiter; Verifikation-Korrekturfaktor vertikal mittig.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="132" t="inlineStr">
         <is>
-          <t>0.13</t>
+          <t>0.15</t>
         </is>
       </c>
       <c r="B66" s="133" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="C66" s="134" t="inlineStr">
         <is>
-          <t>• Strömungsbereich dreistufig: laminar (Re &lt; 2300), Übergangsbereich (2300–4000), turbulent (Re &gt; 4000).</t>
+          <t>• Deckblatt-Diagramm aus Excel-Zellen statt Bild – direkt in Excel bearbeitbar.</t>
         </is>
       </c>
     </row>
@@ -3052,51 +3045,59 @@
       <c r="B67" s="135" t="n"/>
       <c r="C67" s="134" t="inlineStr">
         <is>
+          <t>• Auslegung: Beispielräume mit gemischter Heizlast (≤ 50 W/m²); Formelzeichen in Zeile 5 ergänzt (Flächen u. a.).</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="136" t="n"/>
+      <c r="B68" s="136" t="n"/>
+      <c r="C68" s="134" t="inlineStr">
+        <is>
+          <t>• Heizkreisverteiler: zusätzliche Spalte Spreizung [K].</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="132" t="inlineStr">
+        <is>
+          <t>0.14</t>
+        </is>
+      </c>
+      <c r="B69" s="133" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="C69" s="134" t="inlineStr">
+        <is>
+          <t>• Deckblatt als erstes Blatt: Übersichtsdiagramm Eingaben → Verarbeitung → Ergebnisse (inkl. Vereinfachungen).</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="132" t="inlineStr">
+        <is>
+          <t>0.13</t>
+        </is>
+      </c>
+      <c r="B70" s="133" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C70" s="134" t="inlineStr">
+        <is>
+          <t>• Strömungsbereich dreistufig: laminar (Re &lt; 2300), Übergangsbereich (2300–4000), turbulent (Re &gt; 4000).</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="135" t="n"/>
+      <c r="B71" s="135" t="n"/>
+      <c r="C71" s="134" t="inlineStr">
+        <is>
           <t>• Spalte 'Strömungsbereich' ausgeblendet (für die Auslegung nicht relevant) und ohne Färbung.</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="135" t="n"/>
-      <c r="B68" s="135" t="n"/>
-      <c r="C68" s="134" t="inlineStr">
-        <is>
-          <t>• Auslegung schlanker: weitere Zwischenspalten standardmäßig ausgeblendet (jederzeit einblendbar).</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="135" t="n"/>
-      <c r="B69" s="135" t="n"/>
-      <c r="C69" s="134" t="inlineStr">
-        <is>
-          <t>• Verifikation: Korrekturfaktor kleiner dargestellt (passt nun vollständig in die Zelle).</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="136" t="n"/>
-      <c r="B70" s="136" t="n"/>
-      <c r="C70" s="134" t="inlineStr">
-        <is>
-          <t>• Changelog wieder ausführlich.</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="132" t="inlineStr">
-        <is>
-          <t>0.12</t>
-        </is>
-      </c>
-      <c r="B71" s="133" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="C71" s="134" t="inlineStr">
-        <is>
-          <t>• Grundeinstellungen: Bezeichnungen ausgeschrieben (keine Abkürzungen).</t>
         </is>
       </c>
     </row>
@@ -3105,7 +3106,7 @@
       <c r="B72" s="135" t="n"/>
       <c r="C72" s="134" t="inlineStr">
         <is>
-          <t>• Neue Spalte 'spez. Heizlast [W/m²]' (Heizlast bezogen auf die Raumfläche).</t>
+          <t>• Auslegung schlanker: weitere Zwischenspalten standardmäßig ausgeblendet (jederzeit einblendbar).</t>
         </is>
       </c>
     </row>
@@ -3114,42 +3115,42 @@
       <c r="B73" s="135" t="n"/>
       <c r="C73" s="134" t="inlineStr">
         <is>
-          <t>• Massenstrom/Geschwindigkeit/Druckverlust auf Basis min(Leistung; Heizlast) + Verlust nach unten (realer Betriebspunkt).</t>
+          <t>• Verifikation: Korrekturfaktor kleiner dargestellt (passt nun vollständig in die Zelle).</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="135" t="n"/>
-      <c r="B74" s="135" t="n"/>
+      <c r="A74" s="136" t="n"/>
+      <c r="B74" s="136" t="n"/>
       <c r="C74" s="134" t="inlineStr">
         <is>
-          <t>• Heizkreisverteiler zusätzlich mit Massenstrom [kg/h]; Zonen-Kürzel (AZ/RZ/BAD).</t>
+          <t>• Changelog wieder ausführlich.</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="136" t="n"/>
-      <c r="B75" s="136" t="n"/>
+      <c r="A75" s="132" t="inlineStr">
+        <is>
+          <t>0.12</t>
+        </is>
+      </c>
+      <c r="B75" s="133" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
       <c r="C75" s="134" t="inlineStr">
         <is>
-          <t>• Kapazität 200 Räume / 50 Verteiler; Auslegung A3 quer, übrige Blätter A4 hoch.</t>
+          <t>• Grundeinstellungen: Bezeichnungen ausgeschrieben (keine Abkürzungen).</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="132" t="inlineStr">
-        <is>
-          <t>0.11</t>
-        </is>
-      </c>
-      <c r="B76" s="133" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
+      <c r="A76" s="135" t="n"/>
+      <c r="B76" s="135" t="n"/>
       <c r="C76" s="134" t="inlineStr">
         <is>
-          <t>• Bugfixes: Hinweistext wurde als Formel interpretiert (Fehler 501); MAXIFS ersetzt (#NAME? in LibreOffice).</t>
+          <t>• Neue Spalte 'spez. Heizlast [W/m²]' (Heizlast bezogen auf die Raumfläche).</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3159,7 @@
       <c r="B77" s="135" t="n"/>
       <c r="C77" s="134" t="inlineStr">
         <is>
-          <t>• Verifikation: Korrekturfaktor prominent oben; Hersteller-q direkt neben q berechnet.</t>
+          <t>• Massenstrom/Geschwindigkeit/Druckverlust auf Basis min(Leistung; Heizlast) + Verlust nach unten (realer Betriebspunkt).</t>
         </is>
       </c>
     </row>
@@ -3167,7 +3168,7 @@
       <c r="B78" s="135" t="n"/>
       <c r="C78" s="134" t="inlineStr">
         <is>
-          <t>• Konstanten: alle Tabellen untereinander, mit Leerzeilen für weitere Einträge.</t>
+          <t>• Heizkreisverteiler zusätzlich mit Massenstrom [kg/h]; Zonen-Kürzel (AZ/RZ/BAD).</t>
         </is>
       </c>
     </row>
@@ -3176,14 +3177,14 @@
       <c r="B79" s="136" t="n"/>
       <c r="C79" s="134" t="inlineStr">
         <is>
-          <t>• Methodik: Variablen zuerst, dann Formeln mit Erklärung je Schritt; weitere Musterräume (Verwaltungsbau).</t>
+          <t>• Kapazität 200 Räume / 50 Verteiler; Auslegung A3 quer, übrige Blätter A4 hoch.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="132" t="inlineStr">
         <is>
-          <t>0.10</t>
+          <t>0.11</t>
         </is>
       </c>
       <c r="B80" s="133" t="inlineStr">
@@ -3193,7 +3194,7 @@
       </c>
       <c r="C80" s="134" t="inlineStr">
         <is>
-          <t>• Heizkreisverteiler-Liste und Verifikation ohne dynamische Array-Funktionen → läuft in Excel UND LibreOffice.</t>
+          <t>• Bugfixes: Hinweistext wurde als Formel interpretiert (Fehler 501); MAXIFS ersetzt (#NAME? in LibreOffice).</t>
         </is>
       </c>
     </row>
@@ -3202,42 +3203,42 @@
       <c r="B81" s="135" t="n"/>
       <c r="C81" s="134" t="inlineStr">
         <is>
-          <t>• Verifikation mit Liniendiagramm; Konstanten/Bibliotheken in eigenes Blatt ausgelagert.</t>
+          <t>• Verifikation: Korrekturfaktor prominent oben; Hersteller-q direkt neben q berechnet.</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="136" t="n"/>
-      <c r="B82" s="136" t="n"/>
+      <c r="A82" s="135" t="n"/>
+      <c r="B82" s="135" t="n"/>
       <c r="C82" s="134" t="inlineStr">
         <is>
-          <t>• Gewähltes Rohrsystem mit Außen-/Innendurchmesser, Wandstärke und Rauheit im Druckbereich.</t>
+          <t>• Konstanten: alle Tabellen untereinander, mit Leerzeilen für weitere Einträge.</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="132" t="inlineStr">
-        <is>
-          <t>0.9</t>
-        </is>
-      </c>
-      <c r="B83" s="133" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
+      <c r="A83" s="136" t="n"/>
+      <c r="B83" s="136" t="n"/>
       <c r="C83" s="134" t="inlineStr">
         <is>
-          <t>• Neues Blatt 'Heizkreisverteiler' (Leistung, max. Druckverlust, Volumenstrom je HKV).</t>
+          <t>• Methodik: Variablen zuerst, dann Formeln mit Erklärung je Schritt; weitere Musterräume (Verwaltungsbau).</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="135" t="n"/>
-      <c r="B84" s="135" t="n"/>
+      <c r="A84" s="132" t="inlineStr">
+        <is>
+          <t>0.10</t>
+        </is>
+      </c>
+      <c r="B84" s="133" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
       <c r="C84" s="134" t="inlineStr">
         <is>
-          <t>• Spaltenüberschriften der Auslegung dreizeilig (Name / Formelzeichen / Einheit).</t>
+          <t>• Heizkreisverteiler-Liste und Verifikation ohne dynamische Array-Funktionen → läuft in Excel UND LibreOffice.</t>
         </is>
       </c>
     </row>
@@ -3246,7 +3247,7 @@
       <c r="B85" s="135" t="n"/>
       <c r="C85" s="134" t="inlineStr">
         <is>
-          <t>• Korrekturfaktor f wird auf 'Verifikation' eingegeben (mit Vergleichsdiagramm).</t>
+          <t>• Verifikation mit Liniendiagramm; Konstanten/Bibliotheken in eigenes Blatt ausgelagert.</t>
         </is>
       </c>
     </row>
@@ -3255,14 +3256,14 @@
       <c r="B86" s="136" t="n"/>
       <c r="C86" s="134" t="inlineStr">
         <is>
-          <t>• Geschwindigkeits-Grenzwerte v_min/v_max als Grundeinstellung.</t>
+          <t>• Gewähltes Rohrsystem mit Außen-/Innendurchmesser, Wandstärke und Rauheit im Druckbereich.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="132" t="inlineStr">
         <is>
-          <t>0.8</t>
+          <t>0.9</t>
         </is>
       </c>
       <c r="B87" s="133" t="inlineStr">
@@ -3272,7 +3273,7 @@
       </c>
       <c r="C87" s="134" t="inlineStr">
         <is>
-          <t>• Grundeinstellungen für A3 quer optimiert (Einstellungen links, Tabellen rechts).</t>
+          <t>• Neues Blatt 'Heizkreisverteiler' (Leistung, max. Druckverlust, Volumenstrom je HKV).</t>
         </is>
       </c>
     </row>
@@ -3281,7 +3282,7 @@
       <c r="B88" s="135" t="n"/>
       <c r="C88" s="134" t="inlineStr">
         <is>
-          <t>• Auslegung passt auf eine Seite breit; Korrekturfaktor Heizleistung zur Kalibrierung ergänzt.</t>
+          <t>• Spaltenüberschriften der Auslegung dreizeilig (Name / Formelzeichen / Einheit).</t>
         </is>
       </c>
     </row>
@@ -3290,7 +3291,7 @@
       <c r="B89" s="135" t="n"/>
       <c r="C89" s="134" t="inlineStr">
         <is>
-          <t>• Wärmeabgabe nach unten berücksichtigt (Verlust + Gesamtleistung).</t>
+          <t>• Korrekturfaktor f wird auf 'Verifikation' eingegeben (mit Vergleichsdiagramm).</t>
         </is>
       </c>
     </row>
@@ -3299,14 +3300,14 @@
       <c r="B90" s="136" t="n"/>
       <c r="C90" s="134" t="inlineStr">
         <is>
-          <t>• Blätter umbenannt: Raumliste → Auslegung, Übersicht → Kontrolle; zusätzliche Kontrollen.</t>
+          <t>• Geschwindigkeits-Grenzwerte v_min/v_max als Grundeinstellung.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="132" t="inlineStr">
         <is>
-          <t>0.7</t>
+          <t>0.8</t>
         </is>
       </c>
       <c r="B91" s="133" t="inlineStr">
@@ -3316,7 +3317,7 @@
       </c>
       <c r="C91" s="134" t="inlineStr">
         <is>
-          <t>• Deckung-%-Spalte färbt nur noch gefüllte Zellen (leere bleiben farblos).</t>
+          <t>• Grundeinstellungen für A3 quer optimiert (Einstellungen links, Tabellen rechts).</t>
         </is>
       </c>
     </row>
@@ -3325,94 +3326,94 @@
       <c r="B92" s="135" t="n"/>
       <c r="C92" s="134" t="inlineStr">
         <is>
-          <t>• Neues Blatt 'Verifikation'; neue Spalte 'Strömungsbereich' (laminar/turbulent).</t>
+          <t>• Auslegung passt auf eine Seite breit; Korrekturfaktor Heizleistung zur Kalibrierung ergänzt.</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="136" t="n"/>
-      <c r="B93" s="136" t="n"/>
+      <c r="A93" s="135" t="n"/>
+      <c r="B93" s="135" t="n"/>
       <c r="C93" s="134" t="inlineStr">
         <is>
-          <t>• Alle Blätter im A3-Querformat; einheitlicher Kopf je Blatt.</t>
+          <t>• Wärmeabgabe nach unten berücksichtigt (Verlust + Gesamtleistung).</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="132" t="inlineStr">
-        <is>
-          <t>0.6</t>
-        </is>
-      </c>
-      <c r="B94" s="133" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
+      <c r="A94" s="136" t="n"/>
+      <c r="B94" s="136" t="n"/>
       <c r="C94" s="134" t="inlineStr">
         <is>
-          <t>• Bugfix: Zellfärbung (bedingte Formatierung) wird jetzt auch in Excel angezeigt – dxf-Füllfarbe mit voller Deckkraft.</t>
+          <t>• Blätter umbenannt: Raumliste → Auslegung, Übersicht → Kontrolle; zusätzliche Kontrollen.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="132" t="inlineStr">
         <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="B95" s="133" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="C95" s="134" t="inlineStr">
+        <is>
+          <t>• Deckung-%-Spalte färbt nur noch gefüllte Zellen (leere bleiben farblos).</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="135" t="n"/>
+      <c r="B96" s="135" t="n"/>
+      <c r="C96" s="134" t="inlineStr">
+        <is>
+          <t>• Neues Blatt 'Verifikation'; neue Spalte 'Strömungsbereich' (laminar/turbulent).</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="136" t="n"/>
+      <c r="B97" s="136" t="n"/>
+      <c r="C97" s="134" t="inlineStr">
+        <is>
+          <t>• Alle Blätter im A3-Querformat; einheitlicher Kopf je Blatt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="132" t="inlineStr">
+        <is>
+          <t>0.6</t>
+        </is>
+      </c>
+      <c r="B98" s="133" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="C98" s="134" t="inlineStr">
+        <is>
+          <t>• Bugfix: Zellfärbung (bedingte Formatierung) wird jetzt auch in Excel angezeigt – dxf-Füllfarbe mit voller Deckkraft.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="132" t="inlineStr">
+        <is>
           <t>0.5</t>
         </is>
       </c>
-      <c r="B95" s="133" t="inlineStr">
+      <c r="B99" s="133" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
-      <c r="C95" s="134" t="inlineStr">
+      <c r="C99" s="134" t="inlineStr">
         <is>
           <t>• Versionsnummer und Autor werden nur noch im Changelog angezeigt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="136" t="n"/>
-      <c r="B96" s="136" t="n"/>
-      <c r="C96" s="134" t="inlineStr">
-        <is>
-          <t>• Editierbares Bearbeiter-Kürzel rechts oben unter dem Logo (Grundeinstellungen, Auslegung, Kontrolle, HKV).</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="132" t="inlineStr">
-        <is>
-          <t>0.4</t>
-        </is>
-      </c>
-      <c r="B97" s="133" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="C97" s="134" t="inlineStr">
-        <is>
-          <t>• Status-Spalten entfernt – Bewertung erfolgt jetzt direkt als Zellfärbung (grün/rot).</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="135" t="n"/>
-      <c r="B98" s="135" t="n"/>
-      <c r="C98" s="134" t="inlineStr">
-        <is>
-          <t>• Methodik um die Formelzeichen-Legende erweitert.</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="135" t="n"/>
-      <c r="B99" s="135" t="n"/>
-      <c r="C99" s="134" t="inlineStr">
-        <is>
-          <t>• Heizkreisverteiler (HKV) als erste Spalte der Auslegung; Standardwert max. Druckverlust 15.000 Pa.</t>
         </is>
       </c>
     </row>
@@ -3421,14 +3422,14 @@
       <c r="B100" s="136" t="n"/>
       <c r="C100" s="134" t="inlineStr">
         <is>
-          <t>• Versionsschema 0.x eingeführt (1.0 erst nach Test); interner Autor (dh).</t>
+          <t>• Editierbares Bearbeiter-Kürzel rechts oben unter dem Logo (Grundeinstellungen, Auslegung, Kontrolle, HKV).</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="132" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="B101" s="133" t="inlineStr">
@@ -3438,7 +3439,7 @@
       </c>
       <c r="C101" s="134" t="inlineStr">
         <is>
-          <t>• Zonentypen (Aufenthalt/Rand/Bad) mit eigener zulässiger Oberflächentemperatur.</t>
+          <t>• Status-Spalten entfernt – Bewertung erfolgt jetzt direkt als Zellfärbung (grün/rot).</t>
         </is>
       </c>
     </row>
@@ -3447,7 +3448,7 @@
       <c r="B102" s="135" t="n"/>
       <c r="C102" s="134" t="inlineStr">
         <is>
-          <t>• Einheitlicher Kopf: Titel oben links, agn-Logo oben rechts, Projektkopf darunter.</t>
+          <t>• Methodik um die Formelzeichen-Legende erweitert.</t>
         </is>
       </c>
     </row>
@@ -3456,42 +3457,42 @@
       <c r="B103" s="135" t="n"/>
       <c r="C103" s="134" t="inlineStr">
         <is>
-          <t>• Oberflächentemperatur θF und Volumenstrom eingeblendet.</t>
+          <t>• Heizkreisverteiler (HKV) als erste Spalte der Auslegung; Standardwert max. Druckverlust 15.000 Pa.</t>
         </is>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="135" t="n"/>
-      <c r="B104" s="135" t="n"/>
+      <c r="A104" s="136" t="n"/>
+      <c r="B104" s="136" t="n"/>
       <c r="C104" s="134" t="inlineStr">
         <is>
-          <t>• Neue Spalten 'spez. Druckverlust [Pa/m]' und Eingabespalte 'Verteiler (Anbindung)'.</t>
+          <t>• Versionsschema 0.x eingeführt (1.0 erst nach Test); interner Autor (dh).</t>
         </is>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="136" t="n"/>
-      <c r="B105" s="136" t="n"/>
+      <c r="A105" s="132" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="B105" s="133" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
       <c r="C105" s="134" t="inlineStr">
         <is>
-          <t>• Warnung (rot), wenn die aktivierbare Fläche größer als die Raumfläche ist.</t>
+          <t>• Zonentypen (Aufenthalt/Rand/Bad) mit eigener zulässiger Oberflächentemperatur.</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="132" t="inlineStr">
-        <is>
-          <t>0.2</t>
-        </is>
-      </c>
-      <c r="B106" s="133" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
+      <c r="A106" s="135" t="n"/>
+      <c r="B106" s="135" t="n"/>
       <c r="C106" s="134" t="inlineStr">
         <is>
-          <t>• agn-Logo eingebunden und eigenes Changelog-Blatt ergänzt.</t>
+          <t>• Einheitlicher Kopf: Titel oben links, agn-Logo oben rechts, Projektkopf darunter.</t>
         </is>
       </c>
     </row>
@@ -3500,7 +3501,7 @@
       <c r="B107" s="135" t="n"/>
       <c r="C107" s="134" t="inlineStr">
         <is>
-          <t>• Zuschlag Einzelwiderstände (5 %) und fester Verteiler-Aufschlag (500 Pa je Kreis).</t>
+          <t>• Oberflächentemperatur θF und Volumenstrom eingeblendet.</t>
         </is>
       </c>
     </row>
@@ -3509,42 +3510,42 @@
       <c r="B108" s="135" t="n"/>
       <c r="C108" s="134" t="inlineStr">
         <is>
-          <t>• Einheiten als Zellformat; Projektnummer/Projektname erscheinen im Ausdruck.</t>
+          <t>• Neue Spalten 'spez. Druckverlust [Pa/m]' und Eingabespalte 'Verteiler (Anbindung)'.</t>
         </is>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="135" t="n"/>
-      <c r="B109" s="135" t="n"/>
+      <c r="A109" s="136" t="n"/>
+      <c r="B109" s="136" t="n"/>
       <c r="C109" s="134" t="inlineStr">
         <is>
-          <t>• Richtwert-Tabellen für R-Werte und Verlegeabstand-Faktoren; weitere Musterräume.</t>
+          <t>• Warnung (rot), wenn die aktivierbare Fläche größer als die Raumfläche ist.</t>
         </is>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="136" t="n"/>
-      <c r="B110" s="136" t="n"/>
+      <c r="A110" s="132" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="B110" s="133" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
       <c r="C110" s="134" t="inlineStr">
         <is>
-          <t>• Druckaufbereitung für DIN A4.</t>
+          <t>• agn-Logo eingebunden und eigenes Changelog-Blatt ergänzt.</t>
         </is>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="132" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="B111" s="133" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
+      <c r="A111" s="135" t="n"/>
+      <c r="B111" s="135" t="n"/>
       <c r="C111" s="134" t="inlineStr">
         <is>
-          <t>• Ersterstellung mit den Blättern Grundeinstellungen, Raumliste, Übersicht und Methodik.</t>
+          <t>• Zuschlag Einzelwiderstände (5 %) und fester Verteiler-Aufschlag (500 Pa je Kreis).</t>
         </is>
       </c>
     </row>
@@ -3553,7 +3554,7 @@
       <c r="B112" s="135" t="n"/>
       <c r="C112" s="134" t="inlineStr">
         <is>
-          <t>• Heizleistung über die logarithmische Übertemperatur (q = η · K_H · ΔθH).</t>
+          <t>• Einheiten als Zellformat; Projektnummer/Projektname erscheinen im Ausdruck.</t>
         </is>
       </c>
     </row>
@@ -3562,23 +3563,67 @@
       <c r="B113" s="135" t="n"/>
       <c r="C113" s="134" t="inlineStr">
         <is>
+          <t>• Richtwert-Tabellen für R-Werte und Verlegeabstand-Faktoren; weitere Musterräume.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="136" t="n"/>
+      <c r="B114" s="136" t="n"/>
+      <c r="C114" s="134" t="inlineStr">
+        <is>
+          <t>• Druckaufbereitung für DIN A4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="132" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="B115" s="133" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="C115" s="134" t="inlineStr">
+        <is>
+          <t>• Ersterstellung mit den Blättern Grundeinstellungen, Raumliste, Übersicht und Methodik.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="135" t="n"/>
+      <c r="B116" s="135" t="n"/>
+      <c r="C116" s="134" t="inlineStr">
+        <is>
+          <t>• Heizleistung über die logarithmische Übertemperatur (q = η · K_H · ΔθH).</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="135" t="n"/>
+      <c r="B117" s="135" t="n"/>
+      <c r="C117" s="134" t="inlineStr">
+        <is>
           <t>• Druckverlustberechnung nach Darcy-Weisbach.</t>
         </is>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" s="135" t="n"/>
-      <c r="B114" s="135" t="n"/>
-      <c r="C114" s="134" t="inlineStr">
+    <row r="118">
+      <c r="A118" s="135" t="n"/>
+      <c r="B118" s="135" t="n"/>
+      <c r="C118" s="134" t="inlineStr">
         <is>
           <t>• Editierbare Rohrbibliothek und Verlegeabstand-Faktoren.</t>
         </is>
       </c>
     </row>
-    <row r="115">
-      <c r="A115" s="136" t="n"/>
-      <c r="B115" s="136" t="n"/>
-      <c r="C115" s="134" t="inlineStr">
+    <row r="119">
+      <c r="A119" s="136" t="n"/>
+      <c r="B119" s="136" t="n"/>
+      <c r="C119" s="134" t="inlineStr">
         <is>
           <t>• Prüfungen: Oberflächentemperatur, Heizlastdeckung, Kreislänge, Druckverlust.</t>
         </is>
@@ -3586,67 +3631,69 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
-  <mergeCells count="60">
-    <mergeCell ref="A48:A51"/>
-    <mergeCell ref="B97:B100"/>
-    <mergeCell ref="A101:A105"/>
-    <mergeCell ref="A21:A25"/>
-    <mergeCell ref="A26:A28"/>
-    <mergeCell ref="B29:B33"/>
-    <mergeCell ref="B52:B53"/>
-    <mergeCell ref="B12:B15"/>
-    <mergeCell ref="A71:A75"/>
-    <mergeCell ref="A91:A93"/>
-    <mergeCell ref="A54:A55"/>
+  <mergeCells count="62">
+    <mergeCell ref="B49:B51"/>
+    <mergeCell ref="A105:A109"/>
+    <mergeCell ref="A20:A22"/>
+    <mergeCell ref="B30:B32"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="A33:A37"/>
+    <mergeCell ref="A60:A65"/>
     <mergeCell ref="A87:A90"/>
-    <mergeCell ref="B80:B82"/>
-    <mergeCell ref="A62:A64"/>
-    <mergeCell ref="B45:B47"/>
-    <mergeCell ref="A106:A110"/>
-    <mergeCell ref="B56:B61"/>
-    <mergeCell ref="A29:A33"/>
-    <mergeCell ref="B26:B28"/>
-    <mergeCell ref="A12:A15"/>
-    <mergeCell ref="A37:A38"/>
-    <mergeCell ref="A95:A96"/>
-    <mergeCell ref="B16:B18"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="A9:A11"/>
-    <mergeCell ref="B37:B38"/>
-    <mergeCell ref="B48:B51"/>
-    <mergeCell ref="A76:A79"/>
-    <mergeCell ref="A111:A115"/>
-    <mergeCell ref="A39:A41"/>
-    <mergeCell ref="A45:A47"/>
-    <mergeCell ref="B62:B64"/>
-    <mergeCell ref="A56:A61"/>
-    <mergeCell ref="B66:B70"/>
-    <mergeCell ref="B91:B93"/>
-    <mergeCell ref="B106:B110"/>
+    <mergeCell ref="B84:B86"/>
+    <mergeCell ref="A16:A19"/>
+    <mergeCell ref="B58:B59"/>
+    <mergeCell ref="A13:A15"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="B39:B40"/>
+    <mergeCell ref="B52:B55"/>
+    <mergeCell ref="A115:A119"/>
+    <mergeCell ref="A43:A45"/>
+    <mergeCell ref="A56:A57"/>
+    <mergeCell ref="B33:B37"/>
+    <mergeCell ref="B20:B22"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="B95:B97"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="B66:B68"/>
+    <mergeCell ref="A99:A100"/>
+    <mergeCell ref="B70:B74"/>
+    <mergeCell ref="A80:A83"/>
+    <mergeCell ref="A49:A51"/>
+    <mergeCell ref="B101:B104"/>
+    <mergeCell ref="B110:B114"/>
+    <mergeCell ref="A30:A32"/>
+    <mergeCell ref="A101:A104"/>
+    <mergeCell ref="B115:B119"/>
+    <mergeCell ref="B43:B45"/>
+    <mergeCell ref="B25:B29"/>
+    <mergeCell ref="B60:B65"/>
+    <mergeCell ref="A84:A86"/>
     <mergeCell ref="B87:B90"/>
-    <mergeCell ref="B71:B75"/>
-    <mergeCell ref="B83:B86"/>
-    <mergeCell ref="B6:B8"/>
-    <mergeCell ref="A97:A100"/>
-    <mergeCell ref="B95:B96"/>
-    <mergeCell ref="A6:A8"/>
-    <mergeCell ref="B42:B44"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="B54:B55"/>
-    <mergeCell ref="B111:B115"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="B101:B105"/>
-    <mergeCell ref="B39:B41"/>
-    <mergeCell ref="B21:B25"/>
-    <mergeCell ref="A66:A70"/>
-    <mergeCell ref="A52:A53"/>
-    <mergeCell ref="A16:A18"/>
-    <mergeCell ref="A83:A86"/>
-    <mergeCell ref="B9:B11"/>
-    <mergeCell ref="A80:A82"/>
-    <mergeCell ref="B76:B79"/>
-    <mergeCell ref="A42:A44"/>
-    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="A91:A94"/>
+    <mergeCell ref="B6:B9"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A75:A79"/>
+    <mergeCell ref="B99:B100"/>
+    <mergeCell ref="B46:B48"/>
+    <mergeCell ref="B75:B79"/>
+    <mergeCell ref="B80:B83"/>
+    <mergeCell ref="A110:A114"/>
+    <mergeCell ref="A66:A68"/>
+    <mergeCell ref="A70:A74"/>
+    <mergeCell ref="B105:B109"/>
+    <mergeCell ref="B10:B12"/>
+    <mergeCell ref="A25:A29"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="B56:B57"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="A46:A48"/>
+    <mergeCell ref="B91:B94"/>
+    <mergeCell ref="A58:A59"/>
+    <mergeCell ref="A95:A97"/>
+    <mergeCell ref="B16:B19"/>
+    <mergeCell ref="A52:A55"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -4998,7 +5045,7 @@
             <rPr>
               <rFont val="Arial"/>
               <b val="1"/>
-              <color rgb="001A1A1A"/>
+              <color rgb="00000000"/>
               <sz val="13"/>
               <vertAlign val="subscript"/>
             </rPr>
@@ -5025,7 +5072,7 @@
             <rPr>
               <rFont val="Arial"/>
               <b val="1"/>
-              <color rgb="001A1A1A"/>
+              <color rgb="00000000"/>
               <sz val="13"/>
               <vertAlign val="subscript"/>
             </rPr>
@@ -5042,7 +5089,7 @@
             <rPr>
               <rFont val="Arial"/>
               <b val="1"/>
-              <color rgb="001A1A1A"/>
+              <color rgb="00000000"/>
               <sz val="13"/>
               <vertAlign val="subscript"/>
             </rPr>
@@ -5059,7 +5106,7 @@
             <rPr>
               <rFont val="Arial"/>
               <b val="1"/>
-              <color rgb="001A1A1A"/>
+              <color rgb="00000000"/>
               <sz val="13"/>
               <vertAlign val="subscript"/>
             </rPr>
@@ -5086,7 +5133,7 @@
             <rPr>
               <rFont val="Arial"/>
               <b val="1"/>
-              <color rgb="001A1A1A"/>
+              <color rgb="00000000"/>
               <sz val="13"/>
               <vertAlign val="subscript"/>
             </rPr>
@@ -5109,7 +5156,7 @@
             <rPr>
               <rFont val="Arial"/>
               <b val="1"/>
-              <color rgb="001A1A1A"/>
+              <color rgb="00000000"/>
               <sz val="13"/>
               <vertAlign val="subscript"/>
             </rPr>
@@ -5146,7 +5193,7 @@
             <rPr>
               <rFont val="Arial"/>
               <b val="1"/>
-              <color rgb="001A1A1A"/>
+              <color rgb="00000000"/>
               <sz val="13"/>
               <vertAlign val="subscript"/>
             </rPr>
@@ -5169,7 +5216,7 @@
             <rPr>
               <rFont val="Arial"/>
               <b val="1"/>
-              <color rgb="001A1A1A"/>
+              <color rgb="00000000"/>
               <sz val="13"/>
               <vertAlign val="subscript"/>
             </rPr>
@@ -5186,7 +5233,7 @@
             <rPr>
               <rFont val="Arial"/>
               <b val="1"/>
-              <color rgb="001A1A1A"/>
+              <color rgb="00000000"/>
               <sz val="13"/>
               <vertAlign val="subscript"/>
             </rPr>
@@ -5203,7 +5250,7 @@
             <rPr>
               <rFont val="Arial"/>
               <b val="1"/>
-              <color rgb="001A1A1A"/>
+              <color rgb="00000000"/>
               <sz val="13"/>
               <vertAlign val="subscript"/>
             </rPr>
@@ -5220,7 +5267,7 @@
             <rPr>
               <rFont val="Arial"/>
               <b val="1"/>
-              <color rgb="001A1A1A"/>
+              <color rgb="00000000"/>
               <sz val="13"/>
               <vertAlign val="subscript"/>
             </rPr>
@@ -5237,7 +5284,7 @@
             <rPr>
               <rFont val="Arial"/>
               <b val="1"/>
-              <color rgb="001A1A1A"/>
+              <color rgb="00000000"/>
               <sz val="13"/>
               <vertAlign val="subscript"/>
             </rPr>
@@ -5254,7 +5301,7 @@
             <rPr>
               <rFont val="Arial"/>
               <b val="1"/>
-              <color rgb="001A1A1A"/>
+              <color rgb="00000000"/>
               <sz val="13"/>
               <vertAlign val="subscript"/>
             </rPr>
@@ -5297,7 +5344,7 @@
             <rPr>
               <rFont val="Arial"/>
               <b val="1"/>
-              <color rgb="001A1A1A"/>
+              <color rgb="00000000"/>
               <sz val="13"/>
               <vertAlign val="subscript"/>
             </rPr>
@@ -28576,7 +28623,8 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
+  <autoFilter ref="A6:AK206"/>
   <mergeCells count="1">
     <mergeCell ref="AB2:AK2"/>
   </mergeCells>
@@ -28641,6 +28689,16 @@
       <formula>AND($H7&lt;&gt;"",$D7&lt;&gt;"",$H7&gt;$D7)</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="A7:A206 B7:B206 C7:C206 D7:D206 E7:E206 F7:F206 G7:G206 I7:I206 J7:J206 K7:K206 L7:L206 M7:M206">
+    <cfRule type="expression" priority="16" dxfId="2">
+      <formula>AND($B7&lt;&gt;"",MOD(SUBTOTAL(103,$B$7:$B7),2)=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N7:N206 O7:O206 P7:P206 Q7:Q206 S7:S206 U7:U206 W7:W206 X7:X206 Y7:Y206 Z7:Z206 AA7:AA206 AC7:AC206 AF7:AF206 AG7:AG206 AH7:AH206 AI7:AI206 AJ7:AJ206">
+    <cfRule type="expression" priority="17" dxfId="3">
+      <formula>AND($B7&lt;&gt;"",MOD(SUBTOTAL(103,$B$7:$B7),2)=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation sqref="M7:M206" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>='Konstanten'!$E$6:$E$13</formula1>
@@ -29066,50 +29124,50 @@
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
   <conditionalFormatting sqref="B20">
-    <cfRule type="expression" priority="1" dxfId="2">
+    <cfRule type="expression" priority="1" dxfId="4">
       <formula>$B$20&gt;0</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="3">
+    <cfRule type="expression" priority="2" dxfId="5">
       <formula>$B$20=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B21">
-    <cfRule type="expression" priority="3" dxfId="2">
+    <cfRule type="expression" priority="3" dxfId="4">
       <formula>$B$21&gt;0</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" dxfId="3">
+    <cfRule type="expression" priority="4" dxfId="5">
       <formula>$B$21=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22">
-    <cfRule type="expression" priority="5" dxfId="2">
+    <cfRule type="expression" priority="5" dxfId="4">
       <formula>$B$22&gt;0</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" dxfId="3">
+    <cfRule type="expression" priority="6" dxfId="5">
       <formula>$B$22=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B23">
-    <cfRule type="expression" priority="7" dxfId="2">
+    <cfRule type="expression" priority="7" dxfId="4">
       <formula>$B$23&gt;0</formula>
     </cfRule>
-    <cfRule type="expression" priority="8" dxfId="3">
+    <cfRule type="expression" priority="8" dxfId="5">
       <formula>$B$23=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B24">
-    <cfRule type="expression" priority="9" dxfId="2">
+    <cfRule type="expression" priority="9" dxfId="4">
       <formula>$B$24&gt;0</formula>
     </cfRule>
-    <cfRule type="expression" priority="10" dxfId="3">
+    <cfRule type="expression" priority="10" dxfId="5">
       <formula>$B$24=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B25">
-    <cfRule type="expression" priority="11" dxfId="2">
+    <cfRule type="expression" priority="11" dxfId="4">
       <formula>$B$25&gt;0</formula>
     </cfRule>
-    <cfRule type="expression" priority="12" dxfId="3">
+    <cfRule type="expression" priority="12" dxfId="5">
       <formula>$B$25=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -31919,18 +31977,18 @@
     <mergeCell ref="A21:G21"/>
   </mergeCells>
   <conditionalFormatting sqref="I9:I20">
-    <cfRule type="expression" priority="1" dxfId="2">
+    <cfRule type="expression" priority="1" dxfId="4">
       <formula>AND($I9&lt;&gt;"",ABS($I9)&gt;0.1)</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="3">
+    <cfRule type="expression" priority="2" dxfId="5">
       <formula>AND($I9&lt;&gt;"",ABS($I9)&lt;=0.1)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I21">
-    <cfRule type="expression" priority="3" dxfId="2">
+    <cfRule type="expression" priority="3" dxfId="4">
       <formula>AND($I21&lt;&gt;"",ABS($I21)&gt;0.03)</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" dxfId="3">
+    <cfRule type="expression" priority="4" dxfId="5">
       <formula>AND($I21&lt;&gt;"",ABS($I21)&lt;=0.03)</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>